<commit_message>
Recalcul automatique de la colonne Mention pour les anciennes interventions
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_CDF_EFK.xlsx
+++ b/Objets_parlementaires_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="650" uniqueCount="650">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="649">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -573,9 +573,6 @@
   </si>
   <si>
     <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20253835</t>
-  </si>
-  <si>
-    <t xml:space="preserve">À recalculer</t>
   </si>
   <si>
     <t xml:space="preserve">25.3845</t>
@@ -3296,7 +3293,7 @@
         <v>186</v>
       </c>
       <c r="L26" t="s">
-        <v>187</v>
+        <v>22</v>
       </c>
     </row>
     <row r="27">
@@ -3304,7 +3301,7 @@
         <v>20253845</v>
       </c>
       <c r="B27" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C27" t="s">
         <v>32</v>
@@ -3319,22 +3316,22 @@
         <v>16</v>
       </c>
       <c r="G27" t="s">
+        <v>188</v>
+      </c>
+      <c r="H27" t="s">
         <v>189</v>
-      </c>
-      <c r="H27" t="s">
-        <v>190</v>
       </c>
       <c r="I27" t="s">
         <v>68</v>
       </c>
       <c r="J27" t="s">
+        <v>190</v>
+      </c>
+      <c r="K27" t="s">
         <v>191</v>
       </c>
-      <c r="K27" t="s">
-        <v>192</v>
-      </c>
       <c r="L27" t="s">
-        <v>187</v>
+        <v>22</v>
       </c>
     </row>
     <row r="28">
@@ -3342,13 +3339,13 @@
         <v>20253855</v>
       </c>
       <c r="B28" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C28" t="s">
         <v>13</v>
       </c>
       <c r="D28" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E28" t="s">
         <v>182</v>
@@ -3366,13 +3363,13 @@
         <v>145</v>
       </c>
       <c r="J28" t="s">
+        <v>194</v>
+      </c>
+      <c r="K28" t="s">
         <v>195</v>
       </c>
-      <c r="K28" t="s">
-        <v>196</v>
-      </c>
       <c r="L28" t="s">
-        <v>187</v>
+        <v>22</v>
       </c>
     </row>
     <row r="29">
@@ -3380,13 +3377,13 @@
         <v>20253880</v>
       </c>
       <c r="B29" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C29" t="s">
         <v>32</v>
       </c>
       <c r="D29" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E29" t="s">
         <v>182</v>
@@ -3395,22 +3392,22 @@
         <v>16</v>
       </c>
       <c r="G29" t="s">
+        <v>198</v>
+      </c>
+      <c r="H29" t="s">
         <v>199</v>
-      </c>
-      <c r="H29" t="s">
-        <v>200</v>
       </c>
       <c r="I29" t="s">
         <v>68</v>
       </c>
       <c r="J29" t="s">
+        <v>200</v>
+      </c>
+      <c r="K29" t="s">
         <v>201</v>
       </c>
-      <c r="K29" t="s">
-        <v>202</v>
-      </c>
       <c r="L29" t="s">
-        <v>187</v>
+        <v>22</v>
       </c>
     </row>
     <row r="30">
@@ -3418,13 +3415,13 @@
         <v>20253892</v>
       </c>
       <c r="B30" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C30" t="s">
         <v>32</v>
       </c>
       <c r="D30" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="E30" t="s">
         <v>182</v>
@@ -3433,22 +3430,22 @@
         <v>16</v>
       </c>
       <c r="G30" t="s">
+        <v>204</v>
+      </c>
+      <c r="H30" t="s">
         <v>205</v>
-      </c>
-      <c r="H30" t="s">
-        <v>206</v>
       </c>
       <c r="I30" t="s">
         <v>68</v>
       </c>
       <c r="J30" t="s">
+        <v>206</v>
+      </c>
+      <c r="K30" t="s">
         <v>207</v>
       </c>
-      <c r="K30" t="s">
-        <v>208</v>
-      </c>
       <c r="L30" t="s">
-        <v>187</v>
+        <v>22</v>
       </c>
     </row>
     <row r="31">
@@ -3456,13 +3453,13 @@
         <v>20253893</v>
       </c>
       <c r="B31" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C31" t="s">
         <v>63</v>
       </c>
       <c r="D31" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E31" t="s">
         <v>182</v>
@@ -3471,22 +3468,22 @@
         <v>16</v>
       </c>
       <c r="G31" t="s">
+        <v>210</v>
+      </c>
+      <c r="H31" t="s">
         <v>211</v>
-      </c>
-      <c r="H31" t="s">
-        <v>212</v>
       </c>
       <c r="I31" t="s">
         <v>68</v>
       </c>
       <c r="J31" t="s">
+        <v>212</v>
+      </c>
+      <c r="K31" t="s">
         <v>213</v>
       </c>
-      <c r="K31" t="s">
-        <v>214</v>
-      </c>
       <c r="L31" t="s">
-        <v>187</v>
+        <v>54</v>
       </c>
     </row>
     <row r="32">
@@ -3494,37 +3491,37 @@
         <v>20253730</v>
       </c>
       <c r="B32" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C32" t="s">
         <v>13</v>
       </c>
       <c r="D32" t="s">
+        <v>215</v>
+      </c>
+      <c r="E32" t="s">
         <v>216</v>
       </c>
-      <c r="E32" t="s">
+      <c r="F32" t="s">
+        <v>16</v>
+      </c>
+      <c r="G32" t="s">
         <v>217</v>
       </c>
-      <c r="F32" t="s">
-        <v>16</v>
-      </c>
-      <c r="G32" t="s">
+      <c r="H32" t="s">
         <v>218</v>
-      </c>
-      <c r="H32" t="s">
-        <v>219</v>
       </c>
       <c r="I32" t="s">
         <v>68</v>
       </c>
       <c r="J32" t="s">
+        <v>219</v>
+      </c>
+      <c r="K32" t="s">
         <v>220</v>
       </c>
-      <c r="K32" t="s">
-        <v>221</v>
-      </c>
       <c r="L32" t="s">
-        <v>187</v>
+        <v>47</v>
       </c>
     </row>
     <row r="33">
@@ -3532,37 +3529,37 @@
         <v>20253630</v>
       </c>
       <c r="B33" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C33" t="s">
         <v>32</v>
       </c>
       <c r="D33" t="s">
+        <v>222</v>
+      </c>
+      <c r="E33" t="s">
         <v>223</v>
-      </c>
-      <c r="E33" t="s">
-        <v>224</v>
       </c>
       <c r="F33" t="s">
         <v>26</v>
       </c>
       <c r="G33" t="s">
+        <v>224</v>
+      </c>
+      <c r="H33" t="s">
         <v>225</v>
-      </c>
-      <c r="H33" t="s">
-        <v>226</v>
       </c>
       <c r="I33" t="s">
         <v>44</v>
       </c>
       <c r="J33" t="s">
+        <v>226</v>
+      </c>
+      <c r="K33" t="s">
         <v>227</v>
       </c>
-      <c r="K33" t="s">
-        <v>228</v>
-      </c>
       <c r="L33" t="s">
-        <v>187</v>
+        <v>22</v>
       </c>
     </row>
     <row r="34">
@@ -3570,37 +3567,37 @@
         <v>20253637</v>
       </c>
       <c r="B34" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C34" t="s">
         <v>13</v>
       </c>
       <c r="D34" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E34" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="F34" t="s">
         <v>26</v>
       </c>
       <c r="G34" t="s">
+        <v>230</v>
+      </c>
+      <c r="H34" t="s">
         <v>231</v>
       </c>
-      <c r="H34" t="s">
+      <c r="I34" t="s">
         <v>232</v>
       </c>
-      <c r="I34" t="s">
+      <c r="J34" t="s">
         <v>233</v>
       </c>
-      <c r="J34" t="s">
+      <c r="K34" t="s">
         <v>234</v>
       </c>
-      <c r="K34" t="s">
-        <v>235</v>
-      </c>
       <c r="L34" t="s">
-        <v>187</v>
+        <v>47</v>
       </c>
     </row>
     <row r="35">
@@ -3608,37 +3605,37 @@
         <v>20257355</v>
       </c>
       <c r="B35" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C35" t="s">
         <v>39</v>
       </c>
       <c r="D35" t="s">
+        <v>236</v>
+      </c>
+      <c r="E35" t="s">
         <v>237</v>
       </c>
-      <c r="E35" t="s">
+      <c r="F35" t="s">
+        <v>16</v>
+      </c>
+      <c r="G35" t="s">
         <v>238</v>
       </c>
-      <c r="F35" t="s">
-        <v>16</v>
-      </c>
-      <c r="G35" t="s">
+      <c r="H35" t="s">
         <v>239</v>
-      </c>
-      <c r="H35" t="s">
-        <v>240</v>
       </c>
       <c r="I35" t="s">
         <v>44</v>
       </c>
       <c r="J35" t="s">
+        <v>240</v>
+      </c>
+      <c r="K35" t="s">
         <v>241</v>
       </c>
-      <c r="K35" t="s">
-        <v>242</v>
-      </c>
       <c r="L35" t="s">
-        <v>187</v>
+        <v>47</v>
       </c>
     </row>
     <row r="36">
@@ -3646,37 +3643,37 @@
         <v>20257419</v>
       </c>
       <c r="B36" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C36" t="s">
         <v>39</v>
       </c>
       <c r="D36" t="s">
+        <v>243</v>
+      </c>
+      <c r="E36" t="s">
+        <v>237</v>
+      </c>
+      <c r="F36" t="s">
+        <v>16</v>
+      </c>
+      <c r="G36" t="s">
         <v>244</v>
       </c>
-      <c r="E36" t="s">
-        <v>238</v>
-      </c>
-      <c r="F36" t="s">
-        <v>16</v>
-      </c>
-      <c r="G36" t="s">
+      <c r="H36" t="s">
         <v>245</v>
-      </c>
-      <c r="H36" t="s">
-        <v>246</v>
       </c>
       <c r="I36" t="s">
         <v>44</v>
       </c>
       <c r="J36" t="s">
+        <v>246</v>
+      </c>
+      <c r="K36" t="s">
         <v>247</v>
       </c>
-      <c r="K36" t="s">
-        <v>248</v>
-      </c>
       <c r="L36" t="s">
-        <v>187</v>
+        <v>47</v>
       </c>
     </row>
     <row r="37">
@@ -3684,37 +3681,37 @@
         <v>20253479</v>
       </c>
       <c r="B37" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C37" t="s">
         <v>32</v>
       </c>
       <c r="D37" t="s">
+        <v>249</v>
+      </c>
+      <c r="E37" t="s">
         <v>250</v>
       </c>
-      <c r="E37" t="s">
+      <c r="F37" t="s">
+        <v>16</v>
+      </c>
+      <c r="G37" t="s">
         <v>251</v>
       </c>
-      <c r="F37" t="s">
-        <v>16</v>
-      </c>
-      <c r="G37" t="s">
+      <c r="H37" t="s">
         <v>252</v>
-      </c>
-      <c r="H37" t="s">
-        <v>253</v>
       </c>
       <c r="I37" t="s">
         <v>68</v>
       </c>
       <c r="J37" t="s">
+        <v>253</v>
+      </c>
+      <c r="K37" t="s">
         <v>254</v>
       </c>
-      <c r="K37" t="s">
-        <v>255</v>
-      </c>
       <c r="L37" t="s">
-        <v>187</v>
+        <v>22</v>
       </c>
     </row>
     <row r="38">
@@ -3722,37 +3719,37 @@
         <v>20253444</v>
       </c>
       <c r="B38" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C38" t="s">
         <v>13</v>
       </c>
       <c r="D38" t="s">
+        <v>256</v>
+      </c>
+      <c r="E38" t="s">
         <v>257</v>
       </c>
-      <c r="E38" t="s">
+      <c r="F38" t="s">
+        <v>16</v>
+      </c>
+      <c r="G38" t="s">
         <v>258</v>
       </c>
-      <c r="F38" t="s">
-        <v>16</v>
-      </c>
-      <c r="G38" t="s">
+      <c r="H38" t="s">
         <v>259</v>
-      </c>
-      <c r="H38" t="s">
-        <v>260</v>
       </c>
       <c r="I38" t="s">
         <v>68</v>
       </c>
       <c r="J38" t="s">
+        <v>260</v>
+      </c>
+      <c r="K38" t="s">
         <v>261</v>
       </c>
-      <c r="K38" t="s">
-        <v>262</v>
-      </c>
       <c r="L38" t="s">
-        <v>187</v>
+        <v>54</v>
       </c>
     </row>
     <row r="39">
@@ -3760,35 +3757,35 @@
         <v>20253425</v>
       </c>
       <c r="B39" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C39" t="s">
         <v>13</v>
       </c>
       <c r="D39"/>
       <c r="E39" t="s">
+        <v>263</v>
+      </c>
+      <c r="F39" t="s">
+        <v>16</v>
+      </c>
+      <c r="G39" t="s">
         <v>264</v>
       </c>
-      <c r="F39" t="s">
-        <v>16</v>
-      </c>
-      <c r="G39" t="s">
+      <c r="H39" t="s">
         <v>265</v>
-      </c>
-      <c r="H39" t="s">
-        <v>266</v>
       </c>
       <c r="I39" t="s">
         <v>68</v>
       </c>
       <c r="J39" t="s">
+        <v>266</v>
+      </c>
+      <c r="K39" t="s">
         <v>267</v>
       </c>
-      <c r="K39" t="s">
-        <v>268</v>
-      </c>
       <c r="L39" t="s">
-        <v>187</v>
+        <v>22</v>
       </c>
     </row>
     <row r="40">
@@ -3796,7 +3793,7 @@
         <v>20253309</v>
       </c>
       <c r="B40" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C40" t="s">
         <v>13</v>
@@ -3805,28 +3802,28 @@
         <v>124</v>
       </c>
       <c r="E40" t="s">
+        <v>269</v>
+      </c>
+      <c r="F40" t="s">
+        <v>16</v>
+      </c>
+      <c r="G40" t="s">
         <v>270</v>
       </c>
-      <c r="F40" t="s">
-        <v>16</v>
-      </c>
-      <c r="G40" t="s">
+      <c r="H40" t="s">
         <v>271</v>
-      </c>
-      <c r="H40" t="s">
-        <v>272</v>
       </c>
       <c r="I40" t="s">
         <v>68</v>
       </c>
       <c r="J40" t="s">
+        <v>272</v>
+      </c>
+      <c r="K40" t="s">
         <v>273</v>
       </c>
-      <c r="K40" t="s">
-        <v>274</v>
-      </c>
       <c r="L40" t="s">
-        <v>187</v>
+        <v>22</v>
       </c>
     </row>
     <row r="41">
@@ -3834,37 +3831,37 @@
         <v>20253399</v>
       </c>
       <c r="B41" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C41" t="s">
         <v>32</v>
       </c>
       <c r="D41" t="s">
+        <v>275</v>
+      </c>
+      <c r="E41" t="s">
+        <v>269</v>
+      </c>
+      <c r="F41" t="s">
+        <v>16</v>
+      </c>
+      <c r="G41" t="s">
         <v>276</v>
       </c>
-      <c r="E41" t="s">
-        <v>270</v>
-      </c>
-      <c r="F41" t="s">
-        <v>16</v>
-      </c>
-      <c r="G41" t="s">
+      <c r="H41" t="s">
         <v>277</v>
-      </c>
-      <c r="H41" t="s">
-        <v>278</v>
       </c>
       <c r="I41" t="s">
         <v>68</v>
       </c>
       <c r="J41" t="s">
+        <v>278</v>
+      </c>
+      <c r="K41" t="s">
         <v>279</v>
       </c>
-      <c r="K41" t="s">
-        <v>280</v>
-      </c>
       <c r="L41" t="s">
-        <v>187</v>
+        <v>54</v>
       </c>
     </row>
     <row r="42">
@@ -3872,37 +3869,37 @@
         <v>20253404</v>
       </c>
       <c r="B42" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C42" t="s">
         <v>13</v>
       </c>
       <c r="D42" t="s">
+        <v>281</v>
+      </c>
+      <c r="E42" t="s">
+        <v>269</v>
+      </c>
+      <c r="F42" t="s">
+        <v>16</v>
+      </c>
+      <c r="G42" t="s">
         <v>282</v>
       </c>
-      <c r="E42" t="s">
-        <v>270</v>
-      </c>
-      <c r="F42" t="s">
-        <v>16</v>
-      </c>
-      <c r="G42" t="s">
+      <c r="H42" t="s">
         <v>283</v>
-      </c>
-      <c r="H42" t="s">
-        <v>284</v>
       </c>
       <c r="I42" t="s">
         <v>68</v>
       </c>
       <c r="J42" t="s">
+        <v>284</v>
+      </c>
+      <c r="K42" t="s">
         <v>285</v>
       </c>
-      <c r="K42" t="s">
-        <v>286</v>
-      </c>
       <c r="L42" t="s">
-        <v>187</v>
+        <v>47</v>
       </c>
     </row>
     <row r="43">
@@ -3910,37 +3907,37 @@
         <v>20253417</v>
       </c>
       <c r="B43" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C43" t="s">
         <v>13</v>
       </c>
       <c r="D43" t="s">
+        <v>287</v>
+      </c>
+      <c r="E43" t="s">
+        <v>269</v>
+      </c>
+      <c r="F43" t="s">
+        <v>16</v>
+      </c>
+      <c r="G43" t="s">
         <v>288</v>
       </c>
-      <c r="E43" t="s">
-        <v>270</v>
-      </c>
-      <c r="F43" t="s">
-        <v>16</v>
-      </c>
-      <c r="G43" t="s">
+      <c r="H43" t="s">
         <v>289</v>
-      </c>
-      <c r="H43" t="s">
-        <v>290</v>
       </c>
       <c r="I43" t="s">
         <v>68</v>
       </c>
       <c r="J43" t="s">
+        <v>290</v>
+      </c>
+      <c r="K43" t="s">
         <v>291</v>
       </c>
-      <c r="K43" t="s">
-        <v>292</v>
-      </c>
       <c r="L43" t="s">
-        <v>187</v>
+        <v>47</v>
       </c>
     </row>
     <row r="44">
@@ -3948,37 +3945,37 @@
         <v>20251011</v>
       </c>
       <c r="B44" t="s">
+        <v>292</v>
+      </c>
+      <c r="C44" t="s">
         <v>293</v>
       </c>
-      <c r="C44" t="s">
+      <c r="D44" t="s">
         <v>294</v>
       </c>
-      <c r="D44" t="s">
+      <c r="E44" t="s">
         <v>295</v>
-      </c>
-      <c r="E44" t="s">
-        <v>296</v>
       </c>
       <c r="F44" t="s">
         <v>26</v>
       </c>
       <c r="G44" t="s">
+        <v>296</v>
+      </c>
+      <c r="H44" t="s">
         <v>297</v>
-      </c>
-      <c r="H44" t="s">
-        <v>298</v>
       </c>
       <c r="I44" t="s">
         <v>44</v>
       </c>
       <c r="J44" t="s">
+        <v>298</v>
+      </c>
+      <c r="K44" t="s">
         <v>299</v>
       </c>
-      <c r="K44" t="s">
-        <v>300</v>
-      </c>
       <c r="L44" t="s">
-        <v>187</v>
+        <v>47</v>
       </c>
     </row>
     <row r="45">
@@ -3986,37 +3983,37 @@
         <v>20253194</v>
       </c>
       <c r="B45" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C45" t="s">
         <v>32</v>
       </c>
       <c r="D45" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="E45" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="F45" t="s">
         <v>26</v>
       </c>
       <c r="G45" t="s">
+        <v>302</v>
+      </c>
+      <c r="H45" t="s">
         <v>303</v>
-      </c>
-      <c r="H45" t="s">
-        <v>304</v>
       </c>
       <c r="I45" t="s">
         <v>44</v>
       </c>
       <c r="J45" t="s">
+        <v>304</v>
+      </c>
+      <c r="K45" t="s">
         <v>305</v>
       </c>
-      <c r="K45" t="s">
-        <v>306</v>
-      </c>
       <c r="L45" t="s">
-        <v>187</v>
+        <v>47</v>
       </c>
     </row>
     <row r="46">
@@ -4024,37 +4021,37 @@
         <v>20253203</v>
       </c>
       <c r="B46" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C46" t="s">
         <v>32</v>
       </c>
       <c r="D46" t="s">
+        <v>307</v>
+      </c>
+      <c r="E46" t="s">
+        <v>295</v>
+      </c>
+      <c r="F46" t="s">
+        <v>16</v>
+      </c>
+      <c r="G46" t="s">
         <v>308</v>
       </c>
-      <c r="E46" t="s">
-        <v>296</v>
-      </c>
-      <c r="F46" t="s">
-        <v>16</v>
-      </c>
-      <c r="G46" t="s">
+      <c r="H46" t="s">
         <v>309</v>
-      </c>
-      <c r="H46" t="s">
-        <v>310</v>
       </c>
       <c r="I46" t="s">
         <v>44</v>
       </c>
       <c r="J46" t="s">
+        <v>310</v>
+      </c>
+      <c r="K46" t="s">
         <v>311</v>
       </c>
-      <c r="K46" t="s">
-        <v>312</v>
-      </c>
       <c r="L46" t="s">
-        <v>187</v>
+        <v>54</v>
       </c>
     </row>
     <row r="47">
@@ -4062,37 +4059,37 @@
         <v>20253213</v>
       </c>
       <c r="B47" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="C47" t="s">
         <v>32</v>
       </c>
       <c r="D47" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E47" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="F47" t="s">
         <v>26</v>
       </c>
       <c r="G47" t="s">
+        <v>314</v>
+      </c>
+      <c r="H47" t="s">
         <v>315</v>
-      </c>
-      <c r="H47" t="s">
-        <v>316</v>
       </c>
       <c r="I47" t="s">
         <v>44</v>
       </c>
       <c r="J47" t="s">
+        <v>316</v>
+      </c>
+      <c r="K47" t="s">
         <v>317</v>
       </c>
-      <c r="K47" t="s">
-        <v>318</v>
-      </c>
       <c r="L47" t="s">
-        <v>187</v>
+        <v>47</v>
       </c>
     </row>
     <row r="48">
@@ -4100,37 +4097,37 @@
         <v>20253214</v>
       </c>
       <c r="B48" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C48" t="s">
         <v>32</v>
       </c>
       <c r="D48" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="E48" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="F48" t="s">
         <v>16</v>
       </c>
       <c r="G48" t="s">
+        <v>319</v>
+      </c>
+      <c r="H48" t="s">
         <v>320</v>
-      </c>
-      <c r="H48" t="s">
-        <v>321</v>
       </c>
       <c r="I48" t="s">
         <v>44</v>
       </c>
       <c r="J48" t="s">
+        <v>321</v>
+      </c>
+      <c r="K48" t="s">
         <v>322</v>
       </c>
-      <c r="K48" t="s">
-        <v>323</v>
-      </c>
       <c r="L48" t="s">
-        <v>187</v>
+        <v>47</v>
       </c>
     </row>
     <row r="49">
@@ -4138,37 +4135,37 @@
         <v>20253246</v>
       </c>
       <c r="B49" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C49" t="s">
         <v>13</v>
       </c>
       <c r="D49" t="s">
+        <v>324</v>
+      </c>
+      <c r="E49" t="s">
+        <v>295</v>
+      </c>
+      <c r="F49" t="s">
+        <v>16</v>
+      </c>
+      <c r="G49" t="s">
         <v>325</v>
       </c>
-      <c r="E49" t="s">
-        <v>296</v>
-      </c>
-      <c r="F49" t="s">
-        <v>16</v>
-      </c>
-      <c r="G49" t="s">
+      <c r="H49" t="s">
         <v>326</v>
-      </c>
-      <c r="H49" t="s">
-        <v>327</v>
       </c>
       <c r="I49" t="s">
         <v>145</v>
       </c>
       <c r="J49" t="s">
+        <v>327</v>
+      </c>
+      <c r="K49" t="s">
         <v>328</v>
       </c>
-      <c r="K49" t="s">
-        <v>329</v>
-      </c>
       <c r="L49" t="s">
-        <v>187</v>
+        <v>22</v>
       </c>
     </row>
     <row r="50">
@@ -4176,37 +4173,37 @@
         <v>20253093</v>
       </c>
       <c r="B50" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="C50" t="s">
         <v>32</v>
       </c>
       <c r="D50" t="s">
+        <v>330</v>
+      </c>
+      <c r="E50" t="s">
         <v>331</v>
       </c>
-      <c r="E50" t="s">
+      <c r="F50" t="s">
+        <v>16</v>
+      </c>
+      <c r="G50" t="s">
         <v>332</v>
       </c>
-      <c r="F50" t="s">
-        <v>16</v>
-      </c>
-      <c r="G50" t="s">
+      <c r="H50" t="s">
         <v>333</v>
-      </c>
-      <c r="H50" t="s">
-        <v>334</v>
       </c>
       <c r="I50" t="s">
         <v>68</v>
       </c>
       <c r="J50" t="s">
+        <v>334</v>
+      </c>
+      <c r="K50" t="s">
         <v>335</v>
       </c>
-      <c r="K50" t="s">
-        <v>336</v>
-      </c>
       <c r="L50" t="s">
-        <v>187</v>
+        <v>22</v>
       </c>
     </row>
     <row r="51">
@@ -4214,37 +4211,37 @@
         <v>20257213</v>
       </c>
       <c r="B51" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="C51" t="s">
         <v>39</v>
       </c>
       <c r="D51" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="E51" t="s">
+        <v>337</v>
+      </c>
+      <c r="F51" t="s">
+        <v>16</v>
+      </c>
+      <c r="G51" t="s">
         <v>338</v>
       </c>
-      <c r="F51" t="s">
-        <v>16</v>
-      </c>
-      <c r="G51" t="s">
+      <c r="H51" t="s">
         <v>339</v>
-      </c>
-      <c r="H51" t="s">
-        <v>340</v>
       </c>
       <c r="I51" t="s">
         <v>44</v>
       </c>
       <c r="J51" t="s">
+        <v>340</v>
+      </c>
+      <c r="K51" t="s">
         <v>341</v>
       </c>
-      <c r="K51" t="s">
-        <v>342</v>
-      </c>
       <c r="L51" t="s">
-        <v>187</v>
+        <v>22</v>
       </c>
     </row>
     <row r="52">
@@ -4252,37 +4249,37 @@
         <v>20253054</v>
       </c>
       <c r="B52" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="C52" t="s">
         <v>13</v>
       </c>
       <c r="D52" t="s">
+        <v>343</v>
+      </c>
+      <c r="E52" t="s">
         <v>344</v>
       </c>
-      <c r="E52" t="s">
+      <c r="F52" t="s">
+        <v>16</v>
+      </c>
+      <c r="G52" t="s">
         <v>345</v>
       </c>
-      <c r="F52" t="s">
-        <v>16</v>
-      </c>
-      <c r="G52" t="s">
+      <c r="H52" t="s">
         <v>346</v>
-      </c>
-      <c r="H52" t="s">
-        <v>347</v>
       </c>
       <c r="I52" t="s">
         <v>68</v>
       </c>
       <c r="J52" t="s">
+        <v>347</v>
+      </c>
+      <c r="K52" t="s">
         <v>348</v>
       </c>
-      <c r="K52" t="s">
-        <v>349</v>
-      </c>
       <c r="L52" t="s">
-        <v>187</v>
+        <v>47</v>
       </c>
     </row>
     <row r="53">
@@ -4290,7 +4287,7 @@
         <v>20257102</v>
       </c>
       <c r="B53" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="C53" t="s">
         <v>39</v>
@@ -4299,28 +4296,28 @@
         <v>111</v>
       </c>
       <c r="E53" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="F53" t="s">
         <v>16</v>
       </c>
       <c r="G53" t="s">
+        <v>350</v>
+      </c>
+      <c r="H53" t="s">
         <v>351</v>
-      </c>
-      <c r="H53" t="s">
-        <v>352</v>
       </c>
       <c r="I53" t="s">
         <v>44</v>
       </c>
       <c r="J53" t="s">
+        <v>352</v>
+      </c>
+      <c r="K53" t="s">
         <v>353</v>
       </c>
-      <c r="K53" t="s">
-        <v>354</v>
-      </c>
       <c r="L53" t="s">
-        <v>187</v>
+        <v>47</v>
       </c>
     </row>
     <row r="54">
@@ -4328,37 +4325,37 @@
         <v>20257129</v>
       </c>
       <c r="B54" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C54" t="s">
         <v>39</v>
       </c>
       <c r="D54" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E54" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="F54" t="s">
         <v>16</v>
       </c>
       <c r="G54" t="s">
+        <v>355</v>
+      </c>
+      <c r="H54" t="s">
         <v>356</v>
-      </c>
-      <c r="H54" t="s">
-        <v>357</v>
       </c>
       <c r="I54" t="s">
         <v>44</v>
       </c>
       <c r="J54" t="s">
+        <v>357</v>
+      </c>
+      <c r="K54" t="s">
         <v>358</v>
       </c>
-      <c r="K54" t="s">
-        <v>359</v>
-      </c>
       <c r="L54" t="s">
-        <v>187</v>
+        <v>22</v>
       </c>
     </row>
     <row r="55">
@@ -4366,37 +4363,37 @@
         <v>20257138</v>
       </c>
       <c r="B55" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C55" t="s">
         <v>39</v>
       </c>
       <c r="D55" t="s">
+        <v>360</v>
+      </c>
+      <c r="E55" t="s">
+        <v>344</v>
+      </c>
+      <c r="F55" t="s">
+        <v>16</v>
+      </c>
+      <c r="G55" t="s">
         <v>361</v>
       </c>
-      <c r="E55" t="s">
-        <v>345</v>
-      </c>
-      <c r="F55" t="s">
-        <v>16</v>
-      </c>
-      <c r="G55" t="s">
+      <c r="H55" t="s">
         <v>362</v>
-      </c>
-      <c r="H55" t="s">
-        <v>363</v>
       </c>
       <c r="I55" t="s">
         <v>44</v>
       </c>
       <c r="J55" t="s">
+        <v>363</v>
+      </c>
+      <c r="K55" t="s">
         <v>364</v>
       </c>
-      <c r="K55" t="s">
-        <v>365</v>
-      </c>
       <c r="L55" t="s">
-        <v>187</v>
+        <v>47</v>
       </c>
     </row>
     <row r="56">
@@ -4404,37 +4401,37 @@
         <v>20253031</v>
       </c>
       <c r="B56" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="C56" t="s">
         <v>32</v>
       </c>
       <c r="D56" t="s">
+        <v>366</v>
+      </c>
+      <c r="E56" t="s">
         <v>367</v>
       </c>
-      <c r="E56" t="s">
+      <c r="F56" t="s">
+        <v>16</v>
+      </c>
+      <c r="G56" t="s">
         <v>368</v>
       </c>
-      <c r="F56" t="s">
-        <v>16</v>
-      </c>
-      <c r="G56" t="s">
+      <c r="H56" t="s">
         <v>369</v>
-      </c>
-      <c r="H56" t="s">
-        <v>370</v>
       </c>
       <c r="I56" t="s">
         <v>68</v>
       </c>
       <c r="J56" t="s">
+        <v>370</v>
+      </c>
+      <c r="K56" t="s">
         <v>371</v>
       </c>
-      <c r="K56" t="s">
-        <v>372</v>
-      </c>
       <c r="L56" t="s">
-        <v>187</v>
+        <v>47</v>
       </c>
     </row>
     <row r="57">
@@ -4442,37 +4439,37 @@
         <v>20257012</v>
       </c>
       <c r="B57" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="C57" t="s">
         <v>39</v>
       </c>
       <c r="D57" t="s">
+        <v>373</v>
+      </c>
+      <c r="E57" t="s">
+        <v>367</v>
+      </c>
+      <c r="F57" t="s">
+        <v>16</v>
+      </c>
+      <c r="G57" t="s">
         <v>374</v>
       </c>
-      <c r="E57" t="s">
-        <v>368</v>
-      </c>
-      <c r="F57" t="s">
-        <v>16</v>
-      </c>
-      <c r="G57" t="s">
+      <c r="H57" t="s">
         <v>375</v>
-      </c>
-      <c r="H57" t="s">
-        <v>376</v>
       </c>
       <c r="I57" t="s">
         <v>44</v>
       </c>
       <c r="J57" t="s">
+        <v>376</v>
+      </c>
+      <c r="K57" t="s">
         <v>377</v>
       </c>
-      <c r="K57" t="s">
-        <v>378</v>
-      </c>
       <c r="L57" t="s">
-        <v>187</v>
+        <v>54</v>
       </c>
     </row>
     <row r="58">
@@ -4480,35 +4477,35 @@
         <v>20253008</v>
       </c>
       <c r="B58" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C58" t="s">
         <v>13</v>
       </c>
       <c r="D58"/>
       <c r="E58" t="s">
+        <v>379</v>
+      </c>
+      <c r="F58" t="s">
+        <v>16</v>
+      </c>
+      <c r="G58" t="s">
         <v>380</v>
       </c>
-      <c r="F58" t="s">
-        <v>16</v>
-      </c>
-      <c r="G58" t="s">
+      <c r="H58" t="s">
         <v>381</v>
-      </c>
-      <c r="H58" t="s">
-        <v>382</v>
       </c>
       <c r="I58" t="s">
         <v>44</v>
       </c>
       <c r="J58" t="s">
+        <v>382</v>
+      </c>
+      <c r="K58" t="s">
         <v>383</v>
       </c>
-      <c r="K58" t="s">
-        <v>384</v>
-      </c>
       <c r="L58" t="s">
-        <v>187</v>
+        <v>47</v>
       </c>
     </row>
     <row r="59">
@@ -4516,37 +4513,37 @@
         <v>20244404</v>
       </c>
       <c r="B59" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="C59" t="s">
         <v>32</v>
       </c>
       <c r="D59" t="s">
+        <v>385</v>
+      </c>
+      <c r="E59" t="s">
         <v>386</v>
       </c>
-      <c r="E59" t="s">
+      <c r="F59" t="s">
+        <v>16</v>
+      </c>
+      <c r="G59" t="s">
         <v>387</v>
       </c>
-      <c r="F59" t="s">
-        <v>16</v>
-      </c>
-      <c r="G59" t="s">
+      <c r="H59" t="s">
         <v>388</v>
-      </c>
-      <c r="H59" t="s">
-        <v>389</v>
       </c>
       <c r="I59" t="s">
         <v>44</v>
       </c>
       <c r="J59" t="s">
+        <v>389</v>
+      </c>
+      <c r="K59" t="s">
         <v>390</v>
       </c>
-      <c r="K59" t="s">
-        <v>391</v>
-      </c>
       <c r="L59" t="s">
-        <v>187</v>
+        <v>47</v>
       </c>
     </row>
     <row r="60">
@@ -4554,37 +4551,37 @@
         <v>20244419</v>
       </c>
       <c r="B60" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="C60" t="s">
         <v>32</v>
       </c>
       <c r="D60" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E60" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="F60" t="s">
         <v>26</v>
       </c>
       <c r="G60" t="s">
+        <v>392</v>
+      </c>
+      <c r="H60" t="s">
         <v>393</v>
-      </c>
-      <c r="H60" t="s">
-        <v>394</v>
       </c>
       <c r="I60" t="s">
         <v>44</v>
       </c>
       <c r="J60" t="s">
+        <v>394</v>
+      </c>
+      <c r="K60" t="s">
         <v>395</v>
       </c>
-      <c r="K60" t="s">
-        <v>396</v>
-      </c>
       <c r="L60" t="s">
-        <v>187</v>
+        <v>47</v>
       </c>
     </row>
     <row r="61">
@@ -4592,37 +4589,37 @@
         <v>20247975</v>
       </c>
       <c r="B61" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="C61" t="s">
         <v>39</v>
       </c>
       <c r="D61" t="s">
+        <v>397</v>
+      </c>
+      <c r="E61" t="s">
         <v>398</v>
       </c>
-      <c r="E61" t="s">
+      <c r="F61" t="s">
+        <v>16</v>
+      </c>
+      <c r="G61" t="s">
         <v>399</v>
       </c>
-      <c r="F61" t="s">
-        <v>16</v>
-      </c>
-      <c r="G61" t="s">
+      <c r="H61" t="s">
         <v>400</v>
-      </c>
-      <c r="H61" t="s">
-        <v>401</v>
       </c>
       <c r="I61" t="s">
         <v>44</v>
       </c>
       <c r="J61" t="s">
+        <v>401</v>
+      </c>
+      <c r="K61" t="s">
         <v>402</v>
       </c>
-      <c r="K61" t="s">
-        <v>403</v>
-      </c>
       <c r="L61" t="s">
-        <v>187</v>
+        <v>22</v>
       </c>
     </row>
     <row r="62">
@@ -4630,37 +4627,37 @@
         <v>20248043</v>
       </c>
       <c r="B62" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="C62" t="s">
         <v>39</v>
       </c>
       <c r="D62" t="s">
+        <v>404</v>
+      </c>
+      <c r="E62" t="s">
+        <v>398</v>
+      </c>
+      <c r="F62" t="s">
+        <v>16</v>
+      </c>
+      <c r="G62" t="s">
         <v>405</v>
       </c>
-      <c r="E62" t="s">
-        <v>399</v>
-      </c>
-      <c r="F62" t="s">
-        <v>16</v>
-      </c>
-      <c r="G62" t="s">
+      <c r="H62" t="s">
         <v>406</v>
-      </c>
-      <c r="H62" t="s">
-        <v>407</v>
       </c>
       <c r="I62" t="s">
         <v>44</v>
       </c>
       <c r="J62" t="s">
+        <v>407</v>
+      </c>
+      <c r="K62" t="s">
         <v>408</v>
       </c>
-      <c r="K62" t="s">
-        <v>409</v>
-      </c>
       <c r="L62" t="s">
-        <v>187</v>
+        <v>22</v>
       </c>
     </row>
     <row r="63">
@@ -4668,37 +4665,37 @@
         <v>20244290</v>
       </c>
       <c r="B63" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="C63" t="s">
         <v>32</v>
       </c>
       <c r="D63" t="s">
+        <v>410</v>
+      </c>
+      <c r="E63" t="s">
         <v>411</v>
       </c>
-      <c r="E63" t="s">
+      <c r="F63" t="s">
+        <v>16</v>
+      </c>
+      <c r="G63" t="s">
         <v>412</v>
       </c>
-      <c r="F63" t="s">
-        <v>16</v>
-      </c>
-      <c r="G63" t="s">
+      <c r="H63" t="s">
         <v>413</v>
-      </c>
-      <c r="H63" t="s">
-        <v>414</v>
       </c>
       <c r="I63" t="s">
         <v>68</v>
       </c>
       <c r="J63" t="s">
+        <v>414</v>
+      </c>
+      <c r="K63" t="s">
         <v>415</v>
       </c>
-      <c r="K63" t="s">
-        <v>416</v>
-      </c>
       <c r="L63" t="s">
-        <v>187</v>
+        <v>47</v>
       </c>
     </row>
     <row r="64">
@@ -4706,37 +4703,37 @@
         <v>20244278</v>
       </c>
       <c r="B64" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="C64" t="s">
         <v>32</v>
       </c>
       <c r="D64" t="s">
+        <v>417</v>
+      </c>
+      <c r="E64" t="s">
         <v>418</v>
       </c>
-      <c r="E64" t="s">
+      <c r="F64" t="s">
+        <v>16</v>
+      </c>
+      <c r="G64" t="s">
         <v>419</v>
       </c>
-      <c r="F64" t="s">
-        <v>16</v>
-      </c>
-      <c r="G64" t="s">
+      <c r="H64" t="s">
         <v>420</v>
-      </c>
-      <c r="H64" t="s">
-        <v>421</v>
       </c>
       <c r="I64" t="s">
         <v>68</v>
       </c>
       <c r="J64" t="s">
+        <v>421</v>
+      </c>
+      <c r="K64" t="s">
         <v>422</v>
       </c>
-      <c r="K64" t="s">
-        <v>423</v>
-      </c>
       <c r="L64" t="s">
-        <v>187</v>
+        <v>22</v>
       </c>
     </row>
     <row r="65">
@@ -4744,37 +4741,37 @@
         <v>20244082</v>
       </c>
       <c r="B65" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="C65" t="s">
         <v>32</v>
       </c>
       <c r="D65" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="E65" t="s">
+        <v>424</v>
+      </c>
+      <c r="F65" t="s">
+        <v>16</v>
+      </c>
+      <c r="G65" t="s">
         <v>425</v>
       </c>
-      <c r="F65" t="s">
-        <v>16</v>
-      </c>
-      <c r="G65" t="s">
+      <c r="H65" t="s">
         <v>426</v>
-      </c>
-      <c r="H65" t="s">
-        <v>427</v>
       </c>
       <c r="I65" t="s">
         <v>68</v>
       </c>
       <c r="J65" t="s">
+        <v>427</v>
+      </c>
+      <c r="K65" t="s">
         <v>428</v>
       </c>
-      <c r="K65" t="s">
-        <v>429</v>
-      </c>
       <c r="L65" t="s">
-        <v>187</v>
+        <v>47</v>
       </c>
     </row>
     <row r="66">
@@ -4782,37 +4779,37 @@
         <v>20244112</v>
       </c>
       <c r="B66" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="C66" t="s">
         <v>32</v>
       </c>
       <c r="D66" t="s">
+        <v>430</v>
+      </c>
+      <c r="E66" t="s">
+        <v>424</v>
+      </c>
+      <c r="F66" t="s">
+        <v>16</v>
+      </c>
+      <c r="G66" t="s">
         <v>431</v>
       </c>
-      <c r="E66" t="s">
-        <v>425</v>
-      </c>
-      <c r="F66" t="s">
-        <v>16</v>
-      </c>
-      <c r="G66" t="s">
+      <c r="H66" t="s">
         <v>432</v>
-      </c>
-      <c r="H66" t="s">
-        <v>433</v>
       </c>
       <c r="I66" t="s">
         <v>68</v>
       </c>
       <c r="J66" t="s">
+        <v>433</v>
+      </c>
+      <c r="K66" t="s">
         <v>434</v>
       </c>
-      <c r="K66" t="s">
-        <v>435</v>
-      </c>
       <c r="L66" t="s">
-        <v>187</v>
+        <v>54</v>
       </c>
     </row>
     <row r="67">
@@ -4820,7 +4817,7 @@
         <v>20244131</v>
       </c>
       <c r="B67" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="C67" t="s">
         <v>32</v>
@@ -4829,28 +4826,28 @@
         <v>49</v>
       </c>
       <c r="E67" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F67" t="s">
         <v>16</v>
       </c>
       <c r="G67" t="s">
+        <v>436</v>
+      </c>
+      <c r="H67" t="s">
         <v>437</v>
-      </c>
-      <c r="H67" t="s">
-        <v>438</v>
       </c>
       <c r="I67" t="s">
         <v>68</v>
       </c>
       <c r="J67" t="s">
+        <v>438</v>
+      </c>
+      <c r="K67" t="s">
         <v>439</v>
       </c>
-      <c r="K67" t="s">
-        <v>440</v>
-      </c>
       <c r="L67" t="s">
-        <v>187</v>
+        <v>47</v>
       </c>
     </row>
     <row r="68">
@@ -4858,7 +4855,7 @@
         <v>20244132</v>
       </c>
       <c r="B68" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="C68" t="s">
         <v>63</v>
@@ -4867,28 +4864,28 @@
         <v>124</v>
       </c>
       <c r="E68" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F68" t="s">
         <v>16</v>
       </c>
       <c r="G68" t="s">
+        <v>441</v>
+      </c>
+      <c r="H68" t="s">
         <v>442</v>
-      </c>
-      <c r="H68" t="s">
-        <v>443</v>
       </c>
       <c r="I68" t="s">
         <v>68</v>
       </c>
       <c r="J68" t="s">
+        <v>443</v>
+      </c>
+      <c r="K68" t="s">
         <v>444</v>
       </c>
-      <c r="K68" t="s">
-        <v>445</v>
-      </c>
       <c r="L68" t="s">
-        <v>187</v>
+        <v>54</v>
       </c>
     </row>
     <row r="69">
@@ -4896,7 +4893,7 @@
         <v>20244133</v>
       </c>
       <c r="B69" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="C69" t="s">
         <v>13</v>
@@ -4905,28 +4902,28 @@
         <v>124</v>
       </c>
       <c r="E69" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F69" t="s">
         <v>16</v>
       </c>
       <c r="G69" t="s">
+        <v>446</v>
+      </c>
+      <c r="H69" t="s">
         <v>447</v>
-      </c>
-      <c r="H69" t="s">
-        <v>448</v>
       </c>
       <c r="I69" t="s">
         <v>68</v>
       </c>
       <c r="J69" t="s">
+        <v>448</v>
+      </c>
+      <c r="K69" t="s">
         <v>449</v>
       </c>
-      <c r="K69" t="s">
-        <v>450</v>
-      </c>
       <c r="L69" t="s">
-        <v>187</v>
+        <v>54</v>
       </c>
     </row>
     <row r="70">
@@ -4934,37 +4931,37 @@
         <v>20244137</v>
       </c>
       <c r="B70" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="C70" t="s">
         <v>32</v>
       </c>
       <c r="D70" t="s">
+        <v>451</v>
+      </c>
+      <c r="E70" t="s">
+        <v>424</v>
+      </c>
+      <c r="F70" t="s">
+        <v>16</v>
+      </c>
+      <c r="G70" t="s">
         <v>452</v>
       </c>
-      <c r="E70" t="s">
-        <v>425</v>
-      </c>
-      <c r="F70" t="s">
-        <v>16</v>
-      </c>
-      <c r="G70" t="s">
+      <c r="H70" t="s">
         <v>453</v>
-      </c>
-      <c r="H70" t="s">
-        <v>454</v>
       </c>
       <c r="I70" t="s">
         <v>68</v>
       </c>
       <c r="J70" t="s">
+        <v>454</v>
+      </c>
+      <c r="K70" t="s">
         <v>455</v>
       </c>
-      <c r="K70" t="s">
-        <v>456</v>
-      </c>
       <c r="L70" t="s">
-        <v>187</v>
+        <v>54</v>
       </c>
     </row>
     <row r="71">
@@ -4972,37 +4969,37 @@
         <v>20243937</v>
       </c>
       <c r="B71" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="C71" t="s">
         <v>13</v>
       </c>
       <c r="D71" t="s">
+        <v>457</v>
+      </c>
+      <c r="E71" t="s">
         <v>458</v>
-      </c>
-      <c r="E71" t="s">
-        <v>459</v>
       </c>
       <c r="F71" t="s">
         <v>26</v>
       </c>
       <c r="G71" t="s">
+        <v>459</v>
+      </c>
+      <c r="H71" t="s">
         <v>460</v>
-      </c>
-      <c r="H71" t="s">
-        <v>461</v>
       </c>
       <c r="I71" t="s">
         <v>177</v>
       </c>
       <c r="J71" t="s">
+        <v>461</v>
+      </c>
+      <c r="K71" t="s">
         <v>462</v>
       </c>
-      <c r="K71" t="s">
-        <v>463</v>
-      </c>
       <c r="L71" t="s">
-        <v>187</v>
+        <v>22</v>
       </c>
     </row>
     <row r="72">
@@ -5010,37 +5007,37 @@
         <v>20243948</v>
       </c>
       <c r="B72" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="C72" t="s">
         <v>32</v>
       </c>
       <c r="D72" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="E72" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="F72" t="s">
         <v>26</v>
       </c>
       <c r="G72" t="s">
+        <v>465</v>
+      </c>
+      <c r="H72" t="s">
         <v>466</v>
-      </c>
-      <c r="H72" t="s">
-        <v>467</v>
       </c>
       <c r="I72" t="s">
         <v>44</v>
       </c>
       <c r="J72" t="s">
+        <v>467</v>
+      </c>
+      <c r="K72" t="s">
         <v>468</v>
       </c>
-      <c r="K72" t="s">
-        <v>469</v>
-      </c>
       <c r="L72" t="s">
-        <v>187</v>
+        <v>47</v>
       </c>
     </row>
     <row r="73">
@@ -5048,37 +5045,37 @@
         <v>20247720</v>
       </c>
       <c r="B73" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="C73" t="s">
         <v>39</v>
       </c>
       <c r="D73" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E73" t="s">
+        <v>470</v>
+      </c>
+      <c r="F73" t="s">
+        <v>16</v>
+      </c>
+      <c r="G73" t="s">
         <v>471</v>
       </c>
-      <c r="F73" t="s">
-        <v>16</v>
-      </c>
-      <c r="G73" t="s">
+      <c r="H73" t="s">
         <v>472</v>
-      </c>
-      <c r="H73" t="s">
-        <v>473</v>
       </c>
       <c r="I73" t="s">
         <v>44</v>
       </c>
       <c r="J73" t="s">
+        <v>473</v>
+      </c>
+      <c r="K73" t="s">
         <v>474</v>
       </c>
-      <c r="K73" t="s">
-        <v>475</v>
-      </c>
       <c r="L73" t="s">
-        <v>187</v>
+        <v>22</v>
       </c>
     </row>
     <row r="74">
@@ -5086,37 +5083,37 @@
         <v>20247726</v>
       </c>
       <c r="B74" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="C74" t="s">
         <v>39</v>
       </c>
       <c r="D74" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="E74" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="F74" t="s">
         <v>16</v>
       </c>
       <c r="G74" t="s">
+        <v>476</v>
+      </c>
+      <c r="H74" t="s">
         <v>477</v>
-      </c>
-      <c r="H74" t="s">
-        <v>478</v>
       </c>
       <c r="I74" t="s">
         <v>44</v>
       </c>
       <c r="J74" t="s">
+        <v>478</v>
+      </c>
+      <c r="K74" t="s">
         <v>479</v>
       </c>
-      <c r="K74" t="s">
-        <v>480</v>
-      </c>
       <c r="L74" t="s">
-        <v>187</v>
+        <v>47</v>
       </c>
     </row>
     <row r="75">
@@ -5124,7 +5121,7 @@
         <v>20247773</v>
       </c>
       <c r="B75" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="C75" t="s">
         <v>39</v>
@@ -5133,28 +5130,28 @@
         <v>118</v>
       </c>
       <c r="E75" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="F75" t="s">
         <v>16</v>
       </c>
       <c r="G75" t="s">
+        <v>481</v>
+      </c>
+      <c r="H75" t="s">
         <v>482</v>
-      </c>
-      <c r="H75" t="s">
-        <v>483</v>
       </c>
       <c r="I75" t="s">
         <v>44</v>
       </c>
       <c r="J75" t="s">
+        <v>483</v>
+      </c>
+      <c r="K75" t="s">
         <v>484</v>
       </c>
-      <c r="K75" t="s">
-        <v>485</v>
-      </c>
       <c r="L75" t="s">
-        <v>187</v>
+        <v>54</v>
       </c>
     </row>
     <row r="76">
@@ -5162,7 +5159,7 @@
         <v>20247774</v>
       </c>
       <c r="B76" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="C76" t="s">
         <v>39</v>
@@ -5171,28 +5168,28 @@
         <v>118</v>
       </c>
       <c r="E76" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="F76" t="s">
         <v>16</v>
       </c>
       <c r="G76" t="s">
+        <v>486</v>
+      </c>
+      <c r="H76" t="s">
         <v>487</v>
-      </c>
-      <c r="H76" t="s">
-        <v>488</v>
       </c>
       <c r="I76" t="s">
         <v>44</v>
       </c>
       <c r="J76" t="s">
+        <v>488</v>
+      </c>
+      <c r="K76" t="s">
         <v>489</v>
       </c>
-      <c r="K76" t="s">
-        <v>490</v>
-      </c>
       <c r="L76" t="s">
-        <v>187</v>
+        <v>54</v>
       </c>
     </row>
     <row r="77">
@@ -5200,37 +5197,37 @@
         <v>20243858</v>
       </c>
       <c r="B77" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C77" t="s">
         <v>32</v>
       </c>
       <c r="D77" t="s">
+        <v>491</v>
+      </c>
+      <c r="E77" t="s">
         <v>492</v>
       </c>
-      <c r="E77" t="s">
+      <c r="F77" t="s">
+        <v>16</v>
+      </c>
+      <c r="G77" t="s">
         <v>493</v>
       </c>
-      <c r="F77" t="s">
-        <v>16</v>
-      </c>
-      <c r="G77" t="s">
+      <c r="H77" t="s">
         <v>494</v>
-      </c>
-      <c r="H77" t="s">
-        <v>495</v>
       </c>
       <c r="I77" t="s">
         <v>68</v>
       </c>
       <c r="J77" t="s">
+        <v>495</v>
+      </c>
+      <c r="K77" t="s">
         <v>496</v>
       </c>
-      <c r="K77" t="s">
-        <v>497</v>
-      </c>
       <c r="L77" t="s">
-        <v>187</v>
+        <v>22</v>
       </c>
     </row>
     <row r="78">
@@ -5238,37 +5235,37 @@
         <v>20243877</v>
       </c>
       <c r="B78" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="C78" t="s">
         <v>32</v>
       </c>
       <c r="D78" t="s">
+        <v>498</v>
+      </c>
+      <c r="E78" t="s">
+        <v>492</v>
+      </c>
+      <c r="F78" t="s">
+        <v>16</v>
+      </c>
+      <c r="G78" t="s">
         <v>499</v>
       </c>
-      <c r="E78" t="s">
-        <v>493</v>
-      </c>
-      <c r="F78" t="s">
-        <v>16</v>
-      </c>
-      <c r="G78" t="s">
+      <c r="H78" t="s">
         <v>500</v>
-      </c>
-      <c r="H78" t="s">
-        <v>501</v>
       </c>
       <c r="I78" t="s">
         <v>68</v>
       </c>
       <c r="J78" t="s">
+        <v>501</v>
+      </c>
+      <c r="K78" t="s">
         <v>502</v>
       </c>
-      <c r="K78" t="s">
-        <v>503</v>
-      </c>
       <c r="L78" t="s">
-        <v>187</v>
+        <v>47</v>
       </c>
     </row>
     <row r="79">
@@ -5276,7 +5273,7 @@
         <v>20247622</v>
       </c>
       <c r="B79" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="C79" t="s">
         <v>39</v>
@@ -5285,28 +5282,28 @@
         <v>49</v>
       </c>
       <c r="E79" t="s">
+        <v>504</v>
+      </c>
+      <c r="F79" t="s">
+        <v>16</v>
+      </c>
+      <c r="G79" t="s">
         <v>505</v>
       </c>
-      <c r="F79" t="s">
-        <v>16</v>
-      </c>
-      <c r="G79" t="s">
+      <c r="H79" t="s">
         <v>506</v>
-      </c>
-      <c r="H79" t="s">
-        <v>507</v>
       </c>
       <c r="I79" t="s">
         <v>44</v>
       </c>
       <c r="J79" t="s">
+        <v>507</v>
+      </c>
+      <c r="K79" t="s">
         <v>508</v>
       </c>
-      <c r="K79" t="s">
-        <v>509</v>
-      </c>
       <c r="L79" t="s">
-        <v>187</v>
+        <v>47</v>
       </c>
     </row>
     <row r="80">
@@ -5314,37 +5311,37 @@
         <v>20247649</v>
       </c>
       <c r="B80" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="C80" t="s">
         <v>39</v>
       </c>
       <c r="D80" t="s">
+        <v>510</v>
+      </c>
+      <c r="E80" t="s">
+        <v>504</v>
+      </c>
+      <c r="F80" t="s">
+        <v>16</v>
+      </c>
+      <c r="G80" t="s">
         <v>511</v>
       </c>
-      <c r="E80" t="s">
-        <v>505</v>
-      </c>
-      <c r="F80" t="s">
-        <v>16</v>
-      </c>
-      <c r="G80" t="s">
+      <c r="H80" t="s">
         <v>512</v>
-      </c>
-      <c r="H80" t="s">
-        <v>513</v>
       </c>
       <c r="I80" t="s">
         <v>44</v>
       </c>
       <c r="J80" t="s">
+        <v>513</v>
+      </c>
+      <c r="K80" t="s">
         <v>514</v>
       </c>
-      <c r="K80" t="s">
-        <v>515</v>
-      </c>
       <c r="L80" t="s">
-        <v>187</v>
+        <v>47</v>
       </c>
     </row>
     <row r="81">
@@ -5352,37 +5349,37 @@
         <v>20243709</v>
       </c>
       <c r="B81" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="C81" t="s">
         <v>32</v>
       </c>
       <c r="D81" t="s">
+        <v>516</v>
+      </c>
+      <c r="E81" t="s">
         <v>517</v>
       </c>
-      <c r="E81" t="s">
+      <c r="F81" t="s">
+        <v>16</v>
+      </c>
+      <c r="G81" t="s">
         <v>518</v>
       </c>
-      <c r="F81" t="s">
-        <v>16</v>
-      </c>
-      <c r="G81" t="s">
+      <c r="H81" t="s">
         <v>519</v>
-      </c>
-      <c r="H81" t="s">
-        <v>520</v>
       </c>
       <c r="I81" t="s">
         <v>68</v>
       </c>
       <c r="J81" t="s">
+        <v>520</v>
+      </c>
+      <c r="K81" t="s">
         <v>521</v>
       </c>
-      <c r="K81" t="s">
-        <v>522</v>
-      </c>
       <c r="L81" t="s">
-        <v>187</v>
+        <v>54</v>
       </c>
     </row>
     <row r="82">
@@ -5390,37 +5387,37 @@
         <v>20243773</v>
       </c>
       <c r="B82" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="C82" t="s">
         <v>32</v>
       </c>
       <c r="D82" t="s">
+        <v>523</v>
+      </c>
+      <c r="E82" t="s">
+        <v>517</v>
+      </c>
+      <c r="F82" t="s">
+        <v>16</v>
+      </c>
+      <c r="G82" t="s">
         <v>524</v>
       </c>
-      <c r="E82" t="s">
-        <v>518</v>
-      </c>
-      <c r="F82" t="s">
-        <v>16</v>
-      </c>
-      <c r="G82" t="s">
+      <c r="H82" t="s">
         <v>525</v>
-      </c>
-      <c r="H82" t="s">
-        <v>526</v>
       </c>
       <c r="I82" t="s">
         <v>68</v>
       </c>
       <c r="J82" t="s">
+        <v>526</v>
+      </c>
+      <c r="K82" t="s">
         <v>527</v>
       </c>
-      <c r="K82" t="s">
-        <v>528</v>
-      </c>
       <c r="L82" t="s">
-        <v>187</v>
+        <v>47</v>
       </c>
     </row>
     <row r="83">
@@ -5428,37 +5425,37 @@
         <v>20243776</v>
       </c>
       <c r="B83" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="C83" t="s">
         <v>13</v>
       </c>
       <c r="D83" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="E83" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="F83" t="s">
         <v>16</v>
       </c>
       <c r="G83" t="s">
+        <v>529</v>
+      </c>
+      <c r="H83" t="s">
         <v>530</v>
-      </c>
-      <c r="H83" t="s">
-        <v>531</v>
       </c>
       <c r="I83" t="s">
         <v>44</v>
       </c>
       <c r="J83" t="s">
+        <v>531</v>
+      </c>
+      <c r="K83" t="s">
         <v>532</v>
       </c>
-      <c r="K83" t="s">
-        <v>533</v>
-      </c>
       <c r="L83" t="s">
-        <v>187</v>
+        <v>22</v>
       </c>
     </row>
     <row r="84">
@@ -5466,37 +5463,37 @@
         <v>20243609</v>
       </c>
       <c r="B84" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="C84" t="s">
         <v>13</v>
       </c>
       <c r="D84" t="s">
+        <v>534</v>
+      </c>
+      <c r="E84" t="s">
         <v>535</v>
       </c>
-      <c r="E84" t="s">
+      <c r="F84" t="s">
+        <v>16</v>
+      </c>
+      <c r="G84" t="s">
         <v>536</v>
       </c>
-      <c r="F84" t="s">
-        <v>16</v>
-      </c>
-      <c r="G84" t="s">
+      <c r="H84" t="s">
         <v>537</v>
       </c>
-      <c r="H84" t="s">
+      <c r="I84" t="s">
         <v>538</v>
       </c>
-      <c r="I84" t="s">
+      <c r="J84" t="s">
         <v>539</v>
       </c>
-      <c r="J84" t="s">
+      <c r="K84" t="s">
         <v>540</v>
       </c>
-      <c r="K84" t="s">
-        <v>541</v>
-      </c>
       <c r="L84" t="s">
-        <v>187</v>
+        <v>47</v>
       </c>
     </row>
     <row r="85">
@@ -5504,37 +5501,37 @@
         <v>20243574</v>
       </c>
       <c r="B85" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="C85" t="s">
         <v>32</v>
       </c>
       <c r="D85" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E85" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="F85" t="s">
         <v>26</v>
       </c>
       <c r="G85" t="s">
+        <v>543</v>
+      </c>
+      <c r="H85" t="s">
         <v>544</v>
-      </c>
-      <c r="H85" t="s">
-        <v>545</v>
       </c>
       <c r="I85" t="s">
         <v>44</v>
       </c>
       <c r="J85" t="s">
+        <v>545</v>
+      </c>
+      <c r="K85" t="s">
         <v>546</v>
       </c>
-      <c r="K85" t="s">
-        <v>547</v>
-      </c>
       <c r="L85" t="s">
-        <v>187</v>
+        <v>22</v>
       </c>
     </row>
     <row r="86">
@@ -5542,37 +5539,37 @@
         <v>20243557</v>
       </c>
       <c r="B86" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="C86" t="s">
         <v>32</v>
       </c>
       <c r="D86" t="s">
+        <v>548</v>
+      </c>
+      <c r="E86" t="s">
         <v>549</v>
       </c>
-      <c r="E86" t="s">
+      <c r="F86" t="s">
+        <v>16</v>
+      </c>
+      <c r="G86" t="s">
         <v>550</v>
       </c>
-      <c r="F86" t="s">
-        <v>16</v>
-      </c>
-      <c r="G86" t="s">
+      <c r="H86" t="s">
         <v>551</v>
-      </c>
-      <c r="H86" t="s">
-        <v>552</v>
       </c>
       <c r="I86" t="s">
         <v>44</v>
       </c>
       <c r="J86" t="s">
+        <v>552</v>
+      </c>
+      <c r="K86" t="s">
         <v>553</v>
       </c>
-      <c r="K86" t="s">
-        <v>554</v>
-      </c>
       <c r="L86" t="s">
-        <v>187</v>
+        <v>47</v>
       </c>
     </row>
     <row r="87">
@@ -5580,35 +5577,35 @@
         <v>20243471</v>
       </c>
       <c r="B87" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="C87" t="s">
         <v>13</v>
       </c>
       <c r="D87"/>
       <c r="E87" t="s">
+        <v>555</v>
+      </c>
+      <c r="F87" t="s">
+        <v>16</v>
+      </c>
+      <c r="G87" t="s">
         <v>556</v>
       </c>
-      <c r="F87" t="s">
-        <v>16</v>
-      </c>
-      <c r="G87" t="s">
+      <c r="H87" t="s">
         <v>557</v>
-      </c>
-      <c r="H87" t="s">
-        <v>558</v>
       </c>
       <c r="I87" t="s">
         <v>44</v>
       </c>
       <c r="J87" t="s">
+        <v>558</v>
+      </c>
+      <c r="K87" t="s">
         <v>559</v>
       </c>
-      <c r="K87" t="s">
-        <v>560</v>
-      </c>
       <c r="L87" t="s">
-        <v>187</v>
+        <v>22</v>
       </c>
     </row>
     <row r="88">
@@ -5616,35 +5613,35 @@
         <v>20243468</v>
       </c>
       <c r="B88" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="C88" t="s">
         <v>63</v>
       </c>
       <c r="D88"/>
       <c r="E88" t="s">
+        <v>561</v>
+      </c>
+      <c r="F88" t="s">
+        <v>16</v>
+      </c>
+      <c r="G88" t="s">
         <v>562</v>
       </c>
-      <c r="F88" t="s">
-        <v>16</v>
-      </c>
-      <c r="G88" t="s">
+      <c r="H88" t="s">
         <v>563</v>
-      </c>
-      <c r="H88" t="s">
-        <v>564</v>
       </c>
       <c r="I88" t="s">
         <v>177</v>
       </c>
       <c r="J88" t="s">
+        <v>564</v>
+      </c>
+      <c r="K88" t="s">
         <v>565</v>
       </c>
-      <c r="K88" t="s">
-        <v>566</v>
-      </c>
       <c r="L88" t="s">
-        <v>187</v>
+        <v>47</v>
       </c>
     </row>
     <row r="89">
@@ -5652,35 +5649,35 @@
         <v>20243467</v>
       </c>
       <c r="B89" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="C89" t="s">
         <v>13</v>
       </c>
       <c r="D89"/>
       <c r="E89" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="F89" t="s">
         <v>26</v>
       </c>
       <c r="G89" t="s">
+        <v>568</v>
+      </c>
+      <c r="H89" t="s">
         <v>569</v>
-      </c>
-      <c r="H89" t="s">
-        <v>570</v>
       </c>
       <c r="I89" t="s">
         <v>44</v>
       </c>
       <c r="J89" t="s">
+        <v>570</v>
+      </c>
+      <c r="K89" t="s">
         <v>571</v>
       </c>
-      <c r="K89" t="s">
-        <v>572</v>
-      </c>
       <c r="L89" t="s">
-        <v>187</v>
+        <v>47</v>
       </c>
     </row>
     <row r="90">
@@ -5688,37 +5685,37 @@
         <v>20243318</v>
       </c>
       <c r="B90" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="C90" t="s">
         <v>32</v>
       </c>
       <c r="D90" t="s">
+        <v>573</v>
+      </c>
+      <c r="E90" t="s">
         <v>574</v>
       </c>
-      <c r="E90" t="s">
+      <c r="F90" t="s">
+        <v>16</v>
+      </c>
+      <c r="G90" t="s">
         <v>575</v>
       </c>
-      <c r="F90" t="s">
-        <v>16</v>
-      </c>
-      <c r="G90" t="s">
+      <c r="H90" t="s">
         <v>576</v>
-      </c>
-      <c r="H90" t="s">
-        <v>577</v>
       </c>
       <c r="I90" t="s">
         <v>68</v>
       </c>
       <c r="J90" t="s">
+        <v>577</v>
+      </c>
+      <c r="K90" t="s">
         <v>578</v>
       </c>
-      <c r="K90" t="s">
-        <v>579</v>
-      </c>
       <c r="L90" t="s">
-        <v>187</v>
+        <v>54</v>
       </c>
     </row>
     <row r="91">
@@ -5726,37 +5723,37 @@
         <v>20243234</v>
       </c>
       <c r="B91" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="C91" t="s">
         <v>13</v>
       </c>
       <c r="D91" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="E91" t="s">
+        <v>580</v>
+      </c>
+      <c r="F91" t="s">
+        <v>16</v>
+      </c>
+      <c r="G91" t="s">
         <v>581</v>
       </c>
-      <c r="F91" t="s">
-        <v>16</v>
-      </c>
-      <c r="G91" t="s">
+      <c r="H91" t="s">
         <v>582</v>
-      </c>
-      <c r="H91" t="s">
-        <v>583</v>
       </c>
       <c r="I91" t="s">
         <v>44</v>
       </c>
       <c r="J91" t="s">
+        <v>583</v>
+      </c>
+      <c r="K91" t="s">
         <v>584</v>
       </c>
-      <c r="K91" t="s">
-        <v>585</v>
-      </c>
       <c r="L91" t="s">
-        <v>187</v>
+        <v>47</v>
       </c>
     </row>
     <row r="92">
@@ -5764,37 +5761,37 @@
         <v>20243259</v>
       </c>
       <c r="B92" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="C92" t="s">
         <v>32</v>
       </c>
       <c r="D92" t="s">
+        <v>586</v>
+      </c>
+      <c r="E92" t="s">
+        <v>580</v>
+      </c>
+      <c r="F92" t="s">
+        <v>16</v>
+      </c>
+      <c r="G92" t="s">
         <v>587</v>
       </c>
-      <c r="E92" t="s">
-        <v>581</v>
-      </c>
-      <c r="F92" t="s">
-        <v>16</v>
-      </c>
-      <c r="G92" t="s">
+      <c r="H92" t="s">
         <v>588</v>
-      </c>
-      <c r="H92" t="s">
-        <v>589</v>
       </c>
       <c r="I92" t="s">
         <v>44</v>
       </c>
       <c r="J92" t="s">
+        <v>589</v>
+      </c>
+      <c r="K92" t="s">
         <v>590</v>
       </c>
-      <c r="K92" t="s">
-        <v>591</v>
-      </c>
       <c r="L92" t="s">
-        <v>187</v>
+        <v>47</v>
       </c>
     </row>
     <row r="93">
@@ -5802,37 +5799,37 @@
         <v>20243169</v>
       </c>
       <c r="B93" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="C93" t="s">
         <v>13</v>
       </c>
       <c r="D93" t="s">
+        <v>592</v>
+      </c>
+      <c r="E93" t="s">
         <v>593</v>
       </c>
-      <c r="E93" t="s">
+      <c r="F93" t="s">
+        <v>16</v>
+      </c>
+      <c r="G93" t="s">
         <v>594</v>
       </c>
-      <c r="F93" t="s">
-        <v>16</v>
-      </c>
-      <c r="G93" t="s">
+      <c r="H93" t="s">
         <v>595</v>
-      </c>
-      <c r="H93" t="s">
-        <v>596</v>
       </c>
       <c r="I93" t="s">
         <v>44</v>
       </c>
       <c r="J93" t="s">
+        <v>596</v>
+      </c>
+      <c r="K93" t="s">
         <v>597</v>
       </c>
-      <c r="K93" t="s">
-        <v>598</v>
-      </c>
       <c r="L93" t="s">
-        <v>187</v>
+        <v>47</v>
       </c>
     </row>
     <row r="94">
@@ -5840,7 +5837,7 @@
         <v>20243077</v>
       </c>
       <c r="B94" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="C94" t="s">
         <v>13</v>
@@ -5849,28 +5846,28 @@
         <v>14</v>
       </c>
       <c r="E94" t="s">
+        <v>599</v>
+      </c>
+      <c r="F94" t="s">
+        <v>16</v>
+      </c>
+      <c r="G94" t="s">
         <v>600</v>
       </c>
-      <c r="F94" t="s">
-        <v>16</v>
-      </c>
-      <c r="G94" t="s">
+      <c r="H94" t="s">
         <v>601</v>
-      </c>
-      <c r="H94" t="s">
-        <v>602</v>
       </c>
       <c r="I94" t="s">
         <v>68</v>
       </c>
       <c r="J94" t="s">
+        <v>602</v>
+      </c>
+      <c r="K94" t="s">
         <v>603</v>
       </c>
-      <c r="K94" t="s">
-        <v>604</v>
-      </c>
       <c r="L94" t="s">
-        <v>187</v>
+        <v>47</v>
       </c>
     </row>
     <row r="95">
@@ -5878,37 +5875,37 @@
         <v>20247112</v>
       </c>
       <c r="B95" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="C95" t="s">
         <v>39</v>
       </c>
       <c r="D95" t="s">
+        <v>605</v>
+      </c>
+      <c r="E95" t="s">
         <v>606</v>
       </c>
-      <c r="E95" t="s">
+      <c r="F95" t="s">
+        <v>16</v>
+      </c>
+      <c r="G95" t="s">
         <v>607</v>
       </c>
-      <c r="F95" t="s">
-        <v>16</v>
-      </c>
-      <c r="G95" t="s">
+      <c r="H95" t="s">
         <v>608</v>
-      </c>
-      <c r="H95" t="s">
-        <v>609</v>
       </c>
       <c r="I95" t="s">
         <v>44</v>
       </c>
       <c r="J95" t="s">
+        <v>609</v>
+      </c>
+      <c r="K95" t="s">
         <v>610</v>
       </c>
-      <c r="K95" t="s">
-        <v>611</v>
-      </c>
       <c r="L95" t="s">
-        <v>187</v>
+        <v>54</v>
       </c>
     </row>
     <row r="96">
@@ -5916,37 +5913,37 @@
         <v>20247015</v>
       </c>
       <c r="B96" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="C96" t="s">
         <v>39</v>
       </c>
       <c r="D96" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E96" t="s">
+        <v>612</v>
+      </c>
+      <c r="F96" t="s">
+        <v>16</v>
+      </c>
+      <c r="G96" t="s">
         <v>613</v>
       </c>
-      <c r="F96" t="s">
-        <v>16</v>
-      </c>
-      <c r="G96" t="s">
+      <c r="H96" t="s">
         <v>614</v>
-      </c>
-      <c r="H96" t="s">
-        <v>615</v>
       </c>
       <c r="I96" t="s">
         <v>44</v>
       </c>
       <c r="J96" t="s">
+        <v>615</v>
+      </c>
+      <c r="K96" t="s">
         <v>616</v>
       </c>
-      <c r="K96" t="s">
-        <v>617</v>
-      </c>
       <c r="L96" t="s">
-        <v>187</v>
+        <v>22</v>
       </c>
     </row>
     <row r="97">
@@ -5954,7 +5951,7 @@
         <v>20234494</v>
       </c>
       <c r="B97" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="C97" t="s">
         <v>32</v>
@@ -5963,28 +5960,28 @@
         <v>130</v>
       </c>
       <c r="E97" t="s">
+        <v>618</v>
+      </c>
+      <c r="F97" t="s">
+        <v>16</v>
+      </c>
+      <c r="G97" t="s">
         <v>619</v>
       </c>
-      <c r="F97" t="s">
-        <v>16</v>
-      </c>
-      <c r="G97" t="s">
+      <c r="H97" t="s">
         <v>620</v>
-      </c>
-      <c r="H97" t="s">
-        <v>621</v>
       </c>
       <c r="I97" t="s">
         <v>44</v>
       </c>
       <c r="J97" t="s">
+        <v>621</v>
+      </c>
+      <c r="K97" t="s">
         <v>622</v>
       </c>
-      <c r="K97" t="s">
-        <v>623</v>
-      </c>
       <c r="L97" t="s">
-        <v>187</v>
+        <v>22</v>
       </c>
     </row>
     <row r="98">
@@ -5992,7 +5989,7 @@
         <v>20234461</v>
       </c>
       <c r="B98" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="C98" t="s">
         <v>32</v>
@@ -6001,28 +5998,28 @@
         <v>92</v>
       </c>
       <c r="E98" t="s">
+        <v>624</v>
+      </c>
+      <c r="F98" t="s">
+        <v>16</v>
+      </c>
+      <c r="G98" t="s">
         <v>625</v>
       </c>
-      <c r="F98" t="s">
-        <v>16</v>
-      </c>
-      <c r="G98" t="s">
+      <c r="H98" t="s">
         <v>626</v>
-      </c>
-      <c r="H98" t="s">
-        <v>627</v>
       </c>
       <c r="I98" t="s">
         <v>44</v>
       </c>
       <c r="J98" t="s">
+        <v>627</v>
+      </c>
+      <c r="K98" t="s">
         <v>628</v>
       </c>
-      <c r="K98" t="s">
-        <v>629</v>
-      </c>
       <c r="L98" t="s">
-        <v>187</v>
+        <v>47</v>
       </c>
     </row>
     <row r="99">
@@ -6030,37 +6027,37 @@
         <v>20234375</v>
       </c>
       <c r="B99" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="C99" t="s">
         <v>32</v>
       </c>
       <c r="D99" t="s">
+        <v>630</v>
+      </c>
+      <c r="E99" t="s">
         <v>631</v>
       </c>
-      <c r="E99" t="s">
+      <c r="F99" t="s">
+        <v>16</v>
+      </c>
+      <c r="G99" t="s">
         <v>632</v>
       </c>
-      <c r="F99" t="s">
-        <v>16</v>
-      </c>
-      <c r="G99" t="s">
+      <c r="H99" t="s">
         <v>633</v>
-      </c>
-      <c r="H99" t="s">
-        <v>634</v>
       </c>
       <c r="I99" t="s">
         <v>44</v>
       </c>
       <c r="J99" t="s">
+        <v>634</v>
+      </c>
+      <c r="K99" t="s">
         <v>635</v>
       </c>
-      <c r="K99" t="s">
-        <v>636</v>
-      </c>
       <c r="L99" t="s">
-        <v>187</v>
+        <v>22</v>
       </c>
     </row>
     <row r="100">
@@ -6068,37 +6065,37 @@
         <v>20234353</v>
       </c>
       <c r="B100" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="C100" t="s">
         <v>32</v>
       </c>
       <c r="D100" t="s">
+        <v>637</v>
+      </c>
+      <c r="E100" t="s">
         <v>638</v>
       </c>
-      <c r="E100" t="s">
+      <c r="F100" t="s">
+        <v>16</v>
+      </c>
+      <c r="G100" t="s">
         <v>639</v>
       </c>
-      <c r="F100" t="s">
-        <v>16</v>
-      </c>
-      <c r="G100" t="s">
+      <c r="H100" t="s">
         <v>640</v>
-      </c>
-      <c r="H100" t="s">
-        <v>641</v>
       </c>
       <c r="I100" t="s">
         <v>44</v>
       </c>
       <c r="J100" t="s">
+        <v>641</v>
+      </c>
+      <c r="K100" t="s">
         <v>642</v>
       </c>
-      <c r="K100" t="s">
-        <v>643</v>
-      </c>
       <c r="L100" t="s">
-        <v>187</v>
+        <v>47</v>
       </c>
     </row>
     <row r="101">
@@ -6106,35 +6103,35 @@
         <v>20234346</v>
       </c>
       <c r="B101" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="C101" t="s">
         <v>13</v>
       </c>
       <c r="D101"/>
       <c r="E101" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="F101" t="s">
         <v>26</v>
       </c>
       <c r="G101" t="s">
+        <v>645</v>
+      </c>
+      <c r="H101" t="s">
         <v>646</v>
-      </c>
-      <c r="H101" t="s">
-        <v>647</v>
       </c>
       <c r="I101" t="s">
         <v>44</v>
       </c>
       <c r="J101" t="s">
+        <v>647</v>
+      </c>
+      <c r="K101" t="s">
         <v>648</v>
       </c>
-      <c r="K101" t="s">
-        <v>649</v>
-      </c>
       <c r="L101" t="s">
-        <v>187</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ajout des noms de commissions pour les objets parlementaires déposés par une commission
- Récupération automatique du nom de la commission via BusinessRole et Committee
- Les objets sans auteur (SubmittedBy = NA) sont maintenant complétés avec le nom de la commission
- Recalcul automatique des objets existants sans auteur
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_CDF_EFK.xlsx
+++ b/Objets_parlementaires_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="649">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="655" uniqueCount="655">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -803,6 +803,9 @@
     <t xml:space="preserve">25.3425</t>
   </si>
   <si>
+    <t xml:space="preserve">Commission des finances Conseil national</t>
+  </si>
+  <si>
     <t xml:space="preserve">2025-04-04</t>
   </si>
   <si>
@@ -1151,6 +1154,9 @@
     <t xml:space="preserve">25.3008</t>
   </si>
   <si>
+    <t xml:space="preserve">Commission de l'économie et des redevances Conseil national</t>
+  </si>
+  <si>
     <t xml:space="preserve">2025-01-21</t>
   </si>
   <si>
@@ -1679,6 +1685,9 @@
     <t xml:space="preserve">24.3471</t>
   </si>
   <si>
+    <t xml:space="preserve">Commission de la sécurité sociale et de la santé publique Conseil national</t>
+  </si>
+  <si>
     <t xml:space="preserve">2024-05-02</t>
   </si>
   <si>
@@ -1697,6 +1706,9 @@
     <t xml:space="preserve">24.3468</t>
   </si>
   <si>
+    <t xml:space="preserve">Commission des transports et des télécommunications Conseil national</t>
+  </si>
+  <si>
     <t xml:space="preserve">2024-04-30</t>
   </si>
   <si>
@@ -1715,6 +1727,9 @@
     <t xml:space="preserve">24.3467</t>
   </si>
   <si>
+    <t xml:space="preserve">Commission de la politique de sécurité Conseil des États</t>
+  </si>
+  <si>
     <t xml:space="preserve">2024-04-25</t>
   </si>
   <si>
@@ -1944,6 +1959,9 @@
   </si>
   <si>
     <t xml:space="preserve">23.4346</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commission des institutions politiques Conseil des États</t>
   </si>
   <si>
     <t xml:space="preserve">2023-11-20</t>
@@ -3762,27 +3780,29 @@
       <c r="C39" t="s">
         <v>13</v>
       </c>
-      <c r="D39"/>
+      <c r="D39" t="s">
+        <v>263</v>
+      </c>
       <c r="E39" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="F39" t="s">
         <v>16</v>
       </c>
       <c r="G39" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="H39" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="I39" t="s">
         <v>68</v>
       </c>
       <c r="J39" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="K39" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="L39" t="s">
         <v>22</v>
@@ -3793,7 +3813,7 @@
         <v>20253309</v>
       </c>
       <c r="B40" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C40" t="s">
         <v>13</v>
@@ -3802,25 +3822,25 @@
         <v>124</v>
       </c>
       <c r="E40" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="F40" t="s">
         <v>16</v>
       </c>
       <c r="G40" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="H40" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="I40" t="s">
         <v>68</v>
       </c>
       <c r="J40" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="K40" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="L40" t="s">
         <v>22</v>
@@ -3831,34 +3851,34 @@
         <v>20253399</v>
       </c>
       <c r="B41" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C41" t="s">
         <v>32</v>
       </c>
       <c r="D41" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E41" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="F41" t="s">
         <v>16</v>
       </c>
       <c r="G41" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="H41" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="I41" t="s">
         <v>68</v>
       </c>
       <c r="J41" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="K41" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="L41" t="s">
         <v>54</v>
@@ -3869,34 +3889,34 @@
         <v>20253404</v>
       </c>
       <c r="B42" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C42" t="s">
         <v>13</v>
       </c>
       <c r="D42" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E42" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="F42" t="s">
         <v>16</v>
       </c>
       <c r="G42" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="H42" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="I42" t="s">
         <v>68</v>
       </c>
       <c r="J42" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="K42" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="L42" t="s">
         <v>47</v>
@@ -3907,34 +3927,34 @@
         <v>20253417</v>
       </c>
       <c r="B43" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C43" t="s">
         <v>13</v>
       </c>
       <c r="D43" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="E43" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="F43" t="s">
         <v>16</v>
       </c>
       <c r="G43" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="H43" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="I43" t="s">
         <v>68</v>
       </c>
       <c r="J43" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="K43" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="L43" t="s">
         <v>47</v>
@@ -3945,34 +3965,34 @@
         <v>20251011</v>
       </c>
       <c r="B44" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C44" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D44" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="E44" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F44" t="s">
         <v>26</v>
       </c>
       <c r="G44" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="H44" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="I44" t="s">
         <v>44</v>
       </c>
       <c r="J44" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="K44" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="L44" t="s">
         <v>47</v>
@@ -3983,34 +4003,34 @@
         <v>20253194</v>
       </c>
       <c r="B45" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C45" t="s">
         <v>32</v>
       </c>
       <c r="D45" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="E45" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F45" t="s">
         <v>26</v>
       </c>
       <c r="G45" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="H45" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="I45" t="s">
         <v>44</v>
       </c>
       <c r="J45" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="K45" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="L45" t="s">
         <v>47</v>
@@ -4021,34 +4041,34 @@
         <v>20253203</v>
       </c>
       <c r="B46" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C46" t="s">
         <v>32</v>
       </c>
       <c r="D46" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E46" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F46" t="s">
         <v>16</v>
       </c>
       <c r="G46" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="H46" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="I46" t="s">
         <v>44</v>
       </c>
       <c r="J46" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="K46" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="L46" t="s">
         <v>54</v>
@@ -4059,34 +4079,34 @@
         <v>20253213</v>
       </c>
       <c r="B47" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C47" t="s">
         <v>32</v>
       </c>
       <c r="D47" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E47" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F47" t="s">
         <v>26</v>
       </c>
       <c r="G47" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="H47" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="I47" t="s">
         <v>44</v>
       </c>
       <c r="J47" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="K47" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="L47" t="s">
         <v>47</v>
@@ -4097,34 +4117,34 @@
         <v>20253214</v>
       </c>
       <c r="B48" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C48" t="s">
         <v>32</v>
       </c>
       <c r="D48" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E48" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F48" t="s">
         <v>16</v>
       </c>
       <c r="G48" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="H48" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="I48" t="s">
         <v>44</v>
       </c>
       <c r="J48" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="K48" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="L48" t="s">
         <v>47</v>
@@ -4135,34 +4155,34 @@
         <v>20253246</v>
       </c>
       <c r="B49" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C49" t="s">
         <v>13</v>
       </c>
       <c r="D49" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="E49" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F49" t="s">
         <v>16</v>
       </c>
       <c r="G49" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="H49" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="I49" t="s">
         <v>145</v>
       </c>
       <c r="J49" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="K49" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="L49" t="s">
         <v>22</v>
@@ -4173,34 +4193,34 @@
         <v>20253093</v>
       </c>
       <c r="B50" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C50" t="s">
         <v>32</v>
       </c>
       <c r="D50" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="E50" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="F50" t="s">
         <v>16</v>
       </c>
       <c r="G50" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="H50" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="I50" t="s">
         <v>68</v>
       </c>
       <c r="J50" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="K50" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="L50" t="s">
         <v>22</v>
@@ -4211,34 +4231,34 @@
         <v>20257213</v>
       </c>
       <c r="B51" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C51" t="s">
         <v>39</v>
       </c>
       <c r="D51" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E51" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="F51" t="s">
         <v>16</v>
       </c>
       <c r="G51" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="H51" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="I51" t="s">
         <v>44</v>
       </c>
       <c r="J51" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="K51" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="L51" t="s">
         <v>22</v>
@@ -4249,34 +4269,34 @@
         <v>20253054</v>
       </c>
       <c r="B52" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C52" t="s">
         <v>13</v>
       </c>
       <c r="D52" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="E52" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="F52" t="s">
         <v>16</v>
       </c>
       <c r="G52" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="H52" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="I52" t="s">
         <v>68</v>
       </c>
       <c r="J52" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="K52" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="L52" t="s">
         <v>47</v>
@@ -4287,7 +4307,7 @@
         <v>20257102</v>
       </c>
       <c r="B53" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C53" t="s">
         <v>39</v>
@@ -4296,25 +4316,25 @@
         <v>111</v>
       </c>
       <c r="E53" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="F53" t="s">
         <v>16</v>
       </c>
       <c r="G53" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="H53" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="I53" t="s">
         <v>44</v>
       </c>
       <c r="J53" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="K53" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="L53" t="s">
         <v>47</v>
@@ -4325,7 +4345,7 @@
         <v>20257129</v>
       </c>
       <c r="B54" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C54" t="s">
         <v>39</v>
@@ -4334,25 +4354,25 @@
         <v>256</v>
       </c>
       <c r="E54" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="F54" t="s">
         <v>16</v>
       </c>
       <c r="G54" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="H54" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="I54" t="s">
         <v>44</v>
       </c>
       <c r="J54" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="K54" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="L54" t="s">
         <v>22</v>
@@ -4363,34 +4383,34 @@
         <v>20257138</v>
       </c>
       <c r="B55" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C55" t="s">
         <v>39</v>
       </c>
       <c r="D55" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="E55" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="F55" t="s">
         <v>16</v>
       </c>
       <c r="G55" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="H55" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="I55" t="s">
         <v>44</v>
       </c>
       <c r="J55" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="K55" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="L55" t="s">
         <v>47</v>
@@ -4401,34 +4421,34 @@
         <v>20253031</v>
       </c>
       <c r="B56" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C56" t="s">
         <v>32</v>
       </c>
       <c r="D56" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="E56" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="F56" t="s">
         <v>16</v>
       </c>
       <c r="G56" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="H56" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="I56" t="s">
         <v>68</v>
       </c>
       <c r="J56" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="K56" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="L56" t="s">
         <v>47</v>
@@ -4439,34 +4459,34 @@
         <v>20257012</v>
       </c>
       <c r="B57" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C57" t="s">
         <v>39</v>
       </c>
       <c r="D57" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="E57" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="F57" t="s">
         <v>16</v>
       </c>
       <c r="G57" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="H57" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="I57" t="s">
         <v>44</v>
       </c>
       <c r="J57" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="K57" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="L57" t="s">
         <v>54</v>
@@ -4477,32 +4497,34 @@
         <v>20253008</v>
       </c>
       <c r="B58" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C58" t="s">
         <v>13</v>
       </c>
-      <c r="D58"/>
+      <c r="D58" t="s">
+        <v>380</v>
+      </c>
       <c r="E58" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="F58" t="s">
         <v>16</v>
       </c>
       <c r="G58" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="H58" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="I58" t="s">
         <v>44</v>
       </c>
       <c r="J58" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="K58" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="L58" t="s">
         <v>47</v>
@@ -4513,34 +4535,34 @@
         <v>20244404</v>
       </c>
       <c r="B59" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="C59" t="s">
         <v>32</v>
       </c>
       <c r="D59" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="E59" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="F59" t="s">
         <v>16</v>
       </c>
       <c r="G59" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="H59" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="I59" t="s">
         <v>44</v>
       </c>
       <c r="J59" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="K59" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="L59" t="s">
         <v>47</v>
@@ -4551,7 +4573,7 @@
         <v>20244419</v>
       </c>
       <c r="B60" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="C60" t="s">
         <v>32</v>
@@ -4560,25 +4582,25 @@
         <v>222</v>
       </c>
       <c r="E60" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="F60" t="s">
         <v>26</v>
       </c>
       <c r="G60" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="H60" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="I60" t="s">
         <v>44</v>
       </c>
       <c r="J60" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="K60" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="L60" t="s">
         <v>47</v>
@@ -4589,34 +4611,34 @@
         <v>20247975</v>
       </c>
       <c r="B61" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="C61" t="s">
         <v>39</v>
       </c>
       <c r="D61" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="E61" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="F61" t="s">
         <v>16</v>
       </c>
       <c r="G61" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="H61" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="I61" t="s">
         <v>44</v>
       </c>
       <c r="J61" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="K61" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="L61" t="s">
         <v>22</v>
@@ -4627,34 +4649,34 @@
         <v>20248043</v>
       </c>
       <c r="B62" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="C62" t="s">
         <v>39</v>
       </c>
       <c r="D62" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="E62" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="F62" t="s">
         <v>16</v>
       </c>
       <c r="G62" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="H62" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="I62" t="s">
         <v>44</v>
       </c>
       <c r="J62" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="K62" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="L62" t="s">
         <v>22</v>
@@ -4665,34 +4687,34 @@
         <v>20244290</v>
       </c>
       <c r="B63" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="C63" t="s">
         <v>32</v>
       </c>
       <c r="D63" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="E63" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="F63" t="s">
         <v>16</v>
       </c>
       <c r="G63" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="H63" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="I63" t="s">
         <v>68</v>
       </c>
       <c r="J63" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="K63" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="L63" t="s">
         <v>47</v>
@@ -4703,34 +4725,34 @@
         <v>20244278</v>
       </c>
       <c r="B64" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="C64" t="s">
         <v>32</v>
       </c>
       <c r="D64" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="E64" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="F64" t="s">
         <v>16</v>
       </c>
       <c r="G64" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="H64" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="I64" t="s">
         <v>68</v>
       </c>
       <c r="J64" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="K64" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="L64" t="s">
         <v>22</v>
@@ -4741,34 +4763,34 @@
         <v>20244082</v>
       </c>
       <c r="B65" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="C65" t="s">
         <v>32</v>
       </c>
       <c r="D65" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="E65" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="F65" t="s">
         <v>16</v>
       </c>
       <c r="G65" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="H65" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="I65" t="s">
         <v>68</v>
       </c>
       <c r="J65" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="K65" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="L65" t="s">
         <v>47</v>
@@ -4779,34 +4801,34 @@
         <v>20244112</v>
       </c>
       <c r="B66" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="C66" t="s">
         <v>32</v>
       </c>
       <c r="D66" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="E66" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="F66" t="s">
         <v>16</v>
       </c>
       <c r="G66" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="H66" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="I66" t="s">
         <v>68</v>
       </c>
       <c r="J66" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="K66" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="L66" t="s">
         <v>54</v>
@@ -4817,7 +4839,7 @@
         <v>20244131</v>
       </c>
       <c r="B67" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="C67" t="s">
         <v>32</v>
@@ -4826,25 +4848,25 @@
         <v>49</v>
       </c>
       <c r="E67" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="F67" t="s">
         <v>16</v>
       </c>
       <c r="G67" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="H67" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="I67" t="s">
         <v>68</v>
       </c>
       <c r="J67" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="K67" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="L67" t="s">
         <v>47</v>
@@ -4855,7 +4877,7 @@
         <v>20244132</v>
       </c>
       <c r="B68" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="C68" t="s">
         <v>63</v>
@@ -4864,25 +4886,25 @@
         <v>124</v>
       </c>
       <c r="E68" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="F68" t="s">
         <v>16</v>
       </c>
       <c r="G68" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="H68" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="I68" t="s">
         <v>68</v>
       </c>
       <c r="J68" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="K68" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="L68" t="s">
         <v>54</v>
@@ -4893,7 +4915,7 @@
         <v>20244133</v>
       </c>
       <c r="B69" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="C69" t="s">
         <v>13</v>
@@ -4902,25 +4924,25 @@
         <v>124</v>
       </c>
       <c r="E69" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="F69" t="s">
         <v>16</v>
       </c>
       <c r="G69" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="H69" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="I69" t="s">
         <v>68</v>
       </c>
       <c r="J69" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="K69" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="L69" t="s">
         <v>54</v>
@@ -4931,34 +4953,34 @@
         <v>20244137</v>
       </c>
       <c r="B70" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="C70" t="s">
         <v>32</v>
       </c>
       <c r="D70" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="E70" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="F70" t="s">
         <v>16</v>
       </c>
       <c r="G70" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="H70" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="I70" t="s">
         <v>68</v>
       </c>
       <c r="J70" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="K70" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="L70" t="s">
         <v>54</v>
@@ -4969,34 +4991,34 @@
         <v>20243937</v>
       </c>
       <c r="B71" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="C71" t="s">
         <v>13</v>
       </c>
       <c r="D71" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="E71" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="F71" t="s">
         <v>26</v>
       </c>
       <c r="G71" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="H71" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="I71" t="s">
         <v>177</v>
       </c>
       <c r="J71" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="K71" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="L71" t="s">
         <v>22</v>
@@ -5007,34 +5029,34 @@
         <v>20243948</v>
       </c>
       <c r="B72" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="C72" t="s">
         <v>32</v>
       </c>
       <c r="D72" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="E72" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="F72" t="s">
         <v>26</v>
       </c>
       <c r="G72" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="H72" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="I72" t="s">
         <v>44</v>
       </c>
       <c r="J72" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="K72" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="L72" t="s">
         <v>47</v>
@@ -5045,7 +5067,7 @@
         <v>20247720</v>
       </c>
       <c r="B73" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="C73" t="s">
         <v>39</v>
@@ -5054,25 +5076,25 @@
         <v>256</v>
       </c>
       <c r="E73" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="F73" t="s">
         <v>16</v>
       </c>
       <c r="G73" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="H73" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="I73" t="s">
         <v>44</v>
       </c>
       <c r="J73" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="K73" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="L73" t="s">
         <v>22</v>
@@ -5083,34 +5105,34 @@
         <v>20247726</v>
       </c>
       <c r="B74" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="C74" t="s">
         <v>39</v>
       </c>
       <c r="D74" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="E74" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="F74" t="s">
         <v>16</v>
       </c>
       <c r="G74" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="H74" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="I74" t="s">
         <v>44</v>
       </c>
       <c r="J74" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="K74" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="L74" t="s">
         <v>47</v>
@@ -5121,7 +5143,7 @@
         <v>20247773</v>
       </c>
       <c r="B75" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C75" t="s">
         <v>39</v>
@@ -5130,25 +5152,25 @@
         <v>118</v>
       </c>
       <c r="E75" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="F75" t="s">
         <v>16</v>
       </c>
       <c r="G75" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="H75" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="I75" t="s">
         <v>44</v>
       </c>
       <c r="J75" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="K75" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="L75" t="s">
         <v>54</v>
@@ -5159,7 +5181,7 @@
         <v>20247774</v>
       </c>
       <c r="B76" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="C76" t="s">
         <v>39</v>
@@ -5168,25 +5190,25 @@
         <v>118</v>
       </c>
       <c r="E76" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="F76" t="s">
         <v>16</v>
       </c>
       <c r="G76" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="H76" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="I76" t="s">
         <v>44</v>
       </c>
       <c r="J76" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="K76" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="L76" t="s">
         <v>54</v>
@@ -5197,34 +5219,34 @@
         <v>20243858</v>
       </c>
       <c r="B77" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="C77" t="s">
         <v>32</v>
       </c>
       <c r="D77" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="E77" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="F77" t="s">
         <v>16</v>
       </c>
       <c r="G77" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="H77" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="I77" t="s">
         <v>68</v>
       </c>
       <c r="J77" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="K77" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="L77" t="s">
         <v>22</v>
@@ -5235,34 +5257,34 @@
         <v>20243877</v>
       </c>
       <c r="B78" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="C78" t="s">
         <v>32</v>
       </c>
       <c r="D78" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="E78" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="F78" t="s">
         <v>16</v>
       </c>
       <c r="G78" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="H78" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="I78" t="s">
         <v>68</v>
       </c>
       <c r="J78" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="K78" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="L78" t="s">
         <v>47</v>
@@ -5273,7 +5295,7 @@
         <v>20247622</v>
       </c>
       <c r="B79" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="C79" t="s">
         <v>39</v>
@@ -5282,25 +5304,25 @@
         <v>49</v>
       </c>
       <c r="E79" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="F79" t="s">
         <v>16</v>
       </c>
       <c r="G79" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="H79" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="I79" t="s">
         <v>44</v>
       </c>
       <c r="J79" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="K79" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="L79" t="s">
         <v>47</v>
@@ -5311,34 +5333,34 @@
         <v>20247649</v>
       </c>
       <c r="B80" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="C80" t="s">
         <v>39</v>
       </c>
       <c r="D80" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="E80" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="F80" t="s">
         <v>16</v>
       </c>
       <c r="G80" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="H80" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="I80" t="s">
         <v>44</v>
       </c>
       <c r="J80" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="K80" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="L80" t="s">
         <v>47</v>
@@ -5349,34 +5371,34 @@
         <v>20243709</v>
       </c>
       <c r="B81" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="C81" t="s">
         <v>32</v>
       </c>
       <c r="D81" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="E81" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="F81" t="s">
         <v>16</v>
       </c>
       <c r="G81" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="H81" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="I81" t="s">
         <v>68</v>
       </c>
       <c r="J81" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="K81" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="L81" t="s">
         <v>54</v>
@@ -5387,34 +5409,34 @@
         <v>20243773</v>
       </c>
       <c r="B82" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="C82" t="s">
         <v>32</v>
       </c>
       <c r="D82" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="E82" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="F82" t="s">
         <v>16</v>
       </c>
       <c r="G82" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="H82" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="I82" t="s">
         <v>68</v>
       </c>
       <c r="J82" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="K82" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="L82" t="s">
         <v>47</v>
@@ -5425,34 +5447,34 @@
         <v>20243776</v>
       </c>
       <c r="B83" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="C83" t="s">
         <v>13</v>
       </c>
       <c r="D83" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="E83" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="F83" t="s">
         <v>16</v>
       </c>
       <c r="G83" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="H83" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="I83" t="s">
         <v>44</v>
       </c>
       <c r="J83" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="K83" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="L83" t="s">
         <v>22</v>
@@ -5463,34 +5485,34 @@
         <v>20243609</v>
       </c>
       <c r="B84" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="C84" t="s">
         <v>13</v>
       </c>
       <c r="D84" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="E84" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="F84" t="s">
         <v>16</v>
       </c>
       <c r="G84" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="H84" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="I84" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="J84" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="K84" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="L84" t="s">
         <v>47</v>
@@ -5501,7 +5523,7 @@
         <v>20243574</v>
       </c>
       <c r="B85" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="C85" t="s">
         <v>32</v>
@@ -5510,25 +5532,25 @@
         <v>229</v>
       </c>
       <c r="E85" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="F85" t="s">
         <v>26</v>
       </c>
       <c r="G85" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="H85" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="I85" t="s">
         <v>44</v>
       </c>
       <c r="J85" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="K85" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="L85" t="s">
         <v>22</v>
@@ -5539,34 +5561,34 @@
         <v>20243557</v>
       </c>
       <c r="B86" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="C86" t="s">
         <v>32</v>
       </c>
       <c r="D86" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E86" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="F86" t="s">
         <v>16</v>
       </c>
       <c r="G86" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="H86" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="I86" t="s">
         <v>44</v>
       </c>
       <c r="J86" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="K86" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="L86" t="s">
         <v>47</v>
@@ -5577,32 +5599,34 @@
         <v>20243471</v>
       </c>
       <c r="B87" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="C87" t="s">
         <v>13</v>
       </c>
-      <c r="D87"/>
+      <c r="D87" t="s">
+        <v>557</v>
+      </c>
       <c r="E87" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="F87" t="s">
         <v>16</v>
       </c>
       <c r="G87" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
       <c r="H87" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="I87" t="s">
         <v>44</v>
       </c>
       <c r="J87" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="K87" t="s">
-        <v>559</v>
+        <v>562</v>
       </c>
       <c r="L87" t="s">
         <v>22</v>
@@ -5613,32 +5637,34 @@
         <v>20243468</v>
       </c>
       <c r="B88" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="C88" t="s">
         <v>63</v>
       </c>
-      <c r="D88"/>
+      <c r="D88" t="s">
+        <v>564</v>
+      </c>
       <c r="E88" t="s">
-        <v>561</v>
+        <v>565</v>
       </c>
       <c r="F88" t="s">
         <v>16</v>
       </c>
       <c r="G88" t="s">
-        <v>562</v>
+        <v>566</v>
       </c>
       <c r="H88" t="s">
-        <v>563</v>
+        <v>567</v>
       </c>
       <c r="I88" t="s">
         <v>177</v>
       </c>
       <c r="J88" t="s">
-        <v>564</v>
+        <v>568</v>
       </c>
       <c r="K88" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
       <c r="L88" t="s">
         <v>47</v>
@@ -5649,32 +5675,34 @@
         <v>20243467</v>
       </c>
       <c r="B89" t="s">
-        <v>566</v>
+        <v>570</v>
       </c>
       <c r="C89" t="s">
         <v>13</v>
       </c>
-      <c r="D89"/>
+      <c r="D89" t="s">
+        <v>571</v>
+      </c>
       <c r="E89" t="s">
-        <v>567</v>
+        <v>572</v>
       </c>
       <c r="F89" t="s">
         <v>26</v>
       </c>
       <c r="G89" t="s">
-        <v>568</v>
+        <v>573</v>
       </c>
       <c r="H89" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="I89" t="s">
         <v>44</v>
       </c>
       <c r="J89" t="s">
-        <v>570</v>
+        <v>575</v>
       </c>
       <c r="K89" t="s">
-        <v>571</v>
+        <v>576</v>
       </c>
       <c r="L89" t="s">
         <v>47</v>
@@ -5685,34 +5713,34 @@
         <v>20243318</v>
       </c>
       <c r="B90" t="s">
-        <v>572</v>
+        <v>577</v>
       </c>
       <c r="C90" t="s">
         <v>32</v>
       </c>
       <c r="D90" t="s">
-        <v>573</v>
+        <v>578</v>
       </c>
       <c r="E90" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="F90" t="s">
         <v>16</v>
       </c>
       <c r="G90" t="s">
-        <v>575</v>
+        <v>580</v>
       </c>
       <c r="H90" t="s">
-        <v>576</v>
+        <v>581</v>
       </c>
       <c r="I90" t="s">
         <v>68</v>
       </c>
       <c r="J90" t="s">
-        <v>577</v>
+        <v>582</v>
       </c>
       <c r="K90" t="s">
-        <v>578</v>
+        <v>583</v>
       </c>
       <c r="L90" t="s">
         <v>54</v>
@@ -5723,34 +5751,34 @@
         <v>20243234</v>
       </c>
       <c r="B91" t="s">
-        <v>579</v>
+        <v>584</v>
       </c>
       <c r="C91" t="s">
         <v>13</v>
       </c>
       <c r="D91" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="E91" t="s">
-        <v>580</v>
+        <v>585</v>
       </c>
       <c r="F91" t="s">
         <v>16</v>
       </c>
       <c r="G91" t="s">
-        <v>581</v>
+        <v>586</v>
       </c>
       <c r="H91" t="s">
-        <v>582</v>
+        <v>587</v>
       </c>
       <c r="I91" t="s">
         <v>44</v>
       </c>
       <c r="J91" t="s">
-        <v>583</v>
+        <v>588</v>
       </c>
       <c r="K91" t="s">
-        <v>584</v>
+        <v>589</v>
       </c>
       <c r="L91" t="s">
         <v>47</v>
@@ -5761,34 +5789,34 @@
         <v>20243259</v>
       </c>
       <c r="B92" t="s">
-        <v>585</v>
+        <v>590</v>
       </c>
       <c r="C92" t="s">
         <v>32</v>
       </c>
       <c r="D92" t="s">
-        <v>586</v>
+        <v>591</v>
       </c>
       <c r="E92" t="s">
-        <v>580</v>
+        <v>585</v>
       </c>
       <c r="F92" t="s">
         <v>16</v>
       </c>
       <c r="G92" t="s">
-        <v>587</v>
+        <v>592</v>
       </c>
       <c r="H92" t="s">
-        <v>588</v>
+        <v>593</v>
       </c>
       <c r="I92" t="s">
         <v>44</v>
       </c>
       <c r="J92" t="s">
-        <v>589</v>
+        <v>594</v>
       </c>
       <c r="K92" t="s">
-        <v>590</v>
+        <v>595</v>
       </c>
       <c r="L92" t="s">
         <v>47</v>
@@ -5799,34 +5827,34 @@
         <v>20243169</v>
       </c>
       <c r="B93" t="s">
-        <v>591</v>
+        <v>596</v>
       </c>
       <c r="C93" t="s">
         <v>13</v>
       </c>
       <c r="D93" t="s">
-        <v>592</v>
+        <v>597</v>
       </c>
       <c r="E93" t="s">
-        <v>593</v>
+        <v>598</v>
       </c>
       <c r="F93" t="s">
         <v>16</v>
       </c>
       <c r="G93" t="s">
-        <v>594</v>
+        <v>599</v>
       </c>
       <c r="H93" t="s">
-        <v>595</v>
+        <v>600</v>
       </c>
       <c r="I93" t="s">
         <v>44</v>
       </c>
       <c r="J93" t="s">
-        <v>596</v>
+        <v>601</v>
       </c>
       <c r="K93" t="s">
-        <v>597</v>
+        <v>602</v>
       </c>
       <c r="L93" t="s">
         <v>47</v>
@@ -5837,7 +5865,7 @@
         <v>20243077</v>
       </c>
       <c r="B94" t="s">
-        <v>598</v>
+        <v>603</v>
       </c>
       <c r="C94" t="s">
         <v>13</v>
@@ -5846,25 +5874,25 @@
         <v>14</v>
       </c>
       <c r="E94" t="s">
-        <v>599</v>
+        <v>604</v>
       </c>
       <c r="F94" t="s">
         <v>16</v>
       </c>
       <c r="G94" t="s">
-        <v>600</v>
+        <v>605</v>
       </c>
       <c r="H94" t="s">
-        <v>601</v>
+        <v>606</v>
       </c>
       <c r="I94" t="s">
         <v>68</v>
       </c>
       <c r="J94" t="s">
-        <v>602</v>
+        <v>607</v>
       </c>
       <c r="K94" t="s">
-        <v>603</v>
+        <v>608</v>
       </c>
       <c r="L94" t="s">
         <v>47</v>
@@ -5875,34 +5903,34 @@
         <v>20247112</v>
       </c>
       <c r="B95" t="s">
-        <v>604</v>
+        <v>609</v>
       </c>
       <c r="C95" t="s">
         <v>39</v>
       </c>
       <c r="D95" t="s">
-        <v>605</v>
+        <v>610</v>
       </c>
       <c r="E95" t="s">
-        <v>606</v>
+        <v>611</v>
       </c>
       <c r="F95" t="s">
         <v>16</v>
       </c>
       <c r="G95" t="s">
-        <v>607</v>
+        <v>612</v>
       </c>
       <c r="H95" t="s">
-        <v>608</v>
+        <v>613</v>
       </c>
       <c r="I95" t="s">
         <v>44</v>
       </c>
       <c r="J95" t="s">
-        <v>609</v>
+        <v>614</v>
       </c>
       <c r="K95" t="s">
-        <v>610</v>
+        <v>615</v>
       </c>
       <c r="L95" t="s">
         <v>54</v>
@@ -5913,7 +5941,7 @@
         <v>20247015</v>
       </c>
       <c r="B96" t="s">
-        <v>611</v>
+        <v>616</v>
       </c>
       <c r="C96" t="s">
         <v>39</v>
@@ -5922,25 +5950,25 @@
         <v>256</v>
       </c>
       <c r="E96" t="s">
-        <v>612</v>
+        <v>617</v>
       </c>
       <c r="F96" t="s">
         <v>16</v>
       </c>
       <c r="G96" t="s">
-        <v>613</v>
+        <v>618</v>
       </c>
       <c r="H96" t="s">
-        <v>614</v>
+        <v>619</v>
       </c>
       <c r="I96" t="s">
         <v>44</v>
       </c>
       <c r="J96" t="s">
-        <v>615</v>
+        <v>620</v>
       </c>
       <c r="K96" t="s">
-        <v>616</v>
+        <v>621</v>
       </c>
       <c r="L96" t="s">
         <v>22</v>
@@ -5951,7 +5979,7 @@
         <v>20234494</v>
       </c>
       <c r="B97" t="s">
-        <v>617</v>
+        <v>622</v>
       </c>
       <c r="C97" t="s">
         <v>32</v>
@@ -5960,25 +5988,25 @@
         <v>130</v>
       </c>
       <c r="E97" t="s">
-        <v>618</v>
+        <v>623</v>
       </c>
       <c r="F97" t="s">
         <v>16</v>
       </c>
       <c r="G97" t="s">
-        <v>619</v>
+        <v>624</v>
       </c>
       <c r="H97" t="s">
-        <v>620</v>
+        <v>625</v>
       </c>
       <c r="I97" t="s">
         <v>44</v>
       </c>
       <c r="J97" t="s">
-        <v>621</v>
+        <v>626</v>
       </c>
       <c r="K97" t="s">
-        <v>622</v>
+        <v>627</v>
       </c>
       <c r="L97" t="s">
         <v>22</v>
@@ -5989,7 +6017,7 @@
         <v>20234461</v>
       </c>
       <c r="B98" t="s">
-        <v>623</v>
+        <v>628</v>
       </c>
       <c r="C98" t="s">
         <v>32</v>
@@ -5998,25 +6026,25 @@
         <v>92</v>
       </c>
       <c r="E98" t="s">
-        <v>624</v>
+        <v>629</v>
       </c>
       <c r="F98" t="s">
         <v>16</v>
       </c>
       <c r="G98" t="s">
-        <v>625</v>
+        <v>630</v>
       </c>
       <c r="H98" t="s">
-        <v>626</v>
+        <v>631</v>
       </c>
       <c r="I98" t="s">
         <v>44</v>
       </c>
       <c r="J98" t="s">
-        <v>627</v>
+        <v>632</v>
       </c>
       <c r="K98" t="s">
-        <v>628</v>
+        <v>633</v>
       </c>
       <c r="L98" t="s">
         <v>47</v>
@@ -6027,34 +6055,34 @@
         <v>20234375</v>
       </c>
       <c r="B99" t="s">
-        <v>629</v>
+        <v>634</v>
       </c>
       <c r="C99" t="s">
         <v>32</v>
       </c>
       <c r="D99" t="s">
-        <v>630</v>
+        <v>635</v>
       </c>
       <c r="E99" t="s">
-        <v>631</v>
+        <v>636</v>
       </c>
       <c r="F99" t="s">
         <v>16</v>
       </c>
       <c r="G99" t="s">
-        <v>632</v>
+        <v>637</v>
       </c>
       <c r="H99" t="s">
-        <v>633</v>
+        <v>638</v>
       </c>
       <c r="I99" t="s">
         <v>44</v>
       </c>
       <c r="J99" t="s">
-        <v>634</v>
+        <v>639</v>
       </c>
       <c r="K99" t="s">
-        <v>635</v>
+        <v>640</v>
       </c>
       <c r="L99" t="s">
         <v>22</v>
@@ -6065,34 +6093,34 @@
         <v>20234353</v>
       </c>
       <c r="B100" t="s">
-        <v>636</v>
+        <v>641</v>
       </c>
       <c r="C100" t="s">
         <v>32</v>
       </c>
       <c r="D100" t="s">
-        <v>637</v>
+        <v>642</v>
       </c>
       <c r="E100" t="s">
-        <v>638</v>
+        <v>643</v>
       </c>
       <c r="F100" t="s">
         <v>16</v>
       </c>
       <c r="G100" t="s">
-        <v>639</v>
+        <v>644</v>
       </c>
       <c r="H100" t="s">
-        <v>640</v>
+        <v>645</v>
       </c>
       <c r="I100" t="s">
         <v>44</v>
       </c>
       <c r="J100" t="s">
-        <v>641</v>
+        <v>646</v>
       </c>
       <c r="K100" t="s">
-        <v>642</v>
+        <v>647</v>
       </c>
       <c r="L100" t="s">
         <v>47</v>
@@ -6103,32 +6131,34 @@
         <v>20234346</v>
       </c>
       <c r="B101" t="s">
-        <v>643</v>
+        <v>648</v>
       </c>
       <c r="C101" t="s">
         <v>13</v>
       </c>
-      <c r="D101"/>
+      <c r="D101" t="s">
+        <v>649</v>
+      </c>
       <c r="E101" t="s">
-        <v>644</v>
+        <v>650</v>
       </c>
       <c r="F101" t="s">
         <v>26</v>
       </c>
       <c r="G101" t="s">
-        <v>645</v>
+        <v>651</v>
       </c>
       <c r="H101" t="s">
-        <v>646</v>
+        <v>652</v>
       </c>
       <c r="I101" t="s">
         <v>44</v>
       </c>
       <c r="J101" t="s">
-        <v>647</v>
+        <v>653</v>
       </c>
       <c r="K101" t="s">
-        <v>648</v>
+        <v>654</v>
       </c>
       <c r="L101" t="s">
         <v>22</v>

</xml_diff>

<commit_message>
Mise à jour données parlement - 2026-02-13
- Nouveau fichier Nouveautés avec les vrais changements
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_CDF_EFK.xlsx
+++ b/Objets_parlementaires_CDF_EFK.xlsx
@@ -77,45 +77,51 @@
     <t xml:space="preserve">La rémunération des tâches confiées à l'OFDF dans les aéroports de Genève et Bâle doit profiter à l'OFDF !</t>
   </si>
   <si>
+    <t xml:space="preserve">Stellungnahme zum Vorstoss liegt vor / L’avis relatif à l’intervention est disponible</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254785</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254785</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Élu &amp; Conseil fédéral</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25.4620</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Michel Matthias</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PLR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-12-18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Daten der Bundesverwaltung mehrfach nutzbar machen – als Basis für vertrauenswürdige KI in der Schweiz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Favoriser la fiabilité de l’IA en Suisse en rendant réutilisables les données de l’administration fédérale</t>
+  </si>
+  <si>
     <t xml:space="preserve">Eingereicht / Déposé</t>
   </si>
   <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254785</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254785</t>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254620</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254620</t>
   </si>
   <si>
     <t xml:space="preserve">Élu</t>
   </si>
   <si>
-    <t xml:space="preserve">25.4620</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Michel Matthias</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PLR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-12-18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Daten der Bundesverwaltung mehrfach nutzbar machen – als Basis für vertrauenswürdige KI in der Schweiz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Favoriser la fiabilité de l’IA en Suisse en rendant réutilisables les données de l’administration fédérale</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254620</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254620</t>
-  </si>
-  <si>
     <t xml:space="preserve">25.4696</t>
   </si>
   <si>
@@ -191,9 +197,6 @@
     <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20258273</t>
   </si>
   <si>
-    <t xml:space="preserve">Élu &amp; Conseil fédéral</t>
-  </si>
-  <si>
     <t xml:space="preserve">25.4463</t>
   </si>
   <si>
@@ -234,9 +237,6 @@
   </si>
   <si>
     <t xml:space="preserve">Coordination plus efficace des moyens de transport dans le cadre des programmes d'agglomération</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stellungnahme zum Vorstoss liegt vor / L’avis relatif à l’intervention est disponible</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254281</t>
@@ -2471,16 +2471,16 @@
         <v>31</v>
       </c>
       <c r="J3" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="K3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="L3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="M3" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4">
@@ -2488,16 +2488,16 @@
         <v>20254696</v>
       </c>
       <c r="B4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C4" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F4" t="s">
         <v>28</v>
@@ -2506,19 +2506,19 @@
         <v>18</v>
       </c>
       <c r="H4" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="I4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="J4" t="s">
         <v>21</v>
       </c>
       <c r="K4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="L4" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="M4" t="s">
         <v>24</v>
@@ -2529,40 +2529,40 @@
         <v>20258194</v>
       </c>
       <c r="B5" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C5" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D5" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E5" t="s">
         <v>16</v>
       </c>
       <c r="F5" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G5" t="s">
         <v>18</v>
       </c>
       <c r="H5" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="I5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="J5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K5" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="L5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="M5" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6">
@@ -2570,40 +2570,40 @@
         <v>20258273</v>
       </c>
       <c r="B6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E6" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G6" t="s">
         <v>18</v>
       </c>
       <c r="H6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="I6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="J6" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K6" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="L6" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="M6" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7">
@@ -2611,40 +2611,40 @@
         <v>20254463</v>
       </c>
       <c r="B7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C7" t="s">
         <v>14</v>
       </c>
       <c r="D7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E7" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G7" t="s">
         <v>18</v>
       </c>
       <c r="H7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="J7" t="s">
         <v>21</v>
       </c>
       <c r="K7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="M7" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8">
@@ -2652,31 +2652,31 @@
         <v>20254281</v>
       </c>
       <c r="B8" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C8" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D8" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E8" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G8" t="s">
         <v>18</v>
       </c>
       <c r="H8" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I8" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="J8" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="K8" t="s">
         <v>75</v>
@@ -2685,7 +2685,7 @@
         <v>76</v>
       </c>
       <c r="M8" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9">
@@ -2705,7 +2705,7 @@
         <v>27</v>
       </c>
       <c r="F9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G9" t="s">
         <v>18</v>
@@ -2717,7 +2717,7 @@
         <v>80</v>
       </c>
       <c r="J9" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="K9" t="s">
         <v>81</v>
@@ -2726,7 +2726,7 @@
         <v>82</v>
       </c>
       <c r="M9" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10">
@@ -2758,7 +2758,7 @@
         <v>87</v>
       </c>
       <c r="J10" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K10" t="s">
         <v>88</v>
@@ -2767,7 +2767,7 @@
         <v>89</v>
       </c>
       <c r="M10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11">
@@ -2808,7 +2808,7 @@
         <v>96</v>
       </c>
       <c r="M11" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12">
@@ -2819,13 +2819,13 @@
         <v>97</v>
       </c>
       <c r="C12" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D12" t="s">
         <v>98</v>
       </c>
       <c r="E12" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F12" t="s">
         <v>85</v>
@@ -2840,7 +2840,7 @@
         <v>100</v>
       </c>
       <c r="J12" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="K12" t="s">
         <v>101</v>
@@ -2849,7 +2849,7 @@
         <v>102</v>
       </c>
       <c r="M12" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13">
@@ -2866,7 +2866,7 @@
         <v>104</v>
       </c>
       <c r="E13" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F13" t="s">
         <v>85</v>
@@ -2881,7 +2881,7 @@
         <v>106</v>
       </c>
       <c r="J13" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K13" t="s">
         <v>107</v>
@@ -2890,7 +2890,7 @@
         <v>108</v>
       </c>
       <c r="M13" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14">
@@ -2901,7 +2901,7 @@
         <v>109</v>
       </c>
       <c r="C14" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D14" t="s">
         <v>110</v>
@@ -2922,7 +2922,7 @@
         <v>113</v>
       </c>
       <c r="J14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K14" t="s">
         <v>114</v>
@@ -2931,7 +2931,7 @@
         <v>115</v>
       </c>
       <c r="M14" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="15">
@@ -2942,13 +2942,13 @@
         <v>116</v>
       </c>
       <c r="C15" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D15" t="s">
         <v>117</v>
       </c>
       <c r="E15" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F15" t="s">
         <v>118</v>
@@ -2963,7 +2963,7 @@
         <v>120</v>
       </c>
       <c r="J15" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="K15" t="s">
         <v>121</v>
@@ -2972,7 +2972,7 @@
         <v>122</v>
       </c>
       <c r="M15" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16">
@@ -2983,7 +2983,7 @@
         <v>123</v>
       </c>
       <c r="C16" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D16" t="s">
         <v>124</v>
@@ -3004,7 +3004,7 @@
         <v>127</v>
       </c>
       <c r="J16" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K16" t="s">
         <v>128</v>
@@ -3013,7 +3013,7 @@
         <v>129</v>
       </c>
       <c r="M16" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="17">
@@ -3024,7 +3024,7 @@
         <v>130</v>
       </c>
       <c r="C17" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D17" t="s">
         <v>131</v>
@@ -3045,7 +3045,7 @@
         <v>134</v>
       </c>
       <c r="J17" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K17" t="s">
         <v>135</v>
@@ -3054,7 +3054,7 @@
         <v>136</v>
       </c>
       <c r="M17" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
     </row>
     <row r="18">
@@ -3065,13 +3065,13 @@
         <v>137</v>
       </c>
       <c r="C18" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D18" t="s">
         <v>138</v>
       </c>
       <c r="E18" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F18" t="s">
         <v>118</v>
@@ -3086,7 +3086,7 @@
         <v>140</v>
       </c>
       <c r="J18" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K18" t="s">
         <v>141</v>
@@ -3095,7 +3095,7 @@
         <v>142</v>
       </c>
       <c r="M18" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
     </row>
     <row r="19">
@@ -3106,7 +3106,7 @@
         <v>143</v>
       </c>
       <c r="C19" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D19" t="s">
         <v>144</v>
@@ -3125,7 +3125,7 @@
         <v>147</v>
       </c>
       <c r="J19" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="K19" t="s">
         <v>148</v>
@@ -3134,7 +3134,7 @@
         <v>149</v>
       </c>
       <c r="M19" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="20">
@@ -3173,7 +3173,7 @@
         <v>155</v>
       </c>
       <c r="M20" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="21">
@@ -3184,7 +3184,7 @@
         <v>156</v>
       </c>
       <c r="C21" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D21" t="s">
         <v>15</v>
@@ -3205,7 +3205,7 @@
         <v>158</v>
       </c>
       <c r="J21" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K21" t="s">
         <v>159</v>
@@ -3214,7 +3214,7 @@
         <v>160</v>
       </c>
       <c r="M21" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="22">
@@ -3225,13 +3225,13 @@
         <v>161</v>
       </c>
       <c r="C22" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D22" t="s">
         <v>162</v>
       </c>
       <c r="E22" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F22" t="s">
         <v>152</v>
@@ -3246,7 +3246,7 @@
         <v>164</v>
       </c>
       <c r="J22" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K22" t="s">
         <v>165</v>
@@ -3255,7 +3255,7 @@
         <v>166</v>
       </c>
       <c r="M22" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="23">
@@ -3266,7 +3266,7 @@
         <v>167</v>
       </c>
       <c r="C23" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D23" t="s">
         <v>168</v>
@@ -3287,7 +3287,7 @@
         <v>171</v>
       </c>
       <c r="J23" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K23" t="s">
         <v>172</v>
@@ -3296,7 +3296,7 @@
         <v>173</v>
       </c>
       <c r="M23" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
     </row>
     <row r="24">
@@ -3307,7 +3307,7 @@
         <v>174</v>
       </c>
       <c r="C24" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D24" t="s">
         <v>131</v>
@@ -3328,7 +3328,7 @@
         <v>177</v>
       </c>
       <c r="J24" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K24" t="s">
         <v>178</v>
@@ -3337,7 +3337,7 @@
         <v>179</v>
       </c>
       <c r="M24" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
     </row>
     <row r="25">
@@ -3376,7 +3376,7 @@
         <v>187</v>
       </c>
       <c r="M25" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="26">
@@ -3417,7 +3417,7 @@
         <v>194</v>
       </c>
       <c r="M26" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
     </row>
     <row r="27">
@@ -3428,13 +3428,13 @@
         <v>195</v>
       </c>
       <c r="C27" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D27" t="s">
         <v>138</v>
       </c>
       <c r="E27" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F27" t="s">
         <v>190</v>
@@ -3449,7 +3449,7 @@
         <v>197</v>
       </c>
       <c r="J27" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="K27" t="s">
         <v>198</v>
@@ -3458,7 +3458,7 @@
         <v>199</v>
       </c>
       <c r="M27" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
     </row>
     <row r="28">
@@ -3499,7 +3499,7 @@
         <v>203</v>
       </c>
       <c r="M28" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
     </row>
     <row r="29">
@@ -3510,7 +3510,7 @@
         <v>204</v>
       </c>
       <c r="C29" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D29" t="s">
         <v>205</v>
@@ -3531,7 +3531,7 @@
         <v>207</v>
       </c>
       <c r="J29" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="K29" t="s">
         <v>208</v>
@@ -3540,7 +3540,7 @@
         <v>209</v>
       </c>
       <c r="M29" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
     </row>
     <row r="30">
@@ -3551,7 +3551,7 @@
         <v>210</v>
       </c>
       <c r="C30" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D30" t="s">
         <v>211</v>
@@ -3572,7 +3572,7 @@
         <v>214</v>
       </c>
       <c r="J30" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="K30" t="s">
         <v>215</v>
@@ -3581,7 +3581,7 @@
         <v>216</v>
       </c>
       <c r="M30" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
     </row>
     <row r="31">
@@ -3592,7 +3592,7 @@
         <v>217</v>
       </c>
       <c r="C31" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D31" t="s">
         <v>218</v>
@@ -3613,7 +3613,7 @@
         <v>220</v>
       </c>
       <c r="J31" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="K31" t="s">
         <v>221</v>
@@ -3622,7 +3622,7 @@
         <v>222</v>
       </c>
       <c r="M31" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
     </row>
     <row r="32">
@@ -3639,7 +3639,7 @@
         <v>224</v>
       </c>
       <c r="E32" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F32" t="s">
         <v>225</v>
@@ -3654,7 +3654,7 @@
         <v>227</v>
       </c>
       <c r="J32" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="K32" t="s">
         <v>228</v>
@@ -3663,7 +3663,7 @@
         <v>229</v>
       </c>
       <c r="M32" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="33">
@@ -3674,7 +3674,7 @@
         <v>230</v>
       </c>
       <c r="C33" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D33" t="s">
         <v>231</v>
@@ -3695,7 +3695,7 @@
         <v>234</v>
       </c>
       <c r="J33" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K33" t="s">
         <v>235</v>
@@ -3704,7 +3704,7 @@
         <v>236</v>
       </c>
       <c r="M33" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
     </row>
     <row r="34">
@@ -3745,7 +3745,7 @@
         <v>243</v>
       </c>
       <c r="M34" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="35">
@@ -3756,7 +3756,7 @@
         <v>244</v>
       </c>
       <c r="C35" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D35" t="s">
         <v>245</v>
@@ -3777,7 +3777,7 @@
         <v>248</v>
       </c>
       <c r="J35" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K35" t="s">
         <v>249</v>
@@ -3786,7 +3786,7 @@
         <v>250</v>
       </c>
       <c r="M35" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="36">
@@ -3797,7 +3797,7 @@
         <v>251</v>
       </c>
       <c r="C36" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D36" t="s">
         <v>252</v>
@@ -3818,7 +3818,7 @@
         <v>254</v>
       </c>
       <c r="J36" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K36" t="s">
         <v>255</v>
@@ -3827,7 +3827,7 @@
         <v>256</v>
       </c>
       <c r="M36" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="37">
@@ -3838,13 +3838,13 @@
         <v>257</v>
       </c>
       <c r="C37" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D37" t="s">
         <v>258</v>
       </c>
       <c r="E37" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F37" t="s">
         <v>259</v>
@@ -3859,7 +3859,7 @@
         <v>261</v>
       </c>
       <c r="J37" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="K37" t="s">
         <v>262</v>
@@ -3868,7 +3868,7 @@
         <v>263</v>
       </c>
       <c r="M37" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
     </row>
     <row r="38">
@@ -3900,7 +3900,7 @@
         <v>268</v>
       </c>
       <c r="J38" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="K38" t="s">
         <v>269</v>
@@ -3909,7 +3909,7 @@
         <v>270</v>
       </c>
       <c r="M38" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
     </row>
     <row r="39">
@@ -3939,7 +3939,7 @@
         <v>275</v>
       </c>
       <c r="J39" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="K39" t="s">
         <v>276</v>
@@ -3948,7 +3948,7 @@
         <v>277</v>
       </c>
       <c r="M39" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
     </row>
     <row r="40">
@@ -3980,7 +3980,7 @@
         <v>281</v>
       </c>
       <c r="J40" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="K40" t="s">
         <v>282</v>
@@ -3989,7 +3989,7 @@
         <v>283</v>
       </c>
       <c r="M40" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
     </row>
     <row r="41">
@@ -4000,13 +4000,13 @@
         <v>284</v>
       </c>
       <c r="C41" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D41" t="s">
         <v>285</v>
       </c>
       <c r="E41" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F41" t="s">
         <v>279</v>
@@ -4021,7 +4021,7 @@
         <v>287</v>
       </c>
       <c r="J41" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="K41" t="s">
         <v>288</v>
@@ -4030,7 +4030,7 @@
         <v>289</v>
       </c>
       <c r="M41" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
     </row>
     <row r="42">
@@ -4047,7 +4047,7 @@
         <v>291</v>
       </c>
       <c r="E42" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F42" t="s">
         <v>279</v>
@@ -4062,7 +4062,7 @@
         <v>293</v>
       </c>
       <c r="J42" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="K42" t="s">
         <v>294</v>
@@ -4071,7 +4071,7 @@
         <v>295</v>
       </c>
       <c r="M42" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="43">
@@ -4103,7 +4103,7 @@
         <v>299</v>
       </c>
       <c r="J43" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="K43" t="s">
         <v>300</v>
@@ -4112,7 +4112,7 @@
         <v>301</v>
       </c>
       <c r="M43" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="44">
@@ -4129,7 +4129,7 @@
         <v>304</v>
       </c>
       <c r="E44" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F44" t="s">
         <v>305</v>
@@ -4144,7 +4144,7 @@
         <v>307</v>
       </c>
       <c r="J44" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K44" t="s">
         <v>308</v>
@@ -4153,7 +4153,7 @@
         <v>309</v>
       </c>
       <c r="M44" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="45">
@@ -4164,7 +4164,7 @@
         <v>310</v>
       </c>
       <c r="C45" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D45" t="s">
         <v>311</v>
@@ -4185,7 +4185,7 @@
         <v>313</v>
       </c>
       <c r="J45" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K45" t="s">
         <v>314</v>
@@ -4194,7 +4194,7 @@
         <v>315</v>
       </c>
       <c r="M45" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="46">
@@ -4205,7 +4205,7 @@
         <v>316</v>
       </c>
       <c r="C46" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D46" t="s">
         <v>317</v>
@@ -4226,7 +4226,7 @@
         <v>319</v>
       </c>
       <c r="J46" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K46" t="s">
         <v>320</v>
@@ -4235,7 +4235,7 @@
         <v>321</v>
       </c>
       <c r="M46" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
     </row>
     <row r="47">
@@ -4246,7 +4246,7 @@
         <v>322</v>
       </c>
       <c r="C47" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D47" t="s">
         <v>323</v>
@@ -4267,7 +4267,7 @@
         <v>325</v>
       </c>
       <c r="J47" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K47" t="s">
         <v>326</v>
@@ -4276,7 +4276,7 @@
         <v>327</v>
       </c>
       <c r="M47" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="48">
@@ -4287,7 +4287,7 @@
         <v>328</v>
       </c>
       <c r="C48" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D48" t="s">
         <v>317</v>
@@ -4308,7 +4308,7 @@
         <v>330</v>
       </c>
       <c r="J48" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K48" t="s">
         <v>331</v>
@@ -4317,7 +4317,7 @@
         <v>332</v>
       </c>
       <c r="M48" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="49">
@@ -4358,7 +4358,7 @@
         <v>338</v>
       </c>
       <c r="M49" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
     </row>
     <row r="50">
@@ -4369,13 +4369,13 @@
         <v>339</v>
       </c>
       <c r="C50" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D50" t="s">
         <v>340</v>
       </c>
       <c r="E50" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F50" t="s">
         <v>341</v>
@@ -4390,7 +4390,7 @@
         <v>343</v>
       </c>
       <c r="J50" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="K50" t="s">
         <v>344</v>
@@ -4399,7 +4399,7 @@
         <v>345</v>
       </c>
       <c r="M50" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
     </row>
     <row r="51">
@@ -4410,13 +4410,13 @@
         <v>346</v>
       </c>
       <c r="C51" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D51" t="s">
         <v>285</v>
       </c>
       <c r="E51" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F51" t="s">
         <v>347</v>
@@ -4431,7 +4431,7 @@
         <v>349</v>
       </c>
       <c r="J51" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K51" t="s">
         <v>350</v>
@@ -4440,7 +4440,7 @@
         <v>351</v>
       </c>
       <c r="M51" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
     </row>
     <row r="52">
@@ -4472,7 +4472,7 @@
         <v>357</v>
       </c>
       <c r="J52" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="K52" t="s">
         <v>358</v>
@@ -4481,7 +4481,7 @@
         <v>359</v>
       </c>
       <c r="M52" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="53">
@@ -4492,13 +4492,13 @@
         <v>360</v>
       </c>
       <c r="C53" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D53" t="s">
         <v>117</v>
       </c>
       <c r="E53" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F53" t="s">
         <v>355</v>
@@ -4513,7 +4513,7 @@
         <v>362</v>
       </c>
       <c r="J53" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K53" t="s">
         <v>363</v>
@@ -4522,7 +4522,7 @@
         <v>364</v>
       </c>
       <c r="M53" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="54">
@@ -4533,7 +4533,7 @@
         <v>365</v>
       </c>
       <c r="C54" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D54" t="s">
         <v>265</v>
@@ -4554,7 +4554,7 @@
         <v>367</v>
       </c>
       <c r="J54" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K54" t="s">
         <v>368</v>
@@ -4563,7 +4563,7 @@
         <v>369</v>
       </c>
       <c r="M54" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
     </row>
     <row r="55">
@@ -4574,13 +4574,13 @@
         <v>370</v>
       </c>
       <c r="C55" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D55" t="s">
         <v>371</v>
       </c>
       <c r="E55" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F55" t="s">
         <v>355</v>
@@ -4595,7 +4595,7 @@
         <v>373</v>
       </c>
       <c r="J55" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K55" t="s">
         <v>374</v>
@@ -4604,7 +4604,7 @@
         <v>375</v>
       </c>
       <c r="M55" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="56">
@@ -4615,7 +4615,7 @@
         <v>376</v>
       </c>
       <c r="C56" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D56" t="s">
         <v>377</v>
@@ -4636,7 +4636,7 @@
         <v>381</v>
       </c>
       <c r="J56" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="K56" t="s">
         <v>382</v>
@@ -4645,7 +4645,7 @@
         <v>383</v>
       </c>
       <c r="M56" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="57">
@@ -4656,7 +4656,7 @@
         <v>384</v>
       </c>
       <c r="C57" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D57" t="s">
         <v>385</v>
@@ -4677,7 +4677,7 @@
         <v>387</v>
       </c>
       <c r="J57" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K57" t="s">
         <v>388</v>
@@ -4686,7 +4686,7 @@
         <v>389</v>
       </c>
       <c r="M57" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
     </row>
     <row r="58">
@@ -4716,7 +4716,7 @@
         <v>394</v>
       </c>
       <c r="J58" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K58" t="s">
         <v>395</v>
@@ -4725,7 +4725,7 @@
         <v>396</v>
       </c>
       <c r="M58" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="59">
@@ -4736,7 +4736,7 @@
         <v>397</v>
       </c>
       <c r="C59" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D59" t="s">
         <v>398</v>
@@ -4757,7 +4757,7 @@
         <v>401</v>
       </c>
       <c r="J59" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K59" t="s">
         <v>402</v>
@@ -4766,7 +4766,7 @@
         <v>403</v>
       </c>
       <c r="M59" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="60">
@@ -4777,7 +4777,7 @@
         <v>404</v>
       </c>
       <c r="C60" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D60" t="s">
         <v>231</v>
@@ -4798,7 +4798,7 @@
         <v>406</v>
       </c>
       <c r="J60" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K60" t="s">
         <v>407</v>
@@ -4807,7 +4807,7 @@
         <v>408</v>
       </c>
       <c r="M60" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="61">
@@ -4818,7 +4818,7 @@
         <v>409</v>
       </c>
       <c r="C61" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D61" t="s">
         <v>410</v>
@@ -4839,7 +4839,7 @@
         <v>413</v>
       </c>
       <c r="J61" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K61" t="s">
         <v>414</v>
@@ -4848,7 +4848,7 @@
         <v>415</v>
       </c>
       <c r="M61" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
     </row>
     <row r="62">
@@ -4859,7 +4859,7 @@
         <v>416</v>
       </c>
       <c r="C62" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D62" t="s">
         <v>417</v>
@@ -4880,7 +4880,7 @@
         <v>419</v>
       </c>
       <c r="J62" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K62" t="s">
         <v>420</v>
@@ -4889,7 +4889,7 @@
         <v>421</v>
       </c>
       <c r="M62" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
     </row>
     <row r="63">
@@ -4900,13 +4900,13 @@
         <v>422</v>
       </c>
       <c r="C63" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D63" t="s">
         <v>423</v>
       </c>
       <c r="E63" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F63" t="s">
         <v>424</v>
@@ -4921,7 +4921,7 @@
         <v>426</v>
       </c>
       <c r="J63" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="K63" t="s">
         <v>427</v>
@@ -4930,7 +4930,7 @@
         <v>428</v>
       </c>
       <c r="M63" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="64">
@@ -4941,13 +4941,13 @@
         <v>429</v>
       </c>
       <c r="C64" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D64" t="s">
         <v>430</v>
       </c>
       <c r="E64" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F64" t="s">
         <v>431</v>
@@ -4962,7 +4962,7 @@
         <v>433</v>
       </c>
       <c r="J64" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="K64" t="s">
         <v>434</v>
@@ -4971,7 +4971,7 @@
         <v>435</v>
       </c>
       <c r="M64" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
     </row>
     <row r="65">
@@ -4982,7 +4982,7 @@
         <v>436</v>
       </c>
       <c r="C65" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D65" t="s">
         <v>297</v>
@@ -5003,7 +5003,7 @@
         <v>439</v>
       </c>
       <c r="J65" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="K65" t="s">
         <v>440</v>
@@ -5012,7 +5012,7 @@
         <v>441</v>
       </c>
       <c r="M65" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="66">
@@ -5023,13 +5023,13 @@
         <v>442</v>
       </c>
       <c r="C66" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D66" t="s">
         <v>443</v>
       </c>
       <c r="E66" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F66" t="s">
         <v>437</v>
@@ -5044,7 +5044,7 @@
         <v>445</v>
       </c>
       <c r="J66" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="K66" t="s">
         <v>446</v>
@@ -5053,7 +5053,7 @@
         <v>447</v>
       </c>
       <c r="M66" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
     </row>
     <row r="67">
@@ -5064,13 +5064,13 @@
         <v>448</v>
       </c>
       <c r="C67" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D67" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E67" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F67" t="s">
         <v>437</v>
@@ -5085,7 +5085,7 @@
         <v>450</v>
       </c>
       <c r="J67" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="K67" t="s">
         <v>451</v>
@@ -5094,7 +5094,7 @@
         <v>452</v>
       </c>
       <c r="M67" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="68">
@@ -5105,7 +5105,7 @@
         <v>453</v>
       </c>
       <c r="C68" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D68" t="s">
         <v>131</v>
@@ -5126,7 +5126,7 @@
         <v>455</v>
       </c>
       <c r="J68" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="K68" t="s">
         <v>456</v>
@@ -5135,7 +5135,7 @@
         <v>457</v>
       </c>
       <c r="M68" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
     </row>
     <row r="69">
@@ -5167,7 +5167,7 @@
         <v>460</v>
       </c>
       <c r="J69" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="K69" t="s">
         <v>461</v>
@@ -5176,7 +5176,7 @@
         <v>462</v>
       </c>
       <c r="M69" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
     </row>
     <row r="70">
@@ -5187,13 +5187,13 @@
         <v>463</v>
       </c>
       <c r="C70" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D70" t="s">
         <v>464</v>
       </c>
       <c r="E70" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F70" t="s">
         <v>437</v>
@@ -5208,7 +5208,7 @@
         <v>466</v>
       </c>
       <c r="J70" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="K70" t="s">
         <v>467</v>
@@ -5217,7 +5217,7 @@
         <v>468</v>
       </c>
       <c r="M70" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
     </row>
     <row r="71">
@@ -5258,7 +5258,7 @@
         <v>475</v>
       </c>
       <c r="M71" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
     </row>
     <row r="72">
@@ -5269,13 +5269,13 @@
         <v>476</v>
       </c>
       <c r="C72" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D72" t="s">
         <v>477</v>
       </c>
       <c r="E72" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F72" t="s">
         <v>471</v>
@@ -5290,7 +5290,7 @@
         <v>479</v>
       </c>
       <c r="J72" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K72" t="s">
         <v>480</v>
@@ -5299,7 +5299,7 @@
         <v>481</v>
       </c>
       <c r="M72" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="73">
@@ -5310,7 +5310,7 @@
         <v>482</v>
       </c>
       <c r="C73" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D73" t="s">
         <v>265</v>
@@ -5331,7 +5331,7 @@
         <v>485</v>
       </c>
       <c r="J73" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K73" t="s">
         <v>486</v>
@@ -5340,7 +5340,7 @@
         <v>487</v>
       </c>
       <c r="M73" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
     </row>
     <row r="74">
@@ -5351,7 +5351,7 @@
         <v>488</v>
       </c>
       <c r="C74" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D74" t="s">
         <v>297</v>
@@ -5372,7 +5372,7 @@
         <v>490</v>
       </c>
       <c r="J74" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K74" t="s">
         <v>491</v>
@@ -5381,7 +5381,7 @@
         <v>492</v>
       </c>
       <c r="M74" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="75">
@@ -5392,7 +5392,7 @@
         <v>493</v>
       </c>
       <c r="C75" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D75" t="s">
         <v>124</v>
@@ -5413,7 +5413,7 @@
         <v>495</v>
       </c>
       <c r="J75" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K75" t="s">
         <v>496</v>
@@ -5422,7 +5422,7 @@
         <v>497</v>
       </c>
       <c r="M75" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
     </row>
     <row r="76">
@@ -5433,7 +5433,7 @@
         <v>498</v>
       </c>
       <c r="C76" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D76" t="s">
         <v>124</v>
@@ -5454,7 +5454,7 @@
         <v>500</v>
       </c>
       <c r="J76" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K76" t="s">
         <v>501</v>
@@ -5463,7 +5463,7 @@
         <v>502</v>
       </c>
       <c r="M76" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
     </row>
     <row r="77">
@@ -5474,7 +5474,7 @@
         <v>503</v>
       </c>
       <c r="C77" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D77" t="s">
         <v>504</v>
@@ -5495,7 +5495,7 @@
         <v>507</v>
       </c>
       <c r="J77" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="K77" t="s">
         <v>508</v>
@@ -5504,7 +5504,7 @@
         <v>509</v>
       </c>
       <c r="M77" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
     </row>
     <row r="78">
@@ -5515,7 +5515,7 @@
         <v>510</v>
       </c>
       <c r="C78" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D78" t="s">
         <v>511</v>
@@ -5536,7 +5536,7 @@
         <v>513</v>
       </c>
       <c r="J78" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="K78" t="s">
         <v>514</v>
@@ -5545,7 +5545,7 @@
         <v>515</v>
       </c>
       <c r="M78" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="79">
@@ -5556,13 +5556,13 @@
         <v>516</v>
       </c>
       <c r="C79" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D79" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E79" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F79" t="s">
         <v>517</v>
@@ -5577,7 +5577,7 @@
         <v>519</v>
       </c>
       <c r="J79" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K79" t="s">
         <v>520</v>
@@ -5586,7 +5586,7 @@
         <v>521</v>
       </c>
       <c r="M79" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="80">
@@ -5597,7 +5597,7 @@
         <v>522</v>
       </c>
       <c r="C80" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D80" t="s">
         <v>523</v>
@@ -5618,7 +5618,7 @@
         <v>525</v>
       </c>
       <c r="J80" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K80" t="s">
         <v>526</v>
@@ -5627,7 +5627,7 @@
         <v>527</v>
       </c>
       <c r="M80" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="81">
@@ -5638,13 +5638,13 @@
         <v>528</v>
       </c>
       <c r="C81" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D81" t="s">
         <v>529</v>
       </c>
       <c r="E81" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F81" t="s">
         <v>530</v>
@@ -5659,7 +5659,7 @@
         <v>532</v>
       </c>
       <c r="J81" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="K81" t="s">
         <v>533</v>
@@ -5668,7 +5668,7 @@
         <v>534</v>
       </c>
       <c r="M81" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
     </row>
     <row r="82">
@@ -5679,13 +5679,13 @@
         <v>535</v>
       </c>
       <c r="C82" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D82" t="s">
         <v>536</v>
       </c>
       <c r="E82" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F82" t="s">
         <v>530</v>
@@ -5700,7 +5700,7 @@
         <v>538</v>
       </c>
       <c r="J82" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="K82" t="s">
         <v>539</v>
@@ -5709,7 +5709,7 @@
         <v>540</v>
       </c>
       <c r="M82" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="83">
@@ -5726,7 +5726,7 @@
         <v>536</v>
       </c>
       <c r="E83" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F83" t="s">
         <v>530</v>
@@ -5741,7 +5741,7 @@
         <v>543</v>
       </c>
       <c r="J83" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K83" t="s">
         <v>544</v>
@@ -5750,7 +5750,7 @@
         <v>545</v>
       </c>
       <c r="M83" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
     </row>
     <row r="84">
@@ -5791,7 +5791,7 @@
         <v>553</v>
       </c>
       <c r="M84" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="85">
@@ -5802,7 +5802,7 @@
         <v>554</v>
       </c>
       <c r="C85" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D85" t="s">
         <v>238</v>
@@ -5823,7 +5823,7 @@
         <v>557</v>
       </c>
       <c r="J85" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K85" t="s">
         <v>558</v>
@@ -5832,7 +5832,7 @@
         <v>559</v>
       </c>
       <c r="M85" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
     </row>
     <row r="86">
@@ -5843,7 +5843,7 @@
         <v>560</v>
       </c>
       <c r="C86" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D86" t="s">
         <v>561</v>
@@ -5864,7 +5864,7 @@
         <v>564</v>
       </c>
       <c r="J86" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K86" t="s">
         <v>565</v>
@@ -5873,7 +5873,7 @@
         <v>566</v>
       </c>
       <c r="M86" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="87">
@@ -5903,7 +5903,7 @@
         <v>571</v>
       </c>
       <c r="J87" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K87" t="s">
         <v>572</v>
@@ -5912,7 +5912,7 @@
         <v>573</v>
       </c>
       <c r="M87" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
     </row>
     <row r="88">
@@ -5923,7 +5923,7 @@
         <v>574</v>
       </c>
       <c r="C88" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D88" t="s">
         <v>575</v>
@@ -5951,7 +5951,7 @@
         <v>580</v>
       </c>
       <c r="M88" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="89">
@@ -5981,7 +5981,7 @@
         <v>585</v>
       </c>
       <c r="J89" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K89" t="s">
         <v>586</v>
@@ -5990,7 +5990,7 @@
         <v>587</v>
       </c>
       <c r="M89" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="90">
@@ -6001,13 +6001,13 @@
         <v>588</v>
       </c>
       <c r="C90" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D90" t="s">
         <v>589</v>
       </c>
       <c r="E90" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F90" t="s">
         <v>590</v>
@@ -6022,7 +6022,7 @@
         <v>592</v>
       </c>
       <c r="J90" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="K90" t="s">
         <v>593</v>
@@ -6031,7 +6031,7 @@
         <v>594</v>
       </c>
       <c r="M90" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
     </row>
     <row r="91">
@@ -6063,7 +6063,7 @@
         <v>598</v>
       </c>
       <c r="J91" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K91" t="s">
         <v>599</v>
@@ -6072,7 +6072,7 @@
         <v>600</v>
       </c>
       <c r="M91" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="92">
@@ -6083,13 +6083,13 @@
         <v>601</v>
       </c>
       <c r="C92" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D92" t="s">
         <v>602</v>
       </c>
       <c r="E92" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F92" t="s">
         <v>596</v>
@@ -6104,7 +6104,7 @@
         <v>604</v>
       </c>
       <c r="J92" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K92" t="s">
         <v>605</v>
@@ -6113,7 +6113,7 @@
         <v>606</v>
       </c>
       <c r="M92" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="93">
@@ -6145,7 +6145,7 @@
         <v>611</v>
       </c>
       <c r="J93" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K93" t="s">
         <v>612</v>
@@ -6154,7 +6154,7 @@
         <v>613</v>
       </c>
       <c r="M93" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="94">
@@ -6186,7 +6186,7 @@
         <v>617</v>
       </c>
       <c r="J94" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="K94" t="s">
         <v>618</v>
@@ -6195,7 +6195,7 @@
         <v>619</v>
       </c>
       <c r="M94" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="95">
@@ -6206,13 +6206,13 @@
         <v>620</v>
       </c>
       <c r="C95" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D95" t="s">
         <v>621</v>
       </c>
       <c r="E95" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F95" t="s">
         <v>622</v>
@@ -6227,7 +6227,7 @@
         <v>624</v>
       </c>
       <c r="J95" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K95" t="s">
         <v>625</v>
@@ -6236,7 +6236,7 @@
         <v>626</v>
       </c>
       <c r="M95" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
     </row>
     <row r="96">
@@ -6247,7 +6247,7 @@
         <v>627</v>
       </c>
       <c r="C96" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D96" t="s">
         <v>265</v>
@@ -6268,7 +6268,7 @@
         <v>630</v>
       </c>
       <c r="J96" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K96" t="s">
         <v>631</v>
@@ -6277,7 +6277,7 @@
         <v>632</v>
       </c>
       <c r="M96" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
     </row>
     <row r="97">
@@ -6288,13 +6288,13 @@
         <v>633</v>
       </c>
       <c r="C97" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D97" t="s">
         <v>138</v>
       </c>
       <c r="E97" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F97" t="s">
         <v>634</v>
@@ -6309,7 +6309,7 @@
         <v>636</v>
       </c>
       <c r="J97" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K97" t="s">
         <v>637</v>
@@ -6318,7 +6318,7 @@
         <v>638</v>
       </c>
       <c r="M97" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
     </row>
     <row r="98">
@@ -6329,13 +6329,13 @@
         <v>639</v>
       </c>
       <c r="C98" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D98" t="s">
         <v>98</v>
       </c>
       <c r="E98" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F98" t="s">
         <v>640</v>
@@ -6350,7 +6350,7 @@
         <v>642</v>
       </c>
       <c r="J98" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K98" t="s">
         <v>643</v>
@@ -6359,7 +6359,7 @@
         <v>644</v>
       </c>
       <c r="M98" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="99">
@@ -6370,7 +6370,7 @@
         <v>645</v>
       </c>
       <c r="C99" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D99" t="s">
         <v>646</v>
@@ -6391,7 +6391,7 @@
         <v>649</v>
       </c>
       <c r="J99" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K99" t="s">
         <v>650</v>
@@ -6400,7 +6400,7 @@
         <v>651</v>
       </c>
       <c r="M99" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
     </row>
     <row r="100">
@@ -6411,7 +6411,7 @@
         <v>652</v>
       </c>
       <c r="C100" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D100" t="s">
         <v>653</v>
@@ -6432,7 +6432,7 @@
         <v>656</v>
       </c>
       <c r="J100" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K100" t="s">
         <v>657</v>
@@ -6441,7 +6441,7 @@
         <v>658</v>
       </c>
       <c r="M100" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="101">
@@ -6471,7 +6471,7 @@
         <v>663</v>
       </c>
       <c r="J101" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K101" t="s">
         <v>664</v>
@@ -6480,7 +6480,7 @@
         <v>665</v>
       </c>
       <c r="M101" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update parliament data - 2026-02-15
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_CDF_EFK.xlsx
+++ b/Objets_parlementaires_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="668" uniqueCount="668">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="662" uniqueCount="662">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -92,7 +92,7 @@
     <t xml:space="preserve">Élu &amp; Conseil fédéral</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-02-14</t>
+    <t xml:space="preserve">2026-02-15</t>
   </si>
   <si>
     <t xml:space="preserve">25.4620</t>
@@ -1860,24 +1860,6 @@
   </si>
   <si>
     <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20243169</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24.3077</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024-03-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dringende Wiederherstellung der Verteidigungsfähigkeit der Schweizer Armee</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rétablir d'urgence la capacité de défense de notre armée</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20243077</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20243077</t>
   </si>
   <si>
     <t xml:space="preserve">24.7112</t>
@@ -2074,8 +2056,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:N101" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:N101"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:N100" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:N100"/>
   <tableColumns count="14">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Numéro"/>
@@ -6320,61 +6302,61 @@
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>20243077</v>
+        <v>20247112</v>
       </c>
       <c r="B94" t="s">
         <v>616</v>
       </c>
       <c r="C94" t="s">
-        <v>15</v>
+        <v>47</v>
       </c>
       <c r="D94" t="s">
-        <v>16</v>
+        <v>617</v>
       </c>
       <c r="E94" t="s">
-        <v>17</v>
+        <v>58</v>
       </c>
       <c r="F94" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="G94" t="s">
         <v>19</v>
       </c>
       <c r="H94" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="I94" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="J94" t="s">
-        <v>22</v>
+        <v>52</v>
       </c>
       <c r="K94" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="L94" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="M94" t="s">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="N94"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>20247112</v>
+        <v>20247015</v>
       </c>
       <c r="B95" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="C95" t="s">
         <v>47</v>
       </c>
       <c r="D95" t="s">
-        <v>623</v>
+        <v>267</v>
       </c>
       <c r="E95" t="s">
-        <v>58</v>
+        <v>29</v>
       </c>
       <c r="F95" t="s">
         <v>624</v>
@@ -6398,25 +6380,25 @@
         <v>628</v>
       </c>
       <c r="M95" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="N95"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>20247015</v>
+        <v>20234494</v>
       </c>
       <c r="B96" t="s">
         <v>629</v>
       </c>
       <c r="C96" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="D96" t="s">
-        <v>267</v>
+        <v>140</v>
       </c>
       <c r="E96" t="s">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="F96" t="s">
         <v>630</v>
@@ -6446,7 +6428,7 @@
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>20234494</v>
+        <v>20234461</v>
       </c>
       <c r="B97" t="s">
         <v>635</v>
@@ -6455,7 +6437,7 @@
         <v>39</v>
       </c>
       <c r="D97" t="s">
-        <v>140</v>
+        <v>100</v>
       </c>
       <c r="E97" t="s">
         <v>58</v>
@@ -6482,13 +6464,13 @@
         <v>640</v>
       </c>
       <c r="M97" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="N97"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>20234461</v>
+        <v>20234375</v>
       </c>
       <c r="B98" t="s">
         <v>641</v>
@@ -6497,160 +6479,118 @@
         <v>39</v>
       </c>
       <c r="D98" t="s">
-        <v>100</v>
+        <v>642</v>
       </c>
       <c r="E98" t="s">
-        <v>58</v>
+        <v>17</v>
       </c>
       <c r="F98" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="G98" t="s">
         <v>19</v>
       </c>
       <c r="H98" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="I98" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="J98" t="s">
         <v>52</v>
       </c>
       <c r="K98" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="L98" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="M98" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="N98"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>20234375</v>
+        <v>20234353</v>
       </c>
       <c r="B99" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="C99" t="s">
         <v>39</v>
       </c>
       <c r="D99" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="E99" t="s">
         <v>17</v>
       </c>
       <c r="F99" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="G99" t="s">
         <v>19</v>
       </c>
       <c r="H99" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="I99" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="J99" t="s">
         <v>52</v>
       </c>
       <c r="K99" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="L99" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="M99" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="N99"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>20234353</v>
+        <v>20234346</v>
       </c>
       <c r="B100" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="C100" t="s">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="D100" t="s">
-        <v>655</v>
-      </c>
-      <c r="E100" t="s">
-        <v>17</v>
-      </c>
+        <v>656</v>
+      </c>
+      <c r="E100"/>
       <c r="F100" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="G100" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="H100" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="I100" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="J100" t="s">
         <v>52</v>
       </c>
       <c r="K100" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="L100" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="M100" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="N100"/>
-    </row>
-    <row r="101">
-      <c r="A101" t="n">
-        <v>20234346</v>
-      </c>
-      <c r="B101" t="s">
-        <v>661</v>
-      </c>
-      <c r="C101" t="s">
-        <v>15</v>
-      </c>
-      <c r="D101" t="s">
-        <v>662</v>
-      </c>
-      <c r="E101"/>
-      <c r="F101" t="s">
-        <v>663</v>
-      </c>
-      <c r="G101" t="s">
-        <v>31</v>
-      </c>
-      <c r="H101" t="s">
-        <v>664</v>
-      </c>
-      <c r="I101" t="s">
-        <v>665</v>
-      </c>
-      <c r="J101" t="s">
-        <v>52</v>
-      </c>
-      <c r="K101" t="s">
-        <v>666</v>
-      </c>
-      <c r="L101" t="s">
-        <v>667</v>
-      </c>
-      <c r="M101" t="s">
-        <v>37</v>
-      </c>
-      <c r="N101"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update parliament data - 2026-02-16
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_CDF_EFK.xlsx
+++ b/Objets_parlementaires_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="662" uniqueCount="662">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="668" uniqueCount="668">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -92,7 +92,7 @@
     <t xml:space="preserve">Élu &amp; Conseil fédéral</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-02-15</t>
+    <t xml:space="preserve">2026-02-16</t>
   </si>
   <si>
     <t xml:space="preserve">25.4620</t>
@@ -224,6 +224,36 @@
     <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254463</t>
   </si>
   <si>
+    <t xml:space="preserve">25.479</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pa. Iv.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Golay Roger</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-09-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Genug Bürokratie! Für einen Frühlingsputz der Gesetze und Verordnungen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trop de bureaucratie ! Pour un grand ménage dans les lois et ordonnances</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zugewiesen an die behandelnde Kommission / Attribué à la commission compétente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20250479</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20250479</t>
+  </si>
+  <si>
     <t xml:space="preserve">25.4281</t>
   </si>
   <si>
@@ -236,9 +266,6 @@
     <t xml:space="preserve">PSS</t>
   </si>
   <si>
-    <t xml:space="preserve">2025-09-26</t>
-  </si>
-  <si>
     <t xml:space="preserve">Wirksamere Koordination der Verkehrsmittel im Rahmen von Agglomerationsprogrammen</t>
   </si>
   <si>
@@ -302,9 +329,6 @@
     <t xml:space="preserve">Garantir la sécurité de l'approvisionnement et un accès rapide aux médicaments innovants</t>
   </si>
   <si>
-    <t xml:space="preserve">Zugewiesen an die behandelnde Kommission / Attribué à la commission compétente</t>
-  </si>
-  <si>
     <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254188</t>
   </si>
   <si>
@@ -1077,12 +1101,6 @@
   </si>
   <si>
     <t xml:space="preserve">25.3054</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Golay Roger</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MCG</t>
   </si>
   <si>
     <t xml:space="preserve">2025-03-05</t>
@@ -2056,8 +2074,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:N100" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:N100"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:N101" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:N101"/>
   <tableColumns count="14">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Numéro"/>
@@ -2670,7 +2688,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>20254281</v>
+        <v>20250479</v>
       </c>
       <c r="B8" t="s">
         <v>70</v>
@@ -2697,16 +2715,16 @@
         <v>76</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>22</v>
+        <v>77</v>
       </c>
       <c r="K8" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="L8" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="M8" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="N8" t="s">
         <v>26</v>
@@ -2714,19 +2732,19 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>20254317</v>
+        <v>20254281</v>
       </c>
       <c r="B9" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C9" t="s">
-        <v>15</v>
+        <v>81</v>
       </c>
       <c r="D9" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E9" t="s">
-        <v>29</v>
+        <v>83</v>
       </c>
       <c r="F9" t="s">
         <v>74</v>
@@ -2735,19 +2753,19 @@
         <v>19</v>
       </c>
       <c r="H9" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="I9" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="J9" s="1" t="s">
         <v>22</v>
       </c>
       <c r="K9" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="L9" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="M9" t="s">
         <v>25</v>
@@ -2758,43 +2776,43 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>20254145</v>
+        <v>20254317</v>
       </c>
       <c r="B10" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C10" t="s">
         <v>15</v>
       </c>
       <c r="D10" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="E10" t="s">
         <v>29</v>
       </c>
       <c r="F10" t="s">
-        <v>87</v>
+        <v>74</v>
       </c>
       <c r="G10" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="H10" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="I10" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>52</v>
+        <v>22</v>
       </c>
       <c r="K10" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="L10" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="M10" t="s">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="N10" t="s">
         <v>26</v>
@@ -2802,40 +2820,40 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>20254188</v>
+        <v>20254145</v>
       </c>
       <c r="B11" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C11" t="s">
         <v>15</v>
       </c>
       <c r="D11" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E11" t="s">
         <v>29</v>
       </c>
       <c r="F11" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="G11" t="s">
         <v>31</v>
       </c>
       <c r="H11" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="I11" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>96</v>
+        <v>52</v>
       </c>
       <c r="K11" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="L11" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="M11" t="s">
         <v>55</v>
@@ -2846,43 +2864,43 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>20254225</v>
+        <v>20254188</v>
       </c>
       <c r="B12" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C12" t="s">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="D12" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E12" t="s">
-        <v>58</v>
+        <v>29</v>
       </c>
       <c r="F12" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="G12" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="H12" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="I12" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>22</v>
+        <v>77</v>
       </c>
       <c r="K12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="L12" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="M12" t="s">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="N12" t="s">
         <v>26</v>
@@ -2890,43 +2908,43 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>20254234</v>
+        <v>20254225</v>
       </c>
       <c r="B13" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C13" t="s">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="D13" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E13" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="F13" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="G13" t="s">
         <v>19</v>
       </c>
       <c r="H13" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="I13" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>52</v>
+        <v>22</v>
       </c>
       <c r="K13" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="L13" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="M13" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="N13" t="s">
         <v>26</v>
@@ -2934,43 +2952,43 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>20254071</v>
+        <v>20254234</v>
       </c>
       <c r="B14" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C14" t="s">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="D14" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E14" t="s">
-        <v>29</v>
+        <v>83</v>
       </c>
       <c r="F14" t="s">
-        <v>113</v>
+        <v>96</v>
       </c>
       <c r="G14" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="H14" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I14" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J14" s="1" t="s">
         <v>52</v>
       </c>
       <c r="K14" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="L14" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="M14" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="N14" t="s">
         <v>26</v>
@@ -2978,43 +2996,43 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>20254024</v>
+        <v>20254071</v>
       </c>
       <c r="B15" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C15" t="s">
         <v>39</v>
       </c>
       <c r="D15" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E15" t="s">
-        <v>73</v>
+        <v>29</v>
       </c>
       <c r="F15" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G15" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="H15" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="I15" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>22</v>
+        <v>52</v>
       </c>
       <c r="K15" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="L15" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="M15" t="s">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="N15" t="s">
         <v>26</v>
@@ -3022,43 +3040,43 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>20257863</v>
+        <v>20254024</v>
       </c>
       <c r="B16" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C16" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="D16" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E16" t="s">
-        <v>127</v>
+        <v>83</v>
       </c>
       <c r="F16" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="G16" t="s">
         <v>19</v>
       </c>
       <c r="H16" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="I16" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>52</v>
+        <v>22</v>
       </c>
       <c r="K16" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="L16" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="M16" t="s">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="N16" t="s">
         <v>26</v>
@@ -3066,43 +3084,43 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>20257888</v>
+        <v>20257863</v>
       </c>
       <c r="B17" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C17" t="s">
         <v>47</v>
       </c>
       <c r="D17" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E17" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F17" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="G17" t="s">
         <v>19</v>
       </c>
       <c r="H17" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="I17" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="J17" s="1" t="s">
         <v>52</v>
       </c>
       <c r="K17" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L17" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="M17" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="N17" t="s">
         <v>26</v>
@@ -3110,43 +3128,43 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>20257890</v>
+        <v>20257888</v>
       </c>
       <c r="B18" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C18" t="s">
         <v>47</v>
       </c>
       <c r="D18" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E18" t="s">
-        <v>58</v>
+        <v>142</v>
       </c>
       <c r="F18" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="G18" t="s">
         <v>19</v>
       </c>
       <c r="H18" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="I18" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="J18" s="1" t="s">
         <v>52</v>
       </c>
       <c r="K18" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="L18" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="M18" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="N18" t="s">
         <v>26</v>
@@ -3154,41 +3172,43 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>20254003</v>
+        <v>20257890</v>
       </c>
       <c r="B19" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C19" t="s">
-        <v>71</v>
+        <v>47</v>
       </c>
       <c r="D19" t="s">
-        <v>146</v>
-      </c>
-      <c r="E19"/>
+        <v>148</v>
+      </c>
+      <c r="E19" t="s">
+        <v>58</v>
+      </c>
       <c r="F19" t="s">
-        <v>147</v>
+        <v>128</v>
       </c>
       <c r="G19" t="s">
         <v>19</v>
       </c>
       <c r="H19" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="I19" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>22</v>
+        <v>52</v>
       </c>
       <c r="K19" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="L19" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="M19" t="s">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="N19" t="s">
         <v>26</v>
@@ -3196,38 +3216,38 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>20253984</v>
+        <v>20254003</v>
       </c>
       <c r="B20" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C20" t="s">
-        <v>15</v>
+        <v>81</v>
       </c>
       <c r="D20" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E20"/>
       <c r="F20" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G20" t="s">
         <v>19</v>
       </c>
       <c r="H20" t="s">
-        <v>88</v>
+        <v>156</v>
       </c>
       <c r="I20" t="s">
-        <v>89</v>
+        <v>157</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>155</v>
+        <v>22</v>
       </c>
       <c r="K20" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="L20" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="M20" t="s">
         <v>55</v>
@@ -3238,40 +3258,38 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>20257663</v>
+        <v>20253984</v>
       </c>
       <c r="B21" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C21" t="s">
-        <v>47</v>
+        <v>15</v>
       </c>
       <c r="D21" t="s">
-        <v>16</v>
-      </c>
-      <c r="E21" t="s">
-        <v>17</v>
-      </c>
+        <v>161</v>
+      </c>
+      <c r="E21"/>
       <c r="F21" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="G21" t="s">
         <v>19</v>
       </c>
       <c r="H21" t="s">
-        <v>159</v>
+        <v>97</v>
       </c>
       <c r="I21" t="s">
-        <v>160</v>
+        <v>98</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>52</v>
+        <v>163</v>
       </c>
       <c r="K21" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="L21" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="M21" t="s">
         <v>55</v>
@@ -3282,40 +3300,40 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>20257698</v>
+        <v>20257663</v>
       </c>
       <c r="B22" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="C22" t="s">
         <v>47</v>
       </c>
       <c r="D22" t="s">
-        <v>164</v>
+        <v>16</v>
       </c>
       <c r="E22" t="s">
-        <v>73</v>
+        <v>17</v>
       </c>
       <c r="F22" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="G22" t="s">
         <v>19</v>
       </c>
       <c r="H22" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="I22" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="J22" s="1" t="s">
         <v>52</v>
       </c>
       <c r="K22" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="L22" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="M22" t="s">
         <v>55</v>
@@ -3326,43 +3344,43 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>20253971</v>
+        <v>20257698</v>
       </c>
       <c r="B23" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C23" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="D23" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="E23" t="s">
-        <v>29</v>
+        <v>83</v>
       </c>
       <c r="F23" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="G23" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="H23" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="I23" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J23" s="1" t="s">
         <v>52</v>
       </c>
       <c r="K23" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="L23" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="M23" t="s">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="N23" t="s">
         <v>26</v>
@@ -3370,40 +3388,40 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>20257601</v>
+        <v>20253971</v>
       </c>
       <c r="B24" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C24" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="D24" t="s">
-        <v>133</v>
+        <v>178</v>
       </c>
       <c r="E24" t="s">
-        <v>134</v>
+        <v>29</v>
       </c>
       <c r="F24" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="G24" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="H24" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="I24" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="J24" s="1" t="s">
         <v>52</v>
       </c>
       <c r="K24" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="L24" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="M24" t="s">
         <v>25</v>
@@ -3414,32 +3432,34 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>20253941</v>
+        <v>20257601</v>
       </c>
       <c r="B25" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="C25" t="s">
-        <v>15</v>
+        <v>47</v>
       </c>
       <c r="D25" t="s">
-        <v>183</v>
-      </c>
-      <c r="E25"/>
+        <v>141</v>
+      </c>
+      <c r="E25" t="s">
+        <v>142</v>
+      </c>
       <c r="F25" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G25" t="s">
         <v>19</v>
       </c>
       <c r="H25" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="I25" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>187</v>
+        <v>52</v>
       </c>
       <c r="K25" t="s">
         <v>188</v>
@@ -3448,7 +3468,7 @@
         <v>189</v>
       </c>
       <c r="M25" t="s">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="N25" t="s">
         <v>26</v>
@@ -3456,7 +3476,7 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>20253835</v>
+        <v>20253941</v>
       </c>
       <c r="B26" t="s">
         <v>190</v>
@@ -3467,9 +3487,7 @@
       <c r="D26" t="s">
         <v>191</v>
       </c>
-      <c r="E26" t="s">
-        <v>29</v>
-      </c>
+      <c r="E26"/>
       <c r="F26" t="s">
         <v>192</v>
       </c>
@@ -3482,56 +3500,58 @@
       <c r="I26" t="s">
         <v>194</v>
       </c>
-      <c r="J26" t="s">
-        <v>155</v>
+      <c r="J26" s="1" t="s">
+        <v>195</v>
       </c>
       <c r="K26" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="L26" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="M26" t="s">
-        <v>37</v>
-      </c>
-      <c r="N26"/>
+        <v>55</v>
+      </c>
+      <c r="N26" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>20253845</v>
+        <v>20253835</v>
       </c>
       <c r="B27" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C27" t="s">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="D27" t="s">
-        <v>140</v>
+        <v>199</v>
       </c>
       <c r="E27" t="s">
-        <v>58</v>
+        <v>29</v>
       </c>
       <c r="F27" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="G27" t="s">
         <v>19</v>
       </c>
       <c r="H27" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="I27" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="J27" t="s">
-        <v>22</v>
+        <v>163</v>
       </c>
       <c r="K27" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="L27" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="M27" t="s">
         <v>37</v>
@@ -3540,40 +3560,40 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>20253855</v>
+        <v>20253845</v>
       </c>
       <c r="B28" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="C28" t="s">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="D28" t="s">
-        <v>203</v>
+        <v>148</v>
       </c>
       <c r="E28" t="s">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="F28" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="G28" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="H28" t="s">
-        <v>193</v>
+        <v>206</v>
       </c>
       <c r="I28" t="s">
-        <v>194</v>
+        <v>207</v>
       </c>
       <c r="J28" t="s">
-        <v>155</v>
+        <v>22</v>
       </c>
       <c r="K28" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="L28" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="M28" t="s">
         <v>37</v>
@@ -3582,40 +3602,40 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>20253880</v>
+        <v>20253855</v>
       </c>
       <c r="B29" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="C29" t="s">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="D29" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="E29" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="F29" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="G29" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="H29" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="I29" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="J29" t="s">
-        <v>22</v>
+        <v>163</v>
       </c>
       <c r="K29" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="L29" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="M29" t="s">
         <v>37</v>
@@ -3624,40 +3644,40 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>20253892</v>
+        <v>20253880</v>
       </c>
       <c r="B30" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C30" t="s">
         <v>39</v>
       </c>
       <c r="D30" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="E30" t="s">
-        <v>214</v>
+        <v>17</v>
       </c>
       <c r="F30" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="G30" t="s">
         <v>19</v>
       </c>
       <c r="H30" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="I30" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="J30" t="s">
         <v>22</v>
       </c>
       <c r="K30" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="L30" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="M30" t="s">
         <v>37</v>
@@ -3666,193 +3686,193 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>20253893</v>
+        <v>20253892</v>
       </c>
       <c r="B31" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C31" t="s">
-        <v>71</v>
+        <v>39</v>
       </c>
       <c r="D31" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="E31" t="s">
-        <v>29</v>
+        <v>222</v>
       </c>
       <c r="F31" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="G31" t="s">
         <v>19</v>
       </c>
       <c r="H31" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="I31" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="J31" t="s">
         <v>22</v>
       </c>
       <c r="K31" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="L31" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="M31" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="N31"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>20253730</v>
+        <v>20253893</v>
       </c>
       <c r="B32" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C32" t="s">
-        <v>15</v>
+        <v>81</v>
       </c>
       <c r="D32" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="E32" t="s">
-        <v>58</v>
+        <v>29</v>
       </c>
       <c r="F32" t="s">
-        <v>227</v>
+        <v>200</v>
       </c>
       <c r="G32" t="s">
         <v>19</v>
       </c>
       <c r="H32" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="I32" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="J32" t="s">
         <v>22</v>
       </c>
       <c r="K32" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="L32" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="M32" t="s">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="N32"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>20253630</v>
+        <v>20253730</v>
       </c>
       <c r="B33" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C33" t="s">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="D33" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E33" t="s">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="F33" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G33" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="H33" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="I33" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="J33" t="s">
-        <v>52</v>
+        <v>22</v>
       </c>
       <c r="K33" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="L33" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="M33" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="N33"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>20253637</v>
+        <v>20253630</v>
       </c>
       <c r="B34" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C34" t="s">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="D34" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E34" t="s">
-        <v>214</v>
+        <v>29</v>
       </c>
       <c r="F34" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
       <c r="G34" t="s">
         <v>31</v>
       </c>
       <c r="H34" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="I34" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="J34" t="s">
-        <v>243</v>
+        <v>52</v>
       </c>
       <c r="K34" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="L34" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="M34" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="N34"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>20257355</v>
+        <v>20253637</v>
       </c>
       <c r="B35" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C35" t="s">
-        <v>47</v>
+        <v>15</v>
       </c>
       <c r="D35" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E35" t="s">
-        <v>17</v>
+        <v>222</v>
       </c>
       <c r="F35" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="G35" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="H35" t="s">
         <v>249</v>
@@ -3861,13 +3881,13 @@
         <v>250</v>
       </c>
       <c r="J35" t="s">
-        <v>52</v>
+        <v>251</v>
       </c>
       <c r="K35" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="L35" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="M35" t="s">
         <v>55</v>
@@ -3876,40 +3896,40 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>20257419</v>
+        <v>20257355</v>
       </c>
       <c r="B36" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C36" t="s">
         <v>47</v>
       </c>
       <c r="D36" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E36" t="s">
         <v>17</v>
       </c>
       <c r="F36" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="G36" t="s">
         <v>19</v>
       </c>
       <c r="H36" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="I36" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="J36" t="s">
         <v>52</v>
       </c>
       <c r="K36" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="L36" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="M36" t="s">
         <v>55</v>
@@ -3918,164 +3938,164 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>20253479</v>
+        <v>20257419</v>
       </c>
       <c r="B37" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="C37" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="D37" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="E37" t="s">
-        <v>73</v>
+        <v>17</v>
       </c>
       <c r="F37" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="G37" t="s">
         <v>19</v>
       </c>
       <c r="H37" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="I37" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="J37" t="s">
-        <v>22</v>
+        <v>52</v>
       </c>
       <c r="K37" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="L37" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="M37" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="N37"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>20253444</v>
+        <v>20253479</v>
       </c>
       <c r="B38" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C38" t="s">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="D38" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="E38" t="s">
-        <v>29</v>
+        <v>83</v>
       </c>
       <c r="F38" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="G38" t="s">
         <v>19</v>
       </c>
       <c r="H38" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="I38" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="J38" t="s">
         <v>22</v>
       </c>
       <c r="K38" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="L38" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="M38" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="N38"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>20253425</v>
+        <v>20253444</v>
       </c>
       <c r="B39" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C39" t="s">
         <v>15</v>
       </c>
       <c r="D39" t="s">
-        <v>274</v>
-      </c>
-      <c r="E39"/>
+        <v>275</v>
+      </c>
+      <c r="E39" t="s">
+        <v>29</v>
+      </c>
       <c r="F39" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="G39" t="s">
         <v>19</v>
       </c>
       <c r="H39" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="I39" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="J39" t="s">
         <v>22</v>
       </c>
       <c r="K39" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="L39" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="M39" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="N39"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>20253309</v>
+        <v>20253425</v>
       </c>
       <c r="B40" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C40" t="s">
         <v>15</v>
       </c>
       <c r="D40" t="s">
-        <v>133</v>
-      </c>
-      <c r="E40" t="s">
-        <v>134</v>
-      </c>
+        <v>282</v>
+      </c>
+      <c r="E40"/>
       <c r="F40" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="G40" t="s">
         <v>19</v>
       </c>
       <c r="H40" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="I40" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="J40" t="s">
         <v>22</v>
       </c>
       <c r="K40" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="L40" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="M40" t="s">
         <v>37</v>
@@ -4084,124 +4104,124 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>20253399</v>
+        <v>20253309</v>
       </c>
       <c r="B41" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="C41" t="s">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="D41" t="s">
-        <v>287</v>
+        <v>141</v>
       </c>
       <c r="E41" t="s">
-        <v>73</v>
+        <v>142</v>
       </c>
       <c r="F41" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="G41" t="s">
         <v>19</v>
       </c>
       <c r="H41" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="I41" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="J41" t="s">
         <v>22</v>
       </c>
       <c r="K41" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="L41" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="M41" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="N41"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>20253404</v>
+        <v>20253399</v>
       </c>
       <c r="B42" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C42" t="s">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="D42" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="E42" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="F42" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="G42" t="s">
         <v>19</v>
       </c>
       <c r="H42" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="I42" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="J42" t="s">
         <v>22</v>
       </c>
       <c r="K42" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="L42" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="M42" t="s">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="N42"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>20253417</v>
+        <v>20253404</v>
       </c>
       <c r="B43" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="C43" t="s">
         <v>15</v>
       </c>
       <c r="D43" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="E43" t="s">
-        <v>17</v>
+        <v>83</v>
       </c>
       <c r="F43" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="G43" t="s">
         <v>19</v>
       </c>
       <c r="H43" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="I43" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="J43" t="s">
         <v>22</v>
       </c>
       <c r="K43" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="L43" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="M43" t="s">
         <v>55</v>
@@ -4210,25 +4230,25 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>20251011</v>
+        <v>20253417</v>
       </c>
       <c r="B44" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="C44" t="s">
-        <v>305</v>
+        <v>15</v>
       </c>
       <c r="D44" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="E44" t="s">
-        <v>58</v>
+        <v>17</v>
       </c>
       <c r="F44" t="s">
-        <v>307</v>
+        <v>289</v>
       </c>
       <c r="G44" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="H44" t="s">
         <v>308</v>
@@ -4237,7 +4257,7 @@
         <v>309</v>
       </c>
       <c r="J44" t="s">
-        <v>52</v>
+        <v>22</v>
       </c>
       <c r="K44" t="s">
         <v>310</v>
@@ -4252,40 +4272,40 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>20253194</v>
+        <v>20251011</v>
       </c>
       <c r="B45" t="s">
         <v>312</v>
       </c>
       <c r="C45" t="s">
-        <v>39</v>
+        <v>313</v>
       </c>
       <c r="D45" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E45" t="s">
-        <v>214</v>
+        <v>58</v>
       </c>
       <c r="F45" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="G45" t="s">
         <v>31</v>
       </c>
       <c r="H45" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="I45" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="J45" t="s">
         <v>52</v>
       </c>
       <c r="K45" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="L45" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="M45" t="s">
         <v>55</v>
@@ -4294,124 +4314,124 @@
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>20253203</v>
+        <v>20253194</v>
       </c>
       <c r="B46" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="C46" t="s">
         <v>39</v>
       </c>
       <c r="D46" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="E46" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="F46" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="G46" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="H46" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="I46" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="J46" t="s">
         <v>52</v>
       </c>
       <c r="K46" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="L46" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="M46" t="s">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="N46"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>20253213</v>
+        <v>20253203</v>
       </c>
       <c r="B47" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="C47" t="s">
         <v>39</v>
       </c>
       <c r="D47" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="E47" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="F47" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="G47" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="H47" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="I47" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="J47" t="s">
         <v>52</v>
       </c>
       <c r="K47" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="L47" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="M47" t="s">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="N47"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>20253214</v>
+        <v>20253213</v>
       </c>
       <c r="B48" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="C48" t="s">
         <v>39</v>
       </c>
       <c r="D48" t="s">
-        <v>319</v>
+        <v>333</v>
       </c>
       <c r="E48" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="F48" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="G48" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="H48" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="I48" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="J48" t="s">
         <v>52</v>
       </c>
       <c r="K48" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="L48" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="M48" t="s">
         <v>55</v>
@@ -4420,82 +4440,82 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>20253246</v>
+        <v>20253214</v>
       </c>
       <c r="B49" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="C49" t="s">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="D49" t="s">
-        <v>336</v>
+        <v>327</v>
       </c>
       <c r="E49" t="s">
-        <v>17</v>
+        <v>222</v>
       </c>
       <c r="F49" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="G49" t="s">
         <v>19</v>
       </c>
       <c r="H49" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="I49" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="J49" t="s">
-        <v>155</v>
+        <v>52</v>
       </c>
       <c r="K49" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="L49" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="M49" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="N49"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>20253093</v>
+        <v>20253246</v>
       </c>
       <c r="B50" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="C50" t="s">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="D50" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="E50" t="s">
-        <v>73</v>
+        <v>17</v>
       </c>
       <c r="F50" t="s">
-        <v>343</v>
+        <v>315</v>
       </c>
       <c r="G50" t="s">
         <v>19</v>
       </c>
       <c r="H50" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="I50" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="J50" t="s">
-        <v>22</v>
+        <v>163</v>
       </c>
       <c r="K50" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="L50" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="M50" t="s">
         <v>37</v>
@@ -4504,40 +4524,40 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>20257213</v>
+        <v>20253093</v>
       </c>
       <c r="B51" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="C51" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="D51" t="s">
-        <v>287</v>
+        <v>350</v>
       </c>
       <c r="E51" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="F51" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="G51" t="s">
         <v>19</v>
       </c>
       <c r="H51" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="I51" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="J51" t="s">
-        <v>52</v>
+        <v>22</v>
       </c>
       <c r="K51" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="L51" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="M51" t="s">
         <v>37</v>
@@ -4546,19 +4566,19 @@
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>20253054</v>
+        <v>20257213</v>
       </c>
       <c r="B52" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="C52" t="s">
-        <v>15</v>
+        <v>47</v>
       </c>
       <c r="D52" t="s">
-        <v>355</v>
+        <v>295</v>
       </c>
       <c r="E52" t="s">
-        <v>356</v>
+        <v>83</v>
       </c>
       <c r="F52" t="s">
         <v>357</v>
@@ -4573,7 +4593,7 @@
         <v>359</v>
       </c>
       <c r="J52" t="s">
-        <v>22</v>
+        <v>52</v>
       </c>
       <c r="K52" t="s">
         <v>360</v>
@@ -4582,46 +4602,46 @@
         <v>361</v>
       </c>
       <c r="M52" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="N52"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>20257102</v>
+        <v>20253054</v>
       </c>
       <c r="B53" t="s">
         <v>362</v>
       </c>
       <c r="C53" t="s">
-        <v>47</v>
+        <v>15</v>
       </c>
       <c r="D53" t="s">
-        <v>119</v>
+        <v>72</v>
       </c>
       <c r="E53" t="s">
         <v>73</v>
       </c>
       <c r="F53" t="s">
-        <v>357</v>
+        <v>363</v>
       </c>
       <c r="G53" t="s">
         <v>19</v>
       </c>
       <c r="H53" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="I53" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="J53" t="s">
-        <v>52</v>
+        <v>22</v>
       </c>
       <c r="K53" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="L53" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="M53" t="s">
         <v>55</v>
@@ -4630,64 +4650,64 @@
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>20257129</v>
+        <v>20257102</v>
       </c>
       <c r="B54" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C54" t="s">
         <v>47</v>
       </c>
       <c r="D54" t="s">
-        <v>267</v>
+        <v>127</v>
       </c>
       <c r="E54" t="s">
-        <v>29</v>
+        <v>83</v>
       </c>
       <c r="F54" t="s">
-        <v>357</v>
+        <v>363</v>
       </c>
       <c r="G54" t="s">
         <v>19</v>
       </c>
       <c r="H54" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="I54" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="J54" t="s">
         <v>52</v>
       </c>
       <c r="K54" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="L54" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="M54" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="N54"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>20257138</v>
+        <v>20257129</v>
       </c>
       <c r="B55" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C55" t="s">
         <v>47</v>
       </c>
       <c r="D55" t="s">
-        <v>373</v>
+        <v>275</v>
       </c>
       <c r="E55" t="s">
-        <v>73</v>
+        <v>29</v>
       </c>
       <c r="F55" t="s">
-        <v>357</v>
+        <v>363</v>
       </c>
       <c r="G55" t="s">
         <v>19</v>
@@ -4708,46 +4728,46 @@
         <v>377</v>
       </c>
       <c r="M55" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="N55"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>20253031</v>
+        <v>20257138</v>
       </c>
       <c r="B56" t="s">
         <v>378</v>
       </c>
       <c r="C56" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="D56" t="s">
         <v>379</v>
       </c>
       <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>363</v>
+      </c>
+      <c r="G56" t="s">
+        <v>19</v>
+      </c>
+      <c r="H56" t="s">
         <v>380</v>
       </c>
-      <c r="F56" t="s">
+      <c r="I56" t="s">
         <v>381</v>
       </c>
-      <c r="G56" t="s">
-        <v>19</v>
-      </c>
-      <c r="H56" t="s">
+      <c r="J56" t="s">
+        <v>52</v>
+      </c>
+      <c r="K56" t="s">
         <v>382</v>
       </c>
-      <c r="I56" t="s">
+      <c r="L56" t="s">
         <v>383</v>
-      </c>
-      <c r="J56" t="s">
-        <v>22</v>
-      </c>
-      <c r="K56" t="s">
-        <v>384</v>
-      </c>
-      <c r="L56" t="s">
-        <v>385</v>
       </c>
       <c r="M56" t="s">
         <v>55</v>
@@ -4756,22 +4776,22 @@
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>20257012</v>
+        <v>20253031</v>
       </c>
       <c r="B57" t="s">
+        <v>384</v>
+      </c>
+      <c r="C57" t="s">
+        <v>39</v>
+      </c>
+      <c r="D57" t="s">
+        <v>385</v>
+      </c>
+      <c r="E57" t="s">
         <v>386</v>
       </c>
-      <c r="C57" t="s">
-        <v>47</v>
-      </c>
-      <c r="D57" t="s">
+      <c r="F57" t="s">
         <v>387</v>
-      </c>
-      <c r="E57" t="s">
-        <v>17</v>
-      </c>
-      <c r="F57" t="s">
-        <v>381</v>
       </c>
       <c r="G57" t="s">
         <v>19</v>
@@ -4783,7 +4803,7 @@
         <v>389</v>
       </c>
       <c r="J57" t="s">
-        <v>52</v>
+        <v>22</v>
       </c>
       <c r="K57" t="s">
         <v>390</v>
@@ -4792,86 +4812,86 @@
         <v>391</v>
       </c>
       <c r="M57" t="s">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="N57"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>20253008</v>
+        <v>20257012</v>
       </c>
       <c r="B58" t="s">
         <v>392</v>
       </c>
       <c r="C58" t="s">
-        <v>15</v>
+        <v>47</v>
       </c>
       <c r="D58" t="s">
         <v>393</v>
       </c>
-      <c r="E58"/>
+      <c r="E58" t="s">
+        <v>17</v>
+      </c>
       <c r="F58" t="s">
+        <v>387</v>
+      </c>
+      <c r="G58" t="s">
+        <v>19</v>
+      </c>
+      <c r="H58" t="s">
         <v>394</v>
       </c>
-      <c r="G58" t="s">
-        <v>19</v>
-      </c>
-      <c r="H58" t="s">
+      <c r="I58" t="s">
         <v>395</v>
-      </c>
-      <c r="I58" t="s">
-        <v>396</v>
       </c>
       <c r="J58" t="s">
         <v>52</v>
       </c>
       <c r="K58" t="s">
+        <v>396</v>
+      </c>
+      <c r="L58" t="s">
         <v>397</v>
       </c>
-      <c r="L58" t="s">
-        <v>398</v>
-      </c>
       <c r="M58" t="s">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="N58"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>20244404</v>
+        <v>20253008</v>
       </c>
       <c r="B59" t="s">
+        <v>398</v>
+      </c>
+      <c r="C59" t="s">
+        <v>15</v>
+      </c>
+      <c r="D59" t="s">
         <v>399</v>
       </c>
-      <c r="C59" t="s">
-        <v>39</v>
-      </c>
-      <c r="D59" t="s">
+      <c r="E59"/>
+      <c r="F59" t="s">
         <v>400</v>
       </c>
-      <c r="E59" t="s">
-        <v>214</v>
-      </c>
-      <c r="F59" t="s">
+      <c r="G59" t="s">
+        <v>19</v>
+      </c>
+      <c r="H59" t="s">
         <v>401</v>
       </c>
-      <c r="G59" t="s">
-        <v>19</v>
-      </c>
-      <c r="H59" t="s">
+      <c r="I59" t="s">
         <v>402</v>
-      </c>
-      <c r="I59" t="s">
-        <v>403</v>
       </c>
       <c r="J59" t="s">
         <v>52</v>
       </c>
       <c r="K59" t="s">
+        <v>403</v>
+      </c>
+      <c r="L59" t="s">
         <v>404</v>
-      </c>
-      <c r="L59" t="s">
-        <v>405</v>
       </c>
       <c r="M59" t="s">
         <v>55</v>
@@ -4880,40 +4900,40 @@
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>20244419</v>
+        <v>20244404</v>
       </c>
       <c r="B60" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="C60" t="s">
         <v>39</v>
       </c>
       <c r="D60" t="s">
-        <v>233</v>
+        <v>406</v>
       </c>
       <c r="E60" t="s">
-        <v>29</v>
+        <v>222</v>
       </c>
       <c r="F60" t="s">
-        <v>401</v>
+        <v>407</v>
       </c>
       <c r="G60" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="H60" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="I60" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="J60" t="s">
         <v>52</v>
       </c>
       <c r="K60" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="L60" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="M60" t="s">
         <v>55</v>
@@ -4922,64 +4942,64 @@
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>20247975</v>
+        <v>20244419</v>
       </c>
       <c r="B61" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="C61" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="D61" t="s">
-        <v>412</v>
+        <v>241</v>
       </c>
       <c r="E61" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="F61" t="s">
+        <v>407</v>
+      </c>
+      <c r="G61" t="s">
+        <v>31</v>
+      </c>
+      <c r="H61" t="s">
         <v>413</v>
       </c>
-      <c r="G61" t="s">
-        <v>19</v>
-      </c>
-      <c r="H61" t="s">
+      <c r="I61" t="s">
         <v>414</v>
-      </c>
-      <c r="I61" t="s">
-        <v>415</v>
       </c>
       <c r="J61" t="s">
         <v>52</v>
       </c>
       <c r="K61" t="s">
+        <v>415</v>
+      </c>
+      <c r="L61" t="s">
         <v>416</v>
       </c>
-      <c r="L61" t="s">
-        <v>417</v>
-      </c>
       <c r="M61" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="N61"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>20248043</v>
+        <v>20247975</v>
       </c>
       <c r="B62" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="C62" t="s">
         <v>47</v>
       </c>
       <c r="D62" t="s">
+        <v>418</v>
+      </c>
+      <c r="E62" t="s">
+        <v>17</v>
+      </c>
+      <c r="F62" t="s">
         <v>419</v>
-      </c>
-      <c r="E62" t="s">
-        <v>214</v>
-      </c>
-      <c r="F62" t="s">
-        <v>413</v>
       </c>
       <c r="G62" t="s">
         <v>19</v>
@@ -5006,103 +5026,103 @@
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>20244290</v>
+        <v>20248043</v>
       </c>
       <c r="B63" t="s">
         <v>424</v>
       </c>
       <c r="C63" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="D63" t="s">
         <v>425</v>
       </c>
       <c r="E63" t="s">
-        <v>58</v>
+        <v>222</v>
       </c>
       <c r="F63" t="s">
+        <v>419</v>
+      </c>
+      <c r="G63" t="s">
+        <v>19</v>
+      </c>
+      <c r="H63" t="s">
         <v>426</v>
       </c>
-      <c r="G63" t="s">
-        <v>19</v>
-      </c>
-      <c r="H63" t="s">
+      <c r="I63" t="s">
         <v>427</v>
       </c>
-      <c r="I63" t="s">
+      <c r="J63" t="s">
+        <v>52</v>
+      </c>
+      <c r="K63" t="s">
         <v>428</v>
       </c>
-      <c r="J63" t="s">
-        <v>22</v>
-      </c>
-      <c r="K63" t="s">
+      <c r="L63" t="s">
         <v>429</v>
       </c>
-      <c r="L63" t="s">
-        <v>430</v>
-      </c>
       <c r="M63" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="N63"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>20244278</v>
+        <v>20244290</v>
       </c>
       <c r="B64" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="C64" t="s">
         <v>39</v>
       </c>
       <c r="D64" t="s">
+        <v>431</v>
+      </c>
+      <c r="E64" t="s">
+        <v>58</v>
+      </c>
+      <c r="F64" t="s">
         <v>432</v>
       </c>
-      <c r="E64" t="s">
-        <v>73</v>
-      </c>
-      <c r="F64" t="s">
+      <c r="G64" t="s">
+        <v>19</v>
+      </c>
+      <c r="H64" t="s">
         <v>433</v>
       </c>
-      <c r="G64" t="s">
-        <v>19</v>
-      </c>
-      <c r="H64" t="s">
+      <c r="I64" t="s">
         <v>434</v>
-      </c>
-      <c r="I64" t="s">
-        <v>435</v>
       </c>
       <c r="J64" t="s">
         <v>22</v>
       </c>
       <c r="K64" t="s">
+        <v>435</v>
+      </c>
+      <c r="L64" t="s">
         <v>436</v>
       </c>
-      <c r="L64" t="s">
-        <v>437</v>
-      </c>
       <c r="M64" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="N64"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>20244082</v>
+        <v>20244278</v>
       </c>
       <c r="B65" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C65" t="s">
         <v>39</v>
       </c>
       <c r="D65" t="s">
-        <v>299</v>
+        <v>438</v>
       </c>
       <c r="E65" t="s">
-        <v>17</v>
+        <v>83</v>
       </c>
       <c r="F65" t="s">
         <v>439</v>
@@ -5126,13 +5146,13 @@
         <v>443</v>
       </c>
       <c r="M65" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="N65"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>20244112</v>
+        <v>20244082</v>
       </c>
       <c r="B66" t="s">
         <v>444</v>
@@ -5141,13 +5161,13 @@
         <v>39</v>
       </c>
       <c r="D66" t="s">
+        <v>307</v>
+      </c>
+      <c r="E66" t="s">
+        <v>17</v>
+      </c>
+      <c r="F66" t="s">
         <v>445</v>
-      </c>
-      <c r="E66" t="s">
-        <v>58</v>
-      </c>
-      <c r="F66" t="s">
-        <v>439</v>
       </c>
       <c r="G66" t="s">
         <v>19</v>
@@ -5168,13 +5188,13 @@
         <v>449</v>
       </c>
       <c r="M66" t="s">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="N66"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>20244131</v>
+        <v>20244112</v>
       </c>
       <c r="B67" t="s">
         <v>450</v>
@@ -5183,115 +5203,115 @@
         <v>39</v>
       </c>
       <c r="D67" t="s">
-        <v>57</v>
+        <v>451</v>
       </c>
       <c r="E67" t="s">
         <v>58</v>
       </c>
       <c r="F67" t="s">
-        <v>439</v>
+        <v>445</v>
       </c>
       <c r="G67" t="s">
         <v>19</v>
       </c>
       <c r="H67" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="I67" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="J67" t="s">
         <v>22</v>
       </c>
       <c r="K67" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="L67" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="M67" t="s">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="N67"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>20244132</v>
+        <v>20244131</v>
       </c>
       <c r="B68" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="C68" t="s">
-        <v>71</v>
+        <v>39</v>
       </c>
       <c r="D68" t="s">
-        <v>133</v>
+        <v>57</v>
       </c>
       <c r="E68" t="s">
-        <v>134</v>
+        <v>58</v>
       </c>
       <c r="F68" t="s">
-        <v>439</v>
+        <v>445</v>
       </c>
       <c r="G68" t="s">
         <v>19</v>
       </c>
       <c r="H68" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="I68" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="J68" t="s">
         <v>22</v>
       </c>
       <c r="K68" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="L68" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="M68" t="s">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="N68"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>20244133</v>
+        <v>20244132</v>
       </c>
       <c r="B69" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="C69" t="s">
-        <v>15</v>
+        <v>81</v>
       </c>
       <c r="D69" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E69" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="F69" t="s">
-        <v>439</v>
+        <v>445</v>
       </c>
       <c r="G69" t="s">
         <v>19</v>
       </c>
       <c r="H69" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="I69" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="J69" t="s">
         <v>22</v>
       </c>
       <c r="K69" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="L69" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="M69" t="s">
         <v>25</v>
@@ -5300,22 +5320,22 @@
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>20244137</v>
+        <v>20244133</v>
       </c>
       <c r="B70" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="C70" t="s">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="D70" t="s">
-        <v>466</v>
+        <v>141</v>
       </c>
       <c r="E70" t="s">
-        <v>58</v>
+        <v>142</v>
       </c>
       <c r="F70" t="s">
-        <v>439</v>
+        <v>445</v>
       </c>
       <c r="G70" t="s">
         <v>19</v>
@@ -5342,64 +5362,64 @@
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>20243937</v>
+        <v>20244137</v>
       </c>
       <c r="B71" t="s">
         <v>471</v>
       </c>
       <c r="C71" t="s">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="D71" t="s">
         <v>472</v>
       </c>
       <c r="E71" t="s">
-        <v>214</v>
+        <v>58</v>
       </c>
       <c r="F71" t="s">
+        <v>445</v>
+      </c>
+      <c r="G71" t="s">
+        <v>19</v>
+      </c>
+      <c r="H71" t="s">
         <v>473</v>
       </c>
-      <c r="G71" t="s">
-        <v>31</v>
-      </c>
-      <c r="H71" t="s">
+      <c r="I71" t="s">
         <v>474</v>
       </c>
-      <c r="I71" t="s">
+      <c r="J71" t="s">
+        <v>22</v>
+      </c>
+      <c r="K71" t="s">
         <v>475</v>
       </c>
-      <c r="J71" t="s">
-        <v>187</v>
-      </c>
-      <c r="K71" t="s">
+      <c r="L71" t="s">
         <v>476</v>
       </c>
-      <c r="L71" t="s">
-        <v>477</v>
-      </c>
       <c r="M71" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="N71"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>20243948</v>
+        <v>20243937</v>
       </c>
       <c r="B72" t="s">
+        <v>477</v>
+      </c>
+      <c r="C72" t="s">
+        <v>15</v>
+      </c>
+      <c r="D72" t="s">
         <v>478</v>
       </c>
-      <c r="C72" t="s">
-        <v>39</v>
-      </c>
-      <c r="D72" t="s">
+      <c r="E72" t="s">
+        <v>222</v>
+      </c>
+      <c r="F72" t="s">
         <v>479</v>
-      </c>
-      <c r="E72" t="s">
-        <v>58</v>
-      </c>
-      <c r="F72" t="s">
-        <v>473</v>
       </c>
       <c r="G72" t="s">
         <v>31</v>
@@ -5411,7 +5431,7 @@
         <v>481</v>
       </c>
       <c r="J72" t="s">
-        <v>52</v>
+        <v>195</v>
       </c>
       <c r="K72" t="s">
         <v>482</v>
@@ -5420,31 +5440,31 @@
         <v>483</v>
       </c>
       <c r="M72" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="N72"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>20247720</v>
+        <v>20243948</v>
       </c>
       <c r="B73" t="s">
         <v>484</v>
       </c>
       <c r="C73" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="D73" t="s">
-        <v>267</v>
+        <v>485</v>
       </c>
       <c r="E73" t="s">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="F73" t="s">
-        <v>485</v>
+        <v>479</v>
       </c>
       <c r="G73" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="H73" t="s">
         <v>486</v>
@@ -5462,13 +5482,13 @@
         <v>489</v>
       </c>
       <c r="M73" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="N73"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>20247726</v>
+        <v>20247720</v>
       </c>
       <c r="B74" t="s">
         <v>490</v>
@@ -5477,115 +5497,115 @@
         <v>47</v>
       </c>
       <c r="D74" t="s">
-        <v>299</v>
+        <v>275</v>
       </c>
       <c r="E74" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="F74" t="s">
-        <v>485</v>
+        <v>491</v>
       </c>
       <c r="G74" t="s">
         <v>19</v>
       </c>
       <c r="H74" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="I74" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="J74" t="s">
         <v>52</v>
       </c>
       <c r="K74" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="L74" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="M74" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="N74"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>20247773</v>
+        <v>20247726</v>
       </c>
       <c r="B75" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="C75" t="s">
         <v>47</v>
       </c>
       <c r="D75" t="s">
-        <v>126</v>
+        <v>307</v>
       </c>
       <c r="E75" t="s">
-        <v>127</v>
+        <v>17</v>
       </c>
       <c r="F75" t="s">
-        <v>485</v>
+        <v>491</v>
       </c>
       <c r="G75" t="s">
         <v>19</v>
       </c>
       <c r="H75" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="I75" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="J75" t="s">
         <v>52</v>
       </c>
       <c r="K75" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="L75" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="M75" t="s">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="N75"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>20247774</v>
+        <v>20247773</v>
       </c>
       <c r="B76" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="C76" t="s">
         <v>47</v>
       </c>
       <c r="D76" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="E76" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="F76" t="s">
-        <v>485</v>
+        <v>491</v>
       </c>
       <c r="G76" t="s">
         <v>19</v>
       </c>
       <c r="H76" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="I76" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="J76" t="s">
         <v>52</v>
       </c>
       <c r="K76" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="L76" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="M76" t="s">
         <v>25</v>
@@ -5594,64 +5614,64 @@
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>20243858</v>
+        <v>20247774</v>
       </c>
       <c r="B77" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="C77" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="D77" t="s">
-        <v>506</v>
+        <v>134</v>
       </c>
       <c r="E77" t="s">
-        <v>17</v>
+        <v>135</v>
       </c>
       <c r="F77" t="s">
+        <v>491</v>
+      </c>
+      <c r="G77" t="s">
+        <v>19</v>
+      </c>
+      <c r="H77" t="s">
         <v>507</v>
       </c>
-      <c r="G77" t="s">
-        <v>19</v>
-      </c>
-      <c r="H77" t="s">
+      <c r="I77" t="s">
         <v>508</v>
       </c>
-      <c r="I77" t="s">
+      <c r="J77" t="s">
+        <v>52</v>
+      </c>
+      <c r="K77" t="s">
         <v>509</v>
       </c>
-      <c r="J77" t="s">
-        <v>22</v>
-      </c>
-      <c r="K77" t="s">
+      <c r="L77" t="s">
         <v>510</v>
       </c>
-      <c r="L77" t="s">
-        <v>511</v>
-      </c>
       <c r="M77" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="N77"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>20243877</v>
+        <v>20243858</v>
       </c>
       <c r="B78" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="C78" t="s">
         <v>39</v>
       </c>
       <c r="D78" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="E78" t="s">
         <v>17</v>
       </c>
       <c r="F78" t="s">
-        <v>507</v>
+        <v>513</v>
       </c>
       <c r="G78" t="s">
         <v>19</v>
@@ -5672,28 +5692,28 @@
         <v>517</v>
       </c>
       <c r="M78" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="N78"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>20247622</v>
+        <v>20243877</v>
       </c>
       <c r="B79" t="s">
         <v>518</v>
       </c>
       <c r="C79" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="D79" t="s">
-        <v>57</v>
+        <v>519</v>
       </c>
       <c r="E79" t="s">
-        <v>58</v>
+        <v>17</v>
       </c>
       <c r="F79" t="s">
-        <v>519</v>
+        <v>513</v>
       </c>
       <c r="G79" t="s">
         <v>19</v>
@@ -5705,7 +5725,7 @@
         <v>521</v>
       </c>
       <c r="J79" t="s">
-        <v>52</v>
+        <v>22</v>
       </c>
       <c r="K79" t="s">
         <v>522</v>
@@ -5720,7 +5740,7 @@
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>20247649</v>
+        <v>20247622</v>
       </c>
       <c r="B80" t="s">
         <v>524</v>
@@ -5729,13 +5749,13 @@
         <v>47</v>
       </c>
       <c r="D80" t="s">
+        <v>57</v>
+      </c>
+      <c r="E80" t="s">
+        <v>58</v>
+      </c>
+      <c r="F80" t="s">
         <v>525</v>
-      </c>
-      <c r="E80" t="s">
-        <v>29</v>
-      </c>
-      <c r="F80" t="s">
-        <v>519</v>
       </c>
       <c r="G80" t="s">
         <v>19</v>
@@ -5762,64 +5782,64 @@
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>20243709</v>
+        <v>20247649</v>
       </c>
       <c r="B81" t="s">
         <v>530</v>
       </c>
       <c r="C81" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="D81" t="s">
         <v>531</v>
       </c>
       <c r="E81" t="s">
-        <v>73</v>
+        <v>29</v>
       </c>
       <c r="F81" t="s">
+        <v>525</v>
+      </c>
+      <c r="G81" t="s">
+        <v>19</v>
+      </c>
+      <c r="H81" t="s">
         <v>532</v>
       </c>
-      <c r="G81" t="s">
-        <v>19</v>
-      </c>
-      <c r="H81" t="s">
+      <c r="I81" t="s">
         <v>533</v>
       </c>
-      <c r="I81" t="s">
+      <c r="J81" t="s">
+        <v>52</v>
+      </c>
+      <c r="K81" t="s">
         <v>534</v>
       </c>
-      <c r="J81" t="s">
-        <v>22</v>
-      </c>
-      <c r="K81" t="s">
+      <c r="L81" t="s">
         <v>535</v>
       </c>
-      <c r="L81" t="s">
-        <v>536</v>
-      </c>
       <c r="M81" t="s">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="N81"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>20243773</v>
+        <v>20243709</v>
       </c>
       <c r="B82" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="C82" t="s">
         <v>39</v>
       </c>
       <c r="D82" t="s">
+        <v>537</v>
+      </c>
+      <c r="E82" t="s">
+        <v>83</v>
+      </c>
+      <c r="F82" t="s">
         <v>538</v>
-      </c>
-      <c r="E82" t="s">
-        <v>41</v>
-      </c>
-      <c r="F82" t="s">
-        <v>532</v>
       </c>
       <c r="G82" t="s">
         <v>19</v>
@@ -5840,124 +5860,124 @@
         <v>542</v>
       </c>
       <c r="M82" t="s">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="N82"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>20243776</v>
+        <v>20243773</v>
       </c>
       <c r="B83" t="s">
         <v>543</v>
       </c>
       <c r="C83" t="s">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="D83" t="s">
-        <v>538</v>
+        <v>544</v>
       </c>
       <c r="E83" t="s">
         <v>41</v>
       </c>
       <c r="F83" t="s">
-        <v>532</v>
+        <v>538</v>
       </c>
       <c r="G83" t="s">
         <v>19</v>
       </c>
       <c r="H83" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="I83" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="J83" t="s">
-        <v>52</v>
+        <v>22</v>
       </c>
       <c r="K83" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="L83" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="M83" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="N83"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>20243609</v>
+        <v>20243776</v>
       </c>
       <c r="B84" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="C84" t="s">
         <v>15</v>
       </c>
       <c r="D84" t="s">
-        <v>549</v>
+        <v>544</v>
       </c>
       <c r="E84" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="F84" t="s">
+        <v>538</v>
+      </c>
+      <c r="G84" t="s">
+        <v>19</v>
+      </c>
+      <c r="H84" t="s">
         <v>550</v>
       </c>
-      <c r="G84" t="s">
-        <v>19</v>
-      </c>
-      <c r="H84" t="s">
+      <c r="I84" t="s">
         <v>551</v>
       </c>
-      <c r="I84" t="s">
+      <c r="J84" t="s">
+        <v>52</v>
+      </c>
+      <c r="K84" t="s">
         <v>552</v>
       </c>
-      <c r="J84" t="s">
+      <c r="L84" t="s">
         <v>553</v>
       </c>
-      <c r="K84" t="s">
-        <v>554</v>
-      </c>
-      <c r="L84" t="s">
-        <v>555</v>
-      </c>
       <c r="M84" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="N84"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>20243574</v>
+        <v>20243609</v>
       </c>
       <c r="B85" t="s">
+        <v>554</v>
+      </c>
+      <c r="C85" t="s">
+        <v>15</v>
+      </c>
+      <c r="D85" t="s">
+        <v>555</v>
+      </c>
+      <c r="E85" t="s">
+        <v>17</v>
+      </c>
+      <c r="F85" t="s">
         <v>556</v>
       </c>
-      <c r="C85" t="s">
-        <v>39</v>
-      </c>
-      <c r="D85" t="s">
-        <v>240</v>
-      </c>
-      <c r="E85" t="s">
-        <v>214</v>
-      </c>
-      <c r="F85" t="s">
+      <c r="G85" t="s">
+        <v>19</v>
+      </c>
+      <c r="H85" t="s">
         <v>557</v>
       </c>
-      <c r="G85" t="s">
-        <v>31</v>
-      </c>
-      <c r="H85" t="s">
+      <c r="I85" t="s">
         <v>558</v>
       </c>
-      <c r="I85" t="s">
+      <c r="J85" t="s">
         <v>559</v>
-      </c>
-      <c r="J85" t="s">
-        <v>52</v>
       </c>
       <c r="K85" t="s">
         <v>560</v>
@@ -5966,13 +5986,13 @@
         <v>561</v>
       </c>
       <c r="M85" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="N85"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>20243557</v>
+        <v>20243574</v>
       </c>
       <c r="B86" t="s">
         <v>562</v>
@@ -5981,151 +6001,153 @@
         <v>39</v>
       </c>
       <c r="D86" t="s">
+        <v>248</v>
+      </c>
+      <c r="E86" t="s">
+        <v>222</v>
+      </c>
+      <c r="F86" t="s">
         <v>563</v>
       </c>
-      <c r="E86" t="s">
-        <v>214</v>
-      </c>
-      <c r="F86" t="s">
+      <c r="G86" t="s">
+        <v>31</v>
+      </c>
+      <c r="H86" t="s">
         <v>564</v>
       </c>
-      <c r="G86" t="s">
-        <v>19</v>
-      </c>
-      <c r="H86" t="s">
+      <c r="I86" t="s">
         <v>565</v>
-      </c>
-      <c r="I86" t="s">
-        <v>566</v>
       </c>
       <c r="J86" t="s">
         <v>52</v>
       </c>
       <c r="K86" t="s">
+        <v>566</v>
+      </c>
+      <c r="L86" t="s">
         <v>567</v>
       </c>
-      <c r="L86" t="s">
-        <v>568</v>
-      </c>
       <c r="M86" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="N86"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>20243471</v>
+        <v>20243557</v>
       </c>
       <c r="B87" t="s">
+        <v>568</v>
+      </c>
+      <c r="C87" t="s">
+        <v>39</v>
+      </c>
+      <c r="D87" t="s">
         <v>569</v>
       </c>
-      <c r="C87" t="s">
-        <v>15</v>
-      </c>
-      <c r="D87" t="s">
+      <c r="E87" t="s">
+        <v>222</v>
+      </c>
+      <c r="F87" t="s">
         <v>570</v>
       </c>
-      <c r="E87"/>
-      <c r="F87" t="s">
+      <c r="G87" t="s">
+        <v>19</v>
+      </c>
+      <c r="H87" t="s">
         <v>571</v>
       </c>
-      <c r="G87" t="s">
-        <v>19</v>
-      </c>
-      <c r="H87" t="s">
+      <c r="I87" t="s">
         <v>572</v>
-      </c>
-      <c r="I87" t="s">
-        <v>573</v>
       </c>
       <c r="J87" t="s">
         <v>52</v>
       </c>
       <c r="K87" t="s">
+        <v>573</v>
+      </c>
+      <c r="L87" t="s">
         <v>574</v>
       </c>
-      <c r="L87" t="s">
-        <v>575</v>
-      </c>
       <c r="M87" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="N87"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>20243468</v>
+        <v>20243471</v>
       </c>
       <c r="B88" t="s">
+        <v>575</v>
+      </c>
+      <c r="C88" t="s">
+        <v>15</v>
+      </c>
+      <c r="D88" t="s">
         <v>576</v>
-      </c>
-      <c r="C88" t="s">
-        <v>71</v>
-      </c>
-      <c r="D88" t="s">
-        <v>577</v>
       </c>
       <c r="E88"/>
       <c r="F88" t="s">
+        <v>577</v>
+      </c>
+      <c r="G88" t="s">
+        <v>19</v>
+      </c>
+      <c r="H88" t="s">
         <v>578</v>
       </c>
-      <c r="G88" t="s">
-        <v>19</v>
-      </c>
-      <c r="H88" t="s">
+      <c r="I88" t="s">
         <v>579</v>
       </c>
-      <c r="I88" t="s">
+      <c r="J88" t="s">
+        <v>52</v>
+      </c>
+      <c r="K88" t="s">
         <v>580</v>
       </c>
-      <c r="J88" t="s">
-        <v>187</v>
-      </c>
-      <c r="K88" t="s">
+      <c r="L88" t="s">
         <v>581</v>
       </c>
-      <c r="L88" t="s">
-        <v>582</v>
-      </c>
       <c r="M88" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="N88"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>20243467</v>
+        <v>20243468</v>
       </c>
       <c r="B89" t="s">
+        <v>582</v>
+      </c>
+      <c r="C89" t="s">
+        <v>81</v>
+      </c>
+      <c r="D89" t="s">
         <v>583</v>
-      </c>
-      <c r="C89" t="s">
-        <v>15</v>
-      </c>
-      <c r="D89" t="s">
-        <v>584</v>
       </c>
       <c r="E89"/>
       <c r="F89" t="s">
+        <v>584</v>
+      </c>
+      <c r="G89" t="s">
+        <v>19</v>
+      </c>
+      <c r="H89" t="s">
         <v>585</v>
       </c>
-      <c r="G89" t="s">
-        <v>31</v>
-      </c>
-      <c r="H89" t="s">
+      <c r="I89" t="s">
         <v>586</v>
       </c>
-      <c r="I89" t="s">
+      <c r="J89" t="s">
+        <v>195</v>
+      </c>
+      <c r="K89" t="s">
         <v>587</v>
       </c>
-      <c r="J89" t="s">
-        <v>52</v>
-      </c>
-      <c r="K89" t="s">
+      <c r="L89" t="s">
         <v>588</v>
-      </c>
-      <c r="L89" t="s">
-        <v>589</v>
       </c>
       <c r="M89" t="s">
         <v>55</v>
@@ -6134,61 +6156,59 @@
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>20243318</v>
+        <v>20243467</v>
       </c>
       <c r="B90" t="s">
+        <v>589</v>
+      </c>
+      <c r="C90" t="s">
+        <v>15</v>
+      </c>
+      <c r="D90" t="s">
         <v>590</v>
       </c>
-      <c r="C90" t="s">
-        <v>39</v>
-      </c>
-      <c r="D90" t="s">
+      <c r="E90"/>
+      <c r="F90" t="s">
         <v>591</v>
       </c>
-      <c r="E90" t="s">
-        <v>41</v>
-      </c>
-      <c r="F90" t="s">
+      <c r="G90" t="s">
+        <v>31</v>
+      </c>
+      <c r="H90" t="s">
         <v>592</v>
       </c>
-      <c r="G90" t="s">
-        <v>19</v>
-      </c>
-      <c r="H90" t="s">
+      <c r="I90" t="s">
         <v>593</v>
       </c>
-      <c r="I90" t="s">
+      <c r="J90" t="s">
+        <v>52</v>
+      </c>
+      <c r="K90" t="s">
         <v>594</v>
       </c>
-      <c r="J90" t="s">
-        <v>22</v>
-      </c>
-      <c r="K90" t="s">
+      <c r="L90" t="s">
         <v>595</v>
       </c>
-      <c r="L90" t="s">
-        <v>596</v>
-      </c>
       <c r="M90" t="s">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="N90"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>20243234</v>
+        <v>20243318</v>
       </c>
       <c r="B91" t="s">
+        <v>596</v>
+      </c>
+      <c r="C91" t="s">
+        <v>39</v>
+      </c>
+      <c r="D91" t="s">
         <v>597</v>
       </c>
-      <c r="C91" t="s">
-        <v>15</v>
-      </c>
-      <c r="D91" t="s">
-        <v>299</v>
-      </c>
       <c r="E91" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="F91" t="s">
         <v>598</v>
@@ -6203,7 +6223,7 @@
         <v>600</v>
       </c>
       <c r="J91" t="s">
-        <v>52</v>
+        <v>22</v>
       </c>
       <c r="K91" t="s">
         <v>601</v>
@@ -6212,28 +6232,28 @@
         <v>602</v>
       </c>
       <c r="M91" t="s">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="N91"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>20243259</v>
+        <v>20243234</v>
       </c>
       <c r="B92" t="s">
         <v>603</v>
       </c>
       <c r="C92" t="s">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="D92" t="s">
+        <v>307</v>
+      </c>
+      <c r="E92" t="s">
+        <v>17</v>
+      </c>
+      <c r="F92" t="s">
         <v>604</v>
-      </c>
-      <c r="E92" t="s">
-        <v>73</v>
-      </c>
-      <c r="F92" t="s">
-        <v>598</v>
       </c>
       <c r="G92" t="s">
         <v>19</v>
@@ -6260,40 +6280,40 @@
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>20243169</v>
+        <v>20243259</v>
       </c>
       <c r="B93" t="s">
         <v>609</v>
       </c>
       <c r="C93" t="s">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="D93" t="s">
         <v>610</v>
       </c>
       <c r="E93" t="s">
-        <v>17</v>
+        <v>83</v>
       </c>
       <c r="F93" t="s">
+        <v>604</v>
+      </c>
+      <c r="G93" t="s">
+        <v>19</v>
+      </c>
+      <c r="H93" t="s">
         <v>611</v>
       </c>
-      <c r="G93" t="s">
-        <v>19</v>
-      </c>
-      <c r="H93" t="s">
+      <c r="I93" t="s">
         <v>612</v>
-      </c>
-      <c r="I93" t="s">
-        <v>613</v>
       </c>
       <c r="J93" t="s">
         <v>52</v>
       </c>
       <c r="K93" t="s">
+        <v>613</v>
+      </c>
+      <c r="L93" t="s">
         <v>614</v>
-      </c>
-      <c r="L93" t="s">
-        <v>615</v>
       </c>
       <c r="M93" t="s">
         <v>55</v>
@@ -6302,61 +6322,61 @@
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>20247112</v>
+        <v>20243169</v>
       </c>
       <c r="B94" t="s">
+        <v>615</v>
+      </c>
+      <c r="C94" t="s">
+        <v>15</v>
+      </c>
+      <c r="D94" t="s">
         <v>616</v>
       </c>
-      <c r="C94" t="s">
-        <v>47</v>
-      </c>
-      <c r="D94" t="s">
+      <c r="E94" t="s">
+        <v>17</v>
+      </c>
+      <c r="F94" t="s">
         <v>617</v>
       </c>
-      <c r="E94" t="s">
-        <v>58</v>
-      </c>
-      <c r="F94" t="s">
+      <c r="G94" t="s">
+        <v>19</v>
+      </c>
+      <c r="H94" t="s">
         <v>618</v>
       </c>
-      <c r="G94" t="s">
-        <v>19</v>
-      </c>
-      <c r="H94" t="s">
+      <c r="I94" t="s">
         <v>619</v>
-      </c>
-      <c r="I94" t="s">
-        <v>620</v>
       </c>
       <c r="J94" t="s">
         <v>52</v>
       </c>
       <c r="K94" t="s">
+        <v>620</v>
+      </c>
+      <c r="L94" t="s">
         <v>621</v>
       </c>
-      <c r="L94" t="s">
-        <v>622</v>
-      </c>
       <c r="M94" t="s">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="N94"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>20247015</v>
+        <v>20247112</v>
       </c>
       <c r="B95" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="C95" t="s">
         <v>47</v>
       </c>
       <c r="D95" t="s">
-        <v>267</v>
+        <v>623</v>
       </c>
       <c r="E95" t="s">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="F95" t="s">
         <v>624</v>
@@ -6380,25 +6400,25 @@
         <v>628</v>
       </c>
       <c r="M95" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="N95"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>20234494</v>
+        <v>20247015</v>
       </c>
       <c r="B96" t="s">
         <v>629</v>
       </c>
       <c r="C96" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="D96" t="s">
-        <v>140</v>
+        <v>275</v>
       </c>
       <c r="E96" t="s">
-        <v>58</v>
+        <v>29</v>
       </c>
       <c r="F96" t="s">
         <v>630</v>
@@ -6428,7 +6448,7 @@
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>20234461</v>
+        <v>20234494</v>
       </c>
       <c r="B97" t="s">
         <v>635</v>
@@ -6437,7 +6457,7 @@
         <v>39</v>
       </c>
       <c r="D97" t="s">
-        <v>100</v>
+        <v>148</v>
       </c>
       <c r="E97" t="s">
         <v>58</v>
@@ -6464,13 +6484,13 @@
         <v>640</v>
       </c>
       <c r="M97" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="N97"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>20234375</v>
+        <v>20234461</v>
       </c>
       <c r="B98" t="s">
         <v>641</v>
@@ -6479,118 +6499,160 @@
         <v>39</v>
       </c>
       <c r="D98" t="s">
+        <v>108</v>
+      </c>
+      <c r="E98" t="s">
+        <v>58</v>
+      </c>
+      <c r="F98" t="s">
         <v>642</v>
       </c>
-      <c r="E98" t="s">
-        <v>17</v>
-      </c>
-      <c r="F98" t="s">
+      <c r="G98" t="s">
+        <v>19</v>
+      </c>
+      <c r="H98" t="s">
         <v>643</v>
       </c>
-      <c r="G98" t="s">
-        <v>19</v>
-      </c>
-      <c r="H98" t="s">
+      <c r="I98" t="s">
         <v>644</v>
-      </c>
-      <c r="I98" t="s">
-        <v>645</v>
       </c>
       <c r="J98" t="s">
         <v>52</v>
       </c>
       <c r="K98" t="s">
+        <v>645</v>
+      </c>
+      <c r="L98" t="s">
         <v>646</v>
       </c>
-      <c r="L98" t="s">
-        <v>647</v>
-      </c>
       <c r="M98" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="N98"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>20234353</v>
+        <v>20234375</v>
       </c>
       <c r="B99" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="C99" t="s">
         <v>39</v>
       </c>
       <c r="D99" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="E99" t="s">
         <v>17</v>
       </c>
       <c r="F99" t="s">
+        <v>649</v>
+      </c>
+      <c r="G99" t="s">
+        <v>19</v>
+      </c>
+      <c r="H99" t="s">
         <v>650</v>
       </c>
-      <c r="G99" t="s">
-        <v>19</v>
-      </c>
-      <c r="H99" t="s">
+      <c r="I99" t="s">
         <v>651</v>
-      </c>
-      <c r="I99" t="s">
-        <v>652</v>
       </c>
       <c r="J99" t="s">
         <v>52</v>
       </c>
       <c r="K99" t="s">
+        <v>652</v>
+      </c>
+      <c r="L99" t="s">
         <v>653</v>
       </c>
-      <c r="L99" t="s">
-        <v>654</v>
-      </c>
       <c r="M99" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="N99"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>20234346</v>
+        <v>20234353</v>
       </c>
       <c r="B100" t="s">
+        <v>654</v>
+      </c>
+      <c r="C100" t="s">
+        <v>39</v>
+      </c>
+      <c r="D100" t="s">
         <v>655</v>
       </c>
-      <c r="C100" t="s">
-        <v>15</v>
-      </c>
-      <c r="D100" t="s">
+      <c r="E100" t="s">
+        <v>17</v>
+      </c>
+      <c r="F100" t="s">
         <v>656</v>
       </c>
-      <c r="E100"/>
-      <c r="F100" t="s">
+      <c r="G100" t="s">
+        <v>19</v>
+      </c>
+      <c r="H100" t="s">
         <v>657</v>
       </c>
-      <c r="G100" t="s">
-        <v>31</v>
-      </c>
-      <c r="H100" t="s">
+      <c r="I100" t="s">
         <v>658</v>
-      </c>
-      <c r="I100" t="s">
-        <v>659</v>
       </c>
       <c r="J100" t="s">
         <v>52</v>
       </c>
       <c r="K100" t="s">
+        <v>659</v>
+      </c>
+      <c r="L100" t="s">
         <v>660</v>
       </c>
-      <c r="L100" t="s">
+      <c r="M100" t="s">
+        <v>55</v>
+      </c>
+      <c r="N100"/>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>20234346</v>
+      </c>
+      <c r="B101" t="s">
         <v>661</v>
       </c>
-      <c r="M100" t="s">
+      <c r="C101" t="s">
+        <v>15</v>
+      </c>
+      <c r="D101" t="s">
+        <v>662</v>
+      </c>
+      <c r="E101"/>
+      <c r="F101" t="s">
+        <v>663</v>
+      </c>
+      <c r="G101" t="s">
+        <v>31</v>
+      </c>
+      <c r="H101" t="s">
+        <v>664</v>
+      </c>
+      <c r="I101" t="s">
+        <v>665</v>
+      </c>
+      <c r="J101" t="s">
+        <v>52</v>
+      </c>
+      <c r="K101" t="s">
+        <v>666</v>
+      </c>
+      <c r="L101" t="s">
+        <v>667</v>
+      </c>
+      <c r="M101" t="s">
         <v>37</v>
       </c>
-      <c r="N100"/>
+      <c r="N101"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update parliament data - 2026-02-25
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_CDF_EFK.xlsx
+++ b/Objets_parlementaires_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3621" uniqueCount="3621">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3610" uniqueCount="3610">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -6237,7 +6237,7 @@
     <t xml:space="preserve">&lt;p&gt;Le Conseil fédéral a révisé le 1er novembre 2023 l’ordonnance sur les émoluments perçus par l’autorité fédérale de surveillance des fondations (OEmol-ASF), dont la nouvelle mouture entrera en vigueur le 1er janvier 2024. L’élément central de ce texte est une nouvelle augmentation des émoluments, qui aura des conséquences financières massives pour les fondations concernées. Ce qui m’amène à poser les questions suivantes :&amp;nbsp;&lt;br&gt;- Pourquoi n’est-il pas possible de passer d’un contrôle annuel de comptes annuels déjà révisés à un rythme pluriannuel assorti de contrôles approfondis en cas de suspicion, ce qui permettrait de réduire les dépenses de l’Autorité fédérale de surveillance des fondations (ASF) et par voie de conséquence la charge administrative et financière des fondations ?&lt;br&gt;- Le Conseil fédéral serait-il prêt à réserver un traitement à part aux fondations d’utilité publique dont le total du bilan est faible (&lt; 5 millions de CHF) et à prévoir pour elles une catégorie d’émoluments distincte et plus avantageuse assortie d’un rythme de révision plus lent (par ex. tous les 3 à 5 ans) ?&lt;/p&gt;</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;p&gt;Der Bundesrat hat am 01.11.2023 die Verordnung über die Gebühren der Eidgenössischen Stiftungsaufsicht (GebV-ESA) revidiert. Die neue Verordnung tritt auf den 01.01.2024 in Kraft. Der Kernpunkt der neuen Verordnung ist eine erneute Gebührenerhöhung – mit massiven finanziellen Auswirkungen für die betroffenen Stiftungen. Hierzu stellen sich folgende Fragen:&amp;nbsp;&lt;br&gt;- Warum kann der Aufwand der ESA und damit der finanzielle und administrative Aufwand der Stiftungen nicht reduziert werden, indem von einer alljährlichen Überprüfung bereits revidierter Jahresabschlüsse auf einen Mehrjahresrhythmus gewechselt wird und auf vertiefte Prüfungen in Verdachtsfällen?&lt;br&gt;- Wäre der Bundesrat bereit, gemeinnützigen Stiftungen mit geringer Bilanzsumme (&amp;lt; 5 Mio. CHF) differenziert zu behandeln und eine separate und günstigere Gebührenkategorie mit einem längeren Revisionsrhythmus einzuführen (z.B. alle 3 – 5 Jahre)?&lt;/p&gt;</t>
+    <t xml:space="preserve">&lt;p&gt;Der Bundesrat hat am 01.11.2023 die Verordnung über die Gebühren der Eidgenössischen Stiftungsaufsicht (GebV-ESA) revidiert. Die neue Verordnung tritt auf den 01.01.2024 in Kraft. Der Kernpunkt der neuen Verordnung ist eine erneute Gebührenerhöhung – mit massiven finanziellen Auswirkungen für die betroffenen Stiftungen. Hierzu stellen sich folgende Fragen:&amp;nbsp;&lt;br&gt;- Warum kann der Aufwand der ESA und damit der finanzielle und administrative Aufwand der Stiftungen nicht reduziert werden, indem von einer alljährlichen Überprüfung bereits revidierter Jahresabschlüsse auf einen Mehrjahresrhythmus gewechselt wird und auf vertiefte Prüfungen in Verdachtsfällen?&lt;br&gt;- Wäre der Bundesrat bereit, gemeinnützigen Stiftungen mit geringer Bilanzsumme (&lt; 5 Mio. CHF) differenziert zu behandeln und eine separate und günstigere Gebührenkategorie mit einem längeren Revisionsrhythmus einzuführen (z.B. alle 3 – 5 Jahre)?&lt;/p&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20234353</t>
@@ -10110,9 +10110,6 @@
     <t xml:space="preserve">&lt;p&gt;Der Bundesrat wird beauftragt, die rechtlichen Grundlagen zu erlassen, damit baldmöglichst&amp;nbsp; qualitätsgesicherte, aktuelle und insbesondere international anschlussfähige und vergleichbare strukturierte Daten der Bundesverwaltung zur Mehrfachnutzung (unter anderem durch KI) für Forschung, Planung und Steuerung zur Verfügung gestellt werden.&amp;nbsp;Diesbezügliche verbindliche Standards für die Bundesverwaltung sind zu erlassen.&amp;nbsp;Der Bundesrat wird zudem beauftragt, eine prioritäre Auswahl jener Verwaltungsdaten zu definieren, die für eine zügige und KI-taugliche Mehrfachnutzung zuerst harmonisiert, standardisiert und technisch zugänglich gemacht werden sollen.&amp;nbsp;Insbesondere die öffentliche Bereitstellung weiterer Registerdaten ist zu prüfen. Gezielte Pilotversuche nach Art. 15 EMBAG können dies beschleunigen und sind vom Bundesrat mit den benötigten Mitteln zu beantragen.&lt;/p&gt;</t>
   </si>
   <si>
-    <t xml:space="preserve">Eingereicht / Déposé</t>
-  </si>
-  <si>
     <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254620</t>
   </si>
   <si>
@@ -10846,36 +10843,6 @@
   </si>
   <si>
     <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20253941</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18.032</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BRG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bestand des Bundespersonals auf dem Stand von 2015 einfrieren. Bericht des Bundesrates zur Abschreibung der Motion 15.3494 (FK-SR)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Geler les effectifs de la Confédération au niveau de 2015. Rapport du Conseil fédéral sur le classement de la motion 15.3494 (CdF-CE)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bloccare l'effettivo del personale della Confederazione al livello del 2015. Rapporto del Consiglio federale concernente lo stralcio della mozione 15.3494 (CdF-CS)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20180032</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20180032</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Staatspolitik</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Politique d'Etat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Politica nazionale</t>
   </si>
 </sst>
 </file>
@@ -10923,8 +10890,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:V329" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:V329"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:V328" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:V328"/>
   <tableColumns count="22">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Numéro"/>
@@ -31048,27 +31015,29 @@
         <v>3364</v>
       </c>
       <c r="N303" t="s">
+        <v>1342</v>
+      </c>
+      <c r="O303" t="s">
         <v>3365</v>
       </c>
-      <c r="O303" t="s">
+      <c r="P303" t="s">
         <v>3366</v>
-      </c>
-      <c r="P303" t="s">
-        <v>3367</v>
       </c>
       <c r="Q303" t="s">
         <v>72</v>
       </c>
       <c r="R303"/>
-      <c r="S303"/>
+      <c r="S303" t="s">
+        <v>38</v>
+      </c>
       <c r="T303" t="s">
+        <v>3367</v>
+      </c>
+      <c r="U303" t="s">
         <v>3368</v>
       </c>
-      <c r="U303" t="s">
+      <c r="V303" t="s">
         <v>3369</v>
-      </c>
-      <c r="V303" t="s">
-        <v>3370</v>
       </c>
     </row>
     <row r="304">
@@ -31076,7 +31045,7 @@
         <v>20254696</v>
       </c>
       <c r="B304" t="s">
-        <v>3371</v>
+        <v>3370</v>
       </c>
       <c r="C304" t="s">
         <v>61</v>
@@ -31097,28 +31066,28 @@
         <v>536</v>
       </c>
       <c r="I304" t="s">
+        <v>3371</v>
+      </c>
+      <c r="J304" t="s">
         <v>3372</v>
       </c>
-      <c r="J304" t="s">
+      <c r="K304" t="s">
         <v>3373</v>
       </c>
-      <c r="K304" t="s">
+      <c r="L304" t="s">
         <v>3374</v>
       </c>
-      <c r="L304" t="s">
+      <c r="M304" t="s">
         <v>3375</v>
-      </c>
-      <c r="M304" t="s">
-        <v>3376</v>
       </c>
       <c r="N304" t="s">
         <v>1342</v>
       </c>
       <c r="O304" t="s">
+        <v>3376</v>
+      </c>
+      <c r="P304" t="s">
         <v>3377</v>
-      </c>
-      <c r="P304" t="s">
-        <v>3378</v>
       </c>
       <c r="Q304" t="s">
         <v>55</v>
@@ -31140,7 +31109,7 @@
         <v>20254562</v>
       </c>
       <c r="B305" t="s">
-        <v>3379</v>
+        <v>3378</v>
       </c>
       <c r="C305" t="s">
         <v>205</v>
@@ -31152,7 +31121,7 @@
         <v>45</v>
       </c>
       <c r="F305" t="s">
-        <v>3380</v>
+        <v>3379</v>
       </c>
       <c r="G305" t="s">
         <v>27</v>
@@ -31161,28 +31130,28 @@
         <v>80</v>
       </c>
       <c r="I305" t="s">
+        <v>3380</v>
+      </c>
+      <c r="J305" t="s">
         <v>3381</v>
       </c>
-      <c r="J305" t="s">
+      <c r="K305" t="s">
         <v>3382</v>
       </c>
-      <c r="K305" t="s">
+      <c r="L305" t="s">
         <v>3383</v>
       </c>
-      <c r="L305" t="s">
+      <c r="M305" t="s">
         <v>3384</v>
-      </c>
-      <c r="M305" t="s">
-        <v>3385</v>
       </c>
       <c r="N305" t="s">
         <v>1342</v>
       </c>
       <c r="O305" t="s">
+        <v>3385</v>
+      </c>
+      <c r="P305" t="s">
         <v>3386</v>
-      </c>
-      <c r="P305" t="s">
-        <v>3387</v>
       </c>
       <c r="Q305" t="s">
         <v>37</v>
@@ -31190,13 +31159,13 @@
       <c r="R305"/>
       <c r="S305"/>
       <c r="T305" t="s">
+        <v>3387</v>
+      </c>
+      <c r="U305" t="s">
         <v>3388</v>
       </c>
-      <c r="U305" t="s">
+      <c r="V305" t="s">
         <v>3389</v>
-      </c>
-      <c r="V305" t="s">
-        <v>3390</v>
       </c>
     </row>
     <row r="306">
@@ -31204,19 +31173,19 @@
         <v>20254594</v>
       </c>
       <c r="B306" t="s">
-        <v>3391</v>
+        <v>3390</v>
       </c>
       <c r="C306" t="s">
         <v>61</v>
       </c>
       <c r="D306" t="s">
-        <v>3392</v>
+        <v>3391</v>
       </c>
       <c r="E306" t="s">
         <v>45</v>
       </c>
       <c r="F306" t="s">
-        <v>3380</v>
+        <v>3379</v>
       </c>
       <c r="G306" t="s">
         <v>47</v>
@@ -31225,28 +31194,28 @@
         <v>64</v>
       </c>
       <c r="I306" t="s">
+        <v>3392</v>
+      </c>
+      <c r="J306" t="s">
         <v>3393</v>
       </c>
-      <c r="J306" t="s">
+      <c r="K306" t="s">
         <v>3394</v>
       </c>
-      <c r="K306" t="s">
+      <c r="L306" t="s">
         <v>3395</v>
       </c>
-      <c r="L306" t="s">
+      <c r="M306" t="s">
         <v>3396</v>
-      </c>
-      <c r="M306" t="s">
-        <v>3397</v>
       </c>
       <c r="N306" t="s">
         <v>1342</v>
       </c>
       <c r="O306" t="s">
+        <v>3397</v>
+      </c>
+      <c r="P306" t="s">
         <v>3398</v>
-      </c>
-      <c r="P306" t="s">
-        <v>3399</v>
       </c>
       <c r="Q306" t="s">
         <v>37</v>
@@ -31254,13 +31223,13 @@
       <c r="R306"/>
       <c r="S306"/>
       <c r="T306" t="s">
+        <v>3399</v>
+      </c>
+      <c r="U306" t="s">
         <v>3400</v>
       </c>
-      <c r="U306" t="s">
+      <c r="V306" t="s">
         <v>3401</v>
-      </c>
-      <c r="V306" t="s">
-        <v>3402</v>
       </c>
     </row>
     <row r="307">
@@ -31268,7 +31237,7 @@
         <v>20254614</v>
       </c>
       <c r="B307" t="s">
-        <v>3403</v>
+        <v>3402</v>
       </c>
       <c r="C307" t="s">
         <v>61</v>
@@ -31280,7 +31249,7 @@
         <v>132</v>
       </c>
       <c r="F307" t="s">
-        <v>3380</v>
+        <v>3379</v>
       </c>
       <c r="G307" t="s">
         <v>27</v>
@@ -31289,28 +31258,28 @@
         <v>64</v>
       </c>
       <c r="I307" t="s">
+        <v>3403</v>
+      </c>
+      <c r="J307" t="s">
         <v>3404</v>
       </c>
-      <c r="J307" t="s">
+      <c r="K307" t="s">
         <v>3405</v>
       </c>
-      <c r="K307" t="s">
+      <c r="L307" t="s">
         <v>3406</v>
       </c>
-      <c r="L307" t="s">
+      <c r="M307" t="s">
         <v>3407</v>
-      </c>
-      <c r="M307" t="s">
-        <v>3408</v>
       </c>
       <c r="N307" t="s">
         <v>1342</v>
       </c>
       <c r="O307" t="s">
+        <v>3408</v>
+      </c>
+      <c r="P307" t="s">
         <v>3409</v>
-      </c>
-      <c r="P307" t="s">
-        <v>3410</v>
       </c>
       <c r="Q307" t="s">
         <v>37</v>
@@ -31332,19 +31301,19 @@
         <v>20258194</v>
       </c>
       <c r="B308" t="s">
-        <v>3411</v>
+        <v>3410</v>
       </c>
       <c r="C308" t="s">
         <v>23</v>
       </c>
       <c r="D308" t="s">
-        <v>3412</v>
+        <v>3411</v>
       </c>
       <c r="E308" t="s">
         <v>25</v>
       </c>
       <c r="F308" t="s">
-        <v>3413</v>
+        <v>3412</v>
       </c>
       <c r="G308" t="s">
         <v>27</v>
@@ -31353,26 +31322,26 @@
         <v>64</v>
       </c>
       <c r="I308" t="s">
+        <v>3413</v>
+      </c>
+      <c r="J308" t="s">
         <v>3414</v>
-      </c>
-      <c r="J308" t="s">
-        <v>3415</v>
       </c>
       <c r="K308"/>
       <c r="L308" t="s">
+        <v>3415</v>
+      </c>
+      <c r="M308" t="s">
         <v>3416</v>
-      </c>
-      <c r="M308" t="s">
-        <v>3417</v>
       </c>
       <c r="N308" t="s">
         <v>34</v>
       </c>
       <c r="O308" t="s">
+        <v>3417</v>
+      </c>
+      <c r="P308" t="s">
         <v>3418</v>
-      </c>
-      <c r="P308" t="s">
-        <v>3419</v>
       </c>
       <c r="Q308" t="s">
         <v>37</v>
@@ -31394,7 +31363,7 @@
         <v>20258273</v>
       </c>
       <c r="B309" t="s">
-        <v>3420</v>
+        <v>3419</v>
       </c>
       <c r="C309" t="s">
         <v>23</v>
@@ -31406,7 +31375,7 @@
         <v>633</v>
       </c>
       <c r="F309" t="s">
-        <v>3413</v>
+        <v>3412</v>
       </c>
       <c r="G309" t="s">
         <v>27</v>
@@ -31415,26 +31384,26 @@
         <v>64</v>
       </c>
       <c r="I309" t="s">
+        <v>3420</v>
+      </c>
+      <c r="J309" t="s">
         <v>3421</v>
-      </c>
-      <c r="J309" t="s">
-        <v>3422</v>
       </c>
       <c r="K309"/>
       <c r="L309" t="s">
+        <v>3422</v>
+      </c>
+      <c r="M309" t="s">
         <v>3423</v>
-      </c>
-      <c r="M309" t="s">
-        <v>3424</v>
       </c>
       <c r="N309" t="s">
         <v>34</v>
       </c>
       <c r="O309" t="s">
+        <v>3424</v>
+      </c>
+      <c r="P309" t="s">
         <v>3425</v>
-      </c>
-      <c r="P309" t="s">
-        <v>3426</v>
       </c>
       <c r="Q309" t="s">
         <v>55</v>
@@ -31442,13 +31411,13 @@
       <c r="R309"/>
       <c r="S309"/>
       <c r="T309" t="s">
+        <v>3426</v>
+      </c>
+      <c r="U309" t="s">
         <v>3427</v>
       </c>
-      <c r="U309" t="s">
+      <c r="V309" t="s">
         <v>3428</v>
-      </c>
-      <c r="V309" t="s">
-        <v>3429</v>
       </c>
     </row>
     <row r="310">
@@ -31456,7 +31425,7 @@
         <v>20254463</v>
       </c>
       <c r="B310" t="s">
-        <v>3430</v>
+        <v>3429</v>
       </c>
       <c r="C310" t="s">
         <v>43</v>
@@ -31468,7 +31437,7 @@
         <v>633</v>
       </c>
       <c r="F310" t="s">
-        <v>3431</v>
+        <v>3430</v>
       </c>
       <c r="G310" t="s">
         <v>27</v>
@@ -31477,28 +31446,28 @@
         <v>28</v>
       </c>
       <c r="I310" t="s">
+        <v>3431</v>
+      </c>
+      <c r="J310" t="s">
         <v>3432</v>
       </c>
-      <c r="J310" t="s">
+      <c r="K310" t="s">
         <v>3433</v>
       </c>
-      <c r="K310" t="s">
+      <c r="L310" t="s">
         <v>3434</v>
       </c>
-      <c r="L310" t="s">
+      <c r="M310" t="s">
         <v>3435</v>
-      </c>
-      <c r="M310" t="s">
-        <v>3436</v>
       </c>
       <c r="N310" t="s">
         <v>34</v>
       </c>
       <c r="O310" t="s">
+        <v>3436</v>
+      </c>
+      <c r="P310" t="s">
         <v>3437</v>
-      </c>
-      <c r="P310" t="s">
-        <v>3438</v>
       </c>
       <c r="Q310" t="s">
         <v>72</v>
@@ -31520,19 +31489,19 @@
         <v>20254281</v>
       </c>
       <c r="B311" t="s">
-        <v>3439</v>
+        <v>3438</v>
       </c>
       <c r="C311" t="s">
         <v>205</v>
       </c>
       <c r="D311" t="s">
-        <v>3440</v>
+        <v>3439</v>
       </c>
       <c r="E311" t="s">
         <v>132</v>
       </c>
       <c r="F311" t="s">
-        <v>3441</v>
+        <v>3440</v>
       </c>
       <c r="G311" t="s">
         <v>27</v>
@@ -31541,28 +31510,28 @@
         <v>536</v>
       </c>
       <c r="I311" t="s">
+        <v>3441</v>
+      </c>
+      <c r="J311" t="s">
         <v>3442</v>
       </c>
-      <c r="J311" t="s">
+      <c r="K311" t="s">
         <v>3443</v>
       </c>
-      <c r="K311" t="s">
+      <c r="L311" t="s">
         <v>3444</v>
       </c>
-      <c r="L311" t="s">
+      <c r="M311" t="s">
         <v>3445</v>
-      </c>
-      <c r="M311" t="s">
-        <v>3446</v>
       </c>
       <c r="N311" t="s">
         <v>1342</v>
       </c>
       <c r="O311" t="s">
+        <v>3446</v>
+      </c>
+      <c r="P311" t="s">
         <v>3447</v>
-      </c>
-      <c r="P311" t="s">
-        <v>3448</v>
       </c>
       <c r="Q311" t="s">
         <v>55</v>
@@ -31584,7 +31553,7 @@
         <v>20254317</v>
       </c>
       <c r="B312" t="s">
-        <v>3449</v>
+        <v>3448</v>
       </c>
       <c r="C312" t="s">
         <v>43</v>
@@ -31596,7 +31565,7 @@
         <v>93</v>
       </c>
       <c r="F312" t="s">
-        <v>3441</v>
+        <v>3440</v>
       </c>
       <c r="G312" t="s">
         <v>27</v>
@@ -31605,28 +31574,28 @@
         <v>536</v>
       </c>
       <c r="I312" t="s">
+        <v>3449</v>
+      </c>
+      <c r="J312" t="s">
         <v>3450</v>
       </c>
-      <c r="J312" t="s">
+      <c r="K312" t="s">
         <v>3451</v>
       </c>
-      <c r="K312" t="s">
+      <c r="L312" t="s">
         <v>3452</v>
       </c>
-      <c r="L312" t="s">
+      <c r="M312" t="s">
         <v>3453</v>
-      </c>
-      <c r="M312" t="s">
-        <v>3454</v>
       </c>
       <c r="N312" t="s">
         <v>1342</v>
       </c>
       <c r="O312" t="s">
+        <v>3454</v>
+      </c>
+      <c r="P312" t="s">
         <v>3455</v>
-      </c>
-      <c r="P312" t="s">
-        <v>3456</v>
       </c>
       <c r="Q312" t="s">
         <v>55</v>
@@ -31634,13 +31603,13 @@
       <c r="R312"/>
       <c r="S312"/>
       <c r="T312" t="s">
+        <v>3456</v>
+      </c>
+      <c r="U312" t="s">
         <v>3457</v>
       </c>
-      <c r="U312" t="s">
+      <c r="V312" t="s">
         <v>3458</v>
-      </c>
-      <c r="V312" t="s">
-        <v>3459</v>
       </c>
     </row>
     <row r="313">
@@ -31648,19 +31617,19 @@
         <v>20254145</v>
       </c>
       <c r="B313" t="s">
-        <v>3460</v>
+        <v>3459</v>
       </c>
       <c r="C313" t="s">
         <v>43</v>
       </c>
       <c r="D313" t="s">
-        <v>3461</v>
+        <v>3460</v>
       </c>
       <c r="E313" t="s">
         <v>93</v>
       </c>
       <c r="F313" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="G313" t="s">
         <v>47</v>
@@ -31669,28 +31638,28 @@
         <v>28</v>
       </c>
       <c r="I313" t="s">
+        <v>3462</v>
+      </c>
+      <c r="J313" t="s">
         <v>3463</v>
       </c>
-      <c r="J313" t="s">
+      <c r="K313" t="s">
         <v>3464</v>
       </c>
-      <c r="K313" t="s">
+      <c r="L313" t="s">
         <v>3465</v>
       </c>
-      <c r="L313" t="s">
+      <c r="M313" t="s">
         <v>3466</v>
-      </c>
-      <c r="M313" t="s">
-        <v>3467</v>
       </c>
       <c r="N313" t="s">
         <v>34</v>
       </c>
       <c r="O313" t="s">
+        <v>3467</v>
+      </c>
+      <c r="P313" t="s">
         <v>3468</v>
-      </c>
-      <c r="P313" t="s">
-        <v>3469</v>
       </c>
       <c r="Q313" t="s">
         <v>37</v>
@@ -31712,19 +31681,19 @@
         <v>20254188</v>
       </c>
       <c r="B314" t="s">
-        <v>3470</v>
+        <v>3469</v>
       </c>
       <c r="C314" t="s">
         <v>43</v>
       </c>
       <c r="D314" t="s">
-        <v>3471</v>
+        <v>3470</v>
       </c>
       <c r="E314" t="s">
         <v>93</v>
       </c>
       <c r="F314" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="G314" t="s">
         <v>47</v>
@@ -31733,28 +31702,28 @@
         <v>64</v>
       </c>
       <c r="I314" t="s">
+        <v>3471</v>
+      </c>
+      <c r="J314" t="s">
         <v>3472</v>
       </c>
-      <c r="J314" t="s">
+      <c r="K314" t="s">
         <v>3473</v>
       </c>
-      <c r="K314" t="s">
+      <c r="L314" t="s">
         <v>3474</v>
       </c>
-      <c r="L314" t="s">
+      <c r="M314" t="s">
         <v>3475</v>
       </c>
-      <c r="M314" t="s">
+      <c r="N314" t="s">
         <v>3476</v>
       </c>
-      <c r="N314" t="s">
+      <c r="O314" t="s">
         <v>3477</v>
       </c>
-      <c r="O314" t="s">
+      <c r="P314" t="s">
         <v>3478</v>
-      </c>
-      <c r="P314" t="s">
-        <v>3479</v>
       </c>
       <c r="Q314" t="s">
         <v>37</v>
@@ -31776,7 +31745,7 @@
         <v>20254225</v>
       </c>
       <c r="B315" t="s">
-        <v>3480</v>
+        <v>3479</v>
       </c>
       <c r="C315" t="s">
         <v>61</v>
@@ -31788,7 +31757,7 @@
         <v>633</v>
       </c>
       <c r="F315" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="G315" t="s">
         <v>27</v>
@@ -31797,28 +31766,28 @@
         <v>64</v>
       </c>
       <c r="I315" t="s">
+        <v>3480</v>
+      </c>
+      <c r="J315" t="s">
         <v>3481</v>
       </c>
-      <c r="J315" t="s">
+      <c r="K315" t="s">
         <v>3482</v>
       </c>
-      <c r="K315" t="s">
+      <c r="L315" t="s">
         <v>3483</v>
       </c>
-      <c r="L315" t="s">
+      <c r="M315" t="s">
         <v>3484</v>
-      </c>
-      <c r="M315" t="s">
-        <v>3485</v>
       </c>
       <c r="N315" t="s">
         <v>1342</v>
       </c>
       <c r="O315" t="s">
+        <v>3485</v>
+      </c>
+      <c r="P315" t="s">
         <v>3486</v>
-      </c>
-      <c r="P315" t="s">
-        <v>3487</v>
       </c>
       <c r="Q315" t="s">
         <v>55</v>
@@ -31826,13 +31795,13 @@
       <c r="R315"/>
       <c r="S315"/>
       <c r="T315" t="s">
+        <v>3487</v>
+      </c>
+      <c r="U315" t="s">
         <v>3488</v>
       </c>
-      <c r="U315" t="s">
+      <c r="V315" t="s">
         <v>3489</v>
-      </c>
-      <c r="V315" t="s">
-        <v>3490</v>
       </c>
     </row>
     <row r="316">
@@ -31840,19 +31809,19 @@
         <v>20254234</v>
       </c>
       <c r="B316" t="s">
-        <v>3491</v>
+        <v>3490</v>
       </c>
       <c r="C316" t="s">
         <v>43</v>
       </c>
       <c r="D316" t="s">
-        <v>3492</v>
+        <v>3491</v>
       </c>
       <c r="E316" t="s">
         <v>132</v>
       </c>
       <c r="F316" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="G316" t="s">
         <v>27</v>
@@ -31861,28 +31830,28 @@
         <v>64</v>
       </c>
       <c r="I316" t="s">
+        <v>3492</v>
+      </c>
+      <c r="J316" t="s">
         <v>3493</v>
       </c>
-      <c r="J316" t="s">
+      <c r="K316" t="s">
         <v>3494</v>
       </c>
-      <c r="K316" t="s">
+      <c r="L316" t="s">
         <v>3495</v>
       </c>
-      <c r="L316" t="s">
+      <c r="M316" t="s">
         <v>3496</v>
-      </c>
-      <c r="M316" t="s">
-        <v>3497</v>
       </c>
       <c r="N316" t="s">
         <v>34</v>
       </c>
       <c r="O316" t="s">
+        <v>3497</v>
+      </c>
+      <c r="P316" t="s">
         <v>3498</v>
-      </c>
-      <c r="P316" t="s">
-        <v>3499</v>
       </c>
       <c r="Q316" t="s">
         <v>72</v>
@@ -31890,13 +31859,13 @@
       <c r="R316"/>
       <c r="S316"/>
       <c r="T316" t="s">
+        <v>3499</v>
+      </c>
+      <c r="U316" t="s">
         <v>3500</v>
       </c>
-      <c r="U316" t="s">
+      <c r="V316" t="s">
         <v>3501</v>
-      </c>
-      <c r="V316" t="s">
-        <v>3502</v>
       </c>
     </row>
     <row r="317">
@@ -31904,19 +31873,19 @@
         <v>20254071</v>
       </c>
       <c r="B317" t="s">
-        <v>3503</v>
+        <v>3502</v>
       </c>
       <c r="C317" t="s">
         <v>61</v>
       </c>
       <c r="D317" t="s">
-        <v>3504</v>
+        <v>3503</v>
       </c>
       <c r="E317" t="s">
         <v>93</v>
       </c>
       <c r="F317" t="s">
-        <v>3505</v>
+        <v>3504</v>
       </c>
       <c r="G317" t="s">
         <v>47</v>
@@ -31925,28 +31894,28 @@
         <v>64</v>
       </c>
       <c r="I317" t="s">
+        <v>3505</v>
+      </c>
+      <c r="J317" t="s">
         <v>3506</v>
       </c>
-      <c r="J317" t="s">
+      <c r="K317" t="s">
         <v>3507</v>
       </c>
-      <c r="K317" t="s">
+      <c r="L317" t="s">
         <v>3508</v>
       </c>
-      <c r="L317" t="s">
+      <c r="M317" t="s">
         <v>3509</v>
-      </c>
-      <c r="M317" t="s">
-        <v>3510</v>
       </c>
       <c r="N317" t="s">
         <v>34</v>
       </c>
       <c r="O317" t="s">
+        <v>3510</v>
+      </c>
+      <c r="P317" t="s">
         <v>3511</v>
-      </c>
-      <c r="P317" t="s">
-        <v>3512</v>
       </c>
       <c r="Q317" t="s">
         <v>37</v>
@@ -31954,13 +31923,13 @@
       <c r="R317"/>
       <c r="S317"/>
       <c r="T317" t="s">
+        <v>3512</v>
+      </c>
+      <c r="U317" t="s">
         <v>3513</v>
       </c>
-      <c r="U317" t="s">
+      <c r="V317" t="s">
         <v>3514</v>
-      </c>
-      <c r="V317" t="s">
-        <v>3515</v>
       </c>
     </row>
     <row r="318">
@@ -31968,7 +31937,7 @@
         <v>20254024</v>
       </c>
       <c r="B318" t="s">
-        <v>3516</v>
+        <v>3515</v>
       </c>
       <c r="C318" t="s">
         <v>61</v>
@@ -31980,7 +31949,7 @@
         <v>132</v>
       </c>
       <c r="F318" t="s">
-        <v>3517</v>
+        <v>3516</v>
       </c>
       <c r="G318" t="s">
         <v>27</v>
@@ -31989,28 +31958,28 @@
         <v>119</v>
       </c>
       <c r="I318" t="s">
+        <v>3517</v>
+      </c>
+      <c r="J318" t="s">
         <v>3518</v>
       </c>
-      <c r="J318" t="s">
+      <c r="K318" t="s">
         <v>3519</v>
       </c>
-      <c r="K318" t="s">
+      <c r="L318" t="s">
         <v>3520</v>
       </c>
-      <c r="L318" t="s">
+      <c r="M318" t="s">
         <v>3521</v>
-      </c>
-      <c r="M318" t="s">
-        <v>3522</v>
       </c>
       <c r="N318" t="s">
         <v>1342</v>
       </c>
       <c r="O318" t="s">
+        <v>3522</v>
+      </c>
+      <c r="P318" t="s">
         <v>3523</v>
-      </c>
-      <c r="P318" t="s">
-        <v>3524</v>
       </c>
       <c r="Q318" t="s">
         <v>55</v>
@@ -32032,7 +32001,7 @@
         <v>20257863</v>
       </c>
       <c r="B319" t="s">
-        <v>3525</v>
+        <v>3524</v>
       </c>
       <c r="C319" t="s">
         <v>23</v>
@@ -32044,7 +32013,7 @@
         <v>1826</v>
       </c>
       <c r="F319" t="s">
-        <v>3517</v>
+        <v>3516</v>
       </c>
       <c r="G319" t="s">
         <v>27</v>
@@ -32053,26 +32022,26 @@
         <v>28</v>
       </c>
       <c r="I319" t="s">
+        <v>3525</v>
+      </c>
+      <c r="J319" t="s">
         <v>3526</v>
-      </c>
-      <c r="J319" t="s">
-        <v>3527</v>
       </c>
       <c r="K319"/>
       <c r="L319" t="s">
+        <v>3527</v>
+      </c>
+      <c r="M319" t="s">
         <v>3528</v>
-      </c>
-      <c r="M319" t="s">
-        <v>3529</v>
       </c>
       <c r="N319" t="s">
         <v>34</v>
       </c>
       <c r="O319" t="s">
+        <v>3529</v>
+      </c>
+      <c r="P319" t="s">
         <v>3530</v>
-      </c>
-      <c r="P319" t="s">
-        <v>3531</v>
       </c>
       <c r="Q319" t="s">
         <v>37</v>
@@ -32094,7 +32063,7 @@
         <v>20257888</v>
       </c>
       <c r="B320" t="s">
-        <v>3532</v>
+        <v>3531</v>
       </c>
       <c r="C320" t="s">
         <v>23</v>
@@ -32106,7 +32075,7 @@
         <v>1473</v>
       </c>
       <c r="F320" t="s">
-        <v>3517</v>
+        <v>3516</v>
       </c>
       <c r="G320" t="s">
         <v>27</v>
@@ -32115,26 +32084,26 @@
         <v>119</v>
       </c>
       <c r="I320" t="s">
+        <v>3532</v>
+      </c>
+      <c r="J320" t="s">
         <v>3533</v>
-      </c>
-      <c r="J320" t="s">
-        <v>3534</v>
       </c>
       <c r="K320"/>
       <c r="L320" t="s">
+        <v>3534</v>
+      </c>
+      <c r="M320" t="s">
         <v>3535</v>
-      </c>
-      <c r="M320" t="s">
-        <v>3536</v>
       </c>
       <c r="N320" t="s">
         <v>34</v>
       </c>
       <c r="O320" t="s">
+        <v>3536</v>
+      </c>
+      <c r="P320" t="s">
         <v>3537</v>
-      </c>
-      <c r="P320" t="s">
-        <v>3538</v>
       </c>
       <c r="Q320" t="s">
         <v>72</v>
@@ -32156,7 +32125,7 @@
         <v>20257890</v>
       </c>
       <c r="B321" t="s">
-        <v>3539</v>
+        <v>3538</v>
       </c>
       <c r="C321" t="s">
         <v>23</v>
@@ -32168,7 +32137,7 @@
         <v>633</v>
       </c>
       <c r="F321" t="s">
-        <v>3517</v>
+        <v>3516</v>
       </c>
       <c r="G321" t="s">
         <v>27</v>
@@ -32177,26 +32146,26 @@
         <v>536</v>
       </c>
       <c r="I321" t="s">
+        <v>3539</v>
+      </c>
+      <c r="J321" t="s">
         <v>3540</v>
-      </c>
-      <c r="J321" t="s">
-        <v>3541</v>
       </c>
       <c r="K321"/>
       <c r="L321" t="s">
+        <v>3541</v>
+      </c>
+      <c r="M321" t="s">
         <v>3542</v>
-      </c>
-      <c r="M321" t="s">
-        <v>3543</v>
       </c>
       <c r="N321" t="s">
         <v>34</v>
       </c>
       <c r="O321" t="s">
+        <v>3543</v>
+      </c>
+      <c r="P321" t="s">
         <v>3544</v>
-      </c>
-      <c r="P321" t="s">
-        <v>3545</v>
       </c>
       <c r="Q321" t="s">
         <v>55</v>
@@ -32218,17 +32187,17 @@
         <v>20254003</v>
       </c>
       <c r="B322" t="s">
-        <v>3546</v>
+        <v>3545</v>
       </c>
       <c r="C322" t="s">
         <v>205</v>
       </c>
       <c r="D322" t="s">
-        <v>3547</v>
+        <v>3546</v>
       </c>
       <c r="E322"/>
       <c r="F322" t="s">
-        <v>3548</v>
+        <v>3547</v>
       </c>
       <c r="G322" t="s">
         <v>27</v>
@@ -32237,28 +32206,28 @@
         <v>28</v>
       </c>
       <c r="I322" t="s">
+        <v>3548</v>
+      </c>
+      <c r="J322" t="s">
         <v>3549</v>
       </c>
-      <c r="J322" t="s">
+      <c r="K322" t="s">
         <v>3550</v>
       </c>
-      <c r="K322" t="s">
+      <c r="L322" t="s">
         <v>3551</v>
       </c>
-      <c r="L322" t="s">
+      <c r="M322" t="s">
         <v>3552</v>
-      </c>
-      <c r="M322" t="s">
-        <v>3553</v>
       </c>
       <c r="N322" t="s">
         <v>1342</v>
       </c>
       <c r="O322" t="s">
+        <v>3553</v>
+      </c>
+      <c r="P322" t="s">
         <v>3554</v>
-      </c>
-      <c r="P322" t="s">
-        <v>3555</v>
       </c>
       <c r="Q322" t="s">
         <v>37</v>
@@ -32266,13 +32235,13 @@
       <c r="R322"/>
       <c r="S322"/>
       <c r="T322" t="s">
+        <v>3555</v>
+      </c>
+      <c r="U322" t="s">
         <v>3556</v>
       </c>
-      <c r="U322" t="s">
+      <c r="V322" t="s">
         <v>3557</v>
-      </c>
-      <c r="V322" t="s">
-        <v>3558</v>
       </c>
     </row>
     <row r="323">
@@ -32280,7 +32249,7 @@
         <v>20253984</v>
       </c>
       <c r="B323" t="s">
-        <v>3559</v>
+        <v>3558</v>
       </c>
       <c r="C323" t="s">
         <v>43</v>
@@ -32290,7 +32259,7 @@
       </c>
       <c r="E323"/>
       <c r="F323" t="s">
-        <v>3560</v>
+        <v>3559</v>
       </c>
       <c r="G323" t="s">
         <v>27</v>
@@ -32299,28 +32268,28 @@
         <v>28</v>
       </c>
       <c r="I323" t="s">
+        <v>3462</v>
+      </c>
+      <c r="J323" t="s">
         <v>3463</v>
       </c>
-      <c r="J323" t="s">
+      <c r="K323" t="s">
         <v>3464</v>
       </c>
-      <c r="K323" t="s">
-        <v>3465</v>
-      </c>
       <c r="L323" t="s">
+        <v>3560</v>
+      </c>
+      <c r="M323" t="s">
         <v>3561</v>
-      </c>
-      <c r="M323" t="s">
-        <v>3562</v>
       </c>
       <c r="N323" t="s">
         <v>1329</v>
       </c>
       <c r="O323" t="s">
+        <v>3562</v>
+      </c>
+      <c r="P323" t="s">
         <v>3563</v>
-      </c>
-      <c r="P323" t="s">
-        <v>3564</v>
       </c>
       <c r="Q323" t="s">
         <v>37</v>
@@ -32342,7 +32311,7 @@
         <v>20257663</v>
       </c>
       <c r="B324" t="s">
-        <v>3565</v>
+        <v>3564</v>
       </c>
       <c r="C324" t="s">
         <v>23</v>
@@ -32354,7 +32323,7 @@
         <v>25</v>
       </c>
       <c r="F324" t="s">
-        <v>3560</v>
+        <v>3559</v>
       </c>
       <c r="G324" t="s">
         <v>27</v>
@@ -32363,26 +32332,26 @@
         <v>119</v>
       </c>
       <c r="I324" t="s">
+        <v>3565</v>
+      </c>
+      <c r="J324" t="s">
         <v>3566</v>
-      </c>
-      <c r="J324" t="s">
-        <v>3567</v>
       </c>
       <c r="K324"/>
       <c r="L324" t="s">
+        <v>3567</v>
+      </c>
+      <c r="M324" t="s">
         <v>3568</v>
-      </c>
-      <c r="M324" t="s">
-        <v>3569</v>
       </c>
       <c r="N324" t="s">
         <v>34</v>
       </c>
       <c r="O324" t="s">
+        <v>3569</v>
+      </c>
+      <c r="P324" t="s">
         <v>3570</v>
-      </c>
-      <c r="P324" t="s">
-        <v>3571</v>
       </c>
       <c r="Q324" t="s">
         <v>37</v>
@@ -32390,13 +32359,13 @@
       <c r="R324"/>
       <c r="S324"/>
       <c r="T324" t="s">
+        <v>3571</v>
+      </c>
+      <c r="U324" t="s">
         <v>3572</v>
       </c>
-      <c r="U324" t="s">
+      <c r="V324" t="s">
         <v>3573</v>
-      </c>
-      <c r="V324" t="s">
-        <v>3574</v>
       </c>
     </row>
     <row r="325">
@@ -32404,19 +32373,19 @@
         <v>20257698</v>
       </c>
       <c r="B325" t="s">
-        <v>3575</v>
+        <v>3574</v>
       </c>
       <c r="C325" t="s">
         <v>23</v>
       </c>
       <c r="D325" t="s">
-        <v>3576</v>
+        <v>3575</v>
       </c>
       <c r="E325" t="s">
         <v>132</v>
       </c>
       <c r="F325" t="s">
-        <v>3560</v>
+        <v>3559</v>
       </c>
       <c r="G325" t="s">
         <v>27</v>
@@ -32425,26 +32394,26 @@
         <v>119</v>
       </c>
       <c r="I325" t="s">
+        <v>3576</v>
+      </c>
+      <c r="J325" t="s">
         <v>3577</v>
-      </c>
-      <c r="J325" t="s">
-        <v>3578</v>
       </c>
       <c r="K325"/>
       <c r="L325" t="s">
+        <v>3578</v>
+      </c>
+      <c r="M325" t="s">
         <v>3579</v>
-      </c>
-      <c r="M325" t="s">
-        <v>3580</v>
       </c>
       <c r="N325" t="s">
         <v>34</v>
       </c>
       <c r="O325" t="s">
+        <v>3580</v>
+      </c>
+      <c r="P325" t="s">
         <v>3581</v>
-      </c>
-      <c r="P325" t="s">
-        <v>3582</v>
       </c>
       <c r="Q325" t="s">
         <v>37</v>
@@ -32466,19 +32435,19 @@
         <v>20253971</v>
       </c>
       <c r="B326" t="s">
-        <v>3583</v>
+        <v>3582</v>
       </c>
       <c r="C326" t="s">
         <v>61</v>
       </c>
       <c r="D326" t="s">
-        <v>3584</v>
+        <v>3583</v>
       </c>
       <c r="E326" t="s">
         <v>93</v>
       </c>
       <c r="F326" t="s">
-        <v>3585</v>
+        <v>3584</v>
       </c>
       <c r="G326" t="s">
         <v>47</v>
@@ -32487,28 +32456,28 @@
         <v>536</v>
       </c>
       <c r="I326" t="s">
+        <v>3585</v>
+      </c>
+      <c r="J326" t="s">
         <v>3586</v>
       </c>
-      <c r="J326" t="s">
+      <c r="K326" t="s">
         <v>3587</v>
       </c>
-      <c r="K326" t="s">
+      <c r="L326" t="s">
         <v>3588</v>
       </c>
-      <c r="L326" t="s">
+      <c r="M326" t="s">
         <v>3589</v>
-      </c>
-      <c r="M326" t="s">
-        <v>3590</v>
       </c>
       <c r="N326" t="s">
         <v>34</v>
       </c>
       <c r="O326" t="s">
+        <v>3590</v>
+      </c>
+      <c r="P326" t="s">
         <v>3591</v>
-      </c>
-      <c r="P326" t="s">
-        <v>3592</v>
       </c>
       <c r="Q326" t="s">
         <v>55</v>
@@ -32516,13 +32485,13 @@
       <c r="R326"/>
       <c r="S326"/>
       <c r="T326" t="s">
+        <v>3456</v>
+      </c>
+      <c r="U326" t="s">
         <v>3457</v>
       </c>
-      <c r="U326" t="s">
+      <c r="V326" t="s">
         <v>3458</v>
-      </c>
-      <c r="V326" t="s">
-        <v>3459</v>
       </c>
     </row>
     <row r="327">
@@ -32530,7 +32499,7 @@
         <v>20257601</v>
       </c>
       <c r="B327" t="s">
-        <v>3593</v>
+        <v>3592</v>
       </c>
       <c r="C327" t="s">
         <v>23</v>
@@ -32542,7 +32511,7 @@
         <v>1473</v>
       </c>
       <c r="F327" t="s">
-        <v>3594</v>
+        <v>3593</v>
       </c>
       <c r="G327" t="s">
         <v>27</v>
@@ -32551,26 +32520,26 @@
         <v>64</v>
       </c>
       <c r="I327" t="s">
+        <v>3594</v>
+      </c>
+      <c r="J327" t="s">
         <v>3595</v>
-      </c>
-      <c r="J327" t="s">
-        <v>3596</v>
       </c>
       <c r="K327"/>
       <c r="L327" t="s">
+        <v>3596</v>
+      </c>
+      <c r="M327" t="s">
         <v>3597</v>
-      </c>
-      <c r="M327" t="s">
-        <v>3598</v>
       </c>
       <c r="N327" t="s">
         <v>34</v>
       </c>
       <c r="O327" t="s">
+        <v>3598</v>
+      </c>
+      <c r="P327" t="s">
         <v>3599</v>
-      </c>
-      <c r="P327" t="s">
-        <v>3600</v>
       </c>
       <c r="Q327" t="s">
         <v>55</v>
@@ -32592,17 +32561,17 @@
         <v>20253941</v>
       </c>
       <c r="B328" t="s">
-        <v>3601</v>
+        <v>3600</v>
       </c>
       <c r="C328" t="s">
         <v>43</v>
       </c>
       <c r="D328" t="s">
-        <v>3602</v>
+        <v>3601</v>
       </c>
       <c r="E328"/>
       <c r="F328" t="s">
-        <v>3603</v>
+        <v>3602</v>
       </c>
       <c r="G328" t="s">
         <v>27</v>
@@ -32611,28 +32580,28 @@
         <v>1533</v>
       </c>
       <c r="I328" t="s">
+        <v>3603</v>
+      </c>
+      <c r="J328" t="s">
         <v>3604</v>
       </c>
-      <c r="J328" t="s">
+      <c r="K328" t="s">
         <v>3605</v>
       </c>
-      <c r="K328" t="s">
+      <c r="L328" t="s">
         <v>3606</v>
       </c>
-      <c r="L328" t="s">
+      <c r="M328" t="s">
         <v>3607</v>
-      </c>
-      <c r="M328" t="s">
-        <v>3608</v>
       </c>
       <c r="N328" t="s">
         <v>1965</v>
       </c>
       <c r="O328" t="s">
+        <v>3608</v>
+      </c>
+      <c r="P328" t="s">
         <v>3609</v>
-      </c>
-      <c r="P328" t="s">
-        <v>3610</v>
       </c>
       <c r="Q328" t="s">
         <v>37</v>
@@ -32642,60 +32611,6 @@
       <c r="T328"/>
       <c r="U328"/>
       <c r="V328"/>
-    </row>
-    <row r="329">
-      <c r="A329" t="n">
-        <v>20180032</v>
-      </c>
-      <c r="B329" t="s">
-        <v>3611</v>
-      </c>
-      <c r="C329" t="s">
-        <v>3612</v>
-      </c>
-      <c r="D329"/>
-      <c r="E329"/>
-      <c r="F329" t="s">
-        <v>673</v>
-      </c>
-      <c r="G329"/>
-      <c r="H329" t="s">
-        <v>28</v>
-      </c>
-      <c r="I329" t="s">
-        <v>3613</v>
-      </c>
-      <c r="J329" t="s">
-        <v>3614</v>
-      </c>
-      <c r="K329" t="s">
-        <v>3615</v>
-      </c>
-      <c r="L329"/>
-      <c r="M329"/>
-      <c r="N329" t="s">
-        <v>34</v>
-      </c>
-      <c r="O329" t="s">
-        <v>3616</v>
-      </c>
-      <c r="P329" t="s">
-        <v>3617</v>
-      </c>
-      <c r="Q329" t="s">
-        <v>975</v>
-      </c>
-      <c r="R329"/>
-      <c r="S329"/>
-      <c r="T329" t="s">
-        <v>3618</v>
-      </c>
-      <c r="U329" t="s">
-        <v>3619</v>
-      </c>
-      <c r="V329" t="s">
-        <v>3620</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update parliament data - 2026-02-27
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_CDF_EFK.xlsx
+++ b/Objets_parlementaires_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3619" uniqueCount="3619">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3621" uniqueCount="3621">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -10140,10 +10140,16 @@
     <t xml:space="preserve">&lt;p&gt;Der Bundesrat wird beauftragt, die rechtlichen Grundlagen zu erlassen, damit baldmöglichst&amp;nbsp; qualitätsgesicherte, aktuelle und insbesondere international anschlussfähige und vergleichbare strukturierte Daten der Bundesverwaltung zur Mehrfachnutzung (unter anderem durch KI) für Forschung, Planung und Steuerung zur Verfügung gestellt werden.&amp;nbsp;Diesbezügliche verbindliche Standards für die Bundesverwaltung sind zu erlassen.&amp;nbsp;Der Bundesrat wird zudem beauftragt, eine prioritäre Auswahl jener Verwaltungsdaten zu definieren, die für eine zügige und KI-taugliche Mehrfachnutzung zuerst harmonisiert, standardisiert und technisch zugänglich gemacht werden sollen.&amp;nbsp;Insbesondere die öffentliche Bereitstellung weiterer Registerdaten ist zu prüfen. Gezielte Pilotversuche nach Art. 15 EMBAG können dies beschleunigen und sind vom Bundesrat mit den benötigten Mitteln zu beantragen.&lt;/p&gt;</t>
   </si>
   <si>
+    <t xml:space="preserve">In Ständerat geplant / Planifié au Conseil des Etats</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254620</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254620</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-02-27</t>
   </si>
   <si>
     <t xml:space="preserve">Staatspolitik|Medien und Kommunikation|Menschenrechte</t>
@@ -31108,27 +31114,29 @@
         <v>3374</v>
       </c>
       <c r="N304" t="s">
-        <v>34</v>
+        <v>3375</v>
       </c>
       <c r="O304" t="s">
-        <v>3375</v>
+        <v>3376</v>
       </c>
       <c r="P304" t="s">
-        <v>3376</v>
+        <v>3377</v>
       </c>
       <c r="Q304" t="s">
         <v>89</v>
       </c>
       <c r="R304"/>
-      <c r="S304"/>
+      <c r="S304" t="s">
+        <v>3378</v>
+      </c>
       <c r="T304" t="s">
-        <v>3377</v>
+        <v>3379</v>
       </c>
       <c r="U304" t="s">
-        <v>3378</v>
+        <v>3380</v>
       </c>
       <c r="V304" t="s">
-        <v>3379</v>
+        <v>3381</v>
       </c>
     </row>
     <row r="305">
@@ -31136,7 +31144,7 @@
         <v>20254696</v>
       </c>
       <c r="B305" t="s">
-        <v>3380</v>
+        <v>3382</v>
       </c>
       <c r="C305" t="s">
         <v>23</v>
@@ -31157,28 +31165,28 @@
         <v>548</v>
       </c>
       <c r="I305" t="s">
-        <v>3381</v>
+        <v>3383</v>
       </c>
       <c r="J305" t="s">
-        <v>3382</v>
+        <v>3384</v>
       </c>
       <c r="K305" t="s">
-        <v>3383</v>
+        <v>3385</v>
       </c>
       <c r="L305" t="s">
-        <v>3384</v>
+        <v>3386</v>
       </c>
       <c r="M305" t="s">
-        <v>3385</v>
+        <v>3387</v>
       </c>
       <c r="N305" t="s">
         <v>34</v>
       </c>
       <c r="O305" t="s">
-        <v>3386</v>
+        <v>3388</v>
       </c>
       <c r="P305" t="s">
-        <v>3387</v>
+        <v>3389</v>
       </c>
       <c r="Q305" t="s">
         <v>73</v>
@@ -31200,7 +31208,7 @@
         <v>20254562</v>
       </c>
       <c r="B306" t="s">
-        <v>3388</v>
+        <v>3390</v>
       </c>
       <c r="C306" t="s">
         <v>217</v>
@@ -31221,28 +31229,28 @@
         <v>97</v>
       </c>
       <c r="I306" t="s">
-        <v>3389</v>
+        <v>3391</v>
       </c>
       <c r="J306" t="s">
-        <v>3390</v>
+        <v>3392</v>
       </c>
       <c r="K306" t="s">
-        <v>3391</v>
+        <v>3393</v>
       </c>
       <c r="L306" t="s">
-        <v>3392</v>
+        <v>3394</v>
       </c>
       <c r="M306" t="s">
-        <v>3393</v>
+        <v>3395</v>
       </c>
       <c r="N306" t="s">
         <v>34</v>
       </c>
       <c r="O306" t="s">
-        <v>3394</v>
+        <v>3396</v>
       </c>
       <c r="P306" t="s">
-        <v>3395</v>
+        <v>3397</v>
       </c>
       <c r="Q306" t="s">
         <v>37</v>
@@ -31250,13 +31258,13 @@
       <c r="R306"/>
       <c r="S306"/>
       <c r="T306" t="s">
-        <v>3396</v>
+        <v>3398</v>
       </c>
       <c r="U306" t="s">
-        <v>3397</v>
+        <v>3399</v>
       </c>
       <c r="V306" t="s">
-        <v>3398</v>
+        <v>3400</v>
       </c>
     </row>
     <row r="307">
@@ -31264,13 +31272,13 @@
         <v>20254594</v>
       </c>
       <c r="B307" t="s">
-        <v>3399</v>
+        <v>3401</v>
       </c>
       <c r="C307" t="s">
         <v>23</v>
       </c>
       <c r="D307" t="s">
-        <v>3400</v>
+        <v>3402</v>
       </c>
       <c r="E307" t="s">
         <v>63</v>
@@ -31285,42 +31293,44 @@
         <v>81</v>
       </c>
       <c r="I307" t="s">
-        <v>3401</v>
+        <v>3403</v>
       </c>
       <c r="J307" t="s">
-        <v>3402</v>
+        <v>3404</v>
       </c>
       <c r="K307" t="s">
-        <v>3403</v>
+        <v>3405</v>
       </c>
       <c r="L307" t="s">
-        <v>3404</v>
+        <v>3406</v>
       </c>
       <c r="M307" t="s">
-        <v>3405</v>
+        <v>3407</v>
       </c>
       <c r="N307" t="s">
-        <v>34</v>
+        <v>3375</v>
       </c>
       <c r="O307" t="s">
-        <v>3406</v>
+        <v>3408</v>
       </c>
       <c r="P307" t="s">
-        <v>3407</v>
+        <v>3409</v>
       </c>
       <c r="Q307" t="s">
         <v>37</v>
       </c>
       <c r="R307"/>
-      <c r="S307"/>
+      <c r="S307" t="s">
+        <v>3378</v>
+      </c>
       <c r="T307" t="s">
-        <v>3408</v>
+        <v>3410</v>
       </c>
       <c r="U307" t="s">
-        <v>3409</v>
+        <v>3411</v>
       </c>
       <c r="V307" t="s">
-        <v>3410</v>
+        <v>3412</v>
       </c>
     </row>
     <row r="308">
@@ -31328,7 +31338,7 @@
         <v>20254614</v>
       </c>
       <c r="B308" t="s">
-        <v>3411</v>
+        <v>3413</v>
       </c>
       <c r="C308" t="s">
         <v>23</v>
@@ -31349,28 +31359,28 @@
         <v>81</v>
       </c>
       <c r="I308" t="s">
-        <v>3412</v>
+        <v>3414</v>
       </c>
       <c r="J308" t="s">
-        <v>3413</v>
+        <v>3415</v>
       </c>
       <c r="K308" t="s">
-        <v>3414</v>
+        <v>3416</v>
       </c>
       <c r="L308" t="s">
-        <v>3415</v>
+        <v>3417</v>
       </c>
       <c r="M308" t="s">
-        <v>3416</v>
+        <v>3418</v>
       </c>
       <c r="N308" t="s">
         <v>34</v>
       </c>
       <c r="O308" t="s">
-        <v>3417</v>
+        <v>3419</v>
       </c>
       <c r="P308" t="s">
-        <v>3418</v>
+        <v>3420</v>
       </c>
       <c r="Q308" t="s">
         <v>37</v>
@@ -31392,19 +31402,19 @@
         <v>20258194</v>
       </c>
       <c r="B309" t="s">
-        <v>3419</v>
+        <v>3421</v>
       </c>
       <c r="C309" t="s">
         <v>43</v>
       </c>
       <c r="D309" t="s">
-        <v>3420</v>
+        <v>3422</v>
       </c>
       <c r="E309" t="s">
         <v>45</v>
       </c>
       <c r="F309" t="s">
-        <v>3421</v>
+        <v>3423</v>
       </c>
       <c r="G309" t="s">
         <v>27</v>
@@ -31413,26 +31423,26 @@
         <v>81</v>
       </c>
       <c r="I309" t="s">
-        <v>3422</v>
+        <v>3424</v>
       </c>
       <c r="J309" t="s">
-        <v>3423</v>
+        <v>3425</v>
       </c>
       <c r="K309"/>
       <c r="L309" t="s">
-        <v>3424</v>
+        <v>3426</v>
       </c>
       <c r="M309" t="s">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="N309" t="s">
         <v>53</v>
       </c>
       <c r="O309" t="s">
-        <v>3426</v>
+        <v>3428</v>
       </c>
       <c r="P309" t="s">
-        <v>3427</v>
+        <v>3429</v>
       </c>
       <c r="Q309" t="s">
         <v>37</v>
@@ -31454,7 +31464,7 @@
         <v>20258273</v>
       </c>
       <c r="B310" t="s">
-        <v>3428</v>
+        <v>3430</v>
       </c>
       <c r="C310" t="s">
         <v>43</v>
@@ -31466,7 +31476,7 @@
         <v>645</v>
       </c>
       <c r="F310" t="s">
-        <v>3421</v>
+        <v>3423</v>
       </c>
       <c r="G310" t="s">
         <v>27</v>
@@ -31475,26 +31485,26 @@
         <v>81</v>
       </c>
       <c r="I310" t="s">
-        <v>3429</v>
+        <v>3431</v>
       </c>
       <c r="J310" t="s">
-        <v>3430</v>
+        <v>3432</v>
       </c>
       <c r="K310"/>
       <c r="L310" t="s">
-        <v>3431</v>
+        <v>3433</v>
       </c>
       <c r="M310" t="s">
-        <v>3432</v>
+        <v>3434</v>
       </c>
       <c r="N310" t="s">
         <v>53</v>
       </c>
       <c r="O310" t="s">
-        <v>3433</v>
+        <v>3435</v>
       </c>
       <c r="P310" t="s">
-        <v>3434</v>
+        <v>3436</v>
       </c>
       <c r="Q310" t="s">
         <v>73</v>
@@ -31502,13 +31512,13 @@
       <c r="R310"/>
       <c r="S310"/>
       <c r="T310" t="s">
-        <v>3435</v>
+        <v>3437</v>
       </c>
       <c r="U310" t="s">
-        <v>3436</v>
+        <v>3438</v>
       </c>
       <c r="V310" t="s">
-        <v>3437</v>
+        <v>3439</v>
       </c>
     </row>
     <row r="311">
@@ -31516,7 +31526,7 @@
         <v>20254463</v>
       </c>
       <c r="B311" t="s">
-        <v>3438</v>
+        <v>3440</v>
       </c>
       <c r="C311" t="s">
         <v>61</v>
@@ -31528,7 +31538,7 @@
         <v>645</v>
       </c>
       <c r="F311" t="s">
-        <v>3439</v>
+        <v>3441</v>
       </c>
       <c r="G311" t="s">
         <v>27</v>
@@ -31537,28 +31547,28 @@
         <v>47</v>
       </c>
       <c r="I311" t="s">
-        <v>3440</v>
+        <v>3442</v>
       </c>
       <c r="J311" t="s">
-        <v>3441</v>
+        <v>3443</v>
       </c>
       <c r="K311" t="s">
-        <v>3442</v>
+        <v>3444</v>
       </c>
       <c r="L311" t="s">
-        <v>3443</v>
+        <v>3445</v>
       </c>
       <c r="M311" t="s">
-        <v>3444</v>
+        <v>3446</v>
       </c>
       <c r="N311" t="s">
         <v>53</v>
       </c>
       <c r="O311" t="s">
-        <v>3445</v>
+        <v>3447</v>
       </c>
       <c r="P311" t="s">
-        <v>3446</v>
+        <v>3448</v>
       </c>
       <c r="Q311" t="s">
         <v>89</v>
@@ -31580,19 +31590,19 @@
         <v>20254281</v>
       </c>
       <c r="B312" t="s">
-        <v>3447</v>
+        <v>3449</v>
       </c>
       <c r="C312" t="s">
         <v>217</v>
       </c>
       <c r="D312" t="s">
-        <v>3448</v>
+        <v>3450</v>
       </c>
       <c r="E312" t="s">
         <v>144</v>
       </c>
       <c r="F312" t="s">
-        <v>3449</v>
+        <v>3451</v>
       </c>
       <c r="G312" t="s">
         <v>27</v>
@@ -31601,28 +31611,28 @@
         <v>548</v>
       </c>
       <c r="I312" t="s">
-        <v>3450</v>
+        <v>3452</v>
       </c>
       <c r="J312" t="s">
-        <v>3451</v>
+        <v>3453</v>
       </c>
       <c r="K312" t="s">
-        <v>3452</v>
+        <v>3454</v>
       </c>
       <c r="L312" t="s">
-        <v>3453</v>
+        <v>3455</v>
       </c>
       <c r="M312" t="s">
-        <v>3454</v>
+        <v>3456</v>
       </c>
       <c r="N312" t="s">
         <v>34</v>
       </c>
       <c r="O312" t="s">
-        <v>3455</v>
+        <v>3457</v>
       </c>
       <c r="P312" t="s">
-        <v>3456</v>
+        <v>3458</v>
       </c>
       <c r="Q312" t="s">
         <v>73</v>
@@ -31644,7 +31654,7 @@
         <v>20254317</v>
       </c>
       <c r="B313" t="s">
-        <v>3457</v>
+        <v>3459</v>
       </c>
       <c r="C313" t="s">
         <v>61</v>
@@ -31656,7 +31666,7 @@
         <v>25</v>
       </c>
       <c r="F313" t="s">
-        <v>3449</v>
+        <v>3451</v>
       </c>
       <c r="G313" t="s">
         <v>27</v>
@@ -31665,28 +31675,28 @@
         <v>548</v>
       </c>
       <c r="I313" t="s">
-        <v>3458</v>
+        <v>3460</v>
       </c>
       <c r="J313" t="s">
-        <v>3459</v>
+        <v>3461</v>
       </c>
       <c r="K313" t="s">
-        <v>3460</v>
+        <v>3462</v>
       </c>
       <c r="L313" t="s">
-        <v>3461</v>
+        <v>3463</v>
       </c>
       <c r="M313" t="s">
-        <v>3462</v>
+        <v>3464</v>
       </c>
       <c r="N313" t="s">
         <v>34</v>
       </c>
       <c r="O313" t="s">
-        <v>3463</v>
+        <v>3465</v>
       </c>
       <c r="P313" t="s">
-        <v>3464</v>
+        <v>3466</v>
       </c>
       <c r="Q313" t="s">
         <v>73</v>
@@ -31694,13 +31704,13 @@
       <c r="R313"/>
       <c r="S313"/>
       <c r="T313" t="s">
-        <v>3465</v>
+        <v>3467</v>
       </c>
       <c r="U313" t="s">
-        <v>3466</v>
+        <v>3468</v>
       </c>
       <c r="V313" t="s">
-        <v>3467</v>
+        <v>3469</v>
       </c>
     </row>
     <row r="314">
@@ -31708,19 +31718,19 @@
         <v>20254145</v>
       </c>
       <c r="B314" t="s">
-        <v>3468</v>
+        <v>3470</v>
       </c>
       <c r="C314" t="s">
         <v>61</v>
       </c>
       <c r="D314" t="s">
-        <v>3469</v>
+        <v>3471</v>
       </c>
       <c r="E314" t="s">
         <v>25</v>
       </c>
       <c r="F314" t="s">
-        <v>3470</v>
+        <v>3472</v>
       </c>
       <c r="G314" t="s">
         <v>65</v>
@@ -31729,28 +31739,28 @@
         <v>47</v>
       </c>
       <c r="I314" t="s">
-        <v>3471</v>
+        <v>3473</v>
       </c>
       <c r="J314" t="s">
-        <v>3472</v>
+        <v>3474</v>
       </c>
       <c r="K314" t="s">
-        <v>3473</v>
+        <v>3475</v>
       </c>
       <c r="L314" t="s">
-        <v>3474</v>
+        <v>3476</v>
       </c>
       <c r="M314" t="s">
-        <v>3475</v>
+        <v>3477</v>
       </c>
       <c r="N314" t="s">
         <v>53</v>
       </c>
       <c r="O314" t="s">
-        <v>3476</v>
+        <v>3478</v>
       </c>
       <c r="P314" t="s">
-        <v>3477</v>
+        <v>3479</v>
       </c>
       <c r="Q314" t="s">
         <v>37</v>
@@ -31772,19 +31782,19 @@
         <v>20254188</v>
       </c>
       <c r="B315" t="s">
-        <v>3478</v>
+        <v>3480</v>
       </c>
       <c r="C315" t="s">
         <v>61</v>
       </c>
       <c r="D315" t="s">
-        <v>3479</v>
+        <v>3481</v>
       </c>
       <c r="E315" t="s">
         <v>25</v>
       </c>
       <c r="F315" t="s">
-        <v>3470</v>
+        <v>3472</v>
       </c>
       <c r="G315" t="s">
         <v>65</v>
@@ -31793,28 +31803,28 @@
         <v>81</v>
       </c>
       <c r="I315" t="s">
-        <v>3480</v>
+        <v>3482</v>
       </c>
       <c r="J315" t="s">
-        <v>3481</v>
+        <v>3483</v>
       </c>
       <c r="K315" t="s">
-        <v>3482</v>
+        <v>3484</v>
       </c>
       <c r="L315" t="s">
-        <v>3483</v>
+        <v>3485</v>
       </c>
       <c r="M315" t="s">
-        <v>3484</v>
+        <v>3486</v>
       </c>
       <c r="N315" t="s">
-        <v>3485</v>
+        <v>3487</v>
       </c>
       <c r="O315" t="s">
-        <v>3486</v>
+        <v>3488</v>
       </c>
       <c r="P315" t="s">
-        <v>3487</v>
+        <v>3489</v>
       </c>
       <c r="Q315" t="s">
         <v>37</v>
@@ -31836,7 +31846,7 @@
         <v>20254225</v>
       </c>
       <c r="B316" t="s">
-        <v>3488</v>
+        <v>3490</v>
       </c>
       <c r="C316" t="s">
         <v>23</v>
@@ -31848,7 +31858,7 @@
         <v>645</v>
       </c>
       <c r="F316" t="s">
-        <v>3470</v>
+        <v>3472</v>
       </c>
       <c r="G316" t="s">
         <v>27</v>
@@ -31857,28 +31867,28 @@
         <v>81</v>
       </c>
       <c r="I316" t="s">
-        <v>3489</v>
+        <v>3491</v>
       </c>
       <c r="J316" t="s">
-        <v>3490</v>
+        <v>3492</v>
       </c>
       <c r="K316" t="s">
-        <v>3491</v>
+        <v>3493</v>
       </c>
       <c r="L316" t="s">
-        <v>3492</v>
+        <v>3494</v>
       </c>
       <c r="M316" t="s">
-        <v>3493</v>
+        <v>3495</v>
       </c>
       <c r="N316" t="s">
         <v>34</v>
       </c>
       <c r="O316" t="s">
-        <v>3494</v>
+        <v>3496</v>
       </c>
       <c r="P316" t="s">
-        <v>3495</v>
+        <v>3497</v>
       </c>
       <c r="Q316" t="s">
         <v>73</v>
@@ -31886,13 +31896,13 @@
       <c r="R316"/>
       <c r="S316"/>
       <c r="T316" t="s">
-        <v>3496</v>
+        <v>3498</v>
       </c>
       <c r="U316" t="s">
-        <v>3497</v>
+        <v>3499</v>
       </c>
       <c r="V316" t="s">
-        <v>3498</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="317">
@@ -31900,19 +31910,19 @@
         <v>20254234</v>
       </c>
       <c r="B317" t="s">
-        <v>3499</v>
+        <v>3501</v>
       </c>
       <c r="C317" t="s">
         <v>61</v>
       </c>
       <c r="D317" t="s">
-        <v>3500</v>
+        <v>3502</v>
       </c>
       <c r="E317" t="s">
         <v>144</v>
       </c>
       <c r="F317" t="s">
-        <v>3470</v>
+        <v>3472</v>
       </c>
       <c r="G317" t="s">
         <v>27</v>
@@ -31921,28 +31931,28 @@
         <v>81</v>
       </c>
       <c r="I317" t="s">
-        <v>3501</v>
+        <v>3503</v>
       </c>
       <c r="J317" t="s">
-        <v>3502</v>
+        <v>3504</v>
       </c>
       <c r="K317" t="s">
-        <v>3503</v>
+        <v>3505</v>
       </c>
       <c r="L317" t="s">
-        <v>3504</v>
+        <v>3506</v>
       </c>
       <c r="M317" t="s">
-        <v>3505</v>
+        <v>3507</v>
       </c>
       <c r="N317" t="s">
         <v>53</v>
       </c>
       <c r="O317" t="s">
-        <v>3506</v>
+        <v>3508</v>
       </c>
       <c r="P317" t="s">
-        <v>3507</v>
+        <v>3509</v>
       </c>
       <c r="Q317" t="s">
         <v>89</v>
@@ -31950,13 +31960,13 @@
       <c r="R317"/>
       <c r="S317"/>
       <c r="T317" t="s">
-        <v>3508</v>
+        <v>3510</v>
       </c>
       <c r="U317" t="s">
-        <v>3509</v>
+        <v>3511</v>
       </c>
       <c r="V317" t="s">
-        <v>3510</v>
+        <v>3512</v>
       </c>
     </row>
     <row r="318">
@@ -31964,19 +31974,19 @@
         <v>20254071</v>
       </c>
       <c r="B318" t="s">
-        <v>3511</v>
+        <v>3513</v>
       </c>
       <c r="C318" t="s">
         <v>23</v>
       </c>
       <c r="D318" t="s">
-        <v>3512</v>
+        <v>3514</v>
       </c>
       <c r="E318" t="s">
         <v>25</v>
       </c>
       <c r="F318" t="s">
-        <v>3513</v>
+        <v>3515</v>
       </c>
       <c r="G318" t="s">
         <v>65</v>
@@ -31985,28 +31995,28 @@
         <v>81</v>
       </c>
       <c r="I318" t="s">
-        <v>3514</v>
+        <v>3516</v>
       </c>
       <c r="J318" t="s">
-        <v>3515</v>
+        <v>3517</v>
       </c>
       <c r="K318" t="s">
-        <v>3516</v>
+        <v>3518</v>
       </c>
       <c r="L318" t="s">
-        <v>3517</v>
+        <v>3519</v>
       </c>
       <c r="M318" t="s">
-        <v>3518</v>
+        <v>3520</v>
       </c>
       <c r="N318" t="s">
         <v>53</v>
       </c>
       <c r="O318" t="s">
-        <v>3519</v>
+        <v>3521</v>
       </c>
       <c r="P318" t="s">
-        <v>3520</v>
+        <v>3522</v>
       </c>
       <c r="Q318" t="s">
         <v>37</v>
@@ -32014,13 +32024,13 @@
       <c r="R318"/>
       <c r="S318"/>
       <c r="T318" t="s">
-        <v>3521</v>
+        <v>3523</v>
       </c>
       <c r="U318" t="s">
-        <v>3522</v>
+        <v>3524</v>
       </c>
       <c r="V318" t="s">
-        <v>3523</v>
+        <v>3525</v>
       </c>
     </row>
     <row r="319">
@@ -32028,7 +32038,7 @@
         <v>20254024</v>
       </c>
       <c r="B319" t="s">
-        <v>3524</v>
+        <v>3526</v>
       </c>
       <c r="C319" t="s">
         <v>23</v>
@@ -32040,7 +32050,7 @@
         <v>144</v>
       </c>
       <c r="F319" t="s">
-        <v>3525</v>
+        <v>3527</v>
       </c>
       <c r="G319" t="s">
         <v>27</v>
@@ -32049,28 +32059,28 @@
         <v>28</v>
       </c>
       <c r="I319" t="s">
-        <v>3526</v>
+        <v>3528</v>
       </c>
       <c r="J319" t="s">
-        <v>3527</v>
+        <v>3529</v>
       </c>
       <c r="K319" t="s">
-        <v>3528</v>
+        <v>3530</v>
       </c>
       <c r="L319" t="s">
-        <v>3529</v>
+        <v>3531</v>
       </c>
       <c r="M319" t="s">
-        <v>3530</v>
+        <v>3532</v>
       </c>
       <c r="N319" t="s">
         <v>34</v>
       </c>
       <c r="O319" t="s">
-        <v>3531</v>
+        <v>3533</v>
       </c>
       <c r="P319" t="s">
-        <v>3532</v>
+        <v>3534</v>
       </c>
       <c r="Q319" t="s">
         <v>73</v>
@@ -32092,7 +32102,7 @@
         <v>20257863</v>
       </c>
       <c r="B320" t="s">
-        <v>3533</v>
+        <v>3535</v>
       </c>
       <c r="C320" t="s">
         <v>43</v>
@@ -32104,7 +32114,7 @@
         <v>1836</v>
       </c>
       <c r="F320" t="s">
-        <v>3525</v>
+        <v>3527</v>
       </c>
       <c r="G320" t="s">
         <v>27</v>
@@ -32113,26 +32123,26 @@
         <v>47</v>
       </c>
       <c r="I320" t="s">
-        <v>3534</v>
+        <v>3536</v>
       </c>
       <c r="J320" t="s">
-        <v>3535</v>
+        <v>3537</v>
       </c>
       <c r="K320"/>
       <c r="L320" t="s">
-        <v>3536</v>
+        <v>3538</v>
       </c>
       <c r="M320" t="s">
-        <v>3537</v>
+        <v>3539</v>
       </c>
       <c r="N320" t="s">
         <v>53</v>
       </c>
       <c r="O320" t="s">
-        <v>3538</v>
+        <v>3540</v>
       </c>
       <c r="P320" t="s">
-        <v>3539</v>
+        <v>3541</v>
       </c>
       <c r="Q320" t="s">
         <v>37</v>
@@ -32154,7 +32164,7 @@
         <v>20257888</v>
       </c>
       <c r="B321" t="s">
-        <v>3540</v>
+        <v>3542</v>
       </c>
       <c r="C321" t="s">
         <v>43</v>
@@ -32166,7 +32176,7 @@
         <v>1483</v>
       </c>
       <c r="F321" t="s">
-        <v>3525</v>
+        <v>3527</v>
       </c>
       <c r="G321" t="s">
         <v>27</v>
@@ -32175,26 +32185,26 @@
         <v>28</v>
       </c>
       <c r="I321" t="s">
-        <v>3541</v>
+        <v>3543</v>
       </c>
       <c r="J321" t="s">
-        <v>3542</v>
+        <v>3544</v>
       </c>
       <c r="K321"/>
       <c r="L321" t="s">
-        <v>3543</v>
+        <v>3545</v>
       </c>
       <c r="M321" t="s">
-        <v>3544</v>
+        <v>3546</v>
       </c>
       <c r="N321" t="s">
         <v>53</v>
       </c>
       <c r="O321" t="s">
-        <v>3545</v>
+        <v>3547</v>
       </c>
       <c r="P321" t="s">
-        <v>3546</v>
+        <v>3548</v>
       </c>
       <c r="Q321" t="s">
         <v>89</v>
@@ -32216,7 +32226,7 @@
         <v>20257890</v>
       </c>
       <c r="B322" t="s">
-        <v>3547</v>
+        <v>3549</v>
       </c>
       <c r="C322" t="s">
         <v>43</v>
@@ -32228,7 +32238,7 @@
         <v>645</v>
       </c>
       <c r="F322" t="s">
-        <v>3525</v>
+        <v>3527</v>
       </c>
       <c r="G322" t="s">
         <v>27</v>
@@ -32237,26 +32247,26 @@
         <v>548</v>
       </c>
       <c r="I322" t="s">
-        <v>3548</v>
+        <v>3550</v>
       </c>
       <c r="J322" t="s">
-        <v>3549</v>
+        <v>3551</v>
       </c>
       <c r="K322"/>
       <c r="L322" t="s">
-        <v>3550</v>
+        <v>3552</v>
       </c>
       <c r="M322" t="s">
-        <v>3551</v>
+        <v>3553</v>
       </c>
       <c r="N322" t="s">
         <v>53</v>
       </c>
       <c r="O322" t="s">
-        <v>3552</v>
+        <v>3554</v>
       </c>
       <c r="P322" t="s">
-        <v>3553</v>
+        <v>3555</v>
       </c>
       <c r="Q322" t="s">
         <v>73</v>
@@ -32278,17 +32288,17 @@
         <v>20254003</v>
       </c>
       <c r="B323" t="s">
-        <v>3554</v>
+        <v>3556</v>
       </c>
       <c r="C323" t="s">
         <v>217</v>
       </c>
       <c r="D323" t="s">
-        <v>3555</v>
+        <v>3557</v>
       </c>
       <c r="E323"/>
       <c r="F323" t="s">
-        <v>3556</v>
+        <v>3558</v>
       </c>
       <c r="G323" t="s">
         <v>27</v>
@@ -32297,28 +32307,28 @@
         <v>47</v>
       </c>
       <c r="I323" t="s">
-        <v>3557</v>
+        <v>3559</v>
       </c>
       <c r="J323" t="s">
-        <v>3558</v>
+        <v>3560</v>
       </c>
       <c r="K323" t="s">
-        <v>3559</v>
+        <v>3561</v>
       </c>
       <c r="L323" t="s">
-        <v>3560</v>
+        <v>3562</v>
       </c>
       <c r="M323" t="s">
-        <v>3561</v>
+        <v>3563</v>
       </c>
       <c r="N323" t="s">
         <v>34</v>
       </c>
       <c r="O323" t="s">
-        <v>3562</v>
+        <v>3564</v>
       </c>
       <c r="P323" t="s">
-        <v>3563</v>
+        <v>3565</v>
       </c>
       <c r="Q323" t="s">
         <v>37</v>
@@ -32326,13 +32336,13 @@
       <c r="R323"/>
       <c r="S323"/>
       <c r="T323" t="s">
-        <v>3564</v>
+        <v>3566</v>
       </c>
       <c r="U323" t="s">
-        <v>3565</v>
+        <v>3567</v>
       </c>
       <c r="V323" t="s">
-        <v>3566</v>
+        <v>3568</v>
       </c>
     </row>
     <row r="324">
@@ -32340,7 +32350,7 @@
         <v>20253984</v>
       </c>
       <c r="B324" t="s">
-        <v>3567</v>
+        <v>3569</v>
       </c>
       <c r="C324" t="s">
         <v>61</v>
@@ -32350,7 +32360,7 @@
       </c>
       <c r="E324"/>
       <c r="F324" t="s">
-        <v>3568</v>
+        <v>3570</v>
       </c>
       <c r="G324" t="s">
         <v>27</v>
@@ -32359,34 +32369,36 @@
         <v>47</v>
       </c>
       <c r="I324" t="s">
-        <v>3471</v>
+        <v>3473</v>
       </c>
       <c r="J324" t="s">
-        <v>3472</v>
+        <v>3474</v>
       </c>
       <c r="K324" t="s">
-        <v>3473</v>
+        <v>3475</v>
       </c>
       <c r="L324" t="s">
-        <v>3569</v>
+        <v>3571</v>
       </c>
       <c r="M324" t="s">
-        <v>3570</v>
+        <v>3572</v>
       </c>
       <c r="N324" t="s">
-        <v>1341</v>
+        <v>3375</v>
       </c>
       <c r="O324" t="s">
-        <v>3571</v>
+        <v>3573</v>
       </c>
       <c r="P324" t="s">
-        <v>3572</v>
+        <v>3574</v>
       </c>
       <c r="Q324" t="s">
         <v>37</v>
       </c>
       <c r="R324"/>
-      <c r="S324"/>
+      <c r="S324" t="s">
+        <v>3378</v>
+      </c>
       <c r="T324" t="s">
         <v>117</v>
       </c>
@@ -32402,7 +32414,7 @@
         <v>20257663</v>
       </c>
       <c r="B325" t="s">
-        <v>3573</v>
+        <v>3575</v>
       </c>
       <c r="C325" t="s">
         <v>43</v>
@@ -32414,7 +32426,7 @@
         <v>45</v>
       </c>
       <c r="F325" t="s">
-        <v>3568</v>
+        <v>3570</v>
       </c>
       <c r="G325" t="s">
         <v>27</v>
@@ -32423,26 +32435,26 @@
         <v>28</v>
       </c>
       <c r="I325" t="s">
-        <v>3574</v>
+        <v>3576</v>
       </c>
       <c r="J325" t="s">
-        <v>3575</v>
+        <v>3577</v>
       </c>
       <c r="K325"/>
       <c r="L325" t="s">
-        <v>3576</v>
+        <v>3578</v>
       </c>
       <c r="M325" t="s">
-        <v>3577</v>
+        <v>3579</v>
       </c>
       <c r="N325" t="s">
         <v>53</v>
       </c>
       <c r="O325" t="s">
-        <v>3578</v>
+        <v>3580</v>
       </c>
       <c r="P325" t="s">
-        <v>3579</v>
+        <v>3581</v>
       </c>
       <c r="Q325" t="s">
         <v>37</v>
@@ -32450,13 +32462,13 @@
       <c r="R325"/>
       <c r="S325"/>
       <c r="T325" t="s">
-        <v>3580</v>
+        <v>3582</v>
       </c>
       <c r="U325" t="s">
-        <v>3581</v>
+        <v>3583</v>
       </c>
       <c r="V325" t="s">
-        <v>3582</v>
+        <v>3584</v>
       </c>
     </row>
     <row r="326">
@@ -32464,19 +32476,19 @@
         <v>20257698</v>
       </c>
       <c r="B326" t="s">
-        <v>3583</v>
+        <v>3585</v>
       </c>
       <c r="C326" t="s">
         <v>43</v>
       </c>
       <c r="D326" t="s">
-        <v>3584</v>
+        <v>3586</v>
       </c>
       <c r="E326" t="s">
         <v>144</v>
       </c>
       <c r="F326" t="s">
-        <v>3568</v>
+        <v>3570</v>
       </c>
       <c r="G326" t="s">
         <v>27</v>
@@ -32485,26 +32497,26 @@
         <v>28</v>
       </c>
       <c r="I326" t="s">
-        <v>3585</v>
+        <v>3587</v>
       </c>
       <c r="J326" t="s">
-        <v>3586</v>
+        <v>3588</v>
       </c>
       <c r="K326"/>
       <c r="L326" t="s">
-        <v>3587</v>
+        <v>3589</v>
       </c>
       <c r="M326" t="s">
-        <v>3588</v>
+        <v>3590</v>
       </c>
       <c r="N326" t="s">
         <v>53</v>
       </c>
       <c r="O326" t="s">
-        <v>3589</v>
+        <v>3591</v>
       </c>
       <c r="P326" t="s">
-        <v>3590</v>
+        <v>3592</v>
       </c>
       <c r="Q326" t="s">
         <v>37</v>
@@ -32526,19 +32538,19 @@
         <v>20253971</v>
       </c>
       <c r="B327" t="s">
-        <v>3591</v>
+        <v>3593</v>
       </c>
       <c r="C327" t="s">
         <v>23</v>
       </c>
       <c r="D327" t="s">
-        <v>3592</v>
+        <v>3594</v>
       </c>
       <c r="E327" t="s">
         <v>25</v>
       </c>
       <c r="F327" t="s">
-        <v>3593</v>
+        <v>3595</v>
       </c>
       <c r="G327" t="s">
         <v>65</v>
@@ -32547,28 +32559,28 @@
         <v>548</v>
       </c>
       <c r="I327" t="s">
-        <v>3594</v>
+        <v>3596</v>
       </c>
       <c r="J327" t="s">
-        <v>3595</v>
+        <v>3597</v>
       </c>
       <c r="K327" t="s">
-        <v>3596</v>
+        <v>3598</v>
       </c>
       <c r="L327" t="s">
-        <v>3597</v>
+        <v>3599</v>
       </c>
       <c r="M327" t="s">
-        <v>3598</v>
+        <v>3600</v>
       </c>
       <c r="N327" t="s">
         <v>53</v>
       </c>
       <c r="O327" t="s">
-        <v>3599</v>
+        <v>3601</v>
       </c>
       <c r="P327" t="s">
-        <v>3600</v>
+        <v>3602</v>
       </c>
       <c r="Q327" t="s">
         <v>73</v>
@@ -32576,13 +32588,13 @@
       <c r="R327"/>
       <c r="S327"/>
       <c r="T327" t="s">
-        <v>3465</v>
+        <v>3467</v>
       </c>
       <c r="U327" t="s">
-        <v>3466</v>
+        <v>3468</v>
       </c>
       <c r="V327" t="s">
-        <v>3467</v>
+        <v>3469</v>
       </c>
     </row>
     <row r="328">
@@ -32590,7 +32602,7 @@
         <v>20257601</v>
       </c>
       <c r="B328" t="s">
-        <v>3601</v>
+        <v>3603</v>
       </c>
       <c r="C328" t="s">
         <v>43</v>
@@ -32602,7 +32614,7 @@
         <v>1483</v>
       </c>
       <c r="F328" t="s">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="G328" t="s">
         <v>27</v>
@@ -32611,26 +32623,26 @@
         <v>81</v>
       </c>
       <c r="I328" t="s">
-        <v>3603</v>
+        <v>3605</v>
       </c>
       <c r="J328" t="s">
-        <v>3604</v>
+        <v>3606</v>
       </c>
       <c r="K328"/>
       <c r="L328" t="s">
-        <v>3605</v>
+        <v>3607</v>
       </c>
       <c r="M328" t="s">
-        <v>3606</v>
+        <v>3608</v>
       </c>
       <c r="N328" t="s">
         <v>53</v>
       </c>
       <c r="O328" t="s">
-        <v>3607</v>
+        <v>3609</v>
       </c>
       <c r="P328" t="s">
-        <v>3608</v>
+        <v>3610</v>
       </c>
       <c r="Q328" t="s">
         <v>73</v>
@@ -32652,17 +32664,17 @@
         <v>20253941</v>
       </c>
       <c r="B329" t="s">
-        <v>3609</v>
+        <v>3611</v>
       </c>
       <c r="C329" t="s">
         <v>61</v>
       </c>
       <c r="D329" t="s">
-        <v>3610</v>
+        <v>3612</v>
       </c>
       <c r="E329"/>
       <c r="F329" t="s">
-        <v>3611</v>
+        <v>3613</v>
       </c>
       <c r="G329" t="s">
         <v>27</v>
@@ -32671,28 +32683,28 @@
         <v>1543</v>
       </c>
       <c r="I329" t="s">
-        <v>3612</v>
+        <v>3614</v>
       </c>
       <c r="J329" t="s">
-        <v>3613</v>
+        <v>3615</v>
       </c>
       <c r="K329" t="s">
-        <v>3614</v>
+        <v>3616</v>
       </c>
       <c r="L329" t="s">
-        <v>3615</v>
+        <v>3617</v>
       </c>
       <c r="M329" t="s">
-        <v>3616</v>
+        <v>3618</v>
       </c>
       <c r="N329" t="s">
         <v>1975</v>
       </c>
       <c r="O329" t="s">
-        <v>3617</v>
+        <v>3619</v>
       </c>
       <c r="P329" t="s">
-        <v>3618</v>
+        <v>3620</v>
       </c>
       <c r="Q329" t="s">
         <v>37</v>

</xml_diff>

<commit_message>
Update parliament data - 2026-03-03
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_CDF_EFK.xlsx
+++ b/Objets_parlementaires_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3633" uniqueCount="3633">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3634" uniqueCount="3634">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -10185,9 +10185,6 @@
     <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254620</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-03-03</t>
-  </si>
-  <si>
     <t xml:space="preserve">Staatspolitik|Medien und Kommunikation|Menschenrechte</t>
   </si>
   <si>
@@ -10224,6 +10221,9 @@
     <t xml:space="preserve">25.4562</t>
   </si>
   <si>
+    <t xml:space="preserve">Le Centre</t>
+  </si>
+  <si>
     <t xml:space="preserve">Unbürokratische Entlastung bei invasiven Schadorganismen</t>
   </si>
   <si>
@@ -10294,6 +10294,9 @@
   </si>
   <si>
     <t xml:space="preserve">25.4614</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PS</t>
   </si>
   <si>
     <t xml:space="preserve">Medikamente als Kostentreiber in der obligatorischen Krankenpflegeversicherung?</t>
@@ -31224,17 +31227,15 @@
         <v>35</v>
       </c>
       <c r="R305"/>
-      <c r="S305" t="s">
+      <c r="S305"/>
+      <c r="T305" t="s">
         <v>3390</v>
       </c>
-      <c r="T305" t="s">
+      <c r="U305" t="s">
         <v>3391</v>
       </c>
-      <c r="U305" t="s">
+      <c r="V305" t="s">
         <v>3392</v>
-      </c>
-      <c r="V305" t="s">
-        <v>3393</v>
       </c>
     </row>
     <row r="306">
@@ -31242,7 +31243,7 @@
         <v>20254696</v>
       </c>
       <c r="B306" t="s">
-        <v>3394</v>
+        <v>3393</v>
       </c>
       <c r="C306" t="s">
         <v>40</v>
@@ -31263,28 +31264,28 @@
         <v>563</v>
       </c>
       <c r="I306" t="s">
+        <v>3394</v>
+      </c>
+      <c r="J306" t="s">
         <v>3395</v>
       </c>
-      <c r="J306" t="s">
+      <c r="K306" t="s">
         <v>3396</v>
       </c>
-      <c r="K306" t="s">
+      <c r="L306" t="s">
         <v>3397</v>
       </c>
-      <c r="L306" t="s">
+      <c r="M306" t="s">
         <v>3398</v>
-      </c>
-      <c r="M306" t="s">
-        <v>3399</v>
       </c>
       <c r="N306" t="s">
         <v>50</v>
       </c>
       <c r="O306" t="s">
+        <v>3399</v>
+      </c>
+      <c r="P306" t="s">
         <v>3400</v>
-      </c>
-      <c r="P306" t="s">
-        <v>3401</v>
       </c>
       <c r="Q306" t="s">
         <v>89</v>
@@ -31306,7 +31307,7 @@
         <v>20254562</v>
       </c>
       <c r="B307" t="s">
-        <v>3402</v>
+        <v>3401</v>
       </c>
       <c r="C307" t="s">
         <v>232</v>
@@ -31315,7 +31316,7 @@
         <v>1568</v>
       </c>
       <c r="E307" t="s">
-        <v>79</v>
+        <v>3402</v>
       </c>
       <c r="F307" t="s">
         <v>43</v>
@@ -31379,7 +31380,7 @@
         <v>3414</v>
       </c>
       <c r="E308" t="s">
-        <v>79</v>
+        <v>3402</v>
       </c>
       <c r="F308" t="s">
         <v>43</v>
@@ -31443,7 +31444,7 @@
         <v>2013</v>
       </c>
       <c r="E309" t="s">
-        <v>159</v>
+        <v>3427</v>
       </c>
       <c r="F309" t="s">
         <v>43</v>
@@ -31455,28 +31456,28 @@
         <v>97</v>
       </c>
       <c r="I309" t="s">
-        <v>3427</v>
+        <v>3428</v>
       </c>
       <c r="J309" t="s">
-        <v>3428</v>
+        <v>3429</v>
       </c>
       <c r="K309" t="s">
-        <v>3429</v>
+        <v>3430</v>
       </c>
       <c r="L309" t="s">
-        <v>3430</v>
+        <v>3431</v>
       </c>
       <c r="M309" t="s">
-        <v>3431</v>
+        <v>3432</v>
       </c>
       <c r="N309" t="s">
         <v>50</v>
       </c>
       <c r="O309" t="s">
-        <v>3432</v>
+        <v>3433</v>
       </c>
       <c r="P309" t="s">
-        <v>3433</v>
+        <v>3434</v>
       </c>
       <c r="Q309" t="s">
         <v>53</v>
@@ -31498,19 +31499,19 @@
         <v>20258194</v>
       </c>
       <c r="B310" t="s">
-        <v>3434</v>
+        <v>3435</v>
       </c>
       <c r="C310" t="s">
         <v>59</v>
       </c>
       <c r="D310" t="s">
-        <v>3435</v>
+        <v>3436</v>
       </c>
       <c r="E310" t="s">
         <v>61</v>
       </c>
       <c r="F310" t="s">
-        <v>3436</v>
+        <v>3437</v>
       </c>
       <c r="G310" t="s">
         <v>27</v>
@@ -31519,26 +31520,26 @@
         <v>97</v>
       </c>
       <c r="I310" t="s">
-        <v>3437</v>
+        <v>3438</v>
       </c>
       <c r="J310" t="s">
-        <v>3438</v>
+        <v>3439</v>
       </c>
       <c r="K310"/>
       <c r="L310" t="s">
-        <v>3439</v>
+        <v>3440</v>
       </c>
       <c r="M310" t="s">
-        <v>3440</v>
+        <v>3441</v>
       </c>
       <c r="N310" t="s">
         <v>69</v>
       </c>
       <c r="O310" t="s">
-        <v>3441</v>
+        <v>3442</v>
       </c>
       <c r="P310" t="s">
-        <v>3442</v>
+        <v>3443</v>
       </c>
       <c r="Q310" t="s">
         <v>53</v>
@@ -31560,7 +31561,7 @@
         <v>20258273</v>
       </c>
       <c r="B311" t="s">
-        <v>3443</v>
+        <v>3444</v>
       </c>
       <c r="C311" t="s">
         <v>59</v>
@@ -31572,7 +31573,7 @@
         <v>659</v>
       </c>
       <c r="F311" t="s">
-        <v>3436</v>
+        <v>3437</v>
       </c>
       <c r="G311" t="s">
         <v>27</v>
@@ -31581,26 +31582,26 @@
         <v>97</v>
       </c>
       <c r="I311" t="s">
-        <v>3444</v>
+        <v>3445</v>
       </c>
       <c r="J311" t="s">
-        <v>3445</v>
+        <v>3446</v>
       </c>
       <c r="K311"/>
       <c r="L311" t="s">
-        <v>3446</v>
+        <v>3447</v>
       </c>
       <c r="M311" t="s">
-        <v>3447</v>
+        <v>3448</v>
       </c>
       <c r="N311" t="s">
         <v>69</v>
       </c>
       <c r="O311" t="s">
-        <v>3448</v>
+        <v>3449</v>
       </c>
       <c r="P311" t="s">
-        <v>3449</v>
+        <v>3450</v>
       </c>
       <c r="Q311" t="s">
         <v>89</v>
@@ -31608,13 +31609,13 @@
       <c r="R311"/>
       <c r="S311"/>
       <c r="T311" t="s">
-        <v>3450</v>
+        <v>3451</v>
       </c>
       <c r="U311" t="s">
-        <v>3451</v>
+        <v>3452</v>
       </c>
       <c r="V311" t="s">
-        <v>3452</v>
+        <v>3453</v>
       </c>
     </row>
     <row r="312">
@@ -31622,7 +31623,7 @@
         <v>20254463</v>
       </c>
       <c r="B312" t="s">
-        <v>3453</v>
+        <v>3454</v>
       </c>
       <c r="C312" t="s">
         <v>77</v>
@@ -31634,7 +31635,7 @@
         <v>659</v>
       </c>
       <c r="F312" t="s">
-        <v>3454</v>
+        <v>3455</v>
       </c>
       <c r="G312" t="s">
         <v>27</v>
@@ -31643,28 +31644,28 @@
         <v>63</v>
       </c>
       <c r="I312" t="s">
-        <v>3455</v>
+        <v>3456</v>
       </c>
       <c r="J312" t="s">
-        <v>3456</v>
+        <v>3457</v>
       </c>
       <c r="K312" t="s">
-        <v>3457</v>
+        <v>3458</v>
       </c>
       <c r="L312" t="s">
-        <v>3458</v>
+        <v>3459</v>
       </c>
       <c r="M312" t="s">
-        <v>3459</v>
+        <v>3460</v>
       </c>
       <c r="N312" t="s">
         <v>69</v>
       </c>
       <c r="O312" t="s">
-        <v>3460</v>
+        <v>3461</v>
       </c>
       <c r="P312" t="s">
-        <v>3461</v>
+        <v>3462</v>
       </c>
       <c r="Q312" t="s">
         <v>35</v>
@@ -31686,19 +31687,19 @@
         <v>20254281</v>
       </c>
       <c r="B313" t="s">
-        <v>3462</v>
+        <v>3463</v>
       </c>
       <c r="C313" t="s">
         <v>232</v>
       </c>
       <c r="D313" t="s">
-        <v>3463</v>
+        <v>3464</v>
       </c>
       <c r="E313" t="s">
-        <v>159</v>
+        <v>3427</v>
       </c>
       <c r="F313" t="s">
-        <v>3464</v>
+        <v>3465</v>
       </c>
       <c r="G313" t="s">
         <v>27</v>
@@ -31707,28 +31708,28 @@
         <v>563</v>
       </c>
       <c r="I313" t="s">
-        <v>3465</v>
+        <v>3466</v>
       </c>
       <c r="J313" t="s">
-        <v>3466</v>
+        <v>3467</v>
       </c>
       <c r="K313" t="s">
-        <v>3467</v>
+        <v>3468</v>
       </c>
       <c r="L313" t="s">
-        <v>3468</v>
+        <v>3469</v>
       </c>
       <c r="M313" t="s">
-        <v>3469</v>
+        <v>3470</v>
       </c>
       <c r="N313" t="s">
         <v>50</v>
       </c>
       <c r="O313" t="s">
-        <v>3470</v>
+        <v>3471</v>
       </c>
       <c r="P313" t="s">
-        <v>3471</v>
+        <v>3472</v>
       </c>
       <c r="Q313" t="s">
         <v>89</v>
@@ -31750,7 +31751,7 @@
         <v>20254317</v>
       </c>
       <c r="B314" t="s">
-        <v>3472</v>
+        <v>3473</v>
       </c>
       <c r="C314" t="s">
         <v>77</v>
@@ -31762,7 +31763,7 @@
         <v>42</v>
       </c>
       <c r="F314" t="s">
-        <v>3464</v>
+        <v>3465</v>
       </c>
       <c r="G314" t="s">
         <v>27</v>
@@ -31771,28 +31772,28 @@
         <v>563</v>
       </c>
       <c r="I314" t="s">
-        <v>3473</v>
+        <v>3474</v>
       </c>
       <c r="J314" t="s">
-        <v>3474</v>
+        <v>3475</v>
       </c>
       <c r="K314" t="s">
-        <v>3475</v>
+        <v>3476</v>
       </c>
       <c r="L314" t="s">
-        <v>3476</v>
+        <v>3477</v>
       </c>
       <c r="M314" t="s">
-        <v>3477</v>
+        <v>3478</v>
       </c>
       <c r="N314" t="s">
         <v>50</v>
       </c>
       <c r="O314" t="s">
-        <v>3478</v>
+        <v>3479</v>
       </c>
       <c r="P314" t="s">
-        <v>3479</v>
+        <v>3480</v>
       </c>
       <c r="Q314" t="s">
         <v>89</v>
@@ -31800,13 +31801,13 @@
       <c r="R314"/>
       <c r="S314"/>
       <c r="T314" t="s">
-        <v>3480</v>
+        <v>3481</v>
       </c>
       <c r="U314" t="s">
-        <v>3481</v>
+        <v>3482</v>
       </c>
       <c r="V314" t="s">
-        <v>3482</v>
+        <v>3483</v>
       </c>
     </row>
     <row r="315">
@@ -31814,19 +31815,19 @@
         <v>20254145</v>
       </c>
       <c r="B315" t="s">
-        <v>3483</v>
+        <v>3484</v>
       </c>
       <c r="C315" t="s">
         <v>77</v>
       </c>
       <c r="D315" t="s">
-        <v>3484</v>
+        <v>3485</v>
       </c>
       <c r="E315" t="s">
         <v>42</v>
       </c>
       <c r="F315" t="s">
-        <v>3485</v>
+        <v>3486</v>
       </c>
       <c r="G315" t="s">
         <v>81</v>
@@ -31835,28 +31836,28 @@
         <v>63</v>
       </c>
       <c r="I315" t="s">
-        <v>3486</v>
+        <v>3487</v>
       </c>
       <c r="J315" t="s">
-        <v>3487</v>
+        <v>3488</v>
       </c>
       <c r="K315" t="s">
-        <v>3488</v>
+        <v>3489</v>
       </c>
       <c r="L315" t="s">
-        <v>3489</v>
+        <v>3490</v>
       </c>
       <c r="M315" t="s">
-        <v>3490</v>
+        <v>3491</v>
       </c>
       <c r="N315" t="s">
         <v>69</v>
       </c>
       <c r="O315" t="s">
-        <v>3491</v>
+        <v>3492</v>
       </c>
       <c r="P315" t="s">
-        <v>3492</v>
+        <v>3493</v>
       </c>
       <c r="Q315" t="s">
         <v>53</v>
@@ -31878,19 +31879,19 @@
         <v>20254188</v>
       </c>
       <c r="B316" t="s">
-        <v>3493</v>
+        <v>3494</v>
       </c>
       <c r="C316" t="s">
         <v>77</v>
       </c>
       <c r="D316" t="s">
-        <v>3494</v>
+        <v>3495</v>
       </c>
       <c r="E316" t="s">
         <v>42</v>
       </c>
       <c r="F316" t="s">
-        <v>3485</v>
+        <v>3486</v>
       </c>
       <c r="G316" t="s">
         <v>81</v>
@@ -31899,28 +31900,28 @@
         <v>97</v>
       </c>
       <c r="I316" t="s">
-        <v>3495</v>
+        <v>3496</v>
       </c>
       <c r="J316" t="s">
-        <v>3496</v>
+        <v>3497</v>
       </c>
       <c r="K316" t="s">
-        <v>3497</v>
+        <v>3498</v>
       </c>
       <c r="L316" t="s">
-        <v>3498</v>
+        <v>3499</v>
       </c>
       <c r="M316" t="s">
-        <v>3499</v>
+        <v>3500</v>
       </c>
       <c r="N316" t="s">
         <v>3387</v>
       </c>
       <c r="O316" t="s">
-        <v>3500</v>
+        <v>3501</v>
       </c>
       <c r="P316" t="s">
-        <v>3501</v>
+        <v>3502</v>
       </c>
       <c r="Q316" t="s">
         <v>53</v>
@@ -31942,7 +31943,7 @@
         <v>20254225</v>
       </c>
       <c r="B317" t="s">
-        <v>3502</v>
+        <v>3503</v>
       </c>
       <c r="C317" t="s">
         <v>40</v>
@@ -31954,7 +31955,7 @@
         <v>659</v>
       </c>
       <c r="F317" t="s">
-        <v>3485</v>
+        <v>3486</v>
       </c>
       <c r="G317" t="s">
         <v>27</v>
@@ -31963,28 +31964,28 @@
         <v>97</v>
       </c>
       <c r="I317" t="s">
-        <v>3503</v>
+        <v>3504</v>
       </c>
       <c r="J317" t="s">
-        <v>3504</v>
+        <v>3505</v>
       </c>
       <c r="K317" t="s">
-        <v>3505</v>
+        <v>3506</v>
       </c>
       <c r="L317" t="s">
-        <v>3506</v>
+        <v>3507</v>
       </c>
       <c r="M317" t="s">
-        <v>3507</v>
+        <v>3508</v>
       </c>
       <c r="N317" t="s">
         <v>50</v>
       </c>
       <c r="O317" t="s">
-        <v>3508</v>
+        <v>3509</v>
       </c>
       <c r="P317" t="s">
-        <v>3509</v>
+        <v>3510</v>
       </c>
       <c r="Q317" t="s">
         <v>89</v>
@@ -31992,13 +31993,13 @@
       <c r="R317"/>
       <c r="S317"/>
       <c r="T317" t="s">
-        <v>3510</v>
+        <v>3511</v>
       </c>
       <c r="U317" t="s">
-        <v>3511</v>
+        <v>3512</v>
       </c>
       <c r="V317" t="s">
-        <v>3512</v>
+        <v>3513</v>
       </c>
     </row>
     <row r="318">
@@ -32006,19 +32007,19 @@
         <v>20254234</v>
       </c>
       <c r="B318" t="s">
-        <v>3513</v>
+        <v>3514</v>
       </c>
       <c r="C318" t="s">
         <v>77</v>
       </c>
       <c r="D318" t="s">
-        <v>3514</v>
+        <v>3515</v>
       </c>
       <c r="E318" t="s">
-        <v>159</v>
+        <v>3427</v>
       </c>
       <c r="F318" t="s">
-        <v>3485</v>
+        <v>3486</v>
       </c>
       <c r="G318" t="s">
         <v>27</v>
@@ -32027,28 +32028,28 @@
         <v>97</v>
       </c>
       <c r="I318" t="s">
-        <v>3515</v>
+        <v>3516</v>
       </c>
       <c r="J318" t="s">
-        <v>3516</v>
+        <v>3517</v>
       </c>
       <c r="K318" t="s">
-        <v>3517</v>
+        <v>3518</v>
       </c>
       <c r="L318" t="s">
-        <v>3518</v>
+        <v>3519</v>
       </c>
       <c r="M318" t="s">
-        <v>3519</v>
+        <v>3520</v>
       </c>
       <c r="N318" t="s">
         <v>69</v>
       </c>
       <c r="O318" t="s">
-        <v>3520</v>
+        <v>3521</v>
       </c>
       <c r="P318" t="s">
-        <v>3521</v>
+        <v>3522</v>
       </c>
       <c r="Q318" t="s">
         <v>35</v>
@@ -32056,13 +32057,13 @@
       <c r="R318"/>
       <c r="S318"/>
       <c r="T318" t="s">
-        <v>3522</v>
+        <v>3523</v>
       </c>
       <c r="U318" t="s">
-        <v>3523</v>
+        <v>3524</v>
       </c>
       <c r="V318" t="s">
-        <v>3524</v>
+        <v>3525</v>
       </c>
     </row>
     <row r="319">
@@ -32070,19 +32071,19 @@
         <v>20254071</v>
       </c>
       <c r="B319" t="s">
-        <v>3525</v>
+        <v>3526</v>
       </c>
       <c r="C319" t="s">
         <v>40</v>
       </c>
       <c r="D319" t="s">
-        <v>3526</v>
+        <v>3527</v>
       </c>
       <c r="E319" t="s">
         <v>42</v>
       </c>
       <c r="F319" t="s">
-        <v>3527</v>
+        <v>3528</v>
       </c>
       <c r="G319" t="s">
         <v>81</v>
@@ -32091,28 +32092,28 @@
         <v>97</v>
       </c>
       <c r="I319" t="s">
-        <v>3528</v>
+        <v>3529</v>
       </c>
       <c r="J319" t="s">
-        <v>3529</v>
+        <v>3530</v>
       </c>
       <c r="K319" t="s">
-        <v>3530</v>
+        <v>3531</v>
       </c>
       <c r="L319" t="s">
-        <v>3531</v>
+        <v>3532</v>
       </c>
       <c r="M319" t="s">
-        <v>3532</v>
+        <v>3533</v>
       </c>
       <c r="N319" t="s">
         <v>69</v>
       </c>
       <c r="O319" t="s">
-        <v>3533</v>
+        <v>3534</v>
       </c>
       <c r="P319" t="s">
-        <v>3534</v>
+        <v>3535</v>
       </c>
       <c r="Q319" t="s">
         <v>53</v>
@@ -32120,13 +32121,13 @@
       <c r="R319"/>
       <c r="S319"/>
       <c r="T319" t="s">
-        <v>3535</v>
+        <v>3536</v>
       </c>
       <c r="U319" t="s">
-        <v>3536</v>
+        <v>3537</v>
       </c>
       <c r="V319" t="s">
-        <v>3537</v>
+        <v>3538</v>
       </c>
     </row>
     <row r="320">
@@ -32134,7 +32135,7 @@
         <v>20254024</v>
       </c>
       <c r="B320" t="s">
-        <v>3538</v>
+        <v>3539</v>
       </c>
       <c r="C320" t="s">
         <v>40</v>
@@ -32143,10 +32144,10 @@
         <v>1639</v>
       </c>
       <c r="E320" t="s">
-        <v>159</v>
+        <v>3427</v>
       </c>
       <c r="F320" t="s">
-        <v>3539</v>
+        <v>3540</v>
       </c>
       <c r="G320" t="s">
         <v>27</v>
@@ -32155,28 +32156,28 @@
         <v>44</v>
       </c>
       <c r="I320" t="s">
-        <v>3540</v>
+        <v>3541</v>
       </c>
       <c r="J320" t="s">
-        <v>3541</v>
+        <v>3542</v>
       </c>
       <c r="K320" t="s">
-        <v>3542</v>
+        <v>3543</v>
       </c>
       <c r="L320" t="s">
-        <v>3543</v>
+        <v>3544</v>
       </c>
       <c r="M320" t="s">
-        <v>3544</v>
+        <v>3545</v>
       </c>
       <c r="N320" t="s">
         <v>50</v>
       </c>
       <c r="O320" t="s">
-        <v>3545</v>
+        <v>3546</v>
       </c>
       <c r="P320" t="s">
-        <v>3546</v>
+        <v>3547</v>
       </c>
       <c r="Q320" t="s">
         <v>89</v>
@@ -32198,7 +32199,7 @@
         <v>20257863</v>
       </c>
       <c r="B321" t="s">
-        <v>3547</v>
+        <v>3548</v>
       </c>
       <c r="C321" t="s">
         <v>59</v>
@@ -32210,7 +32211,7 @@
         <v>1848</v>
       </c>
       <c r="F321" t="s">
-        <v>3539</v>
+        <v>3540</v>
       </c>
       <c r="G321" t="s">
         <v>27</v>
@@ -32219,26 +32220,26 @@
         <v>63</v>
       </c>
       <c r="I321" t="s">
-        <v>3548</v>
+        <v>3549</v>
       </c>
       <c r="J321" t="s">
-        <v>3549</v>
+        <v>3550</v>
       </c>
       <c r="K321"/>
       <c r="L321" t="s">
-        <v>3550</v>
+        <v>3551</v>
       </c>
       <c r="M321" t="s">
-        <v>3551</v>
+        <v>3552</v>
       </c>
       <c r="N321" t="s">
         <v>69</v>
       </c>
       <c r="O321" t="s">
-        <v>3552</v>
+        <v>3553</v>
       </c>
       <c r="P321" t="s">
-        <v>3553</v>
+        <v>3554</v>
       </c>
       <c r="Q321" t="s">
         <v>53</v>
@@ -32260,7 +32261,7 @@
         <v>20257888</v>
       </c>
       <c r="B322" t="s">
-        <v>3554</v>
+        <v>3555</v>
       </c>
       <c r="C322" t="s">
         <v>59</v>
@@ -32269,10 +32270,10 @@
         <v>1495</v>
       </c>
       <c r="E322" t="s">
-        <v>1496</v>
+        <v>659</v>
       </c>
       <c r="F322" t="s">
-        <v>3539</v>
+        <v>3540</v>
       </c>
       <c r="G322" t="s">
         <v>27</v>
@@ -32281,26 +32282,26 @@
         <v>44</v>
       </c>
       <c r="I322" t="s">
-        <v>3555</v>
+        <v>3556</v>
       </c>
       <c r="J322" t="s">
-        <v>3556</v>
+        <v>3557</v>
       </c>
       <c r="K322"/>
       <c r="L322" t="s">
-        <v>3557</v>
+        <v>3558</v>
       </c>
       <c r="M322" t="s">
-        <v>3558</v>
+        <v>3559</v>
       </c>
       <c r="N322" t="s">
         <v>69</v>
       </c>
       <c r="O322" t="s">
-        <v>3559</v>
+        <v>3560</v>
       </c>
       <c r="P322" t="s">
-        <v>3560</v>
+        <v>3561</v>
       </c>
       <c r="Q322" t="s">
         <v>35</v>
@@ -32322,7 +32323,7 @@
         <v>20257890</v>
       </c>
       <c r="B323" t="s">
-        <v>3561</v>
+        <v>3562</v>
       </c>
       <c r="C323" t="s">
         <v>59</v>
@@ -32334,7 +32335,7 @@
         <v>659</v>
       </c>
       <c r="F323" t="s">
-        <v>3539</v>
+        <v>3540</v>
       </c>
       <c r="G323" t="s">
         <v>27</v>
@@ -32343,26 +32344,26 @@
         <v>563</v>
       </c>
       <c r="I323" t="s">
-        <v>3562</v>
+        <v>3563</v>
       </c>
       <c r="J323" t="s">
-        <v>3563</v>
+        <v>3564</v>
       </c>
       <c r="K323"/>
       <c r="L323" t="s">
-        <v>3564</v>
+        <v>3565</v>
       </c>
       <c r="M323" t="s">
-        <v>3565</v>
+        <v>3566</v>
       </c>
       <c r="N323" t="s">
         <v>69</v>
       </c>
       <c r="O323" t="s">
-        <v>3566</v>
+        <v>3567</v>
       </c>
       <c r="P323" t="s">
-        <v>3567</v>
+        <v>3568</v>
       </c>
       <c r="Q323" t="s">
         <v>89</v>
@@ -32384,17 +32385,17 @@
         <v>20254003</v>
       </c>
       <c r="B324" t="s">
-        <v>3568</v>
+        <v>3569</v>
       </c>
       <c r="C324" t="s">
         <v>232</v>
       </c>
       <c r="D324" t="s">
-        <v>3569</v>
+        <v>3570</v>
       </c>
       <c r="E324"/>
       <c r="F324" t="s">
-        <v>3570</v>
+        <v>3571</v>
       </c>
       <c r="G324" t="s">
         <v>27</v>
@@ -32403,28 +32404,28 @@
         <v>63</v>
       </c>
       <c r="I324" t="s">
-        <v>3571</v>
+        <v>3572</v>
       </c>
       <c r="J324" t="s">
-        <v>3572</v>
+        <v>3573</v>
       </c>
       <c r="K324" t="s">
-        <v>3573</v>
+        <v>3574</v>
       </c>
       <c r="L324" t="s">
-        <v>3574</v>
+        <v>3575</v>
       </c>
       <c r="M324" t="s">
-        <v>3575</v>
+        <v>3576</v>
       </c>
       <c r="N324" t="s">
         <v>50</v>
       </c>
       <c r="O324" t="s">
-        <v>3576</v>
+        <v>3577</v>
       </c>
       <c r="P324" t="s">
-        <v>3577</v>
+        <v>3578</v>
       </c>
       <c r="Q324" t="s">
         <v>53</v>
@@ -32432,13 +32433,13 @@
       <c r="R324"/>
       <c r="S324"/>
       <c r="T324" t="s">
-        <v>3578</v>
+        <v>3579</v>
       </c>
       <c r="U324" t="s">
-        <v>3579</v>
+        <v>3580</v>
       </c>
       <c r="V324" t="s">
-        <v>3580</v>
+        <v>3581</v>
       </c>
     </row>
     <row r="325">
@@ -32446,7 +32447,7 @@
         <v>20253984</v>
       </c>
       <c r="B325" t="s">
-        <v>3581</v>
+        <v>3582</v>
       </c>
       <c r="C325" t="s">
         <v>77</v>
@@ -32456,7 +32457,7 @@
       </c>
       <c r="E325"/>
       <c r="F325" t="s">
-        <v>3582</v>
+        <v>3583</v>
       </c>
       <c r="G325" t="s">
         <v>27</v>
@@ -32465,28 +32466,28 @@
         <v>63</v>
       </c>
       <c r="I325" t="s">
-        <v>3486</v>
+        <v>3487</v>
       </c>
       <c r="J325" t="s">
-        <v>3487</v>
+        <v>3488</v>
       </c>
       <c r="K325" t="s">
-        <v>3488</v>
+        <v>3489</v>
       </c>
       <c r="L325" t="s">
-        <v>3583</v>
+        <v>3584</v>
       </c>
       <c r="M325" t="s">
-        <v>3584</v>
+        <v>3585</v>
       </c>
       <c r="N325" t="s">
         <v>3420</v>
       </c>
       <c r="O325" t="s">
-        <v>3585</v>
+        <v>3586</v>
       </c>
       <c r="P325" t="s">
-        <v>3586</v>
+        <v>3587</v>
       </c>
       <c r="Q325" t="s">
         <v>53</v>
@@ -32508,7 +32509,7 @@
         <v>20257663</v>
       </c>
       <c r="B326" t="s">
-        <v>3587</v>
+        <v>3588</v>
       </c>
       <c r="C326" t="s">
         <v>59</v>
@@ -32520,7 +32521,7 @@
         <v>61</v>
       </c>
       <c r="F326" t="s">
-        <v>3582</v>
+        <v>3583</v>
       </c>
       <c r="G326" t="s">
         <v>27</v>
@@ -32529,26 +32530,26 @@
         <v>44</v>
       </c>
       <c r="I326" t="s">
-        <v>3588</v>
+        <v>3589</v>
       </c>
       <c r="J326" t="s">
-        <v>3589</v>
+        <v>3590</v>
       </c>
       <c r="K326"/>
       <c r="L326" t="s">
-        <v>3590</v>
+        <v>3591</v>
       </c>
       <c r="M326" t="s">
-        <v>3591</v>
+        <v>3592</v>
       </c>
       <c r="N326" t="s">
         <v>69</v>
       </c>
       <c r="O326" t="s">
-        <v>3592</v>
+        <v>3593</v>
       </c>
       <c r="P326" t="s">
-        <v>3593</v>
+        <v>3594</v>
       </c>
       <c r="Q326" t="s">
         <v>53</v>
@@ -32556,13 +32557,13 @@
       <c r="R326"/>
       <c r="S326"/>
       <c r="T326" t="s">
-        <v>3594</v>
+        <v>3595</v>
       </c>
       <c r="U326" t="s">
-        <v>3595</v>
+        <v>3596</v>
       </c>
       <c r="V326" t="s">
-        <v>3596</v>
+        <v>3597</v>
       </c>
     </row>
     <row r="327">
@@ -32570,19 +32571,19 @@
         <v>20257698</v>
       </c>
       <c r="B327" t="s">
-        <v>3597</v>
+        <v>3598</v>
       </c>
       <c r="C327" t="s">
         <v>59</v>
       </c>
       <c r="D327" t="s">
-        <v>3598</v>
+        <v>3599</v>
       </c>
       <c r="E327" t="s">
-        <v>159</v>
+        <v>3427</v>
       </c>
       <c r="F327" t="s">
-        <v>3582</v>
+        <v>3583</v>
       </c>
       <c r="G327" t="s">
         <v>27</v>
@@ -32591,26 +32592,26 @@
         <v>44</v>
       </c>
       <c r="I327" t="s">
-        <v>3599</v>
+        <v>3600</v>
       </c>
       <c r="J327" t="s">
-        <v>3600</v>
+        <v>3601</v>
       </c>
       <c r="K327"/>
       <c r="L327" t="s">
-        <v>3601</v>
+        <v>3602</v>
       </c>
       <c r="M327" t="s">
-        <v>3602</v>
+        <v>3603</v>
       </c>
       <c r="N327" t="s">
         <v>69</v>
       </c>
       <c r="O327" t="s">
-        <v>3603</v>
+        <v>3604</v>
       </c>
       <c r="P327" t="s">
-        <v>3604</v>
+        <v>3605</v>
       </c>
       <c r="Q327" t="s">
         <v>53</v>
@@ -32632,19 +32633,19 @@
         <v>20253971</v>
       </c>
       <c r="B328" t="s">
-        <v>3605</v>
+        <v>3606</v>
       </c>
       <c r="C328" t="s">
         <v>40</v>
       </c>
       <c r="D328" t="s">
-        <v>3606</v>
+        <v>3607</v>
       </c>
       <c r="E328" t="s">
         <v>42</v>
       </c>
       <c r="F328" t="s">
-        <v>3607</v>
+        <v>3608</v>
       </c>
       <c r="G328" t="s">
         <v>81</v>
@@ -32653,28 +32654,28 @@
         <v>563</v>
       </c>
       <c r="I328" t="s">
-        <v>3608</v>
+        <v>3609</v>
       </c>
       <c r="J328" t="s">
-        <v>3609</v>
+        <v>3610</v>
       </c>
       <c r="K328" t="s">
-        <v>3610</v>
+        <v>3611</v>
       </c>
       <c r="L328" t="s">
-        <v>3611</v>
+        <v>3612</v>
       </c>
       <c r="M328" t="s">
-        <v>3612</v>
+        <v>3613</v>
       </c>
       <c r="N328" t="s">
         <v>69</v>
       </c>
       <c r="O328" t="s">
-        <v>3613</v>
+        <v>3614</v>
       </c>
       <c r="P328" t="s">
-        <v>3614</v>
+        <v>3615</v>
       </c>
       <c r="Q328" t="s">
         <v>89</v>
@@ -32682,13 +32683,13 @@
       <c r="R328"/>
       <c r="S328"/>
       <c r="T328" t="s">
-        <v>3480</v>
+        <v>3481</v>
       </c>
       <c r="U328" t="s">
-        <v>3481</v>
+        <v>3482</v>
       </c>
       <c r="V328" t="s">
-        <v>3482</v>
+        <v>3483</v>
       </c>
     </row>
     <row r="329">
@@ -32696,7 +32697,7 @@
         <v>20257601</v>
       </c>
       <c r="B329" t="s">
-        <v>3615</v>
+        <v>3616</v>
       </c>
       <c r="C329" t="s">
         <v>59</v>
@@ -32705,10 +32706,10 @@
         <v>1495</v>
       </c>
       <c r="E329" t="s">
-        <v>1496</v>
+        <v>659</v>
       </c>
       <c r="F329" t="s">
-        <v>3616</v>
+        <v>3617</v>
       </c>
       <c r="G329" t="s">
         <v>27</v>
@@ -32717,26 +32718,26 @@
         <v>97</v>
       </c>
       <c r="I329" t="s">
-        <v>3617</v>
+        <v>3618</v>
       </c>
       <c r="J329" t="s">
-        <v>3618</v>
+        <v>3619</v>
       </c>
       <c r="K329"/>
       <c r="L329" t="s">
-        <v>3619</v>
+        <v>3620</v>
       </c>
       <c r="M329" t="s">
-        <v>3620</v>
+        <v>3621</v>
       </c>
       <c r="N329" t="s">
         <v>69</v>
       </c>
       <c r="O329" t="s">
-        <v>3621</v>
+        <v>3622</v>
       </c>
       <c r="P329" t="s">
-        <v>3622</v>
+        <v>3623</v>
       </c>
       <c r="Q329" t="s">
         <v>89</v>
@@ -32758,17 +32759,17 @@
         <v>20253941</v>
       </c>
       <c r="B330" t="s">
-        <v>3623</v>
+        <v>3624</v>
       </c>
       <c r="C330" t="s">
         <v>77</v>
       </c>
       <c r="D330" t="s">
-        <v>3624</v>
+        <v>3625</v>
       </c>
       <c r="E330"/>
       <c r="F330" t="s">
-        <v>3625</v>
+        <v>3626</v>
       </c>
       <c r="G330" t="s">
         <v>27</v>
@@ -32777,28 +32778,28 @@
         <v>1556</v>
       </c>
       <c r="I330" t="s">
-        <v>3626</v>
+        <v>3627</v>
       </c>
       <c r="J330" t="s">
-        <v>3627</v>
+        <v>3628</v>
       </c>
       <c r="K330" t="s">
-        <v>3628</v>
+        <v>3629</v>
       </c>
       <c r="L330" t="s">
-        <v>3629</v>
+        <v>3630</v>
       </c>
       <c r="M330" t="s">
-        <v>3630</v>
+        <v>3631</v>
       </c>
       <c r="N330" t="s">
         <v>1987</v>
       </c>
       <c r="O330" t="s">
-        <v>3631</v>
+        <v>3632</v>
       </c>
       <c r="P330" t="s">
-        <v>3632</v>
+        <v>3633</v>
       </c>
       <c r="Q330" t="s">
         <v>53</v>

</xml_diff>

<commit_message>
Update parliament data - 2026-03-07
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_CDF_EFK.xlsx
+++ b/Objets_parlementaires_CDF_EFK.xlsx
@@ -10404,12 +10404,33 @@
     <t xml:space="preserve">Ambiente|Agricoltura</t>
   </si>
   <si>
+    <t xml:space="preserve">25.7863</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-09-17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Steuerdebakel Waadt: Finanzausgleich betroffen?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Débâcle fiscale vaudoise. Conséquences sur la péréquation financière ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Des rapports datant du printemps critiquent le calcul erroné de l’impôt sur la fortune dans le canton de Vaud qui a engendré une perte pouvant se chiffrer en millions de francs. Le canton de Vaud bénéficiant de la péréquation financière nationale, les erreurs pourraient avoir des répercussions sur les autres cantons et la Confédération.&lt;br&gt;- Est-ce que le Conseil fédéral partage cette analyse&amp;nbsp;?&lt;br&gt;- Les paiements compensatoires déjà effectués peuvent-ils être corrigés&amp;nbsp;?&lt;br&gt;- Quelles mesures entend prendre le Conseil fédéral pour éviter, à l’avenir, de telles erreurs&amp;nbsp;?&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Berichte aus dem Frühjahr kritisieren die fehlerhafte Vermögenssteuerberechnung im Kanton Waadt, die ihm mutmasslich mehrere Millionen Franken kostete. Da Waadt Nehmerkanton im nationalen Finanzausgleich ist, könnten die Fehler auch andere Kantone und den Bund betreffen.&lt;br&gt;- Teilt der Bundesrat diese Einschätzung?&lt;br&gt;- Können bereits geleistete Ausgleichszahlungen korrigiert werden?&lt;br&gt;- Welche Massnahmen plant er, um solche Fehler künftig zu verhindern?&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20257863</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20257863</t>
+  </si>
+  <si>
     <t xml:space="preserve">25.4024</t>
   </si>
   <si>
-    <t xml:space="preserve">2025-09-17</t>
-  </si>
-  <si>
     <t xml:space="preserve">Grossprojekte im VBS an externe Dienstleister. Was für eine Strategie wird verfolgt?</t>
   </si>
   <si>
@@ -10431,27 +10452,6 @@
     <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254024</t>
   </si>
   <si>
-    <t xml:space="preserve">25.7863</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Steuerdebakel Waadt: Finanzausgleich betroffen?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Débâcle fiscale vaudoise. Conséquences sur la péréquation financière ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Des rapports datant du printemps critiquent le calcul erroné de l’impôt sur la fortune dans le canton de Vaud qui a engendré une perte pouvant se chiffrer en millions de francs. Le canton de Vaud bénéficiant de la péréquation financière nationale, les erreurs pourraient avoir des répercussions sur les autres cantons et la Confédération.&lt;br&gt;- Est-ce que le Conseil fédéral partage cette analyse&amp;nbsp;?&lt;br&gt;- Les paiements compensatoires déjà effectués peuvent-ils être corrigés&amp;nbsp;?&lt;br&gt;- Quelles mesures entend prendre le Conseil fédéral pour éviter, à l’avenir, de telles erreurs&amp;nbsp;?&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Berichte aus dem Frühjahr kritisieren die fehlerhafte Vermögenssteuerberechnung im Kanton Waadt, die ihm mutmasslich mehrere Millionen Franken kostete. Da Waadt Nehmerkanton im nationalen Finanzausgleich ist, könnten die Fehler auch andere Kantone und den Bund betreffen.&lt;br&gt;- Teilt der Bundesrat diese Einschätzung?&lt;br&gt;- Können bereits geleistete Ausgleichszahlungen korrigiert werden?&lt;br&gt;- Welche Massnahmen plant er, um solche Fehler künftig zu verhindern?&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20257863</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20257863</t>
-  </si>
-  <si>
     <t xml:space="preserve">25.7888</t>
   </si>
   <si>
@@ -10533,12 +10533,66 @@
     <t xml:space="preserve">Economia|Imposte</t>
   </si>
   <si>
+    <t xml:space="preserve">25.7663</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-09-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ruag: Anwaltskosten in Millionenhöhe statt Munition für unsere Armee?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RUAG : des millions pour des avocats au lieu de munition pour notre armée ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;RUAG, entre autres en lien avec certaines irrégularités, aurait engagé plus de 10 millions de francs en frais d'avocats &lt;a href="https://www.blick.ch/politik/neues-ungemach-bei-ruag-bundesfirma-gibt-ueber-10-millionen-franken-fuer-gutachten-aus-id21203936.html."&gt;https://www.blick.ch/politik/neues-ungemach-bei-ruag-bundesfirma-gibt-ueber-10-millionen-franken-fuer-gutachten-aus-id21203936.html.&lt;/a&gt;&lt;br&gt;- Le Conseil fédéral tolère-t-il cette manière de sous-traiter à grands frais des tâches de gouvernance d'entreprise ?&lt;br&gt;- Entend-il prendre des mesures ?&lt;br&gt;- Ces honoraires faramineux ne seraient-ils pas mieux investis dans l'acquisition de munition ?&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Die Ruag soll unter anderem im Zusammenhang mit bestimmten Unregelmässigkeiten mehr als 10 Millionen Franken für Anwaltskosten ausgegeben haben &lt;a href="https://www.blick.ch/politik/neues-ungemach-bei-ruag-bundesfirma-gibt-ueber-10-millionen-franken-fuer-gutachten-aus-id21203936.html."&gt;(https://www.blick.ch/politik/neues-ungemach-bei-ruag-bundesfirma-gibt-ueber-10-millionen-franken-fuer-gutachten-aus-id21203936.html).&lt;/a&gt;&lt;br&gt;– Duldet der Bundesrat diese Art der kostspieligen Auslagerung von Aufgaben der Corporate Governance?&lt;br&gt;– Beabsichtigt der Bundesrat, Massnahmen zu ergreifen?&lt;br&gt;– Wäre es nicht besser, diese enormen Beträge in den Kauf von Munition zu investieren?&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20257663</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20257663</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sicherheitspolitik|Finanzwesen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Politique de sécurité|Finances</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Politica di sicurezza|Finanze</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25.7698</t>
+  </si>
+  <si>
+    <t xml:space="preserve">De Ventura Linda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Untersuchungskosten Ruag-Skandal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coûts de l’enquête sur le scandale RUAG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;D’après la presse, les coûts de l’enquête externe sur le scandale RUAG se montent aujourd’hui à plus de 10&amp;nbsp;millions de francs.&lt;br&gt;- Quel est le montant des coûts engagés jusqu’à présent et à qui cet argent a-t-il été versé&amp;nbsp;?&lt;br&gt;- Le Conseil fédéral juge-t-il ces coûts raisonnables&amp;nbsp;? Comment justifie-t-il une telle dépense&amp;nbsp;?&lt;br&gt;- Comment explique-t-il l’évidente faillite des mécanismes de contrôle internes, à la fois dans l’entreprise RUAG et au DDPS, qui a imposé cette enquête externe&amp;nbsp;?&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Gemäss Medienberichten belaufen sich die Kosten für die externe Untersuchung des RUAG-Skandals inzwischen auf über CHF 10 Millionen.&lt;br&gt;- Wie hoch sind die bisherigen Kosten der Untersuchung und an wen wurden diese Mittel ausbezahlt?&lt;br&gt;- Hält der Bundesrat diese Kosten für verhältnismässig und wie rechtfertigt er sie?&lt;br&gt;- Wie erklärt der Bundesrat das offensichtliche Versagen der internen Kontrollmechanismen innerhalb der RUAG sowie im VBS, das dazu führte, dass diese externe Untersuchung notwendig&amp;nbsp;wurde?&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20257698</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20257698</t>
+  </si>
+  <si>
     <t xml:space="preserve">25.3984</t>
   </si>
   <si>
-    <t xml:space="preserve">2025-09-10</t>
-  </si>
-  <si>
     <t xml:space="preserve">&lt;p&gt;Le Conseil fédéral est chargé d’adapter l’examen des subventions tel qu’il est réglé dans la loi sur les subventions (LSu) de manière à mettre en place un ensemble de mesures permettant de réduire les subventions nuisibles.&lt;/p&gt;</t>
   </si>
   <si>
@@ -10549,60 +10603,6 @@
   </si>
   <si>
     <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20253984</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25.7663</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ruag: Anwaltskosten in Millionenhöhe statt Munition für unsere Armee?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RUAG : des millions pour des avocats au lieu de munition pour notre armée ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;RUAG, entre autres en lien avec certaines irrégularités, aurait engagé plus de 10 millions de francs en frais d'avocats &lt;a href="https://www.blick.ch/politik/neues-ungemach-bei-ruag-bundesfirma-gibt-ueber-10-millionen-franken-fuer-gutachten-aus-id21203936.html."&gt;https://www.blick.ch/politik/neues-ungemach-bei-ruag-bundesfirma-gibt-ueber-10-millionen-franken-fuer-gutachten-aus-id21203936.html.&lt;/a&gt;&lt;br&gt;- Le Conseil fédéral tolère-t-il cette manière de sous-traiter à grands frais des tâches de gouvernance d'entreprise ?&lt;br&gt;- Entend-il prendre des mesures ?&lt;br&gt;- Ces honoraires faramineux ne seraient-ils pas mieux investis dans l'acquisition de munition ?&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Die Ruag soll unter anderem im Zusammenhang mit bestimmten Unregelmässigkeiten mehr als 10 Millionen Franken für Anwaltskosten ausgegeben haben &lt;a href="https://www.blick.ch/politik/neues-ungemach-bei-ruag-bundesfirma-gibt-ueber-10-millionen-franken-fuer-gutachten-aus-id21203936.html."&gt;(https://www.blick.ch/politik/neues-ungemach-bei-ruag-bundesfirma-gibt-ueber-10-millionen-franken-fuer-gutachten-aus-id21203936.html).&lt;/a&gt;&lt;br&gt;– Duldet der Bundesrat diese Art der kostspieligen Auslagerung von Aufgaben der Corporate Governance?&lt;br&gt;– Beabsichtigt der Bundesrat, Massnahmen zu ergreifen?&lt;br&gt;– Wäre es nicht besser, diese enormen Beträge in den Kauf von Munition zu investieren?&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20257663</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20257663</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sicherheitspolitik|Finanzwesen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Politique de sécurité|Finances</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Politica di sicurezza|Finanze</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25.7698</t>
-  </si>
-  <si>
-    <t xml:space="preserve">De Ventura Linda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Untersuchungskosten Ruag-Skandal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coûts de l’enquête sur le scandale RUAG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;D’après la presse, les coûts de l’enquête externe sur le scandale RUAG se montent aujourd’hui à plus de 10&amp;nbsp;millions de francs.&lt;br&gt;- Quel est le montant des coûts engagés jusqu’à présent et à qui cet argent a-t-il été versé&amp;nbsp;?&lt;br&gt;- Le Conseil fédéral juge-t-il ces coûts raisonnables&amp;nbsp;? Comment justifie-t-il une telle dépense&amp;nbsp;?&lt;br&gt;- Comment explique-t-il l’évidente faillite des mécanismes de contrôle internes, à la fois dans l’entreprise RUAG et au DDPS, qui a imposé cette enquête externe&amp;nbsp;?&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Gemäss Medienberichten belaufen sich die Kosten für die externe Untersuchung des RUAG-Skandals inzwischen auf über CHF 10 Millionen.&lt;br&gt;- Wie hoch sind die bisherigen Kosten der Untersuchung und an wen wurden diese Mittel ausbezahlt?&lt;br&gt;- Hält der Bundesrat diese Kosten für verhältnismässig und wie rechtfertigt er sie?&lt;br&gt;- Wie erklärt der Bundesrat das offensichtliche Versagen der internen Kontrollmechanismen innerhalb der RUAG sowie im VBS, das dazu führte, dass diese externe Untersuchung notwendig&amp;nbsp;wurde?&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20257698</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20257698</t>
   </si>
   <si>
     <t xml:space="preserve">25.3971</t>
@@ -31446,19 +31446,19 @@
     </row>
     <row r="313">
       <c r="A313" t="n">
-        <v>20254024</v>
+        <v>20257863</v>
       </c>
       <c r="B313" t="s">
         <v>3463</v>
       </c>
       <c r="C313" t="s">
-        <v>56</v>
+        <v>23</v>
       </c>
       <c r="D313" t="s">
-        <v>1606</v>
+        <v>1814</v>
       </c>
       <c r="E313" t="s">
-        <v>25</v>
+        <v>1815</v>
       </c>
       <c r="F313" t="s">
         <v>3464</v>
@@ -31467,7 +31467,7 @@
         <v>27</v>
       </c>
       <c r="H313" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="I313" t="s">
         <v>3465</v>
@@ -31475,54 +31475,52 @@
       <c r="J313" t="s">
         <v>3466</v>
       </c>
-      <c r="K313" t="s">
+      <c r="K313"/>
+      <c r="L313" t="s">
         <v>3467</v>
       </c>
-      <c r="L313" t="s">
+      <c r="M313" t="s">
         <v>3468</v>
       </c>
-      <c r="M313" t="s">
+      <c r="N313" t="s">
+        <v>84</v>
+      </c>
+      <c r="O313" t="s">
         <v>3469</v>
       </c>
-      <c r="N313" t="s">
-        <v>66</v>
-      </c>
-      <c r="O313" t="s">
+      <c r="P313" t="s">
         <v>3470</v>
       </c>
-      <c r="P313" t="s">
-        <v>3471</v>
-      </c>
       <c r="Q313" t="s">
-        <v>104</v>
+        <v>69</v>
       </c>
       <c r="R313"/>
       <c r="S313"/>
       <c r="T313" t="s">
-        <v>1534</v>
+        <v>942</v>
       </c>
       <c r="U313" t="s">
-        <v>1535</v>
+        <v>943</v>
       </c>
       <c r="V313" t="s">
-        <v>1536</v>
+        <v>944</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="n">
-        <v>20257863</v>
+        <v>20254024</v>
       </c>
       <c r="B314" t="s">
-        <v>3472</v>
+        <v>3471</v>
       </c>
       <c r="C314" t="s">
-        <v>23</v>
+        <v>56</v>
       </c>
       <c r="D314" t="s">
-        <v>1814</v>
+        <v>1606</v>
       </c>
       <c r="E314" t="s">
-        <v>1815</v>
+        <v>25</v>
       </c>
       <c r="F314" t="s">
         <v>3464</v>
@@ -31531,15 +31529,17 @@
         <v>27</v>
       </c>
       <c r="H314" t="s">
-        <v>78</v>
+        <v>60</v>
       </c>
       <c r="I314" t="s">
+        <v>3472</v>
+      </c>
+      <c r="J314" t="s">
         <v>3473</v>
       </c>
-      <c r="J314" t="s">
+      <c r="K314" t="s">
         <v>3474</v>
       </c>
-      <c r="K314"/>
       <c r="L314" t="s">
         <v>3475</v>
       </c>
@@ -31547,7 +31547,7 @@
         <v>3476</v>
       </c>
       <c r="N314" t="s">
-        <v>84</v>
+        <v>66</v>
       </c>
       <c r="O314" t="s">
         <v>3477</v>
@@ -31556,18 +31556,18 @@
         <v>3478</v>
       </c>
       <c r="Q314" t="s">
-        <v>69</v>
+        <v>104</v>
       </c>
       <c r="R314"/>
       <c r="S314"/>
       <c r="T314" t="s">
-        <v>942</v>
+        <v>1534</v>
       </c>
       <c r="U314" t="s">
-        <v>943</v>
+        <v>1535</v>
       </c>
       <c r="V314" t="s">
-        <v>944</v>
+        <v>1536</v>
       </c>
     </row>
     <row r="315">
@@ -31758,18 +31758,20 @@
     </row>
     <row r="318">
       <c r="A318" t="n">
-        <v>20253984</v>
+        <v>20257663</v>
       </c>
       <c r="B318" t="s">
         <v>3506</v>
       </c>
       <c r="C318" t="s">
-        <v>92</v>
+        <v>23</v>
       </c>
       <c r="D318" t="s">
-        <v>623</v>
-      </c>
-      <c r="E318"/>
+        <v>163</v>
+      </c>
+      <c r="E318" t="s">
+        <v>76</v>
+      </c>
       <c r="F318" t="s">
         <v>3507</v>
       </c>
@@ -31777,31 +31779,29 @@
         <v>27</v>
       </c>
       <c r="H318" t="s">
-        <v>78</v>
+        <v>60</v>
       </c>
       <c r="I318" t="s">
-        <v>3411</v>
+        <v>3508</v>
       </c>
       <c r="J318" t="s">
-        <v>3412</v>
-      </c>
-      <c r="K318" t="s">
-        <v>3413</v>
-      </c>
+        <v>3509</v>
+      </c>
+      <c r="K318"/>
       <c r="L318" t="s">
-        <v>3508</v>
+        <v>3510</v>
       </c>
       <c r="M318" t="s">
-        <v>3509</v>
+        <v>3511</v>
       </c>
       <c r="N318" t="s">
-        <v>3345</v>
+        <v>84</v>
       </c>
       <c r="O318" t="s">
-        <v>3510</v>
+        <v>3512</v>
       </c>
       <c r="P318" t="s">
-        <v>3511</v>
+        <v>3513</v>
       </c>
       <c r="Q318" t="s">
         <v>69</v>
@@ -31809,30 +31809,30 @@
       <c r="R318"/>
       <c r="S318"/>
       <c r="T318" t="s">
-        <v>146</v>
+        <v>3514</v>
       </c>
       <c r="U318" t="s">
-        <v>147</v>
+        <v>3515</v>
       </c>
       <c r="V318" t="s">
-        <v>148</v>
+        <v>3516</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="n">
-        <v>20257663</v>
+        <v>20257698</v>
       </c>
       <c r="B319" t="s">
-        <v>3512</v>
+        <v>3517</v>
       </c>
       <c r="C319" t="s">
         <v>23</v>
       </c>
       <c r="D319" t="s">
-        <v>163</v>
+        <v>3518</v>
       </c>
       <c r="E319" t="s">
-        <v>76</v>
+        <v>25</v>
       </c>
       <c r="F319" t="s">
         <v>3507</v>
@@ -31844,26 +31844,26 @@
         <v>60</v>
       </c>
       <c r="I319" t="s">
-        <v>3513</v>
+        <v>3519</v>
       </c>
       <c r="J319" t="s">
-        <v>3514</v>
+        <v>3520</v>
       </c>
       <c r="K319"/>
       <c r="L319" t="s">
-        <v>3515</v>
+        <v>3521</v>
       </c>
       <c r="M319" t="s">
-        <v>3516</v>
+        <v>3522</v>
       </c>
       <c r="N319" t="s">
         <v>84</v>
       </c>
       <c r="O319" t="s">
-        <v>3517</v>
+        <v>3523</v>
       </c>
       <c r="P319" t="s">
-        <v>3518</v>
+        <v>3524</v>
       </c>
       <c r="Q319" t="s">
         <v>69</v>
@@ -31871,31 +31871,29 @@
       <c r="R319"/>
       <c r="S319"/>
       <c r="T319" t="s">
-        <v>3519</v>
+        <v>1499</v>
       </c>
       <c r="U319" t="s">
-        <v>3520</v>
+        <v>1500</v>
       </c>
       <c r="V319" t="s">
-        <v>3521</v>
+        <v>1501</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="n">
-        <v>20257698</v>
+        <v>20253984</v>
       </c>
       <c r="B320" t="s">
-        <v>3522</v>
+        <v>3525</v>
       </c>
       <c r="C320" t="s">
-        <v>23</v>
+        <v>92</v>
       </c>
       <c r="D320" t="s">
-        <v>3523</v>
-      </c>
-      <c r="E320" t="s">
-        <v>25</v>
-      </c>
+        <v>623</v>
+      </c>
+      <c r="E320"/>
       <c r="F320" t="s">
         <v>3507</v>
       </c>
@@ -31903,15 +31901,17 @@
         <v>27</v>
       </c>
       <c r="H320" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="I320" t="s">
-        <v>3524</v>
+        <v>3411</v>
       </c>
       <c r="J320" t="s">
-        <v>3525</v>
-      </c>
-      <c r="K320"/>
+        <v>3412</v>
+      </c>
+      <c r="K320" t="s">
+        <v>3413</v>
+      </c>
       <c r="L320" t="s">
         <v>3526</v>
       </c>
@@ -31919,7 +31919,7 @@
         <v>3527</v>
       </c>
       <c r="N320" t="s">
-        <v>84</v>
+        <v>3345</v>
       </c>
       <c r="O320" t="s">
         <v>3528</v>
@@ -31933,13 +31933,13 @@
       <c r="R320"/>
       <c r="S320"/>
       <c r="T320" t="s">
-        <v>1499</v>
+        <v>146</v>
       </c>
       <c r="U320" t="s">
-        <v>1500</v>
+        <v>147</v>
       </c>
       <c r="V320" t="s">
-        <v>1501</v>
+        <v>148</v>
       </c>
     </row>
     <row r="321">

</xml_diff>

<commit_message>
Update parliament data - 2026-03-08
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_CDF_EFK.xlsx
+++ b/Objets_parlementaires_CDF_EFK.xlsx
@@ -10404,12 +10404,36 @@
     <t xml:space="preserve">Ambiente|Agricoltura</t>
   </si>
   <si>
+    <t xml:space="preserve">25.4024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-09-17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grossprojekte im VBS an externe Dienstleister. Was für eine Strategie wird verfolgt?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le DDPS confie de grands projets à des externes. Quel est l'objectif stratégique ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Progetti di grande portata nel DDPS a fornitori di prestazioni esterni. Quale strategia viene seguita?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;1. Pourquoi le DDPS externalise-t-il intégralement la gestion des risques et de la qualité de ses grands projets au lieu de renforcer des services internes tels que le Contrôle fédéral des finances ou la révision interne&amp;nbsp;?&lt;/p&gt;&lt;p&gt;2. À combien sont estimés les coûts des nouveaux contrats-cadres conclus pour une durée de douze ans&amp;nbsp;? Comment s’assure-t-on que les coûts ne dérapent pas&amp;nbsp;?&lt;/p&gt;&lt;p&gt;3. Pourquoi avoir choisi une durée de contrat aussi longue&amp;nbsp;? Est-il possible de modifier ou de résilier les contrats en cas de besoin&amp;nbsp;?&lt;/p&gt;&lt;p&gt;4. Quels critères ont déterminé le choix des prestataires externes&amp;nbsp;? Comment éviter les conflits d’intérêts et garantir l’indépendance&amp;nbsp;?&lt;/p&gt;&lt;p&gt;5. Quelles leçons le DDPS tire-t-il de précédentes expertises réalisées par des externes comme celle du cabinet d’avocat Homburger sur le F-35, qui a été taxée d’être un rapport de complaisance&amp;nbsp;? Comment la transparence sera-t-il garantie&amp;nbsp;?&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;1. Weshalb lagert das VBS das Qualitäts- und Risikomanagement bei seinen Grossprojekten vollständig an Externe aus, anstatt interne Stellen wie die EFK oder die interne Revision zu stärken?&lt;/p&gt;&lt;p&gt;2. Wie hoch werden die Kosten der neuen Rahmenverträge über zwölf Jahre geschätzt, und wie wird sichergestellt, dass diese nicht aus dem Ruder laufen?&lt;/p&gt;&lt;p&gt;3. Weshalb wurde eine so lange Vertragsdauer gewählt, und welche Möglichkeiten bestehen, Verträge bei Bedarf anzupassen oder zu beenden?&lt;/p&gt;&lt;p&gt;4. Nach welchen Kriterien werden die externen Dienstleister ausgewählt, und wie wird verhindert, dass Interessenkonflikte entstehen oder die Unabhängigkeit beeinträchtigt wird?&lt;/p&gt;&lt;p&gt;5. Welche Lehren zieht das VBS aus früheren externen Gutachten wie jenen der Kanzlei Homburger zum F-35, die als Gefälligkeitsgutachten kritisiert wurden, und wie wird künftig Transparenz garantiert?&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254024</t>
+  </si>
+  <si>
     <t xml:space="preserve">25.7863</t>
   </si>
   <si>
-    <t xml:space="preserve">2025-09-17</t>
-  </si>
-  <si>
     <t xml:space="preserve">Steuerdebakel Waadt: Finanzausgleich betroffen?</t>
   </si>
   <si>
@@ -10428,30 +10452,6 @@
     <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20257863</t>
   </si>
   <si>
-    <t xml:space="preserve">25.4024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Grossprojekte im VBS an externe Dienstleister. Was für eine Strategie wird verfolgt?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Le DDPS confie de grands projets à des externes. Quel est l'objectif stratégique ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Progetti di grande portata nel DDPS a fornitori di prestazioni esterni. Quale strategia viene seguita?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;1. Pourquoi le DDPS externalise-t-il intégralement la gestion des risques et de la qualité de ses grands projets au lieu de renforcer des services internes tels que le Contrôle fédéral des finances ou la révision interne&amp;nbsp;?&lt;/p&gt;&lt;p&gt;2. À combien sont estimés les coûts des nouveaux contrats-cadres conclus pour une durée de douze ans&amp;nbsp;? Comment s’assure-t-on que les coûts ne dérapent pas&amp;nbsp;?&lt;/p&gt;&lt;p&gt;3. Pourquoi avoir choisi une durée de contrat aussi longue&amp;nbsp;? Est-il possible de modifier ou de résilier les contrats en cas de besoin&amp;nbsp;?&lt;/p&gt;&lt;p&gt;4. Quels critères ont déterminé le choix des prestataires externes&amp;nbsp;? Comment éviter les conflits d’intérêts et garantir l’indépendance&amp;nbsp;?&lt;/p&gt;&lt;p&gt;5. Quelles leçons le DDPS tire-t-il de précédentes expertises réalisées par des externes comme celle du cabinet d’avocat Homburger sur le F-35, qui a été taxée d’être un rapport de complaisance&amp;nbsp;? Comment la transparence sera-t-il garantie&amp;nbsp;?&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;1. Weshalb lagert das VBS das Qualitäts- und Risikomanagement bei seinen Grossprojekten vollständig an Externe aus, anstatt interne Stellen wie die EFK oder die interne Revision zu stärken?&lt;/p&gt;&lt;p&gt;2. Wie hoch werden die Kosten der neuen Rahmenverträge über zwölf Jahre geschätzt, und wie wird sichergestellt, dass diese nicht aus dem Ruder laufen?&lt;/p&gt;&lt;p&gt;3. Weshalb wurde eine so lange Vertragsdauer gewählt, und welche Möglichkeiten bestehen, Verträge bei Bedarf anzupassen oder zu beenden?&lt;/p&gt;&lt;p&gt;4. Nach welchen Kriterien werden die externen Dienstleister ausgewählt, und wie wird verhindert, dass Interessenkonflikte entstehen oder die Unabhängigkeit beeinträchtigt wird?&lt;/p&gt;&lt;p&gt;5. Welche Lehren zieht das VBS aus früheren externen Gutachten wie jenen der Kanzlei Homburger zum F-35, die als Gefälligkeitsgutachten kritisiert wurden, und wie wird künftig Transparenz garantiert?&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254024</t>
-  </si>
-  <si>
     <t xml:space="preserve">25.7888</t>
   </si>
   <si>
@@ -10533,12 +10533,27 @@
     <t xml:space="preserve">Economia|Imposte</t>
   </si>
   <si>
+    <t xml:space="preserve">25.3984</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-09-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Le Conseil fédéral est chargé d’adapter l’examen des subventions tel qu’il est réglé dans la loi sur les subventions (LSu) de manière à mettre en place un ensemble de mesures permettant de réduire les subventions nuisibles.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Der Bundesrat wird beauftragt, die Subventionsprüfung gemäss Subventionsgesetz (SuG) so anzupassen, dass daraus ein Paket für einen Abbau von schädlichen Subventionen hervorgeht.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20253984</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20253984</t>
+  </si>
+  <si>
     <t xml:space="preserve">25.7663</t>
   </si>
   <si>
-    <t xml:space="preserve">2025-09-10</t>
-  </si>
-  <si>
     <t xml:space="preserve">Ruag: Anwaltskosten in Millionenhöhe statt Munition für unsere Armee?</t>
   </si>
   <si>
@@ -10588,21 +10603,6 @@
   </si>
   <si>
     <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20257698</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25.3984</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Le Conseil fédéral est chargé d’adapter l’examen des subventions tel qu’il est réglé dans la loi sur les subventions (LSu) de manière à mettre en place un ensemble de mesures permettant de réduire les subventions nuisibles.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Der Bundesrat wird beauftragt, die Subventionsprüfung gemäss Subventionsgesetz (SuG) so anzupassen, dass daraus ein Paket für einen Abbau von schädlichen Subventionen hervorgeht.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20253984</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20253984</t>
   </si>
   <si>
     <t xml:space="preserve">25.3971</t>
@@ -31446,19 +31446,19 @@
     </row>
     <row r="313">
       <c r="A313" t="n">
-        <v>20257863</v>
+        <v>20254024</v>
       </c>
       <c r="B313" t="s">
         <v>3463</v>
       </c>
       <c r="C313" t="s">
-        <v>23</v>
+        <v>56</v>
       </c>
       <c r="D313" t="s">
-        <v>1814</v>
+        <v>1606</v>
       </c>
       <c r="E313" t="s">
-        <v>1815</v>
+        <v>25</v>
       </c>
       <c r="F313" t="s">
         <v>3464</v>
@@ -31467,7 +31467,7 @@
         <v>27</v>
       </c>
       <c r="H313" t="s">
-        <v>78</v>
+        <v>60</v>
       </c>
       <c r="I313" t="s">
         <v>3465</v>
@@ -31475,52 +31475,54 @@
       <c r="J313" t="s">
         <v>3466</v>
       </c>
-      <c r="K313"/>
+      <c r="K313" t="s">
+        <v>3467</v>
+      </c>
       <c r="L313" t="s">
-        <v>3467</v>
+        <v>3468</v>
       </c>
       <c r="M313" t="s">
-        <v>3468</v>
+        <v>3469</v>
       </c>
       <c r="N313" t="s">
-        <v>84</v>
+        <v>66</v>
       </c>
       <c r="O313" t="s">
-        <v>3469</v>
+        <v>3470</v>
       </c>
       <c r="P313" t="s">
-        <v>3470</v>
+        <v>3471</v>
       </c>
       <c r="Q313" t="s">
-        <v>69</v>
+        <v>104</v>
       </c>
       <c r="R313"/>
       <c r="S313"/>
       <c r="T313" t="s">
-        <v>942</v>
+        <v>1534</v>
       </c>
       <c r="U313" t="s">
-        <v>943</v>
+        <v>1535</v>
       </c>
       <c r="V313" t="s">
-        <v>944</v>
+        <v>1536</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="n">
-        <v>20254024</v>
+        <v>20257863</v>
       </c>
       <c r="B314" t="s">
-        <v>3471</v>
+        <v>3472</v>
       </c>
       <c r="C314" t="s">
-        <v>56</v>
+        <v>23</v>
       </c>
       <c r="D314" t="s">
-        <v>1606</v>
+        <v>1814</v>
       </c>
       <c r="E314" t="s">
-        <v>25</v>
+        <v>1815</v>
       </c>
       <c r="F314" t="s">
         <v>3464</v>
@@ -31529,17 +31531,15 @@
         <v>27</v>
       </c>
       <c r="H314" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="I314" t="s">
-        <v>3472</v>
+        <v>3473</v>
       </c>
       <c r="J314" t="s">
-        <v>3473</v>
-      </c>
-      <c r="K314" t="s">
         <v>3474</v>
       </c>
+      <c r="K314"/>
       <c r="L314" t="s">
         <v>3475</v>
       </c>
@@ -31547,7 +31547,7 @@
         <v>3476</v>
       </c>
       <c r="N314" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="O314" t="s">
         <v>3477</v>
@@ -31556,18 +31556,18 @@
         <v>3478</v>
       </c>
       <c r="Q314" t="s">
-        <v>104</v>
+        <v>69</v>
       </c>
       <c r="R314"/>
       <c r="S314"/>
       <c r="T314" t="s">
-        <v>1534</v>
+        <v>942</v>
       </c>
       <c r="U314" t="s">
-        <v>1535</v>
+        <v>943</v>
       </c>
       <c r="V314" t="s">
-        <v>1536</v>
+        <v>944</v>
       </c>
     </row>
     <row r="315">
@@ -31758,20 +31758,18 @@
     </row>
     <row r="318">
       <c r="A318" t="n">
-        <v>20257663</v>
+        <v>20253984</v>
       </c>
       <c r="B318" t="s">
         <v>3506</v>
       </c>
       <c r="C318" t="s">
-        <v>23</v>
+        <v>92</v>
       </c>
       <c r="D318" t="s">
-        <v>163</v>
-      </c>
-      <c r="E318" t="s">
-        <v>76</v>
-      </c>
+        <v>623</v>
+      </c>
+      <c r="E318"/>
       <c r="F318" t="s">
         <v>3507</v>
       </c>
@@ -31779,29 +31777,31 @@
         <v>27</v>
       </c>
       <c r="H318" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="I318" t="s">
+        <v>3411</v>
+      </c>
+      <c r="J318" t="s">
+        <v>3412</v>
+      </c>
+      <c r="K318" t="s">
+        <v>3413</v>
+      </c>
+      <c r="L318" t="s">
         <v>3508</v>
       </c>
-      <c r="J318" t="s">
+      <c r="M318" t="s">
         <v>3509</v>
       </c>
-      <c r="K318"/>
-      <c r="L318" t="s">
+      <c r="N318" t="s">
+        <v>3345</v>
+      </c>
+      <c r="O318" t="s">
         <v>3510</v>
       </c>
-      <c r="M318" t="s">
+      <c r="P318" t="s">
         <v>3511</v>
-      </c>
-      <c r="N318" t="s">
-        <v>84</v>
-      </c>
-      <c r="O318" t="s">
-        <v>3512</v>
-      </c>
-      <c r="P318" t="s">
-        <v>3513</v>
       </c>
       <c r="Q318" t="s">
         <v>69</v>
@@ -31809,30 +31809,30 @@
       <c r="R318"/>
       <c r="S318"/>
       <c r="T318" t="s">
-        <v>3514</v>
+        <v>146</v>
       </c>
       <c r="U318" t="s">
-        <v>3515</v>
+        <v>147</v>
       </c>
       <c r="V318" t="s">
-        <v>3516</v>
+        <v>148</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="n">
-        <v>20257698</v>
+        <v>20257663</v>
       </c>
       <c r="B319" t="s">
-        <v>3517</v>
+        <v>3512</v>
       </c>
       <c r="C319" t="s">
         <v>23</v>
       </c>
       <c r="D319" t="s">
-        <v>3518</v>
+        <v>163</v>
       </c>
       <c r="E319" t="s">
-        <v>25</v>
+        <v>76</v>
       </c>
       <c r="F319" t="s">
         <v>3507</v>
@@ -31844,26 +31844,26 @@
         <v>60</v>
       </c>
       <c r="I319" t="s">
-        <v>3519</v>
+        <v>3513</v>
       </c>
       <c r="J319" t="s">
-        <v>3520</v>
+        <v>3514</v>
       </c>
       <c r="K319"/>
       <c r="L319" t="s">
-        <v>3521</v>
+        <v>3515</v>
       </c>
       <c r="M319" t="s">
-        <v>3522</v>
+        <v>3516</v>
       </c>
       <c r="N319" t="s">
         <v>84</v>
       </c>
       <c r="O319" t="s">
-        <v>3523</v>
+        <v>3517</v>
       </c>
       <c r="P319" t="s">
-        <v>3524</v>
+        <v>3518</v>
       </c>
       <c r="Q319" t="s">
         <v>69</v>
@@ -31871,29 +31871,31 @@
       <c r="R319"/>
       <c r="S319"/>
       <c r="T319" t="s">
-        <v>1499</v>
+        <v>3519</v>
       </c>
       <c r="U319" t="s">
-        <v>1500</v>
+        <v>3520</v>
       </c>
       <c r="V319" t="s">
-        <v>1501</v>
+        <v>3521</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="n">
-        <v>20253984</v>
+        <v>20257698</v>
       </c>
       <c r="B320" t="s">
-        <v>3525</v>
+        <v>3522</v>
       </c>
       <c r="C320" t="s">
-        <v>92</v>
+        <v>23</v>
       </c>
       <c r="D320" t="s">
-        <v>623</v>
-      </c>
-      <c r="E320"/>
+        <v>3523</v>
+      </c>
+      <c r="E320" t="s">
+        <v>25</v>
+      </c>
       <c r="F320" t="s">
         <v>3507</v>
       </c>
@@ -31901,17 +31903,15 @@
         <v>27</v>
       </c>
       <c r="H320" t="s">
-        <v>78</v>
+        <v>60</v>
       </c>
       <c r="I320" t="s">
-        <v>3411</v>
+        <v>3524</v>
       </c>
       <c r="J320" t="s">
-        <v>3412</v>
-      </c>
-      <c r="K320" t="s">
-        <v>3413</v>
-      </c>
+        <v>3525</v>
+      </c>
+      <c r="K320"/>
       <c r="L320" t="s">
         <v>3526</v>
       </c>
@@ -31919,7 +31919,7 @@
         <v>3527</v>
       </c>
       <c r="N320" t="s">
-        <v>3345</v>
+        <v>84</v>
       </c>
       <c r="O320" t="s">
         <v>3528</v>
@@ -31933,13 +31933,13 @@
       <c r="R320"/>
       <c r="S320"/>
       <c r="T320" t="s">
-        <v>146</v>
+        <v>1499</v>
       </c>
       <c r="U320" t="s">
-        <v>147</v>
+        <v>1500</v>
       </c>
       <c r="V320" t="s">
-        <v>148</v>
+        <v>1501</v>
       </c>
     </row>
     <row r="321">

</xml_diff>

<commit_message>
Update parliament data - 2026-03-16
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_CDF_EFK.xlsx
+++ b/Objets_parlementaires_CDF_EFK.xlsx
@@ -113,7 +113,7 @@
     <t xml:space="preserve">&lt;p&gt;Bei der Volksabstimmung vom 8.3.2025 SRG-Initiative hat die SP Schweiz Einnahmen mit angeblichen Rekordkleinstspenden von 1.6 Millionen deklariert. Spenden über 15'000 wurden keine offen gelegt.&amp;nbsp;&lt;br&gt;Kann der Bundesrat bestätigen, dass solche ausserordentlichen Rekordeinnahmen nicht automatisch zu einer Revision führen und dieser Entscheid für eine Revision im Ermessen der EFK liegt?&lt;/p&gt;</t>
   </si>
   <si>
-    <t xml:space="preserve">Eingereicht / Déposé</t>
+    <t xml:space="preserve">Erledigt / Liquidé</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20267185</t>
@@ -125,6 +125,9 @@
     <t xml:space="preserve">Élu</t>
   </si>
   <si>
+    <t xml:space="preserve">2026-03-16</t>
+  </si>
+  <si>
     <t xml:space="preserve">Staatspolitik</t>
   </si>
   <si>
@@ -201,9 +204,6 @@
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Seit Beginn des Projekts im Jahr 2017 hat die Eidgenössische Finanzkontrolle sechs sehr kritische Prüfberichte zur Steuerung des neuen Auszahlungssystems der Arbeitslosenkassen veröffentlicht.&lt;br&gt;Kann uns der Bundesrat mitteilen, ob das SECO die Bemerkungen der Eidgenössischen Finanzkontrolle ausreichend berücksichtigt hat?&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Erledigt / Liquidé</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20267129</t>
@@ -11231,17 +11231,19 @@
         <v>36</v>
       </c>
       <c r="R2" t="s">
-        <v>26</v>
-      </c>
-      <c r="S2"/>
+        <v>37</v>
+      </c>
+      <c r="S2" t="s">
+        <v>37</v>
+      </c>
       <c r="T2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="U2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="V2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3">
@@ -11249,63 +11251,65 @@
         <v>20267161</v>
       </c>
       <c r="B3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C3" t="s">
         <v>23</v>
       </c>
       <c r="D3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G3" t="s">
         <v>27</v>
       </c>
       <c r="H3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="J3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="K3"/>
       <c r="L3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="M3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="N3" t="s">
         <v>33</v>
       </c>
       <c r="O3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="P3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q3" t="s">
         <v>36</v>
       </c>
       <c r="R3" t="s">
-        <v>43</v>
-      </c>
-      <c r="S3"/>
+        <v>37</v>
+      </c>
+      <c r="S3" t="s">
+        <v>37</v>
+      </c>
       <c r="T3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="U3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="V3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4">
@@ -11313,41 +11317,41 @@
         <v>20267129</v>
       </c>
       <c r="B4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C4" t="s">
         <v>23</v>
       </c>
       <c r="D4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G4" t="s">
         <v>27</v>
       </c>
       <c r="H4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="J4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="K4"/>
       <c r="L4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="M4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="N4" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O4" t="s">
         <v>64</v>
@@ -11359,7 +11363,7 @@
         <v>36</v>
       </c>
       <c r="R4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="S4"/>
       <c r="T4" t="s">
@@ -11395,7 +11399,7 @@
         <v>27</v>
       </c>
       <c r="H5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I5" t="s">
         <v>74</v>
@@ -11545,7 +11549,7 @@
         <v>111</v>
       </c>
       <c r="N7" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O7" t="s">
         <v>112</v>
@@ -11659,7 +11663,7 @@
         <v>27</v>
       </c>
       <c r="H9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I9" t="s">
         <v>137</v>
@@ -11791,7 +11795,7 @@
         <v>164</v>
       </c>
       <c r="H11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I11" t="s">
         <v>137</v>
@@ -12055,7 +12059,7 @@
         <v>27</v>
       </c>
       <c r="H15" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I15" t="s">
         <v>209</v>
@@ -12121,7 +12125,7 @@
         <v>164</v>
       </c>
       <c r="H16" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I16" t="s">
         <v>222</v>
@@ -12139,7 +12143,7 @@
         <v>226</v>
       </c>
       <c r="N16" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O16" t="s">
         <v>227</v>
@@ -12269,7 +12273,7 @@
         <v>250</v>
       </c>
       <c r="N18" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O18" t="s">
         <v>251</v>
@@ -12335,7 +12339,7 @@
         <v>262</v>
       </c>
       <c r="N19" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O19" t="s">
         <v>263</v>
@@ -12383,7 +12387,7 @@
         <v>27</v>
       </c>
       <c r="H20" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I20" t="s">
         <v>272</v>
@@ -12449,7 +12453,7 @@
         <v>27</v>
       </c>
       <c r="H21" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I21" t="s">
         <v>285</v>
@@ -12581,7 +12585,7 @@
         <v>27</v>
       </c>
       <c r="H23" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I23" t="s">
         <v>311</v>
@@ -12797,7 +12801,7 @@
         <v>353</v>
       </c>
       <c r="N26" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O26" t="s">
         <v>354</v>
@@ -12863,7 +12867,7 @@
         <v>366</v>
       </c>
       <c r="N27" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O27" t="s">
         <v>367</v>
@@ -12929,7 +12933,7 @@
         <v>378</v>
       </c>
       <c r="N28" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O28" t="s">
         <v>379</v>
@@ -12995,7 +12999,7 @@
         <v>390</v>
       </c>
       <c r="N29" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O29" t="s">
         <v>391</v>
@@ -13061,7 +13065,7 @@
         <v>401</v>
       </c>
       <c r="N30" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O30" t="s">
         <v>402</v>
@@ -13109,7 +13113,7 @@
         <v>27</v>
       </c>
       <c r="H31" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I31" t="s">
         <v>407</v>
@@ -13175,7 +13179,7 @@
         <v>27</v>
       </c>
       <c r="H32" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I32" t="s">
         <v>419</v>
@@ -13191,7 +13195,7 @@
         <v>422</v>
       </c>
       <c r="N32" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O32" t="s">
         <v>423</v>
@@ -13321,7 +13325,7 @@
         <v>446</v>
       </c>
       <c r="N34" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O34" t="s">
         <v>447</v>
@@ -13385,7 +13389,7 @@
         <v>456</v>
       </c>
       <c r="N35" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O35" t="s">
         <v>457</v>
@@ -13449,7 +13453,7 @@
         <v>467</v>
       </c>
       <c r="N36" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O36" t="s">
         <v>468</v>
@@ -13579,7 +13583,7 @@
         <v>490</v>
       </c>
       <c r="N38" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O38" t="s">
         <v>491</v>
@@ -13643,7 +13647,7 @@
         <v>503</v>
       </c>
       <c r="N39" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O39" t="s">
         <v>504</v>
@@ -13709,7 +13713,7 @@
         <v>513</v>
       </c>
       <c r="N40" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O40" t="s">
         <v>514</v>
@@ -13775,7 +13779,7 @@
         <v>524</v>
       </c>
       <c r="N41" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O41" t="s">
         <v>525</v>
@@ -13823,7 +13827,7 @@
         <v>27</v>
       </c>
       <c r="H42" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I42" t="s">
         <v>533</v>
@@ -13839,7 +13843,7 @@
         <v>536</v>
       </c>
       <c r="N42" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O42" t="s">
         <v>537</v>
@@ -14151,7 +14155,7 @@
         <v>27</v>
       </c>
       <c r="H47" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I47" t="s">
         <v>591</v>
@@ -14217,7 +14221,7 @@
         <v>27</v>
       </c>
       <c r="H48" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I48" t="s">
         <v>599</v>
@@ -14283,7 +14287,7 @@
         <v>27</v>
       </c>
       <c r="H49" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I49" t="s">
         <v>610</v>
@@ -14349,7 +14353,7 @@
         <v>27</v>
       </c>
       <c r="H50" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I50" t="s">
         <v>619</v>
@@ -14433,7 +14437,7 @@
         <v>636</v>
       </c>
       <c r="N51" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O51" t="s">
         <v>637</v>
@@ -14497,7 +14501,7 @@
         <v>644</v>
       </c>
       <c r="N52" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O52" t="s">
         <v>645</v>
@@ -14545,7 +14549,7 @@
         <v>27</v>
       </c>
       <c r="H53" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I53" t="s">
         <v>651</v>
@@ -14561,7 +14565,7 @@
         <v>654</v>
       </c>
       <c r="N53" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O53" t="s">
         <v>655</v>
@@ -14609,7 +14613,7 @@
         <v>27</v>
       </c>
       <c r="H54" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I54" t="s">
         <v>663</v>
@@ -14625,7 +14629,7 @@
         <v>666</v>
       </c>
       <c r="N54" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O54" t="s">
         <v>667</v>
@@ -14673,7 +14677,7 @@
         <v>27</v>
       </c>
       <c r="H55" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I55" t="s">
         <v>673</v>
@@ -14689,7 +14693,7 @@
         <v>676</v>
       </c>
       <c r="N55" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O55" t="s">
         <v>677</v>
@@ -14819,7 +14823,7 @@
         <v>697</v>
       </c>
       <c r="N57" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O57" t="s">
         <v>698</v>
@@ -14867,7 +14871,7 @@
         <v>27</v>
       </c>
       <c r="H58" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I58" t="s">
         <v>702</v>
@@ -14883,7 +14887,7 @@
         <v>705</v>
       </c>
       <c r="N58" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O58" t="s">
         <v>706</v>
@@ -14997,7 +15001,7 @@
         <v>27</v>
       </c>
       <c r="H60" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I60" t="s">
         <v>724</v>
@@ -15081,7 +15085,7 @@
         <v>739</v>
       </c>
       <c r="N61" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O61" t="s">
         <v>740</v>
@@ -15147,7 +15151,7 @@
         <v>751</v>
       </c>
       <c r="N62" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O62" t="s">
         <v>752</v>
@@ -15213,7 +15217,7 @@
         <v>761</v>
       </c>
       <c r="N63" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O63" t="s">
         <v>762</v>
@@ -15277,7 +15281,7 @@
         <v>771</v>
       </c>
       <c r="N64" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O64" t="s">
         <v>772</v>
@@ -15323,7 +15327,7 @@
         <v>27</v>
       </c>
       <c r="H65" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I65" t="s">
         <v>777</v>
@@ -15473,7 +15477,7 @@
         <v>804</v>
       </c>
       <c r="N67" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O67" t="s">
         <v>805</v>
@@ -15539,7 +15543,7 @@
         <v>813</v>
       </c>
       <c r="N68" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O68" t="s">
         <v>814</v>
@@ -15605,7 +15609,7 @@
         <v>826</v>
       </c>
       <c r="N69" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O69" t="s">
         <v>827</v>
@@ -15653,7 +15657,7 @@
         <v>27</v>
       </c>
       <c r="H70" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I70" t="s">
         <v>832</v>
@@ -15669,7 +15673,7 @@
         <v>835</v>
       </c>
       <c r="N70" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O70" t="s">
         <v>836</v>
@@ -15733,7 +15737,7 @@
         <v>846</v>
       </c>
       <c r="N71" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O71" t="s">
         <v>847</v>
@@ -15781,7 +15785,7 @@
         <v>27</v>
       </c>
       <c r="H72" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I72" t="s">
         <v>851</v>
@@ -15799,7 +15803,7 @@
         <v>855</v>
       </c>
       <c r="N72" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O72" t="s">
         <v>856</v>
@@ -15865,7 +15869,7 @@
         <v>868</v>
       </c>
       <c r="N73" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O73" t="s">
         <v>869</v>
@@ -15913,7 +15917,7 @@
         <v>27</v>
       </c>
       <c r="H74" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I74" t="s">
         <v>877</v>
@@ -15931,7 +15935,7 @@
         <v>881</v>
       </c>
       <c r="N74" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O74" t="s">
         <v>882</v>
@@ -15997,7 +16001,7 @@
         <v>894</v>
       </c>
       <c r="N75" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O75" t="s">
         <v>895</v>
@@ -16061,7 +16065,7 @@
         <v>907</v>
       </c>
       <c r="N76" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O76" t="s">
         <v>908</v>
@@ -16127,7 +16131,7 @@
         <v>920</v>
       </c>
       <c r="N77" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O77" t="s">
         <v>921</v>
@@ -16169,7 +16173,7 @@
         <v>27</v>
       </c>
       <c r="H78" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I78" t="s">
         <v>925</v>
@@ -16185,7 +16189,7 @@
         <v>928</v>
       </c>
       <c r="N78" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O78" t="s">
         <v>929</v>
@@ -16251,7 +16255,7 @@
         <v>940</v>
       </c>
       <c r="N79" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O79" t="s">
         <v>941</v>
@@ -16299,7 +16303,7 @@
         <v>27</v>
       </c>
       <c r="H80" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I80" t="s">
         <v>944</v>
@@ -16317,7 +16321,7 @@
         <v>948</v>
       </c>
       <c r="N80" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O80" t="s">
         <v>949</v>
@@ -16383,7 +16387,7 @@
         <v>958</v>
       </c>
       <c r="N81" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O81" t="s">
         <v>959</v>
@@ -16515,7 +16519,7 @@
         <v>983</v>
       </c>
       <c r="N83" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O83" t="s">
         <v>984</v>
@@ -16581,7 +16585,7 @@
         <v>995</v>
       </c>
       <c r="N84" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O84" t="s">
         <v>996</v>
@@ -16647,7 +16651,7 @@
         <v>1004</v>
       </c>
       <c r="N85" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O85" t="s">
         <v>1005</v>
@@ -16695,7 +16699,7 @@
         <v>27</v>
       </c>
       <c r="H86" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I86" t="s">
         <v>1011</v>
@@ -16713,7 +16717,7 @@
         <v>1015</v>
       </c>
       <c r="N86" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O86" t="s">
         <v>1016</v>
@@ -16779,7 +16783,7 @@
         <v>1027</v>
       </c>
       <c r="N87" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O87" t="s">
         <v>1028</v>
@@ -16827,7 +16831,7 @@
         <v>27</v>
       </c>
       <c r="H88" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I88" t="s">
         <v>1036</v>
@@ -16845,7 +16849,7 @@
         <v>1040</v>
       </c>
       <c r="N88" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O88" t="s">
         <v>1041</v>
@@ -16893,7 +16897,7 @@
         <v>27</v>
       </c>
       <c r="H89" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I89" t="s">
         <v>1049</v>
@@ -16911,7 +16915,7 @@
         <v>1053</v>
       </c>
       <c r="N89" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O89" t="s">
         <v>1054</v>
@@ -16977,7 +16981,7 @@
         <v>1065</v>
       </c>
       <c r="N90" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O90" t="s">
         <v>1066</v>
@@ -17025,7 +17029,7 @@
         <v>27</v>
       </c>
       <c r="H91" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I91" t="s">
         <v>1072</v>
@@ -17043,7 +17047,7 @@
         <v>1076</v>
       </c>
       <c r="N91" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O91" t="s">
         <v>1077</v>
@@ -17091,7 +17095,7 @@
         <v>27</v>
       </c>
       <c r="H92" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I92" t="s">
         <v>1081</v>
@@ -17109,7 +17113,7 @@
         <v>1085</v>
       </c>
       <c r="N92" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O92" t="s">
         <v>1086</v>
@@ -17175,7 +17179,7 @@
         <v>1095</v>
       </c>
       <c r="N93" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O93" t="s">
         <v>1096</v>
@@ -17211,7 +17215,7 @@
         <v>135</v>
       </c>
       <c r="D94" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E94" t="s">
         <v>270</v>
@@ -17241,7 +17245,7 @@
         <v>1107</v>
       </c>
       <c r="N94" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O94" t="s">
         <v>1108</v>
@@ -17277,7 +17281,7 @@
         <v>135</v>
       </c>
       <c r="D95" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E95" t="s">
         <v>270</v>
@@ -17307,7 +17311,7 @@
         <v>1118</v>
       </c>
       <c r="N95" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O95" t="s">
         <v>1119</v>
@@ -17355,7 +17359,7 @@
         <v>27</v>
       </c>
       <c r="H96" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I96" t="s">
         <v>1127</v>
@@ -17373,7 +17377,7 @@
         <v>1131</v>
       </c>
       <c r="N96" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O96" t="s">
         <v>1132</v>
@@ -17421,7 +17425,7 @@
         <v>27</v>
       </c>
       <c r="H97" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I97" t="s">
         <v>1138</v>
@@ -17439,7 +17443,7 @@
         <v>1142</v>
       </c>
       <c r="N97" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O97" t="s">
         <v>1143</v>
@@ -17505,7 +17509,7 @@
         <v>1153</v>
       </c>
       <c r="N98" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O98" t="s">
         <v>1154</v>
@@ -17553,7 +17557,7 @@
         <v>27</v>
       </c>
       <c r="H99" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I99" t="s">
         <v>1159</v>
@@ -17571,7 +17575,7 @@
         <v>1163</v>
       </c>
       <c r="N99" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O99" t="s">
         <v>1164</v>
@@ -17637,7 +17641,7 @@
         <v>1174</v>
       </c>
       <c r="N100" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O100" t="s">
         <v>1175</v>
@@ -17703,7 +17707,7 @@
         <v>1185</v>
       </c>
       <c r="N101" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O101" t="s">
         <v>1186</v>
@@ -17769,7 +17773,7 @@
         <v>1194</v>
       </c>
       <c r="N102" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O102" t="s">
         <v>1195</v>
@@ -17899,7 +17903,7 @@
         <v>1211</v>
       </c>
       <c r="N104" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O104" t="s">
         <v>1212</v>
@@ -17963,7 +17967,7 @@
         <v>1221</v>
       </c>
       <c r="N105" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O105" t="s">
         <v>1222</v>
@@ -18029,7 +18033,7 @@
         <v>1234</v>
       </c>
       <c r="N106" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O106" t="s">
         <v>1235</v>
@@ -18077,7 +18081,7 @@
         <v>27</v>
       </c>
       <c r="H107" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I107" t="s">
         <v>1241</v>
@@ -18095,7 +18099,7 @@
         <v>1245</v>
       </c>
       <c r="N107" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O107" t="s">
         <v>1246</v>
@@ -18161,7 +18165,7 @@
         <v>1255</v>
       </c>
       <c r="N108" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O108" t="s">
         <v>1256</v>
@@ -18209,7 +18213,7 @@
         <v>27</v>
       </c>
       <c r="H109" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I109" t="s">
         <v>1260</v>
@@ -18227,7 +18231,7 @@
         <v>1264</v>
       </c>
       <c r="N109" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O109" t="s">
         <v>1265</v>
@@ -18275,7 +18279,7 @@
         <v>27</v>
       </c>
       <c r="H110" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I110" t="s">
         <v>1273</v>
@@ -18357,7 +18361,7 @@
         <v>1289</v>
       </c>
       <c r="N111" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O111" t="s">
         <v>1290</v>
@@ -18421,7 +18425,7 @@
         <v>1298</v>
       </c>
       <c r="N112" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O112" t="s">
         <v>1299</v>
@@ -18485,7 +18489,7 @@
         <v>1310</v>
       </c>
       <c r="N113" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O113" t="s">
         <v>1311</v>
@@ -18533,7 +18537,7 @@
         <v>27</v>
       </c>
       <c r="H114" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I114" t="s">
         <v>1316</v>
@@ -18551,7 +18555,7 @@
         <v>1320</v>
       </c>
       <c r="N114" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O114" t="s">
         <v>1321</v>
@@ -18617,7 +18621,7 @@
         <v>1332</v>
       </c>
       <c r="N115" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O115" t="s">
         <v>1333</v>
@@ -18681,7 +18685,7 @@
         <v>1345</v>
       </c>
       <c r="N116" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O116" t="s">
         <v>1346</v>
@@ -18729,7 +18733,7 @@
         <v>27</v>
       </c>
       <c r="H117" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I117" t="s">
         <v>1353</v>
@@ -18745,7 +18749,7 @@
         <v>1356</v>
       </c>
       <c r="N117" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O117" t="s">
         <v>1357</v>
@@ -18811,7 +18815,7 @@
         <v>1369</v>
       </c>
       <c r="N118" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O118" t="s">
         <v>1370</v>
@@ -18877,7 +18881,7 @@
         <v>1382</v>
       </c>
       <c r="N119" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O119" t="s">
         <v>1383</v>
@@ -18925,7 +18929,7 @@
         <v>27</v>
       </c>
       <c r="H120" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I120" t="s">
         <v>1391</v>
@@ -18941,7 +18945,7 @@
         <v>1394</v>
       </c>
       <c r="N120" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O120" t="s">
         <v>1395</v>
@@ -19007,7 +19011,7 @@
         <v>1407</v>
       </c>
       <c r="N121" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O121" t="s">
         <v>1408</v>
@@ -19073,7 +19077,7 @@
         <v>1420</v>
       </c>
       <c r="N122" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O122" t="s">
         <v>1421</v>
@@ -19139,7 +19143,7 @@
         <v>1431</v>
       </c>
       <c r="N123" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O123" t="s">
         <v>1432</v>
@@ -19205,7 +19209,7 @@
         <v>1440</v>
       </c>
       <c r="N124" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O124" t="s">
         <v>1441</v>
@@ -19271,7 +19275,7 @@
         <v>1453</v>
       </c>
       <c r="N125" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O125" t="s">
         <v>1454</v>
@@ -19319,7 +19323,7 @@
         <v>27</v>
       </c>
       <c r="H126" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I126" t="s">
         <v>1461</v>
@@ -19335,7 +19339,7 @@
         <v>1464</v>
       </c>
       <c r="N126" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O126" t="s">
         <v>1465</v>
@@ -19383,7 +19387,7 @@
         <v>27</v>
       </c>
       <c r="H127" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I127" t="s">
         <v>1473</v>
@@ -19399,7 +19403,7 @@
         <v>1476</v>
       </c>
       <c r="N127" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O127" t="s">
         <v>1477</v>
@@ -19529,7 +19533,7 @@
         <v>1495</v>
       </c>
       <c r="N129" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O129" t="s">
         <v>1496</v>
@@ -19577,7 +19581,7 @@
         <v>27</v>
       </c>
       <c r="H130" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I130" t="s">
         <v>1503</v>
@@ -19595,7 +19599,7 @@
         <v>1507</v>
       </c>
       <c r="N130" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O130" t="s">
         <v>1508</v>
@@ -19643,7 +19647,7 @@
         <v>27</v>
       </c>
       <c r="H131" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I131" t="s">
         <v>1514</v>
@@ -19661,7 +19665,7 @@
         <v>1518</v>
       </c>
       <c r="N131" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O131" t="s">
         <v>1519</v>
@@ -19727,7 +19731,7 @@
         <v>1530</v>
       </c>
       <c r="N132" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O132" t="s">
         <v>1531</v>
@@ -19775,7 +19779,7 @@
         <v>164</v>
       </c>
       <c r="H133" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I133" t="s">
         <v>1539</v>
@@ -19841,7 +19845,7 @@
         <v>27</v>
       </c>
       <c r="H134" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I134" t="s">
         <v>1551</v>
@@ -19859,7 +19863,7 @@
         <v>1555</v>
       </c>
       <c r="N134" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O134" t="s">
         <v>1556</v>
@@ -19925,7 +19929,7 @@
         <v>1567</v>
       </c>
       <c r="N135" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O135" t="s">
         <v>1568</v>
@@ -19991,7 +19995,7 @@
         <v>1576</v>
       </c>
       <c r="N136" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O136" t="s">
         <v>1577</v>
@@ -20055,7 +20059,7 @@
         <v>1585</v>
       </c>
       <c r="N137" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O137" t="s">
         <v>1586</v>
@@ -20119,7 +20123,7 @@
         <v>1592</v>
       </c>
       <c r="N138" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O138" t="s">
         <v>1593</v>
@@ -20185,7 +20189,7 @@
         <v>1601</v>
       </c>
       <c r="N139" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O139" t="s">
         <v>1602</v>
@@ -20251,7 +20255,7 @@
         <v>1613</v>
       </c>
       <c r="N140" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O140" t="s">
         <v>1614</v>
@@ -20317,7 +20321,7 @@
         <v>1624</v>
       </c>
       <c r="N141" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O141" t="s">
         <v>1625</v>
@@ -20383,7 +20387,7 @@
         <v>1636</v>
       </c>
       <c r="N142" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O142" t="s">
         <v>1637</v>
@@ -20449,7 +20453,7 @@
         <v>1645</v>
       </c>
       <c r="N143" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O143" t="s">
         <v>1646</v>
@@ -20515,7 +20519,7 @@
         <v>1657</v>
       </c>
       <c r="N144" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O144" t="s">
         <v>1658</v>
@@ -20581,7 +20585,7 @@
         <v>1669</v>
       </c>
       <c r="N145" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O145" t="s">
         <v>1670</v>
@@ -20647,7 +20651,7 @@
         <v>1678</v>
       </c>
       <c r="N146" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O146" t="s">
         <v>1679</v>
@@ -20711,7 +20715,7 @@
         <v>1690</v>
       </c>
       <c r="N147" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O147" t="s">
         <v>1691</v>
@@ -20775,7 +20779,7 @@
         <v>1701</v>
       </c>
       <c r="N148" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O148" t="s">
         <v>1702</v>
@@ -20839,7 +20843,7 @@
         <v>1708</v>
       </c>
       <c r="N149" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O149" t="s">
         <v>1709</v>
@@ -20949,7 +20953,7 @@
         <v>27</v>
       </c>
       <c r="H151" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I151" t="s">
         <v>1724</v>
@@ -20967,7 +20971,7 @@
         <v>1728</v>
       </c>
       <c r="N151" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O151" t="s">
         <v>1729</v>
@@ -21033,7 +21037,7 @@
         <v>1740</v>
       </c>
       <c r="N152" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O152" t="s">
         <v>1741</v>
@@ -21099,7 +21103,7 @@
         <v>1752</v>
       </c>
       <c r="N153" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O153" t="s">
         <v>1753</v>
@@ -21165,7 +21169,7 @@
         <v>1765</v>
       </c>
       <c r="N154" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O154" t="s">
         <v>1766</v>
@@ -21229,7 +21233,7 @@
         <v>1774</v>
       </c>
       <c r="N155" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O155" t="s">
         <v>1775</v>
@@ -21295,7 +21299,7 @@
         <v>1787</v>
       </c>
       <c r="N156" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O156" t="s">
         <v>1788</v>
@@ -21361,7 +21365,7 @@
         <v>1799</v>
       </c>
       <c r="N157" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O157" t="s">
         <v>1800</v>
@@ -21427,7 +21431,7 @@
         <v>1811</v>
       </c>
       <c r="N158" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O158" t="s">
         <v>1812</v>
@@ -21493,7 +21497,7 @@
         <v>1823</v>
       </c>
       <c r="N159" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O159" t="s">
         <v>1824</v>
@@ -21541,7 +21545,7 @@
         <v>27</v>
       </c>
       <c r="H160" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I160" t="s">
         <v>1830</v>
@@ -21559,7 +21563,7 @@
         <v>1834</v>
       </c>
       <c r="N160" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O160" t="s">
         <v>1835</v>
@@ -21607,7 +21611,7 @@
         <v>27</v>
       </c>
       <c r="H161" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I161" t="s">
         <v>1841</v>
@@ -21625,7 +21629,7 @@
         <v>1845</v>
       </c>
       <c r="N161" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O161" t="s">
         <v>1846</v>
@@ -21691,7 +21695,7 @@
         <v>1854</v>
       </c>
       <c r="N162" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O162" t="s">
         <v>1855</v>
@@ -21757,7 +21761,7 @@
         <v>1864</v>
       </c>
       <c r="N163" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O163" t="s">
         <v>1865</v>
@@ -21805,7 +21809,7 @@
         <v>27</v>
       </c>
       <c r="H164" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I164" t="s">
         <v>1872</v>
@@ -21823,7 +21827,7 @@
         <v>1876</v>
       </c>
       <c r="N164" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O164" t="s">
         <v>1877</v>
@@ -21889,7 +21893,7 @@
         <v>1888</v>
       </c>
       <c r="N165" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O165" t="s">
         <v>1889</v>
@@ -21955,7 +21959,7 @@
         <v>1897</v>
       </c>
       <c r="N166" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O166" t="s">
         <v>1898</v>
@@ -22021,7 +22025,7 @@
         <v>1906</v>
       </c>
       <c r="N167" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O167" t="s">
         <v>1907</v>
@@ -22087,7 +22091,7 @@
         <v>1919</v>
       </c>
       <c r="N168" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O168" t="s">
         <v>1920</v>
@@ -22153,7 +22157,7 @@
         <v>1931</v>
       </c>
       <c r="N169" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O169" t="s">
         <v>1932</v>
@@ -22201,7 +22205,7 @@
         <v>27</v>
       </c>
       <c r="H170" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I170" t="s">
         <v>1939</v>
@@ -22219,7 +22223,7 @@
         <v>1943</v>
       </c>
       <c r="N170" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O170" t="s">
         <v>1944</v>
@@ -22267,7 +22271,7 @@
         <v>27</v>
       </c>
       <c r="H171" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I171" t="s">
         <v>1951</v>
@@ -22285,7 +22289,7 @@
         <v>1955</v>
       </c>
       <c r="N171" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O171" t="s">
         <v>1956</v>
@@ -22351,7 +22355,7 @@
         <v>1967</v>
       </c>
       <c r="N172" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O172" t="s">
         <v>1968</v>
@@ -22399,7 +22403,7 @@
         <v>27</v>
       </c>
       <c r="H173" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I173" t="s">
         <v>1973</v>
@@ -22417,7 +22421,7 @@
         <v>1977</v>
       </c>
       <c r="N173" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O173" t="s">
         <v>1978</v>
@@ -22481,7 +22485,7 @@
         <v>1985</v>
       </c>
       <c r="N174" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O174" t="s">
         <v>1986</v>
@@ -22545,7 +22549,7 @@
         <v>1996</v>
       </c>
       <c r="N175" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O175" t="s">
         <v>1997</v>
@@ -22611,7 +22615,7 @@
         <v>2008</v>
       </c>
       <c r="N176" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O176" t="s">
         <v>2009</v>
@@ -22659,7 +22663,7 @@
         <v>27</v>
       </c>
       <c r="H177" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I177" t="s">
         <v>2016</v>
@@ -22677,7 +22681,7 @@
         <v>2020</v>
       </c>
       <c r="N177" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O177" t="s">
         <v>2021</v>
@@ -22725,7 +22729,7 @@
         <v>27</v>
       </c>
       <c r="H178" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I178" t="s">
         <v>2030</v>
@@ -22743,7 +22747,7 @@
         <v>2034</v>
       </c>
       <c r="N178" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O178" t="s">
         <v>2035</v>
@@ -22809,7 +22813,7 @@
         <v>2045</v>
       </c>
       <c r="N179" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O179" t="s">
         <v>2046</v>
@@ -22875,7 +22879,7 @@
         <v>2058</v>
       </c>
       <c r="N180" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O180" t="s">
         <v>2059</v>
@@ -22923,7 +22927,7 @@
         <v>27</v>
       </c>
       <c r="H181" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I181" t="s">
         <v>2067</v>
@@ -22939,7 +22943,7 @@
         <v>2070</v>
       </c>
       <c r="N181" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O181" t="s">
         <v>2071</v>
@@ -22987,7 +22991,7 @@
         <v>27</v>
       </c>
       <c r="H182" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I182" t="s">
         <v>2078</v>
@@ -23005,7 +23009,7 @@
         <v>2082</v>
       </c>
       <c r="N182" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O182" t="s">
         <v>2083</v>
@@ -23071,7 +23075,7 @@
         <v>2094</v>
       </c>
       <c r="N183" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O183" t="s">
         <v>2095</v>
@@ -23135,7 +23139,7 @@
         <v>2103</v>
       </c>
       <c r="N184" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O184" t="s">
         <v>2104</v>
@@ -23183,7 +23187,7 @@
         <v>27</v>
       </c>
       <c r="H185" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I185" t="s">
         <v>2112</v>
@@ -23201,7 +23205,7 @@
         <v>2116</v>
       </c>
       <c r="N185" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O185" t="s">
         <v>2117</v>
@@ -23249,7 +23253,7 @@
         <v>27</v>
       </c>
       <c r="H186" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I186" t="s">
         <v>2125</v>
@@ -23267,7 +23271,7 @@
         <v>2129</v>
       </c>
       <c r="N186" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O186" t="s">
         <v>2130</v>
@@ -23315,7 +23319,7 @@
         <v>27</v>
       </c>
       <c r="H187" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I187" t="s">
         <v>2137</v>
@@ -23331,7 +23335,7 @@
         <v>2140</v>
       </c>
       <c r="N187" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O187" t="s">
         <v>2141</v>
@@ -23379,7 +23383,7 @@
         <v>27</v>
       </c>
       <c r="H188" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I188" t="s">
         <v>2148</v>
@@ -23397,7 +23401,7 @@
         <v>2152</v>
       </c>
       <c r="N188" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O188" t="s">
         <v>2153</v>
@@ -23461,7 +23465,7 @@
         <v>2165</v>
       </c>
       <c r="N189" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O189" t="s">
         <v>2166</v>
@@ -23525,7 +23529,7 @@
         <v>2178</v>
       </c>
       <c r="N190" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O190" t="s">
         <v>2179</v>
@@ -23571,7 +23575,7 @@
         <v>164</v>
       </c>
       <c r="H191" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I191" t="s">
         <v>2185</v>
@@ -23589,7 +23593,7 @@
         <v>2189</v>
       </c>
       <c r="N191" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O191" t="s">
         <v>2190</v>
@@ -23829,7 +23833,7 @@
         <v>27</v>
       </c>
       <c r="H195" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I195" t="s">
         <v>2230</v>
@@ -23884,7 +23888,7 @@
         <v>373</v>
       </c>
       <c r="E196" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F196" t="s">
         <v>89</v>
@@ -23893,7 +23897,7 @@
         <v>27</v>
       </c>
       <c r="H196" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I196" t="s">
         <v>2241</v>
@@ -23948,7 +23952,7 @@
         <v>2252</v>
       </c>
       <c r="E197" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F197" t="s">
         <v>89</v>
@@ -24012,7 +24016,7 @@
         <v>808</v>
       </c>
       <c r="E198" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F198" t="s">
         <v>89</v>
@@ -24101,7 +24105,7 @@
         <v>2278</v>
       </c>
       <c r="N199" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O199" t="s">
         <v>2279</v>
@@ -24163,7 +24167,7 @@
         <v>2285</v>
       </c>
       <c r="N200" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O200" t="s">
         <v>2286</v>
@@ -24227,7 +24231,7 @@
         <v>2297</v>
       </c>
       <c r="N201" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O201" t="s">
         <v>2298</v>
@@ -24264,7 +24268,7 @@
         <v>2301</v>
       </c>
       <c r="E202" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F202" t="s">
         <v>2302</v>
@@ -24273,7 +24277,7 @@
         <v>27</v>
       </c>
       <c r="H202" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I202" t="s">
         <v>2303</v>
@@ -24337,7 +24341,7 @@
         <v>27</v>
       </c>
       <c r="H203" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I203" t="s">
         <v>2311</v>
@@ -24419,7 +24423,7 @@
         <v>2328</v>
       </c>
       <c r="N204" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O204" t="s">
         <v>2329</v>
@@ -24584,7 +24588,7 @@
         <v>2352</v>
       </c>
       <c r="E207" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F207" t="s">
         <v>2323</v>
@@ -24611,7 +24615,7 @@
         <v>2357</v>
       </c>
       <c r="N207" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O207" t="s">
         <v>2358</v>
@@ -24675,7 +24679,7 @@
         <v>2370</v>
       </c>
       <c r="N208" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O208" t="s">
         <v>2371</v>
@@ -24712,7 +24716,7 @@
         <v>442</v>
       </c>
       <c r="E209" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F209" t="s">
         <v>2377</v>
@@ -24801,7 +24805,7 @@
         <v>2389</v>
       </c>
       <c r="N210" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O210" t="s">
         <v>2390</v>
@@ -24863,7 +24867,7 @@
         <v>2396</v>
       </c>
       <c r="N211" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O211" t="s">
         <v>2397</v>
@@ -24909,7 +24913,7 @@
         <v>27</v>
       </c>
       <c r="H212" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I212" t="s">
         <v>2403</v>
@@ -24925,7 +24929,7 @@
         <v>2406</v>
       </c>
       <c r="N212" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O212" t="s">
         <v>2407</v>
@@ -25111,7 +25115,7 @@
         <v>2433</v>
       </c>
       <c r="N215" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O215" t="s">
         <v>2434</v>
@@ -25148,7 +25152,7 @@
         <v>2440</v>
       </c>
       <c r="E216" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F216" t="s">
         <v>2424</v>
@@ -25173,7 +25177,7 @@
         <v>2444</v>
       </c>
       <c r="N216" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O216" t="s">
         <v>2445</v>
@@ -25219,7 +25223,7 @@
         <v>164</v>
       </c>
       <c r="H217" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I217" t="s">
         <v>2450</v>
@@ -25237,7 +25241,7 @@
         <v>2454</v>
       </c>
       <c r="N217" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O217" t="s">
         <v>2455</v>
@@ -25299,7 +25303,7 @@
         <v>2462</v>
       </c>
       <c r="N218" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O218" t="s">
         <v>2463</v>
@@ -25419,7 +25423,7 @@
         <v>2482</v>
       </c>
       <c r="N220" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O220" t="s">
         <v>2483</v>
@@ -25483,7 +25487,7 @@
         <v>2494</v>
       </c>
       <c r="N221" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O221" t="s">
         <v>2495</v>
@@ -25529,7 +25533,7 @@
         <v>27</v>
       </c>
       <c r="H222" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I222" t="s">
         <v>2503</v>
@@ -25547,7 +25551,7 @@
         <v>2507</v>
       </c>
       <c r="N222" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O222" t="s">
         <v>2508</v>
@@ -25609,7 +25613,7 @@
         <v>2518</v>
       </c>
       <c r="N223" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O223" t="s">
         <v>2519</v>
@@ -25655,7 +25659,7 @@
         <v>27</v>
       </c>
       <c r="H224" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I224" t="s">
         <v>2524</v>
@@ -25673,7 +25677,7 @@
         <v>2528</v>
       </c>
       <c r="N224" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O224" t="s">
         <v>2529</v>
@@ -25737,7 +25741,7 @@
         <v>2539</v>
       </c>
       <c r="N225" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O225" t="s">
         <v>2540</v>
@@ -25801,7 +25805,7 @@
         <v>2548</v>
       </c>
       <c r="N226" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O226" t="s">
         <v>2549</v>
@@ -25865,7 +25869,7 @@
         <v>2560</v>
       </c>
       <c r="N227" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O227" t="s">
         <v>2561</v>
@@ -25929,7 +25933,7 @@
         <v>2569</v>
       </c>
       <c r="N228" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O228" t="s">
         <v>2570</v>
@@ -25975,7 +25979,7 @@
         <v>27</v>
       </c>
       <c r="H229" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I229" t="s">
         <v>2574</v>
@@ -25993,7 +25997,7 @@
         <v>2578</v>
       </c>
       <c r="N229" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O229" t="s">
         <v>2579</v>
@@ -26057,7 +26061,7 @@
         <v>2590</v>
       </c>
       <c r="N230" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O230" t="s">
         <v>2591</v>
@@ -26103,7 +26107,7 @@
         <v>27</v>
       </c>
       <c r="H231" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I231" t="s">
         <v>2595</v>
@@ -26121,7 +26125,7 @@
         <v>2599</v>
       </c>
       <c r="N231" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O231" t="s">
         <v>2600</v>
@@ -26185,7 +26189,7 @@
         <v>2612</v>
       </c>
       <c r="N232" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O232" t="s">
         <v>2613</v>
@@ -26247,7 +26251,7 @@
         <v>2623</v>
       </c>
       <c r="N233" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O233" t="s">
         <v>2624</v>
@@ -26311,7 +26315,7 @@
         <v>2635</v>
       </c>
       <c r="N234" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O234" t="s">
         <v>2636</v>
@@ -26375,7 +26379,7 @@
         <v>2648</v>
       </c>
       <c r="N235" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O235" t="s">
         <v>2649</v>
@@ -26439,7 +26443,7 @@
         <v>2659</v>
       </c>
       <c r="N236" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O236" t="s">
         <v>2660</v>
@@ -26485,7 +26489,7 @@
         <v>27</v>
       </c>
       <c r="H237" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I237" t="s">
         <v>2666</v>
@@ -26503,7 +26507,7 @@
         <v>2670</v>
       </c>
       <c r="N237" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O237" t="s">
         <v>2671</v>
@@ -26567,7 +26571,7 @@
         <v>2682</v>
       </c>
       <c r="N238" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O238" t="s">
         <v>2683</v>
@@ -26631,7 +26635,7 @@
         <v>2694</v>
       </c>
       <c r="N239" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O239" t="s">
         <v>2695</v>
@@ -26695,7 +26699,7 @@
         <v>2707</v>
       </c>
       <c r="N240" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O240" t="s">
         <v>2708</v>
@@ -26759,7 +26763,7 @@
         <v>2721</v>
       </c>
       <c r="N241" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O241" t="s">
         <v>2722</v>
@@ -26805,7 +26809,7 @@
         <v>27</v>
       </c>
       <c r="H242" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I242" t="s">
         <v>2727</v>
@@ -26821,7 +26825,7 @@
         <v>2730</v>
       </c>
       <c r="N242" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O242" t="s">
         <v>2731</v>
@@ -26867,7 +26871,7 @@
         <v>27</v>
       </c>
       <c r="H243" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I243" t="s">
         <v>2734</v>
@@ -26883,7 +26887,7 @@
         <v>2737</v>
       </c>
       <c r="N243" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O243" t="s">
         <v>2738</v>
@@ -26929,7 +26933,7 @@
         <v>27</v>
       </c>
       <c r="H244" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I244" t="s">
         <v>2743</v>
@@ -26947,7 +26951,7 @@
         <v>2747</v>
       </c>
       <c r="N244" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O244" t="s">
         <v>2748</v>
@@ -26993,7 +26997,7 @@
         <v>27</v>
       </c>
       <c r="H245" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I245" t="s">
         <v>2753</v>
@@ -27011,7 +27015,7 @@
         <v>2757</v>
       </c>
       <c r="N245" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O245" t="s">
         <v>2758</v>
@@ -27075,7 +27079,7 @@
         <v>2765</v>
       </c>
       <c r="N246" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O246" t="s">
         <v>2766</v>
@@ -27121,7 +27125,7 @@
         <v>27</v>
       </c>
       <c r="H247" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I247" t="s">
         <v>2773</v>
@@ -27137,7 +27141,7 @@
         <v>2776</v>
       </c>
       <c r="N247" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O247" t="s">
         <v>2777</v>
@@ -27199,7 +27203,7 @@
         <v>2784</v>
       </c>
       <c r="N248" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O248" t="s">
         <v>2785</v>
@@ -27261,7 +27265,7 @@
         <v>2794</v>
       </c>
       <c r="N249" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O249" t="s">
         <v>2795</v>
@@ -27305,7 +27309,7 @@
         <v>27</v>
       </c>
       <c r="H250" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I250" t="s">
         <v>2799</v>
@@ -27323,7 +27327,7 @@
         <v>2803</v>
       </c>
       <c r="N250" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O250" t="s">
         <v>2804</v>
@@ -27385,7 +27389,7 @@
         <v>2816</v>
       </c>
       <c r="N251" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O251" t="s">
         <v>2817</v>
@@ -27431,7 +27435,7 @@
         <v>164</v>
       </c>
       <c r="H252" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I252" t="s">
         <v>2825</v>
@@ -27449,7 +27453,7 @@
         <v>2829</v>
       </c>
       <c r="N252" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O252" t="s">
         <v>2830</v>
@@ -27513,7 +27517,7 @@
         <v>2838</v>
       </c>
       <c r="N253" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O253" t="s">
         <v>2839</v>
@@ -27577,7 +27581,7 @@
         <v>2847</v>
       </c>
       <c r="N254" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O254" t="s">
         <v>2848</v>
@@ -27623,7 +27627,7 @@
         <v>27</v>
       </c>
       <c r="H255" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I255" t="s">
         <v>2854</v>
@@ -27641,7 +27645,7 @@
         <v>2858</v>
       </c>
       <c r="N255" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O255" t="s">
         <v>2859</v>
@@ -27687,7 +27691,7 @@
         <v>27</v>
       </c>
       <c r="H256" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I256" t="s">
         <v>2862</v>
@@ -27705,7 +27709,7 @@
         <v>2866</v>
       </c>
       <c r="N256" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O256" t="s">
         <v>2867</v>
@@ -27751,7 +27755,7 @@
         <v>27</v>
       </c>
       <c r="H257" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I257" t="s">
         <v>2871</v>
@@ -27769,7 +27773,7 @@
         <v>2875</v>
       </c>
       <c r="N257" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O257" t="s">
         <v>2876</v>
@@ -27833,7 +27837,7 @@
         <v>2888</v>
       </c>
       <c r="N258" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O258" t="s">
         <v>2889</v>
@@ -27897,7 +27901,7 @@
         <v>2899</v>
       </c>
       <c r="N259" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O259" t="s">
         <v>2900</v>
@@ -27943,7 +27947,7 @@
         <v>27</v>
       </c>
       <c r="H260" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I260" t="s">
         <v>2908</v>
@@ -27961,7 +27965,7 @@
         <v>2912</v>
       </c>
       <c r="N260" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O260" t="s">
         <v>2913</v>
@@ -28007,7 +28011,7 @@
         <v>27</v>
       </c>
       <c r="H261" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I261" t="s">
         <v>2920</v>
@@ -28025,7 +28029,7 @@
         <v>2924</v>
       </c>
       <c r="N261" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O261" t="s">
         <v>2925</v>
@@ -28071,7 +28075,7 @@
         <v>27</v>
       </c>
       <c r="H262" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I262" t="s">
         <v>2928</v>
@@ -28087,7 +28091,7 @@
         <v>2931</v>
       </c>
       <c r="N262" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O262" t="s">
         <v>2932</v>
@@ -28133,7 +28137,7 @@
         <v>27</v>
       </c>
       <c r="H263" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I263" t="s">
         <v>2939</v>
@@ -28151,7 +28155,7 @@
         <v>2943</v>
       </c>
       <c r="N263" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O263" t="s">
         <v>2944</v>
@@ -28195,7 +28199,7 @@
         <v>27</v>
       </c>
       <c r="H264" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I264" t="s">
         <v>2951</v>
@@ -28213,7 +28217,7 @@
         <v>2955</v>
       </c>
       <c r="N264" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O264" t="s">
         <v>2956</v>
@@ -28257,7 +28261,7 @@
         <v>27</v>
       </c>
       <c r="H265" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I265" t="s">
         <v>2960</v>
@@ -28275,7 +28279,7 @@
         <v>2964</v>
       </c>
       <c r="N265" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O265" t="s">
         <v>2965</v>
@@ -28319,7 +28323,7 @@
         <v>27</v>
       </c>
       <c r="H266" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I266" t="s">
         <v>2968</v>
@@ -28337,7 +28341,7 @@
         <v>2972</v>
       </c>
       <c r="N266" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O266" t="s">
         <v>2973</v>
@@ -28381,7 +28385,7 @@
         <v>27</v>
       </c>
       <c r="H267" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I267" t="s">
         <v>2976</v>
@@ -28399,7 +28403,7 @@
         <v>2980</v>
       </c>
       <c r="N267" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O267" t="s">
         <v>2981</v>
@@ -28443,7 +28447,7 @@
         <v>27</v>
       </c>
       <c r="H268" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I268" t="s">
         <v>2986</v>
@@ -28461,7 +28465,7 @@
         <v>2990</v>
       </c>
       <c r="N268" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O268" t="s">
         <v>2991</v>
@@ -28507,7 +28511,7 @@
         <v>27</v>
       </c>
       <c r="H269" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I269" t="s">
         <v>2999</v>
@@ -28525,7 +28529,7 @@
         <v>3003</v>
       </c>
       <c r="N269" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O269" t="s">
         <v>3004</v>
@@ -28589,7 +28593,7 @@
         <v>3013</v>
       </c>
       <c r="N270" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O270" t="s">
         <v>3014</v>
@@ -28651,7 +28655,7 @@
         <v>3024</v>
       </c>
       <c r="N271" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O271" t="s">
         <v>3025</v>
@@ -28697,7 +28701,7 @@
         <v>27</v>
       </c>
       <c r="H272" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I272" t="s">
         <v>3034</v>
@@ -28715,7 +28719,7 @@
         <v>3038</v>
       </c>
       <c r="N272" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O272" t="s">
         <v>3039</v>
@@ -28779,7 +28783,7 @@
         <v>3051</v>
       </c>
       <c r="N273" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O273" t="s">
         <v>3052</v>
@@ -28843,7 +28847,7 @@
         <v>3062</v>
       </c>
       <c r="N274" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O274" t="s">
         <v>3063</v>
@@ -28889,7 +28893,7 @@
         <v>27</v>
       </c>
       <c r="H275" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I275" t="s">
         <v>3066</v>
@@ -28907,7 +28911,7 @@
         <v>3070</v>
       </c>
       <c r="N275" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O275" t="s">
         <v>3071</v>
@@ -28971,7 +28975,7 @@
         <v>3081</v>
       </c>
       <c r="N276" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O276" t="s">
         <v>3082</v>
@@ -29017,7 +29021,7 @@
         <v>27</v>
       </c>
       <c r="H277" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I277" t="s">
         <v>3088</v>
@@ -29035,7 +29039,7 @@
         <v>3092</v>
       </c>
       <c r="N277" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O277" t="s">
         <v>3093</v>
@@ -29099,7 +29103,7 @@
         <v>3103</v>
       </c>
       <c r="N278" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O278" t="s">
         <v>3104</v>
@@ -29163,7 +29167,7 @@
         <v>3111</v>
       </c>
       <c r="N279" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O279" t="s">
         <v>3112</v>
@@ -29227,7 +29231,7 @@
         <v>3120</v>
       </c>
       <c r="N280" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O280" t="s">
         <v>3121</v>
@@ -29291,7 +29295,7 @@
         <v>3129</v>
       </c>
       <c r="N281" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O281" t="s">
         <v>3130</v>
@@ -29353,7 +29357,7 @@
         <v>3137</v>
       </c>
       <c r="N282" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O282" t="s">
         <v>3138</v>
@@ -29399,7 +29403,7 @@
         <v>27</v>
       </c>
       <c r="H283" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I283" t="s">
         <v>3145</v>
@@ -29415,7 +29419,7 @@
         <v>3148</v>
       </c>
       <c r="N283" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O283" t="s">
         <v>3149</v>
@@ -29479,7 +29483,7 @@
         <v>3157</v>
       </c>
       <c r="N284" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O284" t="s">
         <v>3158</v>
@@ -29523,7 +29527,7 @@
         <v>27</v>
       </c>
       <c r="H285" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I285" t="s">
         <v>3165</v>
@@ -29541,7 +29545,7 @@
         <v>3169</v>
       </c>
       <c r="N285" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O285" t="s">
         <v>3170</v>
@@ -29585,7 +29589,7 @@
         <v>27</v>
       </c>
       <c r="H286" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I286" t="s">
         <v>3173</v>
@@ -29603,7 +29607,7 @@
         <v>3177</v>
       </c>
       <c r="N286" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O286" t="s">
         <v>3178</v>
@@ -29647,7 +29651,7 @@
         <v>27</v>
       </c>
       <c r="H287" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I287" t="s">
         <v>3181</v>
@@ -29665,7 +29669,7 @@
         <v>3185</v>
       </c>
       <c r="N287" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O287" t="s">
         <v>3186</v>
@@ -29711,7 +29715,7 @@
         <v>27</v>
       </c>
       <c r="H288" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I288" t="s">
         <v>3189</v>
@@ -29729,7 +29733,7 @@
         <v>3193</v>
       </c>
       <c r="N288" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O288" t="s">
         <v>3194</v>
@@ -29773,7 +29777,7 @@
         <v>27</v>
       </c>
       <c r="H289" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I289" t="s">
         <v>3201</v>
@@ -29791,7 +29795,7 @@
         <v>3205</v>
       </c>
       <c r="N289" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O289" t="s">
         <v>3206</v>
@@ -29855,7 +29859,7 @@
         <v>3215</v>
       </c>
       <c r="N290" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O290" t="s">
         <v>3216</v>
@@ -29901,7 +29905,7 @@
         <v>27</v>
       </c>
       <c r="H291" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I291" t="s">
         <v>3222</v>
@@ -29917,7 +29921,7 @@
         <v>3225</v>
       </c>
       <c r="N291" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O291" t="s">
         <v>3226</v>
@@ -29963,7 +29967,7 @@
         <v>27</v>
       </c>
       <c r="H292" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I292" t="s">
         <v>3231</v>
@@ -29981,7 +29985,7 @@
         <v>3235</v>
       </c>
       <c r="N292" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O292" t="s">
         <v>3236</v>
@@ -30045,7 +30049,7 @@
         <v>3244</v>
       </c>
       <c r="N293" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O293" t="s">
         <v>3245</v>
@@ -30091,7 +30095,7 @@
         <v>27</v>
       </c>
       <c r="H294" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I294" t="s">
         <v>3250</v>
@@ -30109,7 +30113,7 @@
         <v>3254</v>
       </c>
       <c r="N294" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O294" t="s">
         <v>3255</v>
@@ -30173,7 +30177,7 @@
         <v>3265</v>
       </c>
       <c r="N295" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O295" t="s">
         <v>3266</v>
@@ -30237,7 +30241,7 @@
         <v>3277</v>
       </c>
       <c r="N296" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O296" t="s">
         <v>3278</v>
@@ -30299,7 +30303,7 @@
         <v>3286</v>
       </c>
       <c r="N297" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O297" t="s">
         <v>3287</v>
@@ -30361,7 +30365,7 @@
         <v>3298</v>
       </c>
       <c r="N298" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O298" t="s">
         <v>3299</v>
@@ -30425,7 +30429,7 @@
         <v>3310</v>
       </c>
       <c r="N299" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O299" t="s">
         <v>3311</v>
@@ -30489,7 +30493,7 @@
         <v>3319</v>
       </c>
       <c r="N300" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O300" t="s">
         <v>3320</v>
@@ -30553,7 +30557,7 @@
         <v>3329</v>
       </c>
       <c r="N301" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O301" t="s">
         <v>3330</v>
@@ -30599,7 +30603,7 @@
         <v>27</v>
       </c>
       <c r="H302" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I302" t="s">
         <v>3338</v>
@@ -30617,7 +30621,7 @@
         <v>3342</v>
       </c>
       <c r="N302" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O302" t="s">
         <v>3343</v>
@@ -30663,7 +30667,7 @@
         <v>27</v>
       </c>
       <c r="H303" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I303" t="s">
         <v>3350</v>
@@ -30681,7 +30685,7 @@
         <v>3354</v>
       </c>
       <c r="N303" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O303" t="s">
         <v>3355</v>
@@ -30745,7 +30749,7 @@
         <v>3366</v>
       </c>
       <c r="N304" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O304" t="s">
         <v>3367</v>
@@ -30809,7 +30813,7 @@
         <v>3375</v>
       </c>
       <c r="N305" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O305" t="s">
         <v>3376</v>
@@ -30873,7 +30877,7 @@
         <v>3384</v>
       </c>
       <c r="N306" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O306" t="s">
         <v>3385</v>
@@ -30937,7 +30941,7 @@
         <v>3396</v>
       </c>
       <c r="N307" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O307" t="s">
         <v>3397</v>
@@ -30999,7 +31003,7 @@
         <v>3404</v>
       </c>
       <c r="N308" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O308" t="s">
         <v>3405</v>
@@ -31061,7 +31065,7 @@
         <v>3412</v>
       </c>
       <c r="N309" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O309" t="s">
         <v>3413</v>
@@ -31125,7 +31129,7 @@
         <v>3421</v>
       </c>
       <c r="N310" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O310" t="s">
         <v>3422</v>
@@ -31189,7 +31193,7 @@
         <v>3434</v>
       </c>
       <c r="N311" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O311" t="s">
         <v>3435</v>
@@ -31235,7 +31239,7 @@
         <v>27</v>
       </c>
       <c r="H312" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I312" t="s">
         <v>3443</v>
@@ -31253,7 +31257,7 @@
         <v>3447</v>
       </c>
       <c r="N312" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O312" t="s">
         <v>3448</v>
@@ -31317,7 +31321,7 @@
         <v>3457</v>
       </c>
       <c r="N313" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O313" t="s">
         <v>3458</v>
@@ -31381,7 +31385,7 @@
         <v>3466</v>
       </c>
       <c r="N314" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O314" t="s">
         <v>3467</v>
@@ -31445,7 +31449,7 @@
         <v>3475</v>
       </c>
       <c r="N315" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O315" t="s">
         <v>3476</v>
@@ -31491,7 +31495,7 @@
         <v>164</v>
       </c>
       <c r="H316" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I316" t="s">
         <v>3482</v>
@@ -31509,7 +31513,7 @@
         <v>3486</v>
       </c>
       <c r="N316" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O316" t="s">
         <v>3487</v>
@@ -31573,7 +31577,7 @@
         <v>3497</v>
       </c>
       <c r="N317" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O317" t="s">
         <v>3498</v>
@@ -31637,7 +31641,7 @@
         <v>3509</v>
       </c>
       <c r="N318" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O318" t="s">
         <v>3510</v>
@@ -31701,7 +31705,7 @@
         <v>3519</v>
       </c>
       <c r="N319" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O319" t="s">
         <v>3520</v>
@@ -31765,7 +31769,7 @@
         <v>3528</v>
       </c>
       <c r="N320" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O320" t="s">
         <v>3529</v>
@@ -31829,7 +31833,7 @@
         <v>3537</v>
       </c>
       <c r="N321" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O321" t="s">
         <v>3538</v>
@@ -31875,7 +31879,7 @@
         <v>27</v>
       </c>
       <c r="H322" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I322" t="s">
         <v>3542</v>
@@ -31893,7 +31897,7 @@
         <v>3546</v>
       </c>
       <c r="N322" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O322" t="s">
         <v>3547</v>
@@ -31957,7 +31961,7 @@
         <v>3557</v>
       </c>
       <c r="N323" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O323" t="s">
         <v>3558</v>
@@ -32021,7 +32025,7 @@
         <v>3565</v>
       </c>
       <c r="N324" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O324" t="s">
         <v>3566</v>
@@ -32085,7 +32089,7 @@
         <v>3574</v>
       </c>
       <c r="N325" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O325" t="s">
         <v>3575</v>

</xml_diff>

<commit_message>
Update parliament data - 2026-03-17
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_CDF_EFK.xlsx
+++ b/Objets_parlementaires_CDF_EFK.xlsx
@@ -11233,9 +11233,7 @@
       <c r="R2" t="s">
         <v>37</v>
       </c>
-      <c r="S2" t="s">
-        <v>37</v>
-      </c>
+      <c r="S2"/>
       <c r="T2" t="s">
         <v>38</v>
       </c>
@@ -11299,9 +11297,7 @@
       <c r="R3" t="s">
         <v>37</v>
       </c>
-      <c r="S3" t="s">
-        <v>37</v>
-      </c>
+      <c r="S3"/>
       <c r="T3" t="s">
         <v>52</v>
       </c>

</xml_diff>

<commit_message>
Update parliament data - 2026-04-08
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_CDF_EFK.xlsx
+++ b/Objets_parlementaires_CDF_EFK.xlsx
@@ -16724,9 +16724,7 @@
       <c r="D85" t="s">
         <v>1001</v>
       </c>
-      <c r="E85" t="s">
-        <v>44</v>
-      </c>
+      <c r="E85"/>
       <c r="F85" t="s">
         <v>1002</v>
       </c>

</xml_diff>

<commit_message>
Update parliament data - 2026-04-27
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_CDF_EFK.xlsx
+++ b/Objets_parlementaires_CDF_EFK.xlsx
@@ -155,7 +155,7 @@
     <t xml:space="preserve">Un audit externe de l'OFDF pour restaurer la confiance du personnel et de l'économie</t>
   </si>
   <si>
-    <t xml:space="preserve">Una verifica esterna dell’UDSC per ristabilire la fiducia tra il personale e il mondo economico</t>
+    <t xml:space="preserve">Una verifica esterna dell'UDSC per ristabilire la fiducia tra il personale e il mondo economico</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Le Conseil fédéral est chargé de commander, avant que des décisions irréversibles ne soient prises, un audit externe de l’OFDF et de la transformation en cours portant notamment sur les points suivants&amp;nbsp;:&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Adéquation des moyens (budget et personnel) aux multiples tâches de l’OFDF, en particulier pour la surveillance de la frontière terrestre, le contrôle de la migration ou encore la lutte contre les trafics en tous genres (produits agricoles, animaux, plantes envahissantes)&lt;/li&gt;&lt;li&gt;Efficacité de DaziT dans l’encaissement des droits de douanes (recettes en recul en 2025), avec en particulier la fin du contrôle systématique des camions étrangers, et face aux attentes de l’économie (en écho aux critiques très dures du transporteur Marco Tepoorten parlant d’une «&amp;nbsp;désorganisation systémique&amp;nbsp;»)&lt;/li&gt;&lt;li&gt;Flexibiliser Allegra&lt;/li&gt;&lt;li&gt;Taux d’arrêts maladie et de départs de l’OFDF&lt;/li&gt;&lt;li&gt;Attractivité du statut des personnels OFDF&lt;/li&gt;&lt;li&gt;Formation (qui semble enregistrer un taux d’échec inusuel)&lt;/li&gt;&lt;li&gt;Taux de rotation inhabituel parmi les cadres supérieurs de l’OFDF&lt;/li&gt;&lt;li&gt;Avant de continuer à foncer dans une direction discutable, n’y a-t-il pas lieu de tirer les leçons de transformations analogues à l’étranger (Autriche, Canada), surtout de certains échecs ?&lt;/li&gt;&lt;li&gt;Quelles mesures pour restaurer la confiance du personnel et de l'économie et garantir l'efficacité de l'OFDF dans l'exécution de ses tâches ?&lt;/li&gt;&lt;/ul&gt;</t>
@@ -194,10 +194,10 @@
     <t xml:space="preserve">Versucht das Pro-Komitee der SVP-Nachhaltigkeitsinitiative die Transparenzvorschriften zu umgehen?</t>
   </si>
   <si>
-    <t xml:space="preserve">Le comité en faveur de l’initiative de l’UDC pour la durabilité tente-t-il de contourner les règles de transparence ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Iniziativa per la sostenibilità dell’UDC: il comitato promotore tenta di eludere le disposizioni in materia di trasparenza?</t>
+    <t xml:space="preserve">Le comité en faveur de l'initiative de l'UDC pour la durabilité tente-t-il de contourner les règles de transparence ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Iniziativa per la sostenibilità dell'UDC: Il comitato promotore tenta di eludere le disposizioni in materia di trasparenza?</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;ol&gt;&lt;li&gt;Le Conseil fédéral ou le CDF ont-ils au courant des campagnes évoquées plus bas&amp;nbsp;? Lesquelles ont été portées à leur connaissance&amp;nbsp;?&lt;/li&gt;&lt;li&gt;Savent-ils qui est derrière ces campagnes&amp;nbsp;? D’après certains médias, il pourrait s’agir de l’entourage des cadres de l’UDC. Le Conseil fédéral ou le CDF ont-ils des informations à ce sujet&amp;nbsp;?&lt;/li&gt;&lt;li&gt;Le Conseil fédéral partage-t-il le soupçon qu’il s’agit d’une tentative de contourner les règles de transparence applicables aux campagnes de votation&amp;nbsp;? Estime-t-il aussi que les responsables de campagne utilisent une lacune manifeste de l’art.&amp;nbsp;8, al. 1, OFipo (inscription des communications) pour dissimuler l’origine des fonds destinés aux campagnes&amp;nbsp;? Compte-t-il combler cette lacune&amp;nbsp;?&lt;/li&gt;&lt;li&gt;Le Conseil fédéral ou le CDF ont-ils demandé à l’UDC de cesser ses manœuvres visant à dissimuler le financement de ses campagnes&amp;nbsp;?&lt;/li&gt;&lt;/ol&gt;</t>

</xml_diff>

<commit_message>
Update parliament data - 2026-05-06
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_CDF_EFK.xlsx
+++ b/Objets_parlementaires_CDF_EFK.xlsx
@@ -185,6 +185,57 @@
     <t xml:space="preserve">Scienza e ricerca|Ambiente|Salute</t>
   </si>
   <si>
+    <t xml:space="preserve">26.3398</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gredig Corina</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pvl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-03-20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EFD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Einführung eines öffentlichen Registers der Subventionsempfänger</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Créer un registre public des bénéficiaires de subventions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Introduzione di un registro pubblico dei beneficiari di sussidi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Le Conseil fédéral est chargé de créer un registre central public des bénéficiaires de subventions fédérales. Ce registre sera conçu pour compléter la banque de données sur les subventions et sa tenue sera confiée à la Confédération ou au Contrôle fédéral des finances. Il indiquera au minimum le nom du bénéficiaire ou son type, la nature et l’objet de la subvention, le montant annuel versé et l’office fédéral compétent et utilisera les données dont disposent les offices fédéraux.&amp;nbsp;&lt;br&gt;Les restrictions dictées par la protection des données et par la sécurité seront réservées.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Der Bundesrat wird beauftragt, ein öffentlich einsehbares, zentrales Register der &amp;nbsp;Empfängerinnen und Empfänger von Bundessubventionen einzuführen. Das Register soll als Ergänzung zur bestehenden Subventionsdatenbank ausgestaltet und durch Bund oder EFK geführt werden. Es hat mindestens den Namen oder Empfängertyp, Art und Zweck der Subvention, den jährlich ausbezahlten Betrag sowie das zuständige Bundesamt auszuweisen. Es soll bestehenden Daten der Bundesämter nutzen.&amp;nbsp;&lt;br&gt;Datenschutz- und sicherheitsrelevante Einschränkungen bleiben vorbehalten.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eingereicht / Déposé</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263398</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263398</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Staatspolitik|Finanzwesen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Politique d'Etat|Finances</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Politica nazionale|Finanze</t>
+  </si>
+  <si>
     <t xml:space="preserve">26.3485</t>
   </si>
   <si>
@@ -197,12 +248,6 @@
     <t xml:space="preserve">UDC</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-03-20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EFD</t>
-  </si>
-  <si>
     <t xml:space="preserve">Externes Audit des Bundesamts für Zoll und Grenzsicherheit zur Wiederherstellung des Vertrauens des Personals und der Wirtschaft</t>
   </si>
   <si>
@@ -218,9 +263,6 @@
     <t xml:space="preserve">&lt;p&gt;Bevor irreversible Entscheide getroffen werden, wird der Bundesrat beauftragt, ein externes Audit des Bundesamts für Zoll und Grenzsicherheit (BAZG) und dessen laufender Umstrukturierung in Auftrag zu geben, das insbesondere folgende Punkte umfasst:&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Angemessenheit der Mittel (Budget und Personal) für die vielfältigen Aufgaben des BAZG, insbesondere für die Überwachung der Landesgrenze, die Migrationskontrolle und die Bekämpfung von Schmuggel aller Art (landwirtschaftliche Produkte, Tiere, invasive Pflanzen);&lt;/li&gt;&lt;li&gt;Wirksamkeit des Programms Dazit bei der Zollerhebung (rückläufige Einnahmen&amp;nbsp;2025), insbesondere angesichts des Wegfalls der systematischen Kontrolle ausländischer Lastwagen und der Erwartungen der Wirtschaft (in Anlehnung an die sehr harte Kritik des Transportunternehmers Marco Tepoorten, der von einer «systemischen Desorganisation» sprach);&lt;/li&gt;&lt;li&gt;Flexibilisierung von Allegra;&lt;/li&gt;&lt;li&gt;Krankheitsabsenzen und Abgänge beim BAZG;&lt;/li&gt;&lt;li&gt;Attraktivität des BAZG-Personalstatus;&lt;/li&gt;&lt;li&gt;Ausbildung (mit offenbar ungewöhnlich hoher Durchfallquote);&lt;/li&gt;&lt;li&gt;untypische Fluktuationsrate bei den Führungskräften des BAZG;&lt;/li&gt;&lt;li&gt;Wäre es nicht angebracht, Lehren aus vergleichbaren Umstrukturierungen im Ausland (Österreich, Kanada) zu ziehen – insbesondere aus gewissen Misserfolgen –, bevor weiter in eine fragwürdige Richtung vorgeprescht wird?&lt;/li&gt;&lt;li&gt;Welche Massnahmen sind notwendig, um das Vertrauen des Personals und der Wirtschaft wiederherzustellen und die Wirksamkeit des BAZG bei der Aufgabenerfüllung zu gewährleisten?&lt;/li&gt;&lt;/ul&gt;</t>
   </si>
   <si>
-    <t xml:space="preserve">Eingereicht / Déposé</t>
-  </si>
-  <si>
     <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263485</t>
   </si>
   <si>
@@ -234,48 +276,6 @@
   </si>
   <si>
     <t xml:space="preserve">Politica nazionale|Finanze|Occupazione e lavoro</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26.3398</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mo.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gredig Corina</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pvl</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Einführung eines öffentlichen Registers der Subventionsempfänger</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Créer un registre public des bénéficiaires de subventions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Introduzione di un registro pubblico dei beneficiari di sussidi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Le Conseil fédéral est chargé de créer un registre central public des bénéficiaires de subventions fédérales. Ce registre sera conçu pour compléter la banque de données sur les subventions et sa tenue sera confiée à la Confédération ou au Contrôle fédéral des finances. Il indiquera au minimum le nom du bénéficiaire ou son type, la nature et l’objet de la subvention, le montant annuel versé et l’office fédéral compétent et utilisera les données dont disposent les offices fédéraux.&amp;nbsp;&lt;br&gt;Les restrictions dictées par la protection des données et par la sécurité seront réservées.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Der Bundesrat wird beauftragt, ein öffentlich einsehbares, zentrales Register der &amp;nbsp;Empfängerinnen und Empfänger von Bundessubventionen einzuführen. Das Register soll als Ergänzung zur bestehenden Subventionsdatenbank ausgestaltet und durch Bund oder EFK geführt werden. Es hat mindestens den Namen oder Empfängertyp, Art und Zweck der Subvention, den jährlich ausbezahlten Betrag sowie das zuständige Bundesamt auszuweisen. Es soll bestehenden Daten der Bundesämter nutzen.&amp;nbsp;&lt;br&gt;Datenschutz- und sicherheitsrelevante Einschränkungen bleiben vorbehalten.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263398</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263398</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Staatspolitik|Finanzwesen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Politique d'Etat|Finances</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Politica nazionale|Finanze</t>
   </si>
   <si>
     <t xml:space="preserve">26.3487</t>
@@ -11473,7 +11473,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>20263485</v>
+        <v>20263398</v>
       </c>
       <c r="B4" t="s">
         <v>57</v>
@@ -11539,7 +11539,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>20263398</v>
+        <v>20263485</v>
       </c>
       <c r="B5" t="s">
         <v>74</v>
@@ -11749,7 +11749,7 @@
         <v>120</v>
       </c>
       <c r="E8" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="F8" t="s">
         <v>121</v>
@@ -12007,7 +12007,7 @@
         <v>172</v>
       </c>
       <c r="C12" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D12" t="s">
         <v>173</v>
@@ -12269,7 +12269,7 @@
         <v>225</v>
       </c>
       <c r="E16" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F16" t="s">
         <v>226</v>
@@ -12312,13 +12312,13 @@
       </c>
       <c r="S16"/>
       <c r="T16" t="s">
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="U16" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="V16" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
     </row>
     <row r="17">
@@ -12335,7 +12335,7 @@
         <v>237</v>
       </c>
       <c r="E17" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F17" t="s">
         <v>238</v>
@@ -12395,7 +12395,7 @@
         <v>251</v>
       </c>
       <c r="C18" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D18" t="s">
         <v>252</v>
@@ -12527,7 +12527,7 @@
         <v>276</v>
       </c>
       <c r="C20" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D20" t="s">
         <v>277</v>
@@ -12599,7 +12599,7 @@
         <v>283</v>
       </c>
       <c r="E21" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F21" t="s">
         <v>238</v>
@@ -12725,7 +12725,7 @@
         <v>307</v>
       </c>
       <c r="C23" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D23" t="s">
         <v>133</v>
@@ -12791,7 +12791,7 @@
         <v>318</v>
       </c>
       <c r="C24" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D24" t="s">
         <v>319</v>
@@ -12923,7 +12923,7 @@
         <v>344</v>
       </c>
       <c r="C26" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D26" t="s">
         <v>345</v>
@@ -12995,7 +12995,7 @@
         <v>357</v>
       </c>
       <c r="E27" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F27" t="s">
         <v>358</v>
@@ -13059,7 +13059,7 @@
         <v>369</v>
       </c>
       <c r="E28" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F28" t="s">
         <v>358</v>
@@ -13185,7 +13185,7 @@
         <v>394</v>
       </c>
       <c r="C30" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D30" t="s">
         <v>395</v>
@@ -13251,7 +13251,7 @@
         <v>407</v>
       </c>
       <c r="C31" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D31" t="s">
         <v>43</v>
@@ -13383,7 +13383,7 @@
         <v>432</v>
       </c>
       <c r="C33" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D33" t="s">
         <v>433</v>
@@ -13449,13 +13449,13 @@
         <v>445</v>
       </c>
       <c r="C34" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D34" t="s">
         <v>446</v>
       </c>
       <c r="E34" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F34" t="s">
         <v>409</v>
@@ -13975,7 +13975,7 @@
         <v>539</v>
       </c>
       <c r="C42" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D42" t="s">
         <v>540</v>
@@ -14305,7 +14305,7 @@
         <v>597</v>
       </c>
       <c r="E47" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F47" t="s">
         <v>584</v>
@@ -14363,7 +14363,7 @@
         <v>607</v>
       </c>
       <c r="C48" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D48" t="s">
         <v>608</v>
@@ -14761,7 +14761,7 @@
         <v>446</v>
       </c>
       <c r="E54" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F54" t="s">
         <v>680</v>
@@ -14953,7 +14953,7 @@
         <v>709</v>
       </c>
       <c r="C57" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D57" t="s">
         <v>43</v>
@@ -15019,7 +15019,7 @@
         <v>720</v>
       </c>
       <c r="C58" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D58" t="s">
         <v>43</v>
@@ -15287,7 +15287,7 @@
         <v>446</v>
       </c>
       <c r="E62" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F62" t="s">
         <v>751</v>
@@ -15479,7 +15479,7 @@
         <v>794</v>
       </c>
       <c r="E65" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F65" t="s">
         <v>795</v>
@@ -15739,7 +15739,7 @@
         <v>830</v>
       </c>
       <c r="E69" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="F69" t="s">
         <v>821</v>
@@ -15799,13 +15799,13 @@
         <v>841</v>
       </c>
       <c r="C70" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D70" t="s">
         <v>830</v>
       </c>
       <c r="E70" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="F70" t="s">
         <v>821</v>
@@ -15997,7 +15997,7 @@
         <v>871</v>
       </c>
       <c r="C73" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D73" t="s">
         <v>872</v>
@@ -16061,7 +16061,7 @@
         <v>881</v>
       </c>
       <c r="C74" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D74" t="s">
         <v>882</v>
@@ -16128,10 +16128,10 @@
         <v>23</v>
       </c>
       <c r="D75" t="s">
-        <v>76</v>
+        <v>59</v>
       </c>
       <c r="E75" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="F75" t="s">
         <v>893</v>
@@ -16191,13 +16191,13 @@
         <v>904</v>
       </c>
       <c r="C76" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D76" t="s">
         <v>446</v>
       </c>
       <c r="E76" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F76" t="s">
         <v>905</v>
@@ -16323,13 +16323,13 @@
         <v>924</v>
       </c>
       <c r="C78" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D78" t="s">
         <v>925</v>
       </c>
       <c r="E78" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F78" t="s">
         <v>926</v>
@@ -16500,13 +16500,13 @@
       </c>
       <c r="S80"/>
       <c r="T80" t="s">
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="U80" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="V80" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
     </row>
     <row r="81">
@@ -16655,7 +16655,7 @@
         <v>980</v>
       </c>
       <c r="E83" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F83" t="s">
         <v>981</v>
@@ -16721,7 +16721,7 @@
         <v>993</v>
       </c>
       <c r="E84" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F84" t="s">
         <v>994</v>
@@ -16781,7 +16781,7 @@
         <v>1005</v>
       </c>
       <c r="C85" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D85" t="s">
         <v>1006</v>
@@ -16851,7 +16851,7 @@
         <v>1019</v>
       </c>
       <c r="E86" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F86" t="s">
         <v>1020</v>
@@ -16969,13 +16969,13 @@
         <v>1039</v>
       </c>
       <c r="C88" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D88" t="s">
         <v>597</v>
       </c>
       <c r="E88" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F88" t="s">
         <v>1040</v>
@@ -17167,7 +17167,7 @@
         <v>1069</v>
       </c>
       <c r="C91" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D91" t="s">
         <v>1070</v>
@@ -17233,13 +17233,13 @@
         <v>1082</v>
       </c>
       <c r="C92" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D92" t="s">
         <v>1083</v>
       </c>
       <c r="E92" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F92" t="s">
         <v>1071</v>
@@ -17299,7 +17299,7 @@
         <v>1094</v>
       </c>
       <c r="C93" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D93" t="s">
         <v>43</v>
@@ -17348,13 +17348,13 @@
       </c>
       <c r="S93"/>
       <c r="T93" t="s">
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="U93" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="V93" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
     </row>
     <row r="94">
@@ -17365,7 +17365,7 @@
         <v>1103</v>
       </c>
       <c r="C94" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D94" t="s">
         <v>1104</v>
@@ -17497,7 +17497,7 @@
         <v>1126</v>
       </c>
       <c r="C96" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D96" t="s">
         <v>1127</v>
@@ -17701,7 +17701,7 @@
         <v>1164</v>
       </c>
       <c r="E99" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="F99" t="s">
         <v>1152</v>
@@ -17893,7 +17893,7 @@
         <v>1192</v>
       </c>
       <c r="C102" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D102" t="s">
         <v>1193</v>
@@ -17959,7 +17959,7 @@
         <v>1205</v>
       </c>
       <c r="C103" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D103" t="s">
         <v>213</v>
@@ -18025,7 +18025,7 @@
         <v>1217</v>
       </c>
       <c r="C104" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D104" t="s">
         <v>213</v>
@@ -18163,7 +18163,7 @@
         <v>830</v>
       </c>
       <c r="E106" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="F106" t="s">
         <v>1230</v>
@@ -18223,13 +18223,13 @@
         <v>1252</v>
       </c>
       <c r="C107" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D107" t="s">
         <v>446</v>
       </c>
       <c r="E107" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F107" t="s">
         <v>1230</v>
@@ -18272,13 +18272,13 @@
       </c>
       <c r="S107"/>
       <c r="T107" t="s">
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="U107" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="V107" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
     </row>
     <row r="108">
@@ -18355,7 +18355,7 @@
         <v>1273</v>
       </c>
       <c r="C109" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D109" t="s">
         <v>967</v>
@@ -18553,13 +18553,13 @@
         <v>1301</v>
       </c>
       <c r="C112" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D112" t="s">
         <v>1302</v>
       </c>
       <c r="E112" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F112" t="s">
         <v>1293</v>
@@ -19011,13 +19011,13 @@
         <v>1374</v>
       </c>
       <c r="C119" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D119" t="s">
         <v>1375</v>
       </c>
       <c r="E119" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F119" t="s">
         <v>1376</v>
@@ -19077,7 +19077,7 @@
         <v>1387</v>
       </c>
       <c r="C120" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D120" t="s">
         <v>1388</v>
@@ -19211,7 +19211,7 @@
         <v>1409</v>
       </c>
       <c r="E122" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F122" t="s">
         <v>1410</v>
@@ -19269,7 +19269,7 @@
         <v>1417</v>
       </c>
       <c r="C123" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D123" t="s">
         <v>1418</v>
@@ -19601,7 +19601,7 @@
         <v>1480</v>
       </c>
       <c r="E128" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F128" t="s">
         <v>1481</v>
@@ -19989,7 +19989,7 @@
         <v>1550</v>
       </c>
       <c r="C134" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D134" t="s">
         <v>1551</v>
@@ -20061,7 +20061,7 @@
         <v>1564</v>
       </c>
       <c r="E135" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F135" t="s">
         <v>1552</v>
@@ -20125,7 +20125,7 @@
         <v>120</v>
       </c>
       <c r="E136" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="F136" t="s">
         <v>1575</v>
@@ -20183,7 +20183,7 @@
         <v>1582</v>
       </c>
       <c r="C137" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D137" t="s">
         <v>872</v>
@@ -20313,7 +20313,7 @@
         <v>1604</v>
       </c>
       <c r="C139" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D139" t="s">
         <v>967</v>
@@ -20379,13 +20379,13 @@
         <v>1616</v>
       </c>
       <c r="C140" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D140" t="s">
         <v>1480</v>
       </c>
       <c r="E140" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F140" t="s">
         <v>1605</v>
@@ -20451,7 +20451,7 @@
         <v>1628</v>
       </c>
       <c r="E141" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F141" t="s">
         <v>1605</v>
@@ -20511,13 +20511,13 @@
         <v>1639</v>
       </c>
       <c r="C142" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D142" t="s">
         <v>1640</v>
       </c>
       <c r="E142" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F142" t="s">
         <v>1641</v>
@@ -20649,7 +20649,7 @@
         <v>1302</v>
       </c>
       <c r="E144" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F144" t="s">
         <v>1665</v>
@@ -20969,7 +20969,7 @@
         <v>1710</v>
       </c>
       <c r="C149" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D149" t="s">
         <v>1711</v>
@@ -21035,7 +21035,7 @@
         <v>1722</v>
       </c>
       <c r="C150" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D150" t="s">
         <v>43</v>
@@ -21299,7 +21299,7 @@
         <v>1766</v>
       </c>
       <c r="C154" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D154" t="s">
         <v>1767</v>
@@ -21623,7 +21623,7 @@
         <v>1814</v>
       </c>
       <c r="C159" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D159" t="s">
         <v>1815</v>
@@ -21687,7 +21687,7 @@
         <v>1825</v>
       </c>
       <c r="C160" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D160" t="s">
         <v>608</v>
@@ -21817,7 +21817,7 @@
         <v>1849</v>
       </c>
       <c r="C162" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D162" t="s">
         <v>1104</v>
@@ -21883,7 +21883,7 @@
         <v>1861</v>
       </c>
       <c r="C163" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D163" t="s">
         <v>1862</v>
@@ -22085,7 +22085,7 @@
         <v>1897</v>
       </c>
       <c r="E166" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F166" t="s">
         <v>1885</v>
@@ -22145,7 +22145,7 @@
         <v>1908</v>
       </c>
       <c r="C167" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D167" t="s">
         <v>1909</v>
@@ -22283,7 +22283,7 @@
         <v>830</v>
       </c>
       <c r="E169" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="F169" t="s">
         <v>1921</v>
@@ -22343,7 +22343,7 @@
         <v>1943</v>
       </c>
       <c r="C170" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D170" t="s">
         <v>862</v>
@@ -22481,7 +22481,7 @@
         <v>1961</v>
       </c>
       <c r="E172" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F172" t="s">
         <v>1962</v>
@@ -22607,7 +22607,7 @@
         <v>1985</v>
       </c>
       <c r="C174" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D174" t="s">
         <v>1986</v>
@@ -22739,7 +22739,7 @@
         <v>2003</v>
       </c>
       <c r="C176" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D176" t="s">
         <v>2004</v>
@@ -23329,7 +23329,7 @@
         <v>2105</v>
       </c>
       <c r="C185" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D185" t="s">
         <v>1397</v>
@@ -23593,13 +23593,13 @@
         <v>2151</v>
       </c>
       <c r="C189" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D189" t="s">
         <v>2152</v>
       </c>
       <c r="E189" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="F189" t="s">
         <v>2153</v>
@@ -23795,7 +23795,7 @@
         <v>1628</v>
       </c>
       <c r="E192" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F192" t="s">
         <v>2189</v>
@@ -23855,7 +23855,7 @@
         <v>2197</v>
       </c>
       <c r="C193" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D193" t="s">
         <v>608</v>
@@ -24115,13 +24115,13 @@
         <v>2246</v>
       </c>
       <c r="C197" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D197" t="s">
         <v>446</v>
       </c>
       <c r="E197" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F197" t="s">
         <v>2247</v>
@@ -24181,7 +24181,7 @@
         <v>2258</v>
       </c>
       <c r="C198" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D198" t="s">
         <v>2259</v>
@@ -24245,7 +24245,7 @@
         <v>2271</v>
       </c>
       <c r="C199" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D199" t="s">
         <v>2272</v>
@@ -24309,7 +24309,7 @@
         <v>2284</v>
       </c>
       <c r="C200" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D200" t="s">
         <v>2272</v>
@@ -24373,13 +24373,13 @@
         <v>2295</v>
       </c>
       <c r="C201" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D201" t="s">
-        <v>59</v>
+        <v>76</v>
       </c>
       <c r="E201" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F201" t="s">
         <v>226</v>
@@ -24443,7 +24443,7 @@
         <v>830</v>
       </c>
       <c r="E202" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="F202" t="s">
         <v>226</v>
@@ -24501,7 +24501,7 @@
         <v>2314</v>
       </c>
       <c r="C203" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D203" t="s">
         <v>2315</v>
@@ -24565,7 +24565,7 @@
         <v>2327</v>
       </c>
       <c r="C204" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D204" t="s">
         <v>484</v>
@@ -24635,7 +24635,7 @@
         <v>2339</v>
       </c>
       <c r="E205" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F205" t="s">
         <v>2340</v>
@@ -24753,7 +24753,7 @@
         <v>2357</v>
       </c>
       <c r="C207" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D207" t="s">
         <v>1057</v>
@@ -24800,13 +24800,13 @@
       <c r="R207"/>
       <c r="S207"/>
       <c r="T207" t="s">
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="U207" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="V207" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
     </row>
     <row r="208">
@@ -24817,7 +24817,7 @@
         <v>2366</v>
       </c>
       <c r="C208" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D208" t="s">
         <v>2367</v>
@@ -24881,7 +24881,7 @@
         <v>2376</v>
       </c>
       <c r="C209" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D209" t="s">
         <v>188</v>
@@ -24945,7 +24945,7 @@
         <v>2387</v>
       </c>
       <c r="C210" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D210" t="s">
         <v>2388</v>
@@ -24992,13 +24992,13 @@
       <c r="R210"/>
       <c r="S210"/>
       <c r="T210" t="s">
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="U210" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="V210" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
     </row>
     <row r="211">
@@ -25009,7 +25009,7 @@
         <v>2394</v>
       </c>
       <c r="C211" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D211" t="s">
         <v>2395</v>
@@ -25137,7 +25137,7 @@
         <v>2414</v>
       </c>
       <c r="C213" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D213" t="s">
         <v>2415</v>
@@ -25515,7 +25515,7 @@
         <v>2472</v>
       </c>
       <c r="C219" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D219" t="s">
         <v>2473</v>
@@ -25580,10 +25580,10 @@
         <v>187</v>
       </c>
       <c r="D220" t="s">
-        <v>59</v>
+        <v>76</v>
       </c>
       <c r="E220" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F220" t="s">
         <v>174</v>
@@ -25827,7 +25827,7 @@
         <v>2521</v>
       </c>
       <c r="C224" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D224" t="s">
         <v>2522</v>
@@ -25889,7 +25889,7 @@
         <v>2531</v>
       </c>
       <c r="C225" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D225" t="s">
         <v>2532</v>
@@ -25959,7 +25959,7 @@
         <v>1302</v>
       </c>
       <c r="E226" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F226" t="s">
         <v>2545</v>
@@ -26023,7 +26023,7 @@
         <v>2557</v>
       </c>
       <c r="E227" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="F227" t="s">
         <v>2558</v>
@@ -26149,7 +26149,7 @@
         <v>2578</v>
       </c>
       <c r="E229" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F229" t="s">
         <v>2579</v>
@@ -26210,10 +26210,10 @@
         <v>23</v>
       </c>
       <c r="D230" t="s">
-        <v>59</v>
+        <v>76</v>
       </c>
       <c r="E230" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F230" t="s">
         <v>2579</v>
@@ -26341,7 +26341,7 @@
         <v>1628</v>
       </c>
       <c r="E232" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F232" t="s">
         <v>2611</v>
@@ -26655,7 +26655,7 @@
         <v>2658</v>
       </c>
       <c r="C237" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D237" t="s">
         <v>2659</v>
@@ -26851,7 +26851,7 @@
         <v>2695</v>
       </c>
       <c r="E240" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F240" t="s">
         <v>2696</v>
@@ -26909,13 +26909,13 @@
         <v>2707</v>
       </c>
       <c r="C241" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D241" t="s">
         <v>1302</v>
       </c>
       <c r="E241" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F241" t="s">
         <v>2696</v>
@@ -26979,7 +26979,7 @@
         <v>120</v>
       </c>
       <c r="E242" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="F242" t="s">
         <v>2696</v>
@@ -27037,7 +27037,7 @@
         <v>2729</v>
       </c>
       <c r="C243" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D243" t="s">
         <v>2599</v>
@@ -27107,7 +27107,7 @@
         <v>2742</v>
       </c>
       <c r="E244" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F244" t="s">
         <v>2730</v>
@@ -27229,7 +27229,7 @@
         <v>2766</v>
       </c>
       <c r="C246" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D246" t="s">
         <v>2767</v>
@@ -27417,13 +27417,13 @@
         <v>2793</v>
       </c>
       <c r="C249" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D249" t="s">
         <v>2794</v>
       </c>
       <c r="E249" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="F249" t="s">
         <v>2795</v>
@@ -27545,13 +27545,13 @@
         <v>2813</v>
       </c>
       <c r="C251" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D251" t="s">
         <v>120</v>
       </c>
       <c r="E251" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="F251" t="s">
         <v>2805</v>
@@ -27615,7 +27615,7 @@
         <v>2794</v>
       </c>
       <c r="E252" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="F252" t="s">
         <v>2825</v>
@@ -27919,7 +27919,7 @@
         <v>2875</v>
       </c>
       <c r="C257" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D257" t="s">
         <v>2876</v>
@@ -27983,7 +27983,7 @@
         <v>2885</v>
       </c>
       <c r="C258" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D258" t="s">
         <v>1711</v>
@@ -28111,7 +28111,7 @@
         <v>2906</v>
       </c>
       <c r="C260" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D260" t="s">
         <v>574</v>
@@ -28175,7 +28175,7 @@
         <v>2914</v>
       </c>
       <c r="C261" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D261" t="s">
         <v>574</v>
@@ -28239,13 +28239,13 @@
         <v>2922</v>
       </c>
       <c r="C262" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D262" t="s">
         <v>2923</v>
       </c>
       <c r="E262" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F262" t="s">
         <v>2886</v>
@@ -28373,7 +28373,7 @@
         <v>1019</v>
       </c>
       <c r="E264" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F264" t="s">
         <v>2936</v>
@@ -28437,7 +28437,7 @@
         <v>2959</v>
       </c>
       <c r="E265" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F265" t="s">
         <v>2960</v>
@@ -28495,7 +28495,7 @@
         <v>2971</v>
       </c>
       <c r="C266" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D266" t="s">
         <v>2895</v>
@@ -28565,7 +28565,7 @@
         <v>2959</v>
       </c>
       <c r="E267" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F267" t="s">
         <v>2972</v>
@@ -29313,13 +29313,13 @@
         <v>3110</v>
       </c>
       <c r="C279" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D279" t="s">
         <v>1083</v>
       </c>
       <c r="E279" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F279" t="s">
         <v>3098</v>
@@ -29447,7 +29447,7 @@
         <v>2578</v>
       </c>
       <c r="E281" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F281" t="s">
         <v>3098</v>
@@ -29569,7 +29569,7 @@
         <v>3151</v>
       </c>
       <c r="C283" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D283" t="s">
         <v>1353</v>
@@ -29767,7 +29767,7 @@
         <v>2742</v>
       </c>
       <c r="E286" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F286" t="s">
         <v>3177</v>
@@ -29808,13 +29808,13 @@
       <c r="R286"/>
       <c r="S286"/>
       <c r="T286" t="s">
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="U286" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="V286" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
     </row>
     <row r="287">
@@ -30205,7 +30205,7 @@
         <v>2557</v>
       </c>
       <c r="E293" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="F293" t="s">
         <v>3217</v>
@@ -30331,7 +30331,7 @@
         <v>3262</v>
       </c>
       <c r="E295" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F295" t="s">
         <v>3263</v>
@@ -30451,7 +30451,7 @@
         <v>3281</v>
       </c>
       <c r="C297" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D297" t="s">
         <v>3282</v>
@@ -30515,7 +30515,7 @@
         <v>3291</v>
       </c>
       <c r="C298" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D298" t="s">
         <v>3292</v>
@@ -30707,7 +30707,7 @@
         <v>3324</v>
       </c>
       <c r="C301" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D301" t="s">
         <v>1884</v>
@@ -30777,7 +30777,7 @@
         <v>3334</v>
       </c>
       <c r="E302" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F302" t="s">
         <v>3335</v>
@@ -30901,7 +30901,7 @@
         <v>1564</v>
       </c>
       <c r="E304" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F304" t="s">
         <v>3358</v>
@@ -30942,13 +30942,13 @@
       <c r="R304"/>
       <c r="S304"/>
       <c r="T304" t="s">
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="U304" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="V304" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
     </row>
     <row r="305">
@@ -30965,7 +30965,7 @@
         <v>1897</v>
       </c>
       <c r="E305" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F305" t="s">
         <v>3367</v>
@@ -31023,7 +31023,7 @@
         <v>3375</v>
       </c>
       <c r="C306" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D306" t="s">
         <v>3376</v>
@@ -31093,7 +31093,7 @@
         <v>3389</v>
       </c>
       <c r="E307" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F307" t="s">
         <v>3390</v>
@@ -31151,7 +31151,7 @@
         <v>3401</v>
       </c>
       <c r="C308" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D308" t="s">
         <v>2804</v>
@@ -31215,13 +31215,13 @@
         <v>3413</v>
       </c>
       <c r="C309" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D309" t="s">
         <v>1628</v>
       </c>
       <c r="E309" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F309" t="s">
         <v>3414</v>
@@ -31349,7 +31349,7 @@
         <v>2695</v>
       </c>
       <c r="E311" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F311" t="s">
         <v>3432</v>
@@ -31477,7 +31477,7 @@
         <v>2578</v>
       </c>
       <c r="E313" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F313" t="s">
         <v>3453</v>
@@ -31539,7 +31539,7 @@
         <v>1564</v>
       </c>
       <c r="E314" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F314" t="s">
         <v>3461</v>
@@ -31723,7 +31723,7 @@
         <v>3493</v>
       </c>
       <c r="C317" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D317" t="s">
         <v>3494</v>
@@ -31793,7 +31793,7 @@
         <v>3504</v>
       </c>
       <c r="E318" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F318" t="s">
         <v>3505</v>
@@ -31851,7 +31851,7 @@
         <v>3513</v>
       </c>
       <c r="C319" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D319" t="s">
         <v>2599</v>
@@ -31985,7 +31985,7 @@
         <v>2742</v>
       </c>
       <c r="E321" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F321" t="s">
         <v>3514</v>
@@ -32113,7 +32113,7 @@
         <v>1409</v>
       </c>
       <c r="E323" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F323" t="s">
         <v>3557</v>
@@ -32154,13 +32154,13 @@
       <c r="R323"/>
       <c r="S323"/>
       <c r="T323" t="s">
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="U323" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="V323" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
     </row>
     <row r="324">
@@ -32171,7 +32171,7 @@
         <v>3565</v>
       </c>
       <c r="C324" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D324" t="s">
         <v>3566</v>
@@ -32363,13 +32363,13 @@
         <v>3593</v>
       </c>
       <c r="C327" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D327" t="s">
         <v>2959</v>
       </c>
       <c r="E327" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F327" t="s">
         <v>3594</v>

</xml_diff>

<commit_message>
Update parliament data - 2026-06-04
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_CDF_EFK.xlsx
+++ b/Objets_parlementaires_CDF_EFK.xlsx
@@ -17747,9 +17747,15 @@
         <v>354</v>
       </c>
       <c r="S95"/>
-      <c r="T95"/>
-      <c r="U95"/>
-      <c r="V95"/>
+      <c r="T95" t="s">
+        <v>294</v>
+      </c>
+      <c r="U95" t="s">
+        <v>295</v>
+      </c>
+      <c r="V95" t="s">
+        <v>296</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">

</xml_diff>

<commit_message>
Update parliament data - 2026-06-08
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_CDF_EFK.xlsx
+++ b/Objets_parlementaires_CDF_EFK.xlsx
@@ -179,21 +179,54 @@
     <t xml:space="preserve">Politica nazionale|Media e comunicazione|Protezione sociale</t>
   </si>
   <si>
+    <t xml:space="preserve">26.7321</t>
+  </si>
+  <si>
+    <t xml:space="preserve">de Quattro Jacqueline</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PLR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-06-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EJPD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Georgische Staatsangehörige: überdurchschnittlich hohe Gesundheitskosten </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Géorgiens : des coûts médicaux supérieurs à la moyenne </t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Un audit du Contrôle fédéral des finances confirme des coûts médicaux très supérieurs à la moyenne pour les requérants géorgiens, soit 44,40&amp;nbsp;fr par jour et par personne. Entre 2022 et 2025, 26 d’entre eux ont été pris en charge par le SEM pour des traitements lourds. Parmi eux, 17 cas ont bénéficié d’un soutien financier total ou partiel du SEM pour 2,5&amp;nbsp;millions. Avec un cas allant jusqu’à 1,37&amp;nbsp;million. Quand et comment le Conseil fédéral va-t-il enrayer ce tourisme médical ?&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Eine Prüfung der Eidgenössischen Finanzkontrolle zeigt, dass die medizinischen Kosten für georgische Asylsuchende mit Fr.&amp;nbsp;44.40 pro Tag und Person deutlich über dem Durchschnitt liegen. Zwischen 2022 und 2025 benötigten 26&amp;nbsp;Asylsuchende Kostengutsprachen des Staatssekretariats für Migration&amp;nbsp;(SEM) für aufwändige Behandlungen. 17 von ihnen erhielten eine vollständige oder teilweise finanzielle Unterstützung durch das SEM im Gesamtumfang von 2,5&amp;nbsp;Millionen&amp;nbsp;Franken. In einem Fall lagen die Kosten bei bis zu 1,37&amp;nbsp;Millionen&amp;nbsp;Franken. Wann und wie wird der Bundesrat diesem Medizintourismus Einhalt gebieten?&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20267321</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20267321</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Élu &amp; Conseil fédéral</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finanzwesen|Migration|Gesundheit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finances|Politique migratoire|Santé</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finanze|Migrazione|Salute</t>
+  </si>
+  <si>
     <t xml:space="preserve">26.7324</t>
   </si>
   <si>
-    <t xml:space="preserve">de Quattro Jacqueline</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PLR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EJPD</t>
-  </si>
-  <si>
     <t xml:space="preserve">Schwachstellen im Staatssekretariat für Migration </t>
   </si>
   <si>
@@ -267,39 +300,6 @@
   </si>
   <si>
     <t xml:space="preserve">Politica nazionale|Finanze|Media e comunicazione</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26.7321</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Georgische Staatsangehörige: überdurchschnittlich hohe Gesundheitskosten </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Géorgiens : des coûts médicaux supérieurs à la moyenne </t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Un audit du Contrôle fédéral des finances confirme des coûts médicaux très supérieurs à la moyenne pour les requérants géorgiens, soit 44,40&amp;nbsp;fr par jour et par personne. Entre 2022 et 2025, 26 d’entre eux ont été pris en charge par le SEM pour des traitements lourds. Parmi eux, 17 cas ont bénéficié d’un soutien financier total ou partiel du SEM pour 2,5&amp;nbsp;millions. Avec un cas allant jusqu’à 1,37&amp;nbsp;million. Quand et comment le Conseil fédéral va-t-il enrayer ce tourisme médical ?&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Eine Prüfung der Eidgenössischen Finanzkontrolle zeigt, dass die medizinischen Kosten für georgische Asylsuchende mit Fr.&amp;nbsp;44.40 pro Tag und Person deutlich über dem Durchschnitt liegen. Zwischen 2022 und 2025 benötigten 26&amp;nbsp;Asylsuchende Kostengutsprachen des Staatssekretariats für Migration&amp;nbsp;(SEM) für aufwändige Behandlungen. 17 von ihnen erhielten eine vollständige oder teilweise finanzielle Unterstützung durch das SEM im Gesamtumfang von 2,5&amp;nbsp;Millionen&amp;nbsp;Franken. In einem Fall lagen die Kosten bei bis zu 1,37&amp;nbsp;Millionen&amp;nbsp;Franken. Wann und wie wird der Bundesrat diesem Medizintourismus Einhalt gebieten?&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20267321</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20267321</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Élu &amp; Conseil fédéral</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Finanzwesen|Migration|Gesundheit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Finances|Politique migratoire|Santé</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Finanze|Migrazione|Salute</t>
   </si>
   <si>
     <t xml:space="preserve">26.3335</t>
@@ -11838,7 +11838,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>20267324</v>
+        <v>20267321</v>
       </c>
       <c r="B4" t="s">
         <v>55</v>
@@ -11884,124 +11884,124 @@
         <v>65</v>
       </c>
       <c r="Q4" t="s">
-        <v>36</v>
+        <v>66</v>
       </c>
       <c r="R4" t="s">
         <v>37</v>
       </c>
       <c r="S4"/>
       <c r="T4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="U4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="V4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>20263550</v>
+        <v>20267324</v>
       </c>
       <c r="B5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C5" t="s">
-        <v>70</v>
+        <v>23</v>
       </c>
       <c r="D5" t="s">
+        <v>56</v>
+      </c>
+      <c r="E5" t="s">
+        <v>57</v>
+      </c>
+      <c r="F5" t="s">
+        <v>58</v>
+      </c>
+      <c r="G5" t="s">
+        <v>27</v>
+      </c>
+      <c r="H5" t="s">
+        <v>59</v>
+      </c>
+      <c r="I5" t="s">
         <v>71</v>
       </c>
-      <c r="E5" t="s">
+      <c r="J5" t="s">
         <v>72</v>
       </c>
-      <c r="F5" t="s">
-        <v>44</v>
-      </c>
-      <c r="G5" t="s">
+      <c r="K5"/>
+      <c r="L5" t="s">
         <v>73</v>
       </c>
-      <c r="H5"/>
-      <c r="I5" t="s">
+      <c r="M5" t="s">
         <v>74</v>
       </c>
-      <c r="J5" t="s">
+      <c r="N5" t="s">
+        <v>33</v>
+      </c>
+      <c r="O5" t="s">
         <v>75</v>
       </c>
-      <c r="K5" t="s">
+      <c r="P5" t="s">
         <v>76</v>
       </c>
-      <c r="L5"/>
-      <c r="M5" t="s">
-        <v>77</v>
-      </c>
-      <c r="N5" t="s">
-        <v>78</v>
-      </c>
-      <c r="O5" t="s">
-        <v>79</v>
-      </c>
-      <c r="P5" t="s">
-        <v>80</v>
-      </c>
       <c r="Q5" t="s">
-        <v>81</v>
+        <v>36</v>
       </c>
       <c r="R5" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="S5"/>
       <c r="T5" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="U5" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="V5" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>20267321</v>
+        <v>20263550</v>
       </c>
       <c r="B6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C6" t="s">
+        <v>81</v>
+      </c>
+      <c r="D6" t="s">
+        <v>82</v>
+      </c>
+      <c r="E6" t="s">
+        <v>83</v>
+      </c>
+      <c r="F6" t="s">
+        <v>44</v>
+      </c>
+      <c r="G6" t="s">
+        <v>84</v>
+      </c>
+      <c r="H6"/>
+      <c r="I6" t="s">
         <v>85</v>
       </c>
-      <c r="C6" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" t="s">
-        <v>56</v>
-      </c>
-      <c r="E6" t="s">
-        <v>57</v>
-      </c>
-      <c r="F6" t="s">
-        <v>58</v>
-      </c>
-      <c r="G6" t="s">
-        <v>27</v>
-      </c>
-      <c r="H6" t="s">
-        <v>59</v>
-      </c>
-      <c r="I6" t="s">
+      <c r="J6" t="s">
         <v>86</v>
       </c>
-      <c r="J6" t="s">
+      <c r="K6" t="s">
         <v>87</v>
       </c>
-      <c r="K6"/>
-      <c r="L6" t="s">
+      <c r="L6"/>
+      <c r="M6" t="s">
         <v>88</v>
       </c>
-      <c r="M6" t="s">
+      <c r="N6" t="s">
         <v>89</v>
-      </c>
-      <c r="N6" t="s">
-        <v>33</v>
       </c>
       <c r="O6" t="s">
         <v>90</v>
@@ -12013,11 +12013,9 @@
         <v>92</v>
       </c>
       <c r="R6" t="s">
-        <v>37</v>
-      </c>
-      <c r="S6" t="s">
-        <v>37</v>
-      </c>
+        <v>44</v>
+      </c>
+      <c r="S6"/>
       <c r="T6" t="s">
         <v>93</v>
       </c>
@@ -12036,7 +12034,7 @@
         <v>96</v>
       </c>
       <c r="C7" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D7" t="s">
         <v>97</v>
@@ -12180,7 +12178,7 @@
         <v>99</v>
       </c>
       <c r="G9" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H9" t="s">
         <v>45</v>
@@ -12246,7 +12244,7 @@
         <v>99</v>
       </c>
       <c r="G10" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H10" t="s">
         <v>145</v>
@@ -12300,19 +12298,19 @@
         <v>153</v>
       </c>
       <c r="C11" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D11" t="s">
         <v>154</v>
       </c>
       <c r="E11" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F11" t="s">
         <v>155</v>
       </c>
       <c r="G11" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H11" t="s">
         <v>156</v>
@@ -12408,7 +12406,7 @@
         <v>177</v>
       </c>
       <c r="Q12" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R12" t="s">
         <v>178</v>
@@ -12438,7 +12436,7 @@
         <v>183</v>
       </c>
       <c r="E13" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F13" t="s">
         <v>170</v>
@@ -12474,7 +12472,7 @@
         <v>190</v>
       </c>
       <c r="Q13" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R13" t="s">
         <v>178</v>
@@ -12498,7 +12496,7 @@
         <v>194</v>
       </c>
       <c r="C14" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D14" t="s">
         <v>195</v>
@@ -12540,7 +12538,7 @@
         <v>202</v>
       </c>
       <c r="Q14" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R14" t="s">
         <v>178</v>
@@ -12564,13 +12562,13 @@
         <v>206</v>
       </c>
       <c r="C15" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D15" t="s">
         <v>207</v>
       </c>
       <c r="E15" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F15" t="s">
         <v>155</v>
@@ -12630,7 +12628,7 @@
         <v>218</v>
       </c>
       <c r="C16" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D16" t="s">
         <v>219</v>
@@ -12696,7 +12694,7 @@
         <v>231</v>
       </c>
       <c r="C17" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D17" t="s">
         <v>232</v>
@@ -12762,7 +12760,7 @@
         <v>245</v>
       </c>
       <c r="C18" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D18" t="s">
         <v>246</v>
@@ -12804,7 +12802,7 @@
         <v>254</v>
       </c>
       <c r="Q18" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R18" t="s">
         <v>241</v>
@@ -12870,7 +12868,7 @@
         <v>266</v>
       </c>
       <c r="Q19" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R19" t="s">
         <v>170</v>
@@ -12894,7 +12892,7 @@
         <v>270</v>
       </c>
       <c r="C20" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D20" t="s">
         <v>271</v>
@@ -12936,7 +12934,7 @@
         <v>279</v>
       </c>
       <c r="Q20" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R20" t="s">
         <v>170</v>
@@ -12960,7 +12958,7 @@
         <v>283</v>
       </c>
       <c r="C21" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D21" t="s">
         <v>284</v>
@@ -13026,7 +13024,7 @@
         <v>296</v>
       </c>
       <c r="C22" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D22" t="s">
         <v>297</v>
@@ -13092,7 +13090,7 @@
         <v>308</v>
       </c>
       <c r="C23" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D23" t="s">
         <v>309</v>
@@ -13104,7 +13102,7 @@
         <v>285</v>
       </c>
       <c r="G23" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H23" t="s">
         <v>233</v>
@@ -13262,7 +13260,7 @@
         <v>341</v>
       </c>
       <c r="Q25" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R25" t="s">
         <v>342</v>
@@ -13326,7 +13324,7 @@
         <v>351</v>
       </c>
       <c r="Q26" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R26" t="s">
         <v>342</v>
@@ -13390,7 +13388,7 @@
         <v>363</v>
       </c>
       <c r="Q27" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R27" t="s">
         <v>357</v>
@@ -13420,7 +13418,7 @@
         <v>368</v>
       </c>
       <c r="E28" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F28" t="s">
         <v>369</v>
@@ -13486,7 +13484,7 @@
         <v>380</v>
       </c>
       <c r="E29" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F29" t="s">
         <v>381</v>
@@ -13522,7 +13520,7 @@
         <v>389</v>
       </c>
       <c r="Q29" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R29" t="s">
         <v>390</v>
@@ -13588,7 +13586,7 @@
         <v>403</v>
       </c>
       <c r="Q30" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R30" t="s">
         <v>390</v>
@@ -13612,7 +13610,7 @@
         <v>407</v>
       </c>
       <c r="C31" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D31" t="s">
         <v>24</v>
@@ -13654,7 +13652,7 @@
         <v>414</v>
       </c>
       <c r="Q31" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R31" t="s">
         <v>390</v>
@@ -13690,7 +13688,7 @@
         <v>381</v>
       </c>
       <c r="G32" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H32" t="s">
         <v>247</v>
@@ -13720,7 +13718,7 @@
         <v>423</v>
       </c>
       <c r="Q32" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R32" t="s">
         <v>390</v>
@@ -13744,13 +13742,13 @@
         <v>424</v>
       </c>
       <c r="C33" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D33" t="s">
         <v>425</v>
       </c>
       <c r="E33" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F33" t="s">
         <v>381</v>
@@ -13786,7 +13784,7 @@
         <v>432</v>
       </c>
       <c r="Q33" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R33" t="s">
         <v>390</v>
@@ -13810,7 +13808,7 @@
         <v>436</v>
       </c>
       <c r="C34" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D34" t="s">
         <v>437</v>
@@ -13852,7 +13850,7 @@
         <v>445</v>
       </c>
       <c r="Q34" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R34" t="s">
         <v>390</v>
@@ -13918,7 +13916,7 @@
         <v>456</v>
       </c>
       <c r="Q35" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R35" t="s">
         <v>390</v>
@@ -14008,7 +14006,7 @@
         <v>473</v>
       </c>
       <c r="C37" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D37" t="s">
         <v>474</v>
@@ -14020,7 +14018,7 @@
         <v>475</v>
       </c>
       <c r="G37" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H37" t="s">
         <v>247</v>
@@ -14050,7 +14048,7 @@
         <v>482</v>
       </c>
       <c r="Q37" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R37" t="s">
         <v>390</v>
@@ -14086,7 +14084,7 @@
         <v>475</v>
       </c>
       <c r="G38" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H38" t="s">
         <v>233</v>
@@ -14146,7 +14144,7 @@
         <v>499</v>
       </c>
       <c r="E39" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F39" t="s">
         <v>500</v>
@@ -14210,7 +14208,7 @@
         <v>511</v>
       </c>
       <c r="E40" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F40" t="s">
         <v>500</v>
@@ -14228,7 +14226,7 @@
         <v>513</v>
       </c>
       <c r="K40" t="s">
-        <v>76</v>
+        <v>87</v>
       </c>
       <c r="L40" t="s">
         <v>514</v>
@@ -14270,7 +14268,7 @@
         <v>521</v>
       </c>
       <c r="C41" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D41" t="s">
         <v>522</v>
@@ -14312,7 +14310,7 @@
         <v>531</v>
       </c>
       <c r="Q41" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R41" t="s">
         <v>390</v>
@@ -14378,7 +14376,7 @@
         <v>544</v>
       </c>
       <c r="Q42" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R42" t="s">
         <v>390</v>
@@ -14444,7 +14442,7 @@
         <v>557</v>
       </c>
       <c r="Q43" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R43" t="s">
         <v>390</v>
@@ -14468,7 +14466,7 @@
         <v>561</v>
       </c>
       <c r="C44" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D44" t="s">
         <v>562</v>
@@ -14510,7 +14508,7 @@
         <v>569</v>
       </c>
       <c r="Q44" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R44" t="s">
         <v>390</v>
@@ -14606,7 +14604,7 @@
         <v>586</v>
       </c>
       <c r="E46" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F46" t="s">
         <v>550</v>
@@ -14678,7 +14676,7 @@
         <v>599</v>
       </c>
       <c r="G47" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H47" t="s">
         <v>145</v>
@@ -14732,7 +14730,7 @@
         <v>610</v>
       </c>
       <c r="C48" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D48" t="s">
         <v>611</v>
@@ -14744,7 +14742,7 @@
         <v>599</v>
       </c>
       <c r="G48" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H48" t="s">
         <v>59</v>
@@ -14798,7 +14796,7 @@
         <v>622</v>
       </c>
       <c r="C49" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D49" t="s">
         <v>623</v>
@@ -14840,7 +14838,7 @@
         <v>630</v>
       </c>
       <c r="Q49" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R49" t="s">
         <v>390</v>
@@ -14864,7 +14862,7 @@
         <v>634</v>
       </c>
       <c r="C50" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D50" t="s">
         <v>143</v>
@@ -14876,7 +14874,7 @@
         <v>599</v>
       </c>
       <c r="G50" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H50" t="s">
         <v>59</v>
@@ -14930,7 +14928,7 @@
         <v>645</v>
       </c>
       <c r="C51" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D51" t="s">
         <v>623</v>
@@ -14996,7 +14994,7 @@
         <v>653</v>
       </c>
       <c r="C52" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D52" t="s">
         <v>654</v>
@@ -15038,7 +15036,7 @@
         <v>662</v>
       </c>
       <c r="Q52" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R52" t="s">
         <v>390</v>
@@ -15102,7 +15100,7 @@
         <v>673</v>
       </c>
       <c r="Q53" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R53" t="s">
         <v>390</v>
@@ -15296,7 +15294,7 @@
         <v>706</v>
       </c>
       <c r="Q56" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R56" t="s">
         <v>390</v>
@@ -15384,7 +15382,7 @@
         <v>718</v>
       </c>
       <c r="C58" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D58" t="s">
         <v>719</v>
@@ -15456,7 +15454,7 @@
         <v>733</v>
       </c>
       <c r="E59" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F59" t="s">
         <v>721</v>
@@ -15490,7 +15488,7 @@
         <v>739</v>
       </c>
       <c r="Q59" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R59" t="s">
         <v>390</v>
@@ -15578,7 +15576,7 @@
         <v>753</v>
       </c>
       <c r="C61" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D61" t="s">
         <v>754</v>
@@ -15644,7 +15642,7 @@
         <v>766</v>
       </c>
       <c r="C62" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D62" t="s">
         <v>474</v>
@@ -15656,7 +15654,7 @@
         <v>755</v>
       </c>
       <c r="G62" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H62" t="s">
         <v>59</v>
@@ -15750,7 +15748,7 @@
         <v>785</v>
       </c>
       <c r="Q63" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R63" t="s">
         <v>390</v>
@@ -15774,7 +15772,7 @@
         <v>789</v>
       </c>
       <c r="C64" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D64" t="s">
         <v>790</v>
@@ -15840,7 +15838,7 @@
         <v>802</v>
       </c>
       <c r="C65" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D65" t="s">
         <v>803</v>
@@ -15882,7 +15880,7 @@
         <v>811</v>
       </c>
       <c r="Q65" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R65" t="s">
         <v>390</v>
@@ -15906,13 +15904,13 @@
         <v>815</v>
       </c>
       <c r="C66" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D66" t="s">
         <v>586</v>
       </c>
       <c r="E66" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F66" t="s">
         <v>816</v>
@@ -15972,7 +15970,7 @@
         <v>827</v>
       </c>
       <c r="C67" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D67" t="s">
         <v>828</v>
@@ -16014,7 +16012,7 @@
         <v>835</v>
       </c>
       <c r="Q67" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R67" t="s">
         <v>390</v>
@@ -16038,7 +16036,7 @@
         <v>836</v>
       </c>
       <c r="C68" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D68" t="s">
         <v>837</v>
@@ -16146,7 +16144,7 @@
         <v>852</v>
       </c>
       <c r="Q69" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R69" t="s">
         <v>390</v>
@@ -16212,7 +16210,7 @@
         <v>863</v>
       </c>
       <c r="Q70" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R70" t="s">
         <v>390</v>
@@ -16236,7 +16234,7 @@
         <v>864</v>
       </c>
       <c r="C71" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D71" t="s">
         <v>865</v>
@@ -16278,7 +16276,7 @@
         <v>872</v>
       </c>
       <c r="Q71" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R71" t="s">
         <v>390</v>
@@ -16302,7 +16300,7 @@
         <v>876</v>
       </c>
       <c r="C72" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D72" t="s">
         <v>877</v>
@@ -16314,7 +16312,7 @@
         <v>878</v>
       </c>
       <c r="G72" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H72" t="s">
         <v>28</v>
@@ -16408,7 +16406,7 @@
         <v>893</v>
       </c>
       <c r="Q73" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R73" t="s">
         <v>390</v>
@@ -16438,7 +16436,7 @@
         <v>586</v>
       </c>
       <c r="E74" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F74" t="s">
         <v>887</v>
@@ -16536,7 +16534,7 @@
         <v>915</v>
       </c>
       <c r="Q75" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R75" t="s">
         <v>390</v>
@@ -16600,7 +16598,7 @@
         <v>925</v>
       </c>
       <c r="Q76" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R76" t="s">
         <v>390</v>
@@ -16624,13 +16622,13 @@
         <v>929</v>
       </c>
       <c r="C77" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D77" t="s">
         <v>930</v>
       </c>
       <c r="E77" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F77" t="s">
         <v>931</v>
@@ -16818,7 +16816,7 @@
         <v>955</v>
       </c>
       <c r="C80" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D80" t="s">
         <v>956</v>
@@ -16860,7 +16858,7 @@
         <v>964</v>
       </c>
       <c r="Q80" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R80" t="s">
         <v>390</v>
@@ -16884,7 +16882,7 @@
         <v>965</v>
       </c>
       <c r="C81" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D81" t="s">
         <v>966</v>
@@ -16992,7 +16990,7 @@
         <v>984</v>
       </c>
       <c r="Q82" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R82" t="s">
         <v>390</v>
@@ -17016,7 +17014,7 @@
         <v>988</v>
       </c>
       <c r="C83" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D83" t="s">
         <v>487</v>
@@ -17028,7 +17026,7 @@
         <v>989</v>
       </c>
       <c r="G83" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H83" t="s">
         <v>233</v>
@@ -17058,7 +17056,7 @@
         <v>996</v>
       </c>
       <c r="Q83" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R83" t="s">
         <v>390</v>
@@ -17082,7 +17080,7 @@
         <v>997</v>
       </c>
       <c r="C84" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D84" t="s">
         <v>998</v>
@@ -17188,7 +17186,7 @@
         <v>1016</v>
       </c>
       <c r="Q85" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R85" t="s">
         <v>390</v>
@@ -17276,7 +17274,7 @@
         <v>1028</v>
       </c>
       <c r="C87" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D87" t="s">
         <v>168</v>
@@ -17318,7 +17316,7 @@
         <v>1036</v>
       </c>
       <c r="Q87" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R87" t="s">
         <v>390</v>
@@ -17348,7 +17346,7 @@
         <v>586</v>
       </c>
       <c r="E88" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F88" t="s">
         <v>1041</v>
@@ -17408,7 +17406,7 @@
         <v>1049</v>
       </c>
       <c r="C89" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D89" t="s">
         <v>297</v>
@@ -17480,7 +17478,7 @@
         <v>1061</v>
       </c>
       <c r="E90" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F90" t="s">
         <v>1062</v>
@@ -17580,7 +17578,7 @@
         <v>1078</v>
       </c>
       <c r="Q91" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R91" t="s">
         <v>390</v>
@@ -17644,7 +17642,7 @@
         <v>1089</v>
       </c>
       <c r="Q92" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R92" t="s">
         <v>390</v>
@@ -17668,7 +17666,7 @@
         <v>1090</v>
       </c>
       <c r="C93" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D93" t="s">
         <v>24</v>
@@ -17710,7 +17708,7 @@
         <v>1098</v>
       </c>
       <c r="Q93" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R93" t="s">
         <v>390</v>
@@ -17734,7 +17732,7 @@
         <v>1102</v>
       </c>
       <c r="C94" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D94" t="s">
         <v>1103</v>
@@ -17800,13 +17798,13 @@
         <v>1115</v>
       </c>
       <c r="C95" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D95" t="s">
         <v>1116</v>
       </c>
       <c r="E95" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F95" t="s">
         <v>1117</v>
@@ -17842,7 +17840,7 @@
         <v>1124</v>
       </c>
       <c r="Q95" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R95" t="s">
         <v>390</v>
@@ -17866,13 +17864,13 @@
         <v>1128</v>
       </c>
       <c r="C96" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D96" t="s">
         <v>1129</v>
       </c>
       <c r="E96" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F96" t="s">
         <v>1130</v>
@@ -17942,7 +17940,7 @@
         <v>1143</v>
       </c>
       <c r="G97" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H97" t="s">
         <v>59</v>
@@ -17972,7 +17970,7 @@
         <v>1150</v>
       </c>
       <c r="Q97" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R97" t="s">
         <v>390</v>
@@ -17996,13 +17994,13 @@
         <v>1154</v>
       </c>
       <c r="C98" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D98" t="s">
         <v>207</v>
       </c>
       <c r="E98" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F98" t="s">
         <v>1155</v>
@@ -18038,7 +18036,7 @@
         <v>1162</v>
       </c>
       <c r="Q98" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R98" t="s">
         <v>390</v>
@@ -18102,7 +18100,7 @@
         <v>1170</v>
       </c>
       <c r="Q99" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R99" t="s">
         <v>390</v>
@@ -18132,7 +18130,7 @@
         <v>733</v>
       </c>
       <c r="E100" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F100" t="s">
         <v>1175</v>
@@ -18168,7 +18166,7 @@
         <v>1182</v>
       </c>
       <c r="Q100" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R100" t="s">
         <v>390</v>
@@ -18192,7 +18190,7 @@
         <v>1183</v>
       </c>
       <c r="C101" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D101" t="s">
         <v>461</v>
@@ -18234,7 +18232,7 @@
         <v>1190</v>
       </c>
       <c r="Q101" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R101" t="s">
         <v>390</v>
@@ -18258,7 +18256,7 @@
         <v>1191</v>
       </c>
       <c r="C102" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D102" t="s">
         <v>1192</v>
@@ -18300,7 +18298,7 @@
         <v>1200</v>
       </c>
       <c r="Q102" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R102" t="s">
         <v>390</v>
@@ -18366,7 +18364,7 @@
         <v>1213</v>
       </c>
       <c r="Q103" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R103" t="s">
         <v>390</v>
@@ -18393,16 +18391,16 @@
         <v>113</v>
       </c>
       <c r="D104" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
       <c r="E104" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F104" t="s">
         <v>1206</v>
       </c>
       <c r="G104" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H104" t="s">
         <v>115</v>
@@ -18432,7 +18430,7 @@
         <v>1224</v>
       </c>
       <c r="Q104" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R104" t="s">
         <v>390</v>
@@ -18498,7 +18496,7 @@
         <v>1236</v>
       </c>
       <c r="Q105" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R105" t="s">
         <v>390</v>
@@ -18564,7 +18562,7 @@
         <v>1245</v>
       </c>
       <c r="Q106" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R106" t="s">
         <v>390</v>
@@ -18588,7 +18586,7 @@
         <v>1249</v>
       </c>
       <c r="C107" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D107" t="s">
         <v>837</v>
@@ -18630,7 +18628,7 @@
         <v>1256</v>
       </c>
       <c r="Q107" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R107" t="s">
         <v>390</v>
@@ -18720,7 +18718,7 @@
         <v>1272</v>
       </c>
       <c r="C109" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D109" t="s">
         <v>1273</v>
@@ -18786,7 +18784,7 @@
         <v>1285</v>
       </c>
       <c r="C110" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D110" t="s">
         <v>195</v>
@@ -18828,7 +18826,7 @@
         <v>1293</v>
       </c>
       <c r="Q110" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R110" t="s">
         <v>390</v>
@@ -18852,7 +18850,7 @@
         <v>1297</v>
       </c>
       <c r="C111" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D111" t="s">
         <v>1298</v>
@@ -18894,7 +18892,7 @@
         <v>1305</v>
       </c>
       <c r="Q111" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R111" t="s">
         <v>390</v>
@@ -18918,7 +18916,7 @@
         <v>1309</v>
       </c>
       <c r="C112" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D112" t="s">
         <v>908</v>
@@ -18960,7 +18958,7 @@
         <v>1316</v>
       </c>
       <c r="Q112" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R112" t="s">
         <v>390</v>
@@ -18984,7 +18982,7 @@
         <v>1317</v>
       </c>
       <c r="C113" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D113" t="s">
         <v>1318</v>
@@ -19092,7 +19090,7 @@
         <v>1335</v>
       </c>
       <c r="Q114" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R114" t="s">
         <v>390</v>
@@ -19158,7 +19156,7 @@
         <v>1347</v>
       </c>
       <c r="Q115" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R115" t="s">
         <v>390</v>
@@ -19224,7 +19222,7 @@
         <v>1358</v>
       </c>
       <c r="Q116" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R116" t="s">
         <v>390</v>
@@ -19290,20 +19288,20 @@
         <v>1371</v>
       </c>
       <c r="Q117" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R117" t="s">
         <v>390</v>
       </c>
       <c r="S117"/>
       <c r="T117" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="U117" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="V117" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
     </row>
     <row r="118">
@@ -19314,7 +19312,7 @@
         <v>1372</v>
       </c>
       <c r="C118" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D118" t="s">
         <v>966</v>
@@ -19386,7 +19384,7 @@
         <v>586</v>
       </c>
       <c r="E119" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F119" t="s">
         <v>1364</v>
@@ -19446,7 +19444,7 @@
         <v>1391</v>
       </c>
       <c r="C120" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D120" t="s">
         <v>1392</v>
@@ -19578,7 +19576,7 @@
         <v>1415</v>
       </c>
       <c r="C122" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D122" t="s">
         <v>1103</v>
@@ -19644,7 +19642,7 @@
         <v>1423</v>
       </c>
       <c r="C123" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D123" t="s">
         <v>711</v>
@@ -19686,7 +19684,7 @@
         <v>1431</v>
       </c>
       <c r="Q123" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R123" t="s">
         <v>390</v>
@@ -19716,7 +19714,7 @@
         <v>1433</v>
       </c>
       <c r="E124" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F124" t="s">
         <v>1424</v>
@@ -19752,7 +19750,7 @@
         <v>1440</v>
       </c>
       <c r="Q124" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R124" t="s">
         <v>390</v>
@@ -19816,7 +19814,7 @@
         <v>1448</v>
       </c>
       <c r="Q125" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R125" t="s">
         <v>390</v>
@@ -19880,7 +19878,7 @@
         <v>1458</v>
       </c>
       <c r="Q126" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R126" t="s">
         <v>390</v>
@@ -19904,7 +19902,7 @@
         <v>1462</v>
       </c>
       <c r="C127" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D127" t="s">
         <v>1463</v>
@@ -19946,7 +19944,7 @@
         <v>1471</v>
       </c>
       <c r="Q127" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R127" t="s">
         <v>390</v>
@@ -19970,7 +19968,7 @@
         <v>1475</v>
       </c>
       <c r="C128" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D128" t="s">
         <v>908</v>
@@ -20012,7 +20010,7 @@
         <v>1482</v>
       </c>
       <c r="Q128" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R128" t="s">
         <v>390</v>
@@ -20036,7 +20034,7 @@
         <v>1483</v>
       </c>
       <c r="C129" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D129" t="s">
         <v>1484</v>
@@ -20102,7 +20100,7 @@
         <v>1493</v>
       </c>
       <c r="C130" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D130" t="s">
         <v>143</v>
@@ -20174,7 +20172,7 @@
         <v>1506</v>
       </c>
       <c r="E131" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F131" t="s">
         <v>1507</v>
@@ -20338,7 +20336,7 @@
         <v>1535</v>
       </c>
       <c r="Q133" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R133" t="s">
         <v>390</v>
@@ -20368,7 +20366,7 @@
         <v>1540</v>
       </c>
       <c r="E134" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F134" t="s">
         <v>1541</v>
@@ -20402,7 +20400,7 @@
         <v>1547</v>
       </c>
       <c r="Q134" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R134" t="s">
         <v>390</v>
@@ -20468,7 +20466,7 @@
         <v>1557</v>
       </c>
       <c r="Q135" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R135" t="s">
         <v>390</v>
@@ -20492,7 +20490,7 @@
         <v>1561</v>
       </c>
       <c r="C136" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D136" t="s">
         <v>865</v>
@@ -20558,7 +20556,7 @@
         <v>1573</v>
       </c>
       <c r="C137" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D137" t="s">
         <v>1574</v>
@@ -20598,7 +20596,7 @@
         <v>1582</v>
       </c>
       <c r="Q137" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R137" t="s">
         <v>390</v>
@@ -20662,7 +20660,7 @@
         <v>1593</v>
       </c>
       <c r="Q138" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R138" t="s">
         <v>390</v>
@@ -20686,7 +20684,7 @@
         <v>1597</v>
       </c>
       <c r="C139" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D139" t="s">
         <v>56</v>
@@ -20728,7 +20726,7 @@
         <v>1605</v>
       </c>
       <c r="Q139" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R139" t="s">
         <v>390</v>
@@ -20752,13 +20750,13 @@
         <v>1609</v>
       </c>
       <c r="C140" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D140" t="s">
         <v>1610</v>
       </c>
       <c r="E140" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F140" t="s">
         <v>1611</v>
@@ -20882,7 +20880,7 @@
         <v>1633</v>
       </c>
       <c r="C142" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D142" t="s">
         <v>1634</v>
@@ -20894,7 +20892,7 @@
         <v>1635</v>
       </c>
       <c r="G142" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H142" t="s">
         <v>59</v>
@@ -20990,7 +20988,7 @@
         <v>1655</v>
       </c>
       <c r="Q143" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R143" t="s">
         <v>390</v>
@@ -21014,7 +21012,7 @@
         <v>1659</v>
       </c>
       <c r="C144" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D144" t="s">
         <v>711</v>
@@ -21056,7 +21054,7 @@
         <v>1666</v>
       </c>
       <c r="Q144" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R144" t="s">
         <v>390</v>
@@ -21080,7 +21078,7 @@
         <v>1667</v>
       </c>
       <c r="C145" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D145" t="s">
         <v>1668</v>
@@ -21122,7 +21120,7 @@
         <v>1675</v>
       </c>
       <c r="Q145" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R145" t="s">
         <v>390</v>
@@ -21218,7 +21216,7 @@
         <v>1693</v>
       </c>
       <c r="E147" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F147" t="s">
         <v>1681</v>
@@ -21316,7 +21314,7 @@
         <v>1710</v>
       </c>
       <c r="Q148" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R148" t="s">
         <v>390</v>
@@ -21404,7 +21402,7 @@
         <v>1721</v>
       </c>
       <c r="C150" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D150" t="s">
         <v>711</v>
@@ -21446,7 +21444,7 @@
         <v>1729</v>
       </c>
       <c r="Q150" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R150" t="s">
         <v>390</v>
@@ -21512,7 +21510,7 @@
         <v>1741</v>
       </c>
       <c r="Q151" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R151" t="s">
         <v>390</v>
@@ -21542,7 +21540,7 @@
         <v>1610</v>
       </c>
       <c r="E152" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F152" t="s">
         <v>1734</v>
@@ -21602,13 +21600,13 @@
         <v>1756</v>
       </c>
       <c r="C153" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D153" t="s">
         <v>1757</v>
       </c>
       <c r="E153" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F153" t="s">
         <v>1734</v>
@@ -21644,7 +21642,7 @@
         <v>1764</v>
       </c>
       <c r="Q153" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R153" t="s">
         <v>390</v>
@@ -21674,13 +21672,13 @@
         <v>154</v>
       </c>
       <c r="E154" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F154" t="s">
         <v>1769</v>
       </c>
       <c r="G154" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H154" t="s">
         <v>247</v>
@@ -21734,7 +21732,7 @@
         <v>1780</v>
       </c>
       <c r="C155" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D155" t="s">
         <v>1392</v>
@@ -21776,7 +21774,7 @@
         <v>1788</v>
       </c>
       <c r="Q155" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R155" t="s">
         <v>390</v>
@@ -21800,13 +21798,13 @@
         <v>1792</v>
       </c>
       <c r="C156" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D156" t="s">
         <v>1433</v>
       </c>
       <c r="E156" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F156" t="s">
         <v>1793</v>
@@ -21842,7 +21840,7 @@
         <v>1800</v>
       </c>
       <c r="Q156" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R156" t="s">
         <v>390</v>
@@ -21866,7 +21864,7 @@
         <v>1801</v>
       </c>
       <c r="C157" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D157" t="s">
         <v>1071</v>
@@ -21908,7 +21906,7 @@
         <v>1809</v>
       </c>
       <c r="Q157" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R157" t="s">
         <v>390</v>
@@ -21972,20 +21970,20 @@
         <v>1818</v>
       </c>
       <c r="Q158" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R158" t="s">
         <v>390</v>
       </c>
       <c r="S158"/>
       <c r="T158" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="U158" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="V158" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
     </row>
     <row r="159">
@@ -22036,20 +22034,20 @@
         <v>1825</v>
       </c>
       <c r="Q159" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R159" t="s">
         <v>390</v>
       </c>
       <c r="S159"/>
       <c r="T159" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="U159" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="V159" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
     </row>
     <row r="160">
@@ -22060,7 +22058,7 @@
         <v>1826</v>
       </c>
       <c r="C160" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D160" t="s">
         <v>1528</v>
@@ -22102,7 +22100,7 @@
         <v>1834</v>
       </c>
       <c r="Q160" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R160" t="s">
         <v>390</v>
@@ -22168,7 +22166,7 @@
         <v>1843</v>
       </c>
       <c r="Q161" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R161" t="s">
         <v>390</v>
@@ -22234,7 +22232,7 @@
         <v>1854</v>
       </c>
       <c r="Q162" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R162" t="s">
         <v>390</v>
@@ -22258,7 +22256,7 @@
         <v>1858</v>
       </c>
       <c r="C163" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D163" t="s">
         <v>1859</v>
@@ -22300,7 +22298,7 @@
         <v>1866</v>
       </c>
       <c r="Q163" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R163" t="s">
         <v>390</v>
@@ -22324,7 +22322,7 @@
         <v>1867</v>
       </c>
       <c r="C164" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D164" t="s">
         <v>1363</v>
@@ -22366,7 +22364,7 @@
         <v>1875</v>
       </c>
       <c r="Q164" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R164" t="s">
         <v>390</v>
@@ -22390,7 +22388,7 @@
         <v>1879</v>
       </c>
       <c r="C165" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D165" t="s">
         <v>114</v>
@@ -22432,7 +22430,7 @@
         <v>1886</v>
       </c>
       <c r="Q165" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R165" t="s">
         <v>390</v>
@@ -22522,7 +22520,7 @@
         <v>1899</v>
       </c>
       <c r="C167" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D167" t="s">
         <v>97</v>
@@ -22564,7 +22562,7 @@
         <v>1907</v>
       </c>
       <c r="Q167" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R167" t="s">
         <v>390</v>
@@ -22588,7 +22586,7 @@
         <v>1911</v>
       </c>
       <c r="C168" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D168" t="s">
         <v>1574</v>
@@ -22692,7 +22690,7 @@
         <v>1930</v>
       </c>
       <c r="Q169" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R169" t="s">
         <v>390</v>
@@ -22756,7 +22754,7 @@
         <v>1937</v>
       </c>
       <c r="Q170" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R170" t="s">
         <v>390</v>
@@ -22790,7 +22788,7 @@
         <v>1940</v>
       </c>
       <c r="G171" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H171" t="s">
         <v>233</v>
@@ -22820,7 +22818,7 @@
         <v>1948</v>
       </c>
       <c r="Q171" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R171" t="s">
         <v>390</v>
@@ -22884,7 +22882,7 @@
         <v>1957</v>
       </c>
       <c r="Q172" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R172" t="s">
         <v>390</v>
@@ -22908,7 +22906,7 @@
         <v>1961</v>
       </c>
       <c r="C173" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D173" t="s">
         <v>1811</v>
@@ -23082,7 +23080,7 @@
         <v>1994</v>
       </c>
       <c r="Q175" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R175" t="s">
         <v>390</v>
@@ -23182,7 +23180,7 @@
         <v>2009</v>
       </c>
       <c r="G177" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H177" t="s">
         <v>1648</v>
@@ -23212,7 +23210,7 @@
         <v>2016</v>
       </c>
       <c r="Q177" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R177" t="s">
         <v>390</v>
@@ -23236,13 +23234,13 @@
         <v>2020</v>
       </c>
       <c r="C178" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D178" t="s">
         <v>2021</v>
       </c>
       <c r="E178" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F178" t="s">
         <v>2009</v>
@@ -23368,7 +23366,7 @@
         <v>2044</v>
       </c>
       <c r="C180" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D180" t="s">
         <v>1528</v>
@@ -23434,7 +23432,7 @@
         <v>2056</v>
       </c>
       <c r="C181" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D181" t="s">
         <v>966</v>
@@ -23476,7 +23474,7 @@
         <v>2063</v>
       </c>
       <c r="Q181" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R181" t="s">
         <v>390</v>
@@ -23542,20 +23540,20 @@
         <v>2074</v>
       </c>
       <c r="Q182" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R182" t="s">
         <v>390</v>
       </c>
       <c r="S182"/>
       <c r="T182" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="U182" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="V182" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
     </row>
     <row r="183">
@@ -23566,7 +23564,7 @@
         <v>2075</v>
       </c>
       <c r="C183" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D183" t="s">
         <v>246</v>
@@ -23608,7 +23606,7 @@
         <v>2083</v>
       </c>
       <c r="Q183" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R183" t="s">
         <v>390</v>
@@ -23632,13 +23630,13 @@
         <v>2084</v>
       </c>
       <c r="C184" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D184" t="s">
         <v>2085</v>
       </c>
       <c r="E184" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F184" t="s">
         <v>2086</v>
@@ -23674,7 +23672,7 @@
         <v>2093</v>
       </c>
       <c r="Q184" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R184" t="s">
         <v>390</v>
@@ -23698,7 +23696,7 @@
         <v>2097</v>
       </c>
       <c r="C185" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D185" t="s">
         <v>536</v>
@@ -23806,7 +23804,7 @@
         <v>2117</v>
       </c>
       <c r="Q186" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R186" t="s">
         <v>390</v>
@@ -23830,7 +23828,7 @@
         <v>2118</v>
       </c>
       <c r="C187" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D187" t="s">
         <v>246</v>
@@ -23872,7 +23870,7 @@
         <v>2126</v>
       </c>
       <c r="Q187" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R187" t="s">
         <v>390</v>
@@ -23962,7 +23960,7 @@
         <v>2139</v>
       </c>
       <c r="C189" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D189" t="s">
         <v>2140</v>
@@ -24040,7 +24038,7 @@
         <v>2153</v>
       </c>
       <c r="G190" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H190" t="s">
         <v>1648</v>
@@ -24070,7 +24068,7 @@
         <v>2160</v>
       </c>
       <c r="Q190" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R190" t="s">
         <v>390</v>
@@ -24160,7 +24158,7 @@
         <v>2176</v>
       </c>
       <c r="C192" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D192" t="s">
         <v>2177</v>
@@ -24202,7 +24200,7 @@
         <v>2184</v>
       </c>
       <c r="Q192" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R192" t="s">
         <v>390</v>
@@ -24226,7 +24224,7 @@
         <v>2188</v>
       </c>
       <c r="C193" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D193" t="s">
         <v>1986</v>
@@ -24268,7 +24266,7 @@
         <v>2196</v>
       </c>
       <c r="Q193" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R193" t="s">
         <v>390</v>
@@ -24292,7 +24290,7 @@
         <v>2197</v>
       </c>
       <c r="C194" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D194" t="s">
         <v>2198</v>
@@ -24334,7 +24332,7 @@
         <v>2206</v>
       </c>
       <c r="Q194" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R194" t="s">
         <v>390</v>
@@ -24398,7 +24396,7 @@
         <v>2214</v>
       </c>
       <c r="Q195" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R195" t="s">
         <v>390</v>
@@ -24462,7 +24460,7 @@
         <v>2225</v>
       </c>
       <c r="Q196" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R196" t="s">
         <v>390</v>
@@ -24528,7 +24526,7 @@
         <v>2237</v>
       </c>
       <c r="Q197" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R197" t="s">
         <v>390</v>
@@ -24552,7 +24550,7 @@
         <v>2241</v>
       </c>
       <c r="C198" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D198" t="s">
         <v>2242</v>
@@ -24618,7 +24616,7 @@
         <v>2253</v>
       </c>
       <c r="C199" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D199" t="s">
         <v>2254</v>
@@ -24684,7 +24682,7 @@
         <v>2264</v>
       </c>
       <c r="C200" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D200" t="s">
         <v>1891</v>
@@ -24726,7 +24724,7 @@
         <v>2271</v>
       </c>
       <c r="Q200" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R200" t="s">
         <v>390</v>
@@ -24792,7 +24790,7 @@
         <v>2284</v>
       </c>
       <c r="Q201" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R201" t="s">
         <v>390</v>
@@ -24856,7 +24854,7 @@
         <v>2296</v>
       </c>
       <c r="Q202" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R202" t="s">
         <v>390</v>
@@ -24880,7 +24878,7 @@
         <v>2300</v>
       </c>
       <c r="C203" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D203" t="s">
         <v>908</v>
@@ -24946,13 +24944,13 @@
         <v>2312</v>
       </c>
       <c r="C204" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D204" t="s">
         <v>1757</v>
       </c>
       <c r="E204" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F204" t="s">
         <v>2313</v>
@@ -25076,7 +25074,7 @@
         <v>2333</v>
       </c>
       <c r="C206" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D206" t="s">
         <v>2334</v>
@@ -25142,7 +25140,7 @@
         <v>2346</v>
       </c>
       <c r="C207" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D207" t="s">
         <v>2347</v>
@@ -25278,7 +25276,7 @@
         <v>586</v>
       </c>
       <c r="E209" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F209" t="s">
         <v>2371</v>
@@ -25378,7 +25376,7 @@
         <v>2391</v>
       </c>
       <c r="Q210" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R210" t="s">
         <v>390</v>
@@ -25412,7 +25410,7 @@
         <v>2397</v>
       </c>
       <c r="G211" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H211" t="s">
         <v>145</v>
@@ -25442,7 +25440,7 @@
         <v>2404</v>
       </c>
       <c r="Q211" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R211" t="s">
         <v>390</v>
@@ -25476,7 +25474,7 @@
         <v>2397</v>
       </c>
       <c r="G212" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H212" t="s">
         <v>247</v>
@@ -25506,7 +25504,7 @@
         <v>2415</v>
       </c>
       <c r="Q212" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R212" t="s">
         <v>390</v>
@@ -25536,7 +25534,7 @@
         <v>183</v>
       </c>
       <c r="E213" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F213" t="s">
         <v>369</v>
@@ -25572,7 +25570,7 @@
         <v>2426</v>
       </c>
       <c r="Q213" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R213"/>
       <c r="S213"/>
@@ -25594,7 +25592,7 @@
         <v>2430</v>
       </c>
       <c r="C214" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D214" t="s">
         <v>966</v>
@@ -25670,7 +25668,7 @@
         <v>272</v>
       </c>
       <c r="G215" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H215" t="s">
         <v>233</v>
@@ -25700,7 +25698,7 @@
         <v>2447</v>
       </c>
       <c r="Q215" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R215"/>
       <c r="S215"/>
@@ -25792,7 +25790,7 @@
         <v>2463</v>
       </c>
       <c r="E217" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F217" t="s">
         <v>2464</v>
@@ -25888,7 +25886,7 @@
         <v>2477</v>
       </c>
       <c r="Q218" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R218"/>
       <c r="S218"/>
@@ -25952,7 +25950,7 @@
         <v>2489</v>
       </c>
       <c r="Q219" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R219"/>
       <c r="S219"/>
@@ -26016,7 +26014,7 @@
         <v>2499</v>
       </c>
       <c r="Q220" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R220"/>
       <c r="S220"/>
@@ -26080,7 +26078,7 @@
         <v>2507</v>
       </c>
       <c r="Q221" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R221"/>
       <c r="S221"/>
@@ -26114,7 +26112,7 @@
         <v>2513</v>
       </c>
       <c r="G222" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H222" t="s">
         <v>145</v>
@@ -26178,7 +26176,7 @@
         <v>2513</v>
       </c>
       <c r="G223" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H223" t="s">
         <v>233</v>
@@ -26230,7 +26228,7 @@
         <v>2527</v>
       </c>
       <c r="C224" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D224" t="s">
         <v>1103</v>
@@ -26272,7 +26270,7 @@
         <v>2534</v>
       </c>
       <c r="Q224" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R224"/>
       <c r="S224"/>
@@ -26336,7 +26334,7 @@
         <v>2546</v>
       </c>
       <c r="Q225" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R225"/>
       <c r="S225"/>
@@ -26358,7 +26356,7 @@
         <v>2550</v>
       </c>
       <c r="C226" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D226" t="s">
         <v>2551</v>
@@ -26370,7 +26368,7 @@
         <v>2552</v>
       </c>
       <c r="G226" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H226" t="s">
         <v>233</v>
@@ -26422,7 +26420,7 @@
         <v>2563</v>
       </c>
       <c r="C227" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D227" t="s">
         <v>690</v>
@@ -26464,7 +26462,7 @@
         <v>2571</v>
       </c>
       <c r="Q227" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R227"/>
       <c r="S227"/>
@@ -26588,7 +26586,7 @@
         <v>2585</v>
       </c>
       <c r="Q229" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R229"/>
       <c r="S229"/>
@@ -26650,7 +26648,7 @@
         <v>2595</v>
       </c>
       <c r="Q230" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R230"/>
       <c r="S230"/>
@@ -26740,7 +26738,7 @@
         <v>183</v>
       </c>
       <c r="E232" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F232" t="s">
         <v>322</v>
@@ -26858,7 +26856,7 @@
         <v>2627</v>
       </c>
       <c r="C234" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D234" t="s">
         <v>129</v>
@@ -26870,7 +26868,7 @@
         <v>2628</v>
       </c>
       <c r="G234" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H234" t="s">
         <v>247</v>
@@ -26900,7 +26898,7 @@
         <v>2635</v>
       </c>
       <c r="Q234" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R234"/>
       <c r="S234"/>
@@ -26962,7 +26960,7 @@
         <v>2643</v>
       </c>
       <c r="Q235" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R235"/>
       <c r="S235"/>
@@ -27058,7 +27056,7 @@
         <v>2656</v>
       </c>
       <c r="G237" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H237" t="s">
         <v>145</v>
@@ -27088,7 +27086,7 @@
         <v>2663</v>
       </c>
       <c r="Q237" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R237"/>
       <c r="S237"/>
@@ -27110,13 +27108,13 @@
         <v>2667</v>
       </c>
       <c r="C238" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D238" t="s">
         <v>1433</v>
       </c>
       <c r="E238" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F238" t="s">
         <v>2668</v>
@@ -27152,7 +27150,7 @@
         <v>2675</v>
       </c>
       <c r="Q238" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R238"/>
       <c r="S238"/>
@@ -27174,7 +27172,7 @@
         <v>2679</v>
       </c>
       <c r="C239" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D239" t="s">
         <v>2680</v>
@@ -27216,7 +27214,7 @@
         <v>2688</v>
       </c>
       <c r="Q239" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R239"/>
       <c r="S239"/>
@@ -27278,7 +27276,7 @@
         <v>2699</v>
       </c>
       <c r="Q240" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R240"/>
       <c r="S240"/>
@@ -27300,13 +27298,13 @@
         <v>2700</v>
       </c>
       <c r="C241" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D241" t="s">
         <v>2701</v>
       </c>
       <c r="E241" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F241" t="s">
         <v>2702</v>
@@ -27364,13 +27362,13 @@
         <v>2713</v>
       </c>
       <c r="C242" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D242" t="s">
         <v>183</v>
       </c>
       <c r="E242" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F242" t="s">
         <v>2702</v>
@@ -27406,7 +27404,7 @@
         <v>2720</v>
       </c>
       <c r="Q242" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R242"/>
       <c r="S242"/>
@@ -27428,7 +27426,7 @@
         <v>2721</v>
       </c>
       <c r="C243" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D243" t="s">
         <v>2722</v>
@@ -27498,7 +27496,7 @@
         <v>1757</v>
       </c>
       <c r="E244" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F244" t="s">
         <v>2734</v>
@@ -27556,7 +27554,7 @@
         <v>2742</v>
       </c>
       <c r="C245" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D245" t="s">
         <v>2743</v>
@@ -27598,7 +27596,7 @@
         <v>2750</v>
       </c>
       <c r="Q245" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R245"/>
       <c r="S245"/>
@@ -27620,7 +27618,7 @@
         <v>2751</v>
       </c>
       <c r="C246" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D246" t="s">
         <v>2334</v>
@@ -27684,7 +27682,7 @@
         <v>2763</v>
       </c>
       <c r="C247" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D247" t="s">
         <v>2764</v>
@@ -27696,7 +27694,7 @@
         <v>2752</v>
       </c>
       <c r="G247" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H247" t="s">
         <v>115</v>
@@ -27748,7 +27746,7 @@
         <v>2772</v>
       </c>
       <c r="C248" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D248" t="s">
         <v>334</v>
@@ -27790,7 +27788,7 @@
         <v>2780</v>
       </c>
       <c r="Q248" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R248"/>
       <c r="S248"/>
@@ -27916,7 +27914,7 @@
         <v>2801</v>
       </c>
       <c r="Q250" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R250"/>
       <c r="S250"/>
@@ -27938,7 +27936,7 @@
         <v>2805</v>
       </c>
       <c r="C251" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D251" t="s">
         <v>2782</v>
@@ -28002,13 +28000,13 @@
         <v>2817</v>
       </c>
       <c r="C252" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D252" t="s">
         <v>2818</v>
       </c>
       <c r="E252" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F252" t="s">
         <v>2819</v>
@@ -28044,7 +28042,7 @@
         <v>2826</v>
       </c>
       <c r="Q252" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R252"/>
       <c r="S252"/>
@@ -28072,7 +28070,7 @@
         <v>1433</v>
       </c>
       <c r="E253" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F253" t="s">
         <v>2819</v>
@@ -28108,7 +28106,7 @@
         <v>2837</v>
       </c>
       <c r="Q253" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R253"/>
       <c r="S253"/>
@@ -28130,7 +28128,7 @@
         <v>2841</v>
       </c>
       <c r="C254" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D254" t="s">
         <v>271</v>
@@ -28172,7 +28170,7 @@
         <v>2848</v>
       </c>
       <c r="Q254" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R254"/>
       <c r="S254"/>
@@ -28236,7 +28234,7 @@
         <v>2860</v>
       </c>
       <c r="Q255" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R255"/>
       <c r="S255"/>
@@ -28258,19 +28256,19 @@
         <v>2864</v>
       </c>
       <c r="C256" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D256" t="s">
         <v>2865</v>
       </c>
       <c r="E256" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F256" t="s">
         <v>2853</v>
       </c>
       <c r="G256" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H256" t="s">
         <v>145</v>
@@ -28300,7 +28298,7 @@
         <v>2872</v>
       </c>
       <c r="Q256" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R256"/>
       <c r="S256"/>
@@ -28322,7 +28320,7 @@
         <v>2876</v>
       </c>
       <c r="C257" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D257" t="s">
         <v>2877</v>
@@ -28364,7 +28362,7 @@
         <v>2885</v>
       </c>
       <c r="Q257" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R257"/>
       <c r="S257"/>
@@ -28428,7 +28426,7 @@
         <v>2899</v>
       </c>
       <c r="Q258" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R258"/>
       <c r="S258"/>
@@ -28616,7 +28614,7 @@
         <v>2925</v>
       </c>
       <c r="Q261" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R261"/>
       <c r="S261"/>
@@ -28638,7 +28636,7 @@
         <v>2926</v>
       </c>
       <c r="C262" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D262" t="s">
         <v>2927</v>
@@ -28680,7 +28678,7 @@
         <v>2935</v>
       </c>
       <c r="Q262" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R262"/>
       <c r="S262"/>
@@ -28744,7 +28742,7 @@
         <v>2943</v>
       </c>
       <c r="Q263" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R263"/>
       <c r="S263"/>
@@ -28806,7 +28804,7 @@
         <v>2954</v>
       </c>
       <c r="Q264" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R264"/>
       <c r="S264"/>
@@ -28868,7 +28866,7 @@
         <v>2962</v>
       </c>
       <c r="Q265" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R265"/>
       <c r="S265"/>
@@ -28930,7 +28928,7 @@
         <v>2972</v>
       </c>
       <c r="Q266" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R266"/>
       <c r="S266"/>
@@ -28952,7 +28950,7 @@
         <v>2973</v>
       </c>
       <c r="C267" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D267" t="s">
         <v>1519</v>
@@ -29054,7 +29052,7 @@
         <v>2994</v>
       </c>
       <c r="Q268" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R268"/>
       <c r="S268"/>
@@ -29088,7 +29086,7 @@
         <v>3000</v>
       </c>
       <c r="G269" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H269" t="s">
         <v>45</v>
@@ -29118,7 +29116,7 @@
         <v>3007</v>
       </c>
       <c r="Q269" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R269"/>
       <c r="S269"/>
@@ -29182,7 +29180,7 @@
         <v>3016</v>
       </c>
       <c r="Q270" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R270"/>
       <c r="S270"/>
@@ -29204,7 +29202,7 @@
         <v>3017</v>
       </c>
       <c r="C271" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D271" t="s">
         <v>3018</v>
@@ -29246,7 +29244,7 @@
         <v>3025</v>
       </c>
       <c r="Q271" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R271"/>
       <c r="S271"/>
@@ -29402,7 +29400,7 @@
         <v>3046</v>
       </c>
       <c r="E274" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F274" t="s">
         <v>3009</v>
@@ -29460,7 +29458,7 @@
         <v>3057</v>
       </c>
       <c r="C275" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D275" t="s">
         <v>3058</v>
@@ -29502,7 +29500,7 @@
         <v>3066</v>
       </c>
       <c r="Q275" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R275"/>
       <c r="S275"/>
@@ -29524,13 +29522,13 @@
         <v>3070</v>
       </c>
       <c r="C276" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D276" t="s">
         <v>207</v>
       </c>
       <c r="E276" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F276" t="s">
         <v>3059</v>
@@ -29588,13 +29586,13 @@
         <v>3081</v>
       </c>
       <c r="C277" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D277" t="s">
         <v>3082</v>
       </c>
       <c r="E277" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F277" t="s">
         <v>3083</v>
@@ -29630,7 +29628,7 @@
         <v>3090</v>
       </c>
       <c r="Q277" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R277"/>
       <c r="S277"/>
@@ -29694,7 +29692,7 @@
         <v>3102</v>
       </c>
       <c r="Q278" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R278"/>
       <c r="S278"/>
@@ -29722,7 +29720,7 @@
         <v>3082</v>
       </c>
       <c r="E279" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F279" t="s">
         <v>3095</v>
@@ -29756,7 +29754,7 @@
         <v>3109</v>
       </c>
       <c r="Q279" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R279"/>
       <c r="S279"/>
@@ -29778,7 +29776,7 @@
         <v>3113</v>
       </c>
       <c r="C280" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D280" t="s">
         <v>2890</v>
@@ -29820,7 +29818,7 @@
         <v>3121</v>
       </c>
       <c r="Q280" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R280"/>
       <c r="S280"/>
@@ -29882,7 +29880,7 @@
         <v>3133</v>
       </c>
       <c r="Q281" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R281"/>
       <c r="S281"/>
@@ -29944,7 +29942,7 @@
         <v>3142</v>
       </c>
       <c r="Q282" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R282"/>
       <c r="S282"/>
@@ -30006,7 +30004,7 @@
         <v>3150</v>
       </c>
       <c r="Q283" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R283"/>
       <c r="S283"/>
@@ -30068,7 +30066,7 @@
         <v>3158</v>
       </c>
       <c r="Q284" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R284"/>
       <c r="S284"/>
@@ -30130,7 +30128,7 @@
         <v>3168</v>
       </c>
       <c r="Q285" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R285"/>
       <c r="S285"/>
@@ -30152,7 +30150,7 @@
         <v>3172</v>
       </c>
       <c r="C286" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D286" t="s">
         <v>3173</v>
@@ -30194,7 +30192,7 @@
         <v>3181</v>
       </c>
       <c r="Q286" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R286"/>
       <c r="S286"/>
@@ -30216,7 +30214,7 @@
         <v>3182</v>
       </c>
       <c r="C287" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D287" t="s">
         <v>3183</v>
@@ -30342,7 +30340,7 @@
         <v>3206</v>
       </c>
       <c r="C289" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D289" t="s">
         <v>3207</v>
@@ -30448,7 +30446,7 @@
         <v>3229</v>
       </c>
       <c r="Q290" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R290"/>
       <c r="S290"/>
@@ -30473,10 +30471,10 @@
         <v>113</v>
       </c>
       <c r="D291" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
       <c r="E291" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F291" t="s">
         <v>3221</v>
@@ -30534,7 +30532,7 @@
         <v>3241</v>
       </c>
       <c r="C292" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D292" t="s">
         <v>536</v>
@@ -30598,13 +30596,13 @@
         <v>3252</v>
       </c>
       <c r="C293" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D293" t="s">
         <v>2701</v>
       </c>
       <c r="E293" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F293" t="s">
         <v>3221</v>
@@ -30640,7 +30638,7 @@
         <v>3259</v>
       </c>
       <c r="Q293" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R293"/>
       <c r="S293"/>
@@ -30662,7 +30660,7 @@
         <v>3263</v>
       </c>
       <c r="C294" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D294" t="s">
         <v>1261</v>
@@ -30704,7 +30702,7 @@
         <v>3270</v>
       </c>
       <c r="Q294" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R294"/>
       <c r="S294"/>
@@ -30768,7 +30766,7 @@
         <v>3281</v>
       </c>
       <c r="Q295" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R295"/>
       <c r="S295"/>
@@ -30790,7 +30788,7 @@
         <v>3282</v>
       </c>
       <c r="C296" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D296" t="s">
         <v>1836</v>
@@ -30918,19 +30916,19 @@
         <v>3299</v>
       </c>
       <c r="C298" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D298" t="s">
         <v>2865</v>
       </c>
       <c r="E298" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F298" t="s">
         <v>3300</v>
       </c>
       <c r="G298" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H298" t="s">
         <v>145</v>
@@ -30960,7 +30958,7 @@
         <v>3307</v>
       </c>
       <c r="Q298" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R298"/>
       <c r="S298"/>
@@ -31022,7 +31020,7 @@
         <v>3315</v>
       </c>
       <c r="Q299" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R299"/>
       <c r="S299"/>
@@ -31084,7 +31082,7 @@
         <v>3326</v>
       </c>
       <c r="Q300" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R300"/>
       <c r="S300"/>
@@ -31106,7 +31104,7 @@
         <v>3327</v>
       </c>
       <c r="C301" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D301" t="s">
         <v>654</v>
@@ -31272,7 +31270,7 @@
         <v>3355</v>
       </c>
       <c r="Q303" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R303"/>
       <c r="S303"/>
@@ -31356,7 +31354,7 @@
         <v>3364</v>
       </c>
       <c r="C305" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D305" t="s">
         <v>2680</v>
@@ -31398,7 +31396,7 @@
         <v>3371</v>
       </c>
       <c r="Q305" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R305"/>
       <c r="S305"/>
@@ -31482,13 +31480,13 @@
         <v>3384</v>
       </c>
       <c r="C307" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D307" t="s">
         <v>3385</v>
       </c>
       <c r="E307" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F307" t="s">
         <v>3386</v>
@@ -31524,7 +31522,7 @@
         <v>3393</v>
       </c>
       <c r="Q307" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R307"/>
       <c r="S307"/>
@@ -31586,7 +31584,7 @@
         <v>3403</v>
       </c>
       <c r="Q308" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R308"/>
       <c r="S308"/>
@@ -31714,7 +31712,7 @@
         <v>3422</v>
       </c>
       <c r="Q310" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R310"/>
       <c r="S310"/>
@@ -31736,7 +31734,7 @@
         <v>3423</v>
       </c>
       <c r="C311" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D311" t="s">
         <v>3424</v>
@@ -31800,7 +31798,7 @@
         <v>3436</v>
       </c>
       <c r="C312" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D312" t="s">
         <v>2764</v>
@@ -31812,7 +31810,7 @@
         <v>3425</v>
       </c>
       <c r="G312" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H312" t="s">
         <v>145</v>
@@ -31934,7 +31932,7 @@
         <v>3457</v>
       </c>
       <c r="E314" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F314" t="s">
         <v>3458</v>
@@ -32052,13 +32050,13 @@
         <v>3480</v>
       </c>
       <c r="C316" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D316" t="s">
         <v>1693</v>
       </c>
       <c r="E316" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F316" t="s">
         <v>3481</v>
@@ -32116,13 +32114,13 @@
         <v>3489</v>
       </c>
       <c r="C317" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D317" t="s">
         <v>2021</v>
       </c>
       <c r="E317" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F317" t="s">
         <v>3490</v>
@@ -32192,7 +32190,7 @@
         <v>3500</v>
       </c>
       <c r="G318" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H318" t="s">
         <v>115</v>
@@ -32244,13 +32242,13 @@
         <v>3511</v>
       </c>
       <c r="C319" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D319" t="s">
         <v>3512</v>
       </c>
       <c r="E319" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F319" t="s">
         <v>3513</v>
@@ -32378,7 +32376,7 @@
         <v>1757</v>
       </c>
       <c r="E321" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F321" t="s">
         <v>3537</v>
@@ -32436,7 +32434,7 @@
         <v>3545</v>
       </c>
       <c r="C322" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D322" t="s">
         <v>536</v>
@@ -32506,7 +32504,7 @@
         <v>2818</v>
       </c>
       <c r="E323" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F323" t="s">
         <v>3555</v>
@@ -32606,7 +32604,7 @@
         <v>3574</v>
       </c>
       <c r="Q324" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R324"/>
       <c r="S324"/>
@@ -32634,7 +32632,7 @@
         <v>2701</v>
       </c>
       <c r="E325" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F325" t="s">
         <v>3576</v>
@@ -32696,7 +32694,7 @@
         <v>1693</v>
       </c>
       <c r="E326" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F326" t="s">
         <v>3584</v>
@@ -32730,7 +32728,7 @@
         <v>3590</v>
       </c>
       <c r="Q326" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R326"/>
       <c r="S326"/>
@@ -32752,7 +32750,7 @@
         <v>3591</v>
       </c>
       <c r="C327" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D327" t="s">
         <v>3499</v>
@@ -32764,7 +32762,7 @@
         <v>3592</v>
       </c>
       <c r="G327" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H327" t="s">
         <v>115</v>
@@ -32816,7 +32814,7 @@
         <v>3603</v>
       </c>
       <c r="C328" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D328" t="s">
         <v>3604</v>
@@ -32858,7 +32856,7 @@
         <v>3612</v>
       </c>
       <c r="Q328" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R328"/>
       <c r="S328"/>
@@ -32922,7 +32920,7 @@
         <v>3625</v>
       </c>
       <c r="Q329" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R329"/>
       <c r="S329"/>
@@ -32944,13 +32942,13 @@
         <v>3626</v>
       </c>
       <c r="C330" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D330" t="s">
         <v>3627</v>
       </c>
       <c r="E330" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F330" t="s">
         <v>3628</v>
@@ -32986,7 +32984,7 @@
         <v>3635</v>
       </c>
       <c r="Q330" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R330"/>
       <c r="S330"/>
@@ -33050,7 +33048,7 @@
         <v>3644</v>
       </c>
       <c r="Q331" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R331"/>
       <c r="S331"/>
@@ -33072,7 +33070,7 @@
         <v>3645</v>
       </c>
       <c r="C332" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D332" t="s">
         <v>3646</v>
@@ -33136,19 +33134,19 @@
         <v>3657</v>
       </c>
       <c r="C333" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D333" t="s">
         <v>2865</v>
       </c>
       <c r="E333" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F333" t="s">
         <v>3637</v>
       </c>
       <c r="G333" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H333" t="s">
         <v>247</v>
@@ -33200,7 +33198,7 @@
         <v>3668</v>
       </c>
       <c r="C334" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D334" t="s">
         <v>2722</v>
@@ -33242,7 +33240,7 @@
         <v>3675</v>
       </c>
       <c r="Q334" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R334"/>
       <c r="S334"/>
@@ -33264,13 +33262,13 @@
         <v>3679</v>
       </c>
       <c r="C335" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D335" t="s">
         <v>1540</v>
       </c>
       <c r="E335" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F335" t="s">
         <v>3680</v>
@@ -33370,7 +33368,7 @@
         <v>3697</v>
       </c>
       <c r="Q336" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R336"/>
       <c r="S336"/>
@@ -33392,7 +33390,7 @@
         <v>3698</v>
       </c>
       <c r="C337" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D337" t="s">
         <v>536</v>
@@ -33434,7 +33432,7 @@
         <v>3706</v>
       </c>
       <c r="Q337" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R337"/>
       <c r="S337"/>
@@ -33456,7 +33454,7 @@
         <v>3707</v>
       </c>
       <c r="C338" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D338" t="s">
         <v>1811</v>
@@ -33526,7 +33524,7 @@
         <v>3082</v>
       </c>
       <c r="E339" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F339" t="s">
         <v>3717</v>
@@ -33584,7 +33582,7 @@
         <v>3728</v>
       </c>
       <c r="C340" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D340" t="s">
         <v>2033</v>
@@ -33626,7 +33624,7 @@
         <v>3735</v>
       </c>
       <c r="Q340" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R340"/>
       <c r="S340"/>
@@ -33648,7 +33646,7 @@
         <v>3736</v>
       </c>
       <c r="C341" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D341" t="s">
         <v>536</v>

</xml_diff>

<commit_message>
Update parliament data - 2026-06-28
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_CDF_EFK.xlsx
+++ b/Objets_parlementaires_CDF_EFK.xlsx
@@ -1016,10 +1016,10 @@
     <t xml:space="preserve">2025-12-17</t>
   </si>
   <si>
-    <t xml:space="preserve">xml:space="preserve"&amp;gt; Das Ruder wieder übernehmen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">xml:space="preserve"&amp;gt;  Il est temps de reprendre les choses en main</t>
+    <t xml:space="preserve">xml:space="preserve"&gt; Das Ruder wieder übernehmen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">xml:space="preserve"&gt;  Il est temps de reprendre les choses en main</t>
   </si>
   <si>
     <t xml:space="preserve">È tempo di prendere in mano la situazione</t>
@@ -1509,10 +1509,10 @@
     <t xml:space="preserve">25.3893</t>
   </si>
   <si>
-    <t xml:space="preserve">xml:space="preserve"&amp;gt; Transparenz und Rechtfertigung der finanziellen Reserven der Suva und Prüfung durch die Eidgenössische Finanzkontrolle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">xml:space="preserve"&amp;gt; Transparence et justification des réserves financières de la Suva et contrôle du CDF</t>
+    <t xml:space="preserve">xml:space="preserve"&gt; Transparenz und Rechtfertigung der finanziellen Reserven der Suva und Prüfung durch die Eidgenössische Finanzkontrolle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">xml:space="preserve"&gt; Transparence et justification des réserves financières de la Suva et contrôle du CDF</t>
   </si>
   <si>
     <t xml:space="preserve">Trasparenza e giustificazione delle riserve finanziarie della Suva e controllo del CDF</t>
@@ -1848,13 +1848,13 @@
     <t xml:space="preserve">Schmezer Ueli</t>
   </si>
   <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;CO2-Verordnung. Erleichterungsmassnahmen für die Autobranche? </t>
-  </si>
-  <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;Ordonnance sur le CO2. Des mesures d'allègement pour la branche automobile ? </t>
-  </si>
-  <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;Ordinanza sul CO2. Misure di agevolazione per il settore automobilistico? </t>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;CO2-Verordnung. Erleichterungsmassnahmen für die Autobranche? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;Ordonnance sur le CO2. Des mesures d'allègement pour la branche automobile ? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;Ordinanza sul CO2. Misure di agevolazione per il settore automobilistico? </t>
   </si>
   <si>
     <t xml:space="preserve">&amp;amp;lt;p&amp;amp;gt;La révision, ou plus précisément l’adaptation de l’ordonnance sur le CO2 faisant suite à la révision de la loi sur le CO2 (en vigueur depuis le 1.1.2025), revêt une grande importance pour la réalisation des objectifs légaux en matière d'émissions. Cela concerne en particulier les dispositions d'exécution pour les voitures de tourisme.&amp;amp;amp;nbsp;&amp;amp;lt;/p&amp;amp;gt;&amp;amp;lt;p&amp;amp;gt;&amp;amp;amp;nbsp;&amp;amp;lt;/p&amp;amp;gt;&amp;amp;lt;p&amp;amp;gt;Le 17 mars 2025, le Conseil fédéral a laissé entendre pendant l’heure des questions qu'il « adopterait l'ordonnance lors d'une prochaine séance ». Il a répondu de façon évasive aux questions sur cette ordonnance.&amp;amp;lt;/p&amp;amp;gt;&amp;amp;lt;p&amp;amp;gt;&amp;amp;amp;nbsp;&amp;amp;lt;/p&amp;amp;gt;&amp;amp;lt;p&amp;amp;gt;La présente interpellation s’intéresse aux mesures d'allègement des sanctions pécuniaires qui pourraient éventuellement être (une nouvelle fois) accordées à la branche automobile lorsque celle-ci ne parvient pas à atteindre les valeurs cibles.&amp;amp;amp;nbsp;&amp;amp;lt;/p&amp;amp;gt;&amp;amp;lt;p&amp;amp;gt;Concrètement, l’ordonnance sur le CO2 soulève les questions suivantes.&amp;amp;amp;nbsp;&amp;amp;lt;br&amp;amp;gt;&amp;amp;amp;nbsp;&amp;amp;lt;/p&amp;amp;gt;&amp;amp;lt;ol&amp;amp;gt;&amp;amp;lt;li&amp;amp;gt;La procédure de consultation s’est achevée le 17 octobre 2024. Pourquoi cette ordonnance dont nous avons urgemment besoin n'est-elle pas entrée en vigueur en mars 2025&amp;amp;amp;nbsp;? Quels sont les facteurs qui ont conduit à ce retard.&amp;amp;amp;nbsp;&amp;amp;lt;br&amp;amp;gt;&amp;amp;amp;nbsp;&amp;amp;lt;/li&amp;amp;gt;&amp;amp;lt;li&amp;amp;gt;Le projet envoyé en consultation ne prévoyait pas d'alléger les sanctions. Sur les 202 prises de position annoncées par le Conseil fédéral, combien demandaient, dans le délai imparti par la procédure, des allégements en cas de non-respect des objectifs ? Quels étaient leurs principaux arguments ?&amp;amp;amp;nbsp;&amp;amp;lt;br&amp;amp;gt;&amp;amp;amp;nbsp;&amp;amp;lt;/li&amp;amp;gt;&amp;amp;lt;li&amp;amp;gt;Le Contrôle fédéral des finances (CDF) a évalué l'efficacité des sanctions en matière de CO2 pour les voitures de tourisme neuves : il est clair pour lui qu'il faut renoncer à des mesures d'allégement si les objectifs ne sont pas atteints.&amp;amp;amp;nbsp;&amp;amp;lt;br&amp;amp;gt;Le Conseil fédéral partage-t-il l'appréciation du CDF ? Si ce n'est pas le cas, quels sont ses arguments ?&amp;amp;lt;br&amp;amp;gt;&amp;amp;amp;nbsp;&amp;amp;lt;/li&amp;amp;gt;&amp;amp;lt;li&amp;amp;gt;Par le passé (notamment en 2015 et en 2020), des dispositions prévoyant des allégements (supercrédits, phase d’introduction) ont été introduites pour réduire les montants des sanctions en cas de dépassement des objectifs d'émission. Quel est le montant cumulé des dépassements d'objectifs non sanctionnés depuis 2010 en Suisse&amp;amp;amp;nbsp;?&amp;amp;amp;nbsp;&amp;amp;lt;br&amp;amp;gt;&amp;amp;amp;nbsp;&amp;amp;lt;/li&amp;amp;gt;&amp;amp;lt;li&amp;amp;gt;Si le Conseil fédéral introduit des mesures d'allégement dans l'ordonnance : combien de millions de francs d’exonérations cela représentera-t-il pour la branche&amp;amp;amp;nbsp;?&amp;amp;lt;br&amp;amp;gt;&amp;amp;amp;nbsp;&amp;amp;lt;/li&amp;amp;gt;&amp;amp;lt;li&amp;amp;gt;Si le Conseil fédéral introduit des mesures d'allégement dans l'ordonnance : comment sera-t-il possible, d’après lui, d’atteindre les valeurs cibles prévues par la loi&amp;amp;amp;nbsp;?&amp;amp;lt;/li&amp;amp;gt;&amp;amp;lt;/ol&amp;amp;gt;</t>
@@ -2163,10 +2163,10 @@
     <t xml:space="preserve">2025-03-11</t>
   </si>
   <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;Nimmt der Bundesrat die Finanzkontrolle ernst? </t>
-  </si>
-  <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;Le Conseil fédéral prend-il au sérieux le Contrôle fédéral des finances ? </t>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;Nimmt der Bundesrat die Finanzkontrolle ernst? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;Le Conseil fédéral prend-il au sérieux le Contrôle fédéral des finances ? </t>
   </si>
   <si>
     <t xml:space="preserve">&amp;amp;lt;p&amp;amp;gt;L'élaboration de l'ordonnance sur le CO2 revêt une grande importance pour la réalisation des objectifs légaux en matière d'émissions, en particulier les dispositions d'exécution pour les voitures de tourisme.&amp;amp;lt;br&amp;amp;gt;Le Contrôle fédéral des finances a évalué l'efficacité des sanctions en matière de CO2 pour les voitures de tourisme neuves&amp;amp;amp;nbsp;: il est clair pour lui qu'il faut renoncer à des mesures d'allègement si les objectifs ne sont pas atteints.&amp;amp;lt;br&amp;amp;gt;Le Conseil fédéral partage-t-il l'avis du Contrôle fédéral des finances&amp;amp;amp;nbsp;? Dans la négative, pour quelles raisons&amp;amp;amp;nbsp;?&amp;amp;lt;/p&amp;amp;gt;</t>
@@ -2262,10 +2262,10 @@
     <t xml:space="preserve">25.7129</t>
   </si>
   <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;Ist der Kaufpreis für die F-35 fix? </t>
-  </si>
-  <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;Le prix d’achat des F-35, est-il fixe ? </t>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;Ist der Kaufpreis für die F-35 fix? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;Le prix d’achat des F-35, est-il fixe ? </t>
   </si>
   <si>
     <t xml:space="preserve">&amp;amp;lt;p&amp;amp;gt;Selon les informations régulièrement transmises par le DDPS, les Etats-Unis se sont engagés à fournir les 36 F-35 acquis par la Suisse à un prix d’achat fixe. Mais selon un avis du Contrôle fédéral des finances émis le 8 juillet 2022, il n’existe aucune garantie juridique à ce sujet.&amp;amp;lt;br&amp;amp;gt;A notre connaissance, cette dernière information n’a jamais été démentie par le Conseil fédéral.&amp;amp;lt;br&amp;amp;gt;Le Conseil fédéral la confirme-t-il ?&amp;amp;lt;/p&amp;amp;gt;</t>
@@ -2397,13 +2397,13 @@
     <t xml:space="preserve">2025-01-21</t>
   </si>
   <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;Schweizer Depotbank für die Ausgleichfonds von AHV, IV und EO </t>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;Schweizer Depotbank für die Ausgleichfonds von AHV, IV und EO </t>
   </si>
   <si>
     <t xml:space="preserve">Banque dépositaire pour les fonds de compensation AVS/AI/APG</t>
   </si>
   <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;Banca depositaria svizzera per i fondi di compensazione AVS, AI e IPG </t>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;Banca depositaria svizzera per i fondi di compensazione AVS, AI e IPG </t>
   </si>
   <si>
     <t xml:space="preserve">&amp;amp;lt;p&amp;amp;gt;Les fonds de compensation AVS/AI/APG sont responsables de la gestion des liquidités et de la fortune de ces trois assurances. En décembre&amp;amp;amp;nbsp;2023, le conseil d’administration de Compenswiss, l’autorité compétente, a décidé de confier le mandat de banque dépositaire, qui était alors assumé par UBS, à un établissement bancaire américain, la State Street Bank International GmbH. Le transfert à la nouvelle banque dépositaire a eu lieu fin juillet&amp;amp;amp;nbsp;2024.&amp;amp;lt;/p&amp;amp;gt;&amp;amp;lt;p&amp;amp;gt;Le Conseil fédéral est chargé d’encourager Compenswiss à résilier le mandat confié à la State Street Bank International GmbH pour le remettre à une banque suisse. Si, pour des raisons juridiques, cela n’est pas possible, le Conseil fédéral est chargé de créer les conditions légales nécessaires.&amp;amp;lt;/p&amp;amp;gt;&amp;amp;lt;p&amp;amp;gt;Une minorité (Bertschy, Grossen Jürg, Roth David, Ryser, Walti Beat, Wermuth, Widmer Céline) propose de rejeter la motion.&amp;amp;lt;/p&amp;amp;gt;</t>
@@ -2499,10 +2499,10 @@
     <t xml:space="preserve">2024-12-11</t>
   </si>
   <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;ETH-Top vs. ETH-Baumanagement-Flop </t>
-  </si>
-  <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;EPFZ. Un top et un flop </t>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;ETH-Top vs. ETH-Baumanagement-Flop </t>
+  </si>
+  <si>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;EPFZ. Un top et un flop </t>
   </si>
   <si>
     <t xml:space="preserve">&amp;amp;lt;p&amp;amp;gt;Top&amp;amp;amp;nbsp;: 7e place dans le classement mondial des universités 2025. Flop&amp;amp;amp;nbsp;: l’EPFZ comme maître d’ouvrage. 2019&amp;amp;amp;nbsp;: rapport du CDF à propos du projet BSS (Bâle)&amp;amp;amp;nbsp;: «&amp;amp;amp;nbsp;la direction du projet BSS n’a pas mis en œuvre de processus valables pour la gestion du changement&amp;amp;amp;nbsp;»&amp;amp;amp;nbsp;; «&amp;amp;amp;nbsp;il n’existe pas d’instruments continus pour le pilotage financier de l’ensemble du projet ». 2023-2024&amp;amp;amp;nbsp;: projet GLC (Zurich)&amp;amp;amp;nbsp;: une centaine de PME et d’entreprises générales attendent encore le versement de plusieurs millions de francs. L’EPFZ refuse de donner suite aux demandes d’entretien des entreprises générales en vue de résoudre le problème.&amp;amp;lt;br&amp;amp;gt;Que fait le Conseil fédéral pour protéger les entreprises concernées et la réputation de l’EPFZ&amp;amp;amp;nbsp;?&amp;amp;lt;/p&amp;amp;gt;</t>
@@ -3408,10 +3408,10 @@
     <t xml:space="preserve">2024-02-26</t>
   </si>
   <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;Unterstellung von Organisationen ausserhalb der Bundesverwaltung unter die Aufsicht durch die Eidgenössische Finanzkontrolle. Wann wird der Bundesrat seinen Bericht veröffentlichen? </t>
-  </si>
-  <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;Assujettissement des organisations externes à l’administration au Contrôle fédéral des finances. Quand le Conseil fédéral publiera-t-il son rapport ? </t>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;Unterstellung von Organisationen ausserhalb der Bundesverwaltung unter die Aufsicht durch die Eidgenössische Finanzkontrolle. Wann wird der Bundesrat seinen Bericht veröffentlichen? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;Assujettissement des organisations externes à l’administration au Contrôle fédéral des finances. Quand le Conseil fédéral publiera-t-il son rapport ? </t>
   </si>
   <si>
     <t xml:space="preserve">&amp;amp;lt;p&amp;amp;gt;Le postulat 15.4112 intitulé «&amp;amp;amp;nbsp;Examen des critères selon lesquels les organisations externes à l’administration doivent être soumises à la surveillance du Contrôle fédéral des finances&amp;amp;amp;nbsp;» a été accepté par le Conseil national le 18 mars 2016. En réponse à la question 19.5385, le Conseil fédéral a indiqué que le rapport demandé par le postulat serait publié à la fin de l’année 2019. Pour l’heure, le rapport n’a pas encore été publié.&amp;amp;lt;br&amp;amp;gt;Quand le sera-t-il&amp;amp;amp;nbsp;?&amp;amp;amp;nbsp;&amp;amp;lt;/p&amp;amp;gt;</t>
@@ -3594,7 +3594,7 @@
     <t xml:space="preserve">Fonds pour la démocratie et l'état de droit en commémoration de 1848</t>
   </si>
   <si>
-    <t xml:space="preserve">xml:space="preserve"&amp;gt; Fondo per la democrazia e lo Stato di diritto in commemorazione del 1848</t>
+    <t xml:space="preserve">xml:space="preserve"&gt; Fondo per la democrazia e lo Stato di diritto in commemorazione del 1848</t>
   </si>
   <si>
     <t xml:space="preserve">&amp;amp;lt;p&amp;amp;gt;Le Conseil fédéral est invité à élaborer les bases légales pour le financement d’un fonds pour la démocratie et l’État de droit. Ce fonds doit, d’une part, soutenir des activités pouvant renforcer la compréhension et l’engagement pour les institutions politiques de l’État fédéral suisse, en particulier chez les jeunes. D’autre part, afin de renforcer la cohésion de la Suisse, le fonds doit encourager la connaissance et la pratique des langues nationales.&amp;amp;lt;/p&amp;amp;gt;&amp;amp;lt;p&amp;amp;gt;&amp;amp;amp;nbsp;&amp;amp;lt;/p&amp;amp;gt;&amp;amp;lt;p&amp;amp;gt;Le fonds doit être géré par un comité indépendant du Parlement et de l’administration, composé de cinq à neuf personnes au maximum, nommées par le Conseil fédéral pour une durée de quatre ans et rééligibles deux fois au maximum. Les comptes annuels doivent être soumis au Contrôle fédéral des finances pour révision.&amp;amp;lt;/p&amp;amp;gt;</t>
@@ -3630,7 +3630,7 @@
     <t xml:space="preserve">Une manifestation en faveur du pouvoir d'achat doit-elle être considérée comme une manifestation électorale?</t>
   </si>
   <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;Una manifestazione a favore del potere d'acquisto è una manifestazione elettorale o no? </t>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;Una manifestazione a favore del potere d'acquisto è una manifestazione elettorale o no? </t>
   </si>
   <si>
     <t xml:space="preserve">&amp;amp;lt;p&amp;amp;gt;Dans le « Tagesanzeiger » du 22 septembre 2023, le directeur du Contrôle fédéral des finances, Pascal Stirnimann, a affirmé, à propos d’une manifestation en faveur du pouvoir d’achat qui a été organisée par l’Union syndicale suisse (USS) et à laquelle participaient des parlementaires fédéraux socialistes et verts, que si, lors d’une grande manifestation, dix candidats d’un même parti scandaient leurs slogans électoraux, mais que les organisateurs de la manifestation affirmaient néanmoins qu’il ne s’agissait pas d’une campagne électorale, le CDF allait examiner la chose de près.&amp;amp;lt;/p&amp;amp;gt;&amp;amp;lt;p&amp;amp;gt;Dans ce contexte, je prie le Conseil fédéral de répondre aux questions suivantes&amp;amp;amp;nbsp;:&amp;amp;amp;nbsp;&amp;amp;lt;/p&amp;amp;gt;&amp;amp;lt;ol&amp;amp;gt;&amp;amp;lt;li&amp;amp;gt;A-t-on, après la manifestation sur le pouvoir d’achat organisée par les syndicats, ouvert une enquête pour déterminer si la loi sur le financement de la vie politique avait été violée&amp;amp;amp;nbsp;?&amp;amp;lt;br&amp;amp;gt;a. Dans l’affirmative, pourquoi&amp;amp;amp;nbsp;?&amp;amp;lt;br&amp;amp;gt;b. Dans la négative, pourquoi&amp;amp;amp;nbsp;?&amp;amp;lt;/li&amp;amp;gt;&amp;amp;lt;li&amp;amp;gt;Dans le cas où une enquête a été ouverte, quand disposera-t-on, selon le Conseil fédéral, des premiers résultats&amp;amp;amp;nbsp;?&amp;amp;lt;/li&amp;amp;gt;&amp;amp;lt;li&amp;amp;gt;Selon lui, une manifestation disposant d’un budget de 150&amp;amp;amp;nbsp;000&amp;amp;amp;nbsp;francs (comme ce fut le cas pour la manifestation en faveur du pouvoir d’achat) doit-elle faire l’objet d’une déclaration conformément à la loi sur le financement de la vie politique&amp;amp;amp;nbsp;?&amp;amp;amp;nbsp;&amp;amp;lt;br&amp;amp;gt;a. Dans l’affirmative, pourquoi&amp;amp;amp;nbsp;?&amp;amp;lt;br&amp;amp;gt;b. Dans la négative, pourquoi&amp;amp;amp;nbsp;?&amp;amp;amp;nbsp;&amp;amp;amp;nbsp;&amp;amp;lt;/li&amp;amp;gt;&amp;amp;lt;li&amp;amp;gt;Le Conseil fédéral approuve-t-il l’affirmation de Pascal Stirnimann selon laquelle toute personne qui dépense, en vue d’influer sur une élection, des montants dépassant les plafonds fixés par la loi est tenue de les déclarer&amp;amp;amp;nbsp;?&amp;amp;lt;/li&amp;amp;gt;&amp;amp;lt;li&amp;amp;gt;Où se situe, pour le Conseil fédéral, la limite entre une manifestation ne visant pas à influer sur une élection et une manifestation visant une telle fin&amp;amp;amp;nbsp;?&amp;amp;lt;/li&amp;amp;gt;&amp;amp;lt;li&amp;amp;gt;Que pense-t-il de l’argument avancé par le porte-parole de l’USS selon lequel ladite manifestation portait sur les négociations salariales, qu’elle ne constituait pas une manifestation électorale au sens de la loi et qu’elle ne devait, par conséquent, pas faire l’objet d’une déclaration&amp;amp;amp;nbsp;?&amp;amp;amp;nbsp;&amp;amp;lt;/li&amp;amp;gt;&amp;amp;lt;li&amp;amp;gt;Est-il d’avis que toutes les manifestations susceptibles d’être considérées comme des manifestations électorales en raison de leur rayonnement ou du sujet sur lequel elles portent sont soumises à la loi sur le financement de la vie politique&amp;amp;amp;nbsp;?&amp;amp;lt;/li&amp;amp;gt;&amp;amp;lt;/ol&amp;amp;gt;</t>
@@ -4254,7 +4254,7 @@
     <t xml:space="preserve">Die Schweizerische Radio- und Fernsehgesellschaft der Eidgenössischen Finanzkontrolle unterstellen</t>
   </si>
   <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;Soumettre la Société suisse de radiodiffusion et télévision au Contrôle fédéral des finances </t>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;Soumettre la Société suisse de radiodiffusion et télévision au Contrôle fédéral des finances </t>
   </si>
   <si>
     <t xml:space="preserve">Società svizzera di radiotelevisione da sottoporre al Controllo federale delle finanze</t>
@@ -7572,10 +7572,10 @@
     <t xml:space="preserve">25.8273</t>
   </si>
   <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;Kostendeckende Erträge aus dem Artenschutz? </t>
-  </si>
-  <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;Des revenus couvrant les coûts liés à la protection des espèces ? </t>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;Kostendeckende Erträge aus dem Artenschutz? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;Des revenus couvrant les coûts liés à la protection des espèces ? </t>
   </si>
   <si>
     <t xml:space="preserve">&amp;amp;lt;p&amp;amp;gt;Chaque année, la Suisse délivre environ 100&amp;amp;amp;nbsp;000 autorisations pour le commerce d'espèces végétales et animales menacées et effectue quelque 20&amp;amp;amp;nbsp;000 contrôles à l'importation. Elle perçoit à cet effet des émoluments d'environ 4&amp;amp;amp;nbsp;millions de francs. Selon le CDF, ces émoluments ne couvriraient pas les coûts et constitueraient donc une subvention dommageable à la biodiversité.&amp;amp;lt;br&amp;amp;gt;Compte tenu des débats en cours concernant le budget,&amp;amp;lt;br&amp;amp;gt;le Conseil fédéral est-il prêt à introduire des émoluments couvrant les coûts dans ce domaine&amp;amp;amp;nbsp;?&amp;amp;lt;br&amp;amp;gt;Si oui, quand&amp;amp;amp;nbsp;?&amp;amp;lt;br&amp;amp;gt;Si non, pourquoi&amp;amp;amp;nbsp;?&amp;amp;lt;/p&amp;amp;gt;</t>
@@ -7740,10 +7740,10 @@
     <t xml:space="preserve">25.4225</t>
   </si>
   <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;Giftiger Rasen. Warum sind toxische PFAS-Pestizide ausgerechnet zur Anwendung auf Spiel- und Sportplätzen oder in Wohnquartieren zugelassen? </t>
-  </si>
-  <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;Gazon toxique. Pourquoi les pesticides PFAS sont-ils autorisés sur les terrains de jeux et de sport ainsi que dans les quartiers résidentiels ? </t>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;Giftiger Rasen. Warum sind toxische PFAS-Pestizide ausgerechnet zur Anwendung auf Spiel- und Sportplätzen oder in Wohnquartieren zugelassen? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;Gazon toxique. Pourquoi les pesticides PFAS sont-ils autorisés sur les terrains de jeux et de sport ainsi que dans les quartiers résidentiels ? </t>
   </si>
   <si>
     <t xml:space="preserve">Superfici erbose inquinate. Perché i pesticidi tossici contenenti PFAS sono omologati per l'uso sui campi sportivi e da gioco e nei quartieri residenziali?</t>
@@ -7926,10 +7926,10 @@
     <t xml:space="preserve">25.789</t>
   </si>
   <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;Rolle des Bundes bei der Sanierung der Deponie Gamsenried </t>
-  </si>
-  <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;Rôle de la Confédération dans l’assainissement de la décharge de Gamsenried </t>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;Rolle des Bundes bei der Sanierung der Deponie Gamsenried </t>
+  </si>
+  <si>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;Rôle de la Confédération dans l’assainissement de la décharge de Gamsenried </t>
   </si>
   <si>
     <t xml:space="preserve">&amp;amp;lt;p&amp;amp;gt;Concernant le suivi de l’assainissement de cette décharge, le Contrôle fédéral des finances (CDF) souligne «&amp;amp;amp;nbsp;l’absence d’une vision d’ensemble des risques et d’un suivi coordonné des différentes entités fédérales&amp;amp;amp;nbsp;».&amp;amp;lt;br&amp;amp;gt;- Comment le Conseil fédéral réagit-il aux critiques du CDF?&amp;amp;lt;br&amp;amp;gt;- Entend-il réaliser une analyse globale des risques, en tenant compte des interfaces avec l'A9 et la correction du Rhône puis, sur cette base, établir un concept de surveillance avec des responsabilités clairement définies?&amp;amp;lt;/p&amp;amp;gt;</t>
@@ -11430,10 +11430,10 @@
     <t xml:space="preserve">Sottoporre la SUVA alla vigilanza finanziaria del Controllo federale delle finanze</t>
   </si>
   <si>
-    <t xml:space="preserve">&amp;lt;p&amp;gt;Le Conseil fédéral est chargé de proposer aux Chambres fédérales d'abroger l'article 1, alinéa , lettera , de la loi sur le Contrôle des finances (LCF ; RS 614.0) lorsqu'elles procéderont à la prochaine révision de la loi en question.&amp;lt;/p&amp;gt;&amp;lt;p&amp;gt;Une minorité (Gasche, Gilli, Gmür, Gössi, Gschwind, Kiener Nellen, Müller Leo, Schneeberger, Siegenthaler, Vischer Daniel) propose le rejet de la motion.&amp;lt;/p&amp;gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&amp;lt;p&amp;gt;Der Bundesrat wird beauftragt, der Bundesversammlung im Rahmen der nächsten Revision des Finanzkontrollgesetzes (FKG; SR 614.0) die ersatzlose Streichung von Artikel 19 Absatz 1 Buchstabe b vorzulegen.&amp;lt;/p&amp;gt;&amp;lt;p&amp;gt;Eine Minderheit (Gasche, Gilli, Gmür, Gössi, Gschwind, Kiener Nellen, Müller Leo, Schneeberger, Siegenthaler, Vischer Daniel) beantragt die Ablehnung der Motion.&amp;lt;/p&amp;gt;</t>
+    <t xml:space="preserve">&lt;p&gt;Le Conseil fédéral est chargé de proposer aux Chambres fédérales d'abroger l'article 1, alinéa , lettera , de la loi sur le Contrôle des finances (LCF ; RS 614.0) lorsqu'elles procéderont à la prochaine révision de la loi en question.&lt;/p&gt;&lt;p&gt;Une minorité (Gasche, Gilli, Gmür, Gössi, Gschwind, Kiener Nellen, Müller Leo, Schneeberger, Siegenthaler, Vischer Daniel) propose le rejet de la motion.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Der Bundesrat wird beauftragt, der Bundesversammlung im Rahmen der nächsten Revision des Finanzkontrollgesetzes (FKG; SR 614.0) die ersatzlose Streichung von Artikel 19 Absatz 1 Buchstabe b vorzulegen.&lt;/p&gt;&lt;p&gt;Eine Minderheit (Gasche, Gilli, Gmür, Gössi, Gschwind, Kiener Nellen, Müller Leo, Schneeberger, Siegenthaler, Vischer Daniel) beantragt die Ablehnung der Motion.&lt;/p&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20153828</t>
@@ -11472,10 +11472,10 @@
     <t xml:space="preserve">Bloccare l'effettivo del personale della Confederazione al livello del 2015</t>
   </si>
   <si>
-    <t xml:space="preserve">&amp;lt;p&amp;gt;Le Conseil fédéral est chargé de prendre des mesures afin que les effectifs de la Confédération ne dépassent pas le nombre fixé dans le budget 2015 (à savoir 35 000 équivalents plein temps).&amp;lt;/p&amp;gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&amp;lt;p&amp;gt;Der Bundesrat wird beauftragt, Massnahmen zu ergreifen mit dem Ziel, dass der Bundespersonalbestand den Stand gemäss Voranschlag 2015 (35 000 FTE) nicht überschreitet.&amp;lt;/p&amp;gt;</t>
+    <t xml:space="preserve">&lt;p&gt;Le Conseil fédéral est chargé de prendre des mesures afin que les effectifs de la Confédération ne dépassent pas le nombre fixé dans le budget 2015 (à savoir 35 000 équivalents plein temps).&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Der Bundesrat wird beauftragt, Massnahmen zu ergreifen mit dem Ziel, dass der Bundespersonalbestand den Stand gemäss Voranschlag 2015 (35 000 FTE) nicht überschreitet.&lt;/p&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20153494</t>

</xml_diff>

<commit_message>
Update parliament data - 2026-07-06
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_CDF_EFK.xlsx
+++ b/Objets_parlementaires_CDF_EFK.xlsx
@@ -257,10 +257,10 @@
     <t xml:space="preserve">Titel folgt</t>
   </si>
   <si>
-    <t xml:space="preserve">Réintroduction de l’obligation de visas pour les Géorgiens </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reintrodurre l’obbligo del visto per i Georgiani</t>
+    <t xml:space="preserve">Réintroduction de l'obligation de visas pour les Géorgiens </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reintrodurre l'obbligo del visto per i Georgiani</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Le Conseil fédéral est chargé d’intervenir auprès de l’Union européenne afin de demander la réintroduction de l’obligation de visas pour les ressortissants géorgiens. Cette mesure vise à enrayer le tourisme médical qui n’a pas tari.&lt;/p&gt;</t>

</xml_diff>

<commit_message>
Update parliament data - 2026-07-10
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_CDF_EFK.xlsx
+++ b/Objets_parlementaires_CDF_EFK.xlsx
@@ -104,7 +104,7 @@
     <t xml:space="preserve">UVEK</t>
   </si>
   <si>
-    <t xml:space="preserve">Gotthard-Eisenbahnachse: Plant der Bundesrat, die bei der Ausarbeitung der Botschaft 2027 aufgetretenen Mängel zu beheben?</t>
+    <t xml:space="preserve">Gotthard-Eisenbahnachse. Plant der Bundesrat, die bei der Ausarbeitung der Botschaft 2027 aufgetretenen Mängel zu beheben?</t>
   </si>
   <si>
     <t xml:space="preserve">Axe ferroviaire du Saint-Gothard. Le Conseil fédéral a-t-il l'intention de remédier aux lacunes constatées lors de la préparation du message 2027 ?</t>
@@ -248,7 +248,7 @@
     <t xml:space="preserve">Titre suit</t>
   </si>
   <si>
-    <t xml:space="preserve">Attuazione coerente dell’Agenda 2030 nelle politiche settoriali</t>
+    <t xml:space="preserve">Attuazione coerente dell'Agenda 2030 nelle politiche settoriali</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Der Bundesrat wird beauftragt, Massnahmen zu ergreifen, um eine umfassende, kohärente und wirkungsvolle Umsetzung der Agenda 2030 in den Sektoralpolitiken sicherzustellen:&amp;nbsp;&lt;/p&gt;&lt;ol style="list-style-type:decimal;"&gt;&lt;li&gt;Auf Basis des Länderberichts (Voluntary National Review) 2026 ist eine gezielte Analyse der notwendigen Massnahmen vorzunehmen, um die festgestellten Lücken zu schliessen.&amp;nbsp;&lt;/li&gt;&lt;li&gt;Der Bundesrat muss sicherstellen, dass das Direktionskomitee Agenda 2030 seine koordinierende und steuernde Rolle wahrnimmt und die Agenda 2030 kohärent in die Sektoralpolitiken übersetzt.&amp;nbsp;&lt;/li&gt;&lt;li&gt;Der Bundesrat muss dem Parlament in regelmässigen Abständen über die zusätzlichen Massnahmen berichten.&amp;nbsp;&lt;/li&gt;&lt;/ol&gt;</t>

</xml_diff>

<commit_message>
Update parliament data - 2026-08-13
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_CDF_EFK.xlsx
+++ b/Objets_parlementaires_CDF_EFK.xlsx
@@ -12025,9 +12025,7 @@
       <c r="R2" t="s">
         <v>39</v>
       </c>
-      <c r="S2" t="s">
-        <v>39</v>
-      </c>
+      <c r="S2"/>
       <c r="T2" t="s">
         <v>40</v>
       </c>

</xml_diff>